<commit_message>
Outputs RAG 14B final
</commit_message>
<xml_diff>
--- a/results/manual_eval_qwen14B_rag_validation.xlsx
+++ b/results/manual_eval_qwen14B_rag_validation.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H201"/>
+  <dimension ref="A1:E201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -440,21 +440,6 @@
       <c r="E1" t="inlineStr">
         <is>
           <t>retrieved_ctx</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>topk_idx</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>topk_scores</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>topk_chunks</t>
         </is>
       </c>
     </row>
@@ -501,21 +486,6 @@
 2 mixtures only if they are breathed during aerobic exercise.</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>[10, 0, 86, 710, 472]</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>[0.8685173988342285, 0.8574632406234741, 0.8220016956329346, 0.8164328336715698, 0.8055824041366577]</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>["Uptake of O\n2 from the air is the essential purpose of respiration, so oxygen supplementation is used in medicine. Treatment not only increases oxygen levels in the patient's blood, but has the secondary effect of decreasing resistance to blood flow in many types of diseased lungs, easing work load on the heart. Oxygen therapy is used to treat emphysema, pneumonia, some heart disorders (congestive heart failure), some disorders that cause increased pulmonary artery pressure, and any disease that impairs the body's ability to take up and use gaseous oxygen.", "Hyperbaric (high-pressure) medicine uses special oxygen chambers to increase the partial pressure of O\n2 around the patient and, when needed, the medical staff. Carbon monoxide poisoning, gas gangrene, and decompression sickness (the 'bends') are sometimes treated using these devices. Increased O\n2 concentration in the lungs helps to displace carbon monoxide from the heme group of hemoglobin. Oxygen gas is poisonous to the anaerobic bacteria that cause gas gangrene, so increasing its partial pressure helps kill them. Decompression sickness occurs in divers who decompress too quickly after a dive, resulting in bubbles of inert gas, mostly nitrogen and helium, forming in their blood. Increasing the pressure of O\n2 as soon as possible is part of the treatment.", "Oxygen toxicity to the lungs and central nervous system can also occur in deep scuba diving and surface supplied diving. Prolonged breathing of an air mixture with an O\n2 partial pressure more than 60 kPa can eventually lead to permanent pulmonary fibrosis. Exposure to a O\n2 partial pressures greater than 160 kPa (about 1.6 atm) may lead to convulsions (normally fatal for divers). Acute oxygen toxicity (causing seizures, its most feared effect for divers) can occur by breathing an air mixture with 21% O\n2 at 66 m or more of depth; the same thing can occur by breathing 100% O\n2 at only 6 m.", "Oxygen gas (O\n2) can be toxic at elevated partial pressures, leading to convulsions and other health problems.[j] Oxygen toxicity usually begins to occur at partial pressures more than 50 kilopascals (kPa), equal to about 50% oxygen composition at standard pressure or 2.5 times the normal sea-level O\n2 partial pressure of about 21 kPa. This is not a problem except for patients on mechanical ventilators, since gas supplied through oxygen masks in medical applications is typically composed of only 30%–50% O\n2 by volume (about 30 kPa at standard pressure). (although this figure also is subject to wide variation, depending on type of mask).", "Oxygen, as a supposed mild euphoric, has a history of recreational use in oxygen bars and in sports. Oxygen bars are establishments, found in Japan, California, and Las Vegas, Nevada since the late 1990s that offer higher than normal O\n2 exposure for a fee. Professional athletes, especially in American football, also sometimes go off field between plays to wear oxygen masks in order to get a \"boost\" in performance. The pharmacological effect is doubtful; a placebo effect is a more likely explanation. Available studies support a performance boost from enriched O\n2 mixtures only if they are breathed during aerobic exercise."]</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -547,21 +517,6 @@
 BSkyB has no veto over the presence of channels on their EPG, with open access being an enforced part of their operating licence from Ofcom. Any channel which can get carriage on a suitable beam of a satellite at 28° East is entitled to access to BSkyB's EPG for a fee, ranging from £15–100,000. Third-party channels which opt for encryption receive discounts ranging from reduced price to free EPG entries, free carriage on a BSkyB leased transponder, or actual payment for being carried. However, even in this case, BSkyB does not carry any control over the channel's content or carriage issues such as picture quality.</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>[1, 658, 541, 624, 421]</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>[0.7888264060020447, 0.7863542437553406, 0.7717632055282593, 0.7635020613670349, 0.7415463328361511]</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>["The agreements include fixed annual carriage fees of £30m for the channels with both channel suppliers able to secure additional capped payments if their channels meet certain performance-related targets. Currently there is no indication as to whether the new deal includes the additional Video On Demand and High Definition content which had previously been offered by BSkyB. As part of the agreements, both BSkyB and Virgin Media agreed to terminate all High Court proceedings against each other relating to the carriage of their respective basic channels.", "Provided is a universal Ku band LNB (9.75/10.600 GHz) which is fitted at the end of the dish and pointed at the correct satellite constellation; most digital receivers will receive the free to air channels. Some broadcasts are free-to-air and unencrypted, some are encrypted but do not require a monthly subscription (known as free-to-view), some are encrypted and require a monthly subscription, and some are pay-per-view services. To view the encrypted content a VideoGuard UK equipped receiver (all of which are dedicated to the Sky service, and cannot be used to decrypt other services) needs to be used. Unofficial CAMs are now available to view the service, although use of them breaks the user's contract with Sky and invalidates the user's rights to use the card.", "The service started on 1 September 1993 based on the idea from the then chief executive officer, Sam Chisholm and Rupert Murdoch, of converting the company business strategy to an entirely fee-based concept. The new package included four channels formerly available free-to-air, broadcasting on Astra's satellites, as well as introducing new channels. The service continued until the closure of BSkyB's analogue service on 27 September 2001, due to the launch and expansion of the Sky Digital platform. Some of the channels did broadcast either in the clear or soft encrypted (whereby a Videocrypt decoder was required to decode, without a subscription card) prior to their addition to the Sky Multichannels package. Within two months of the launch, BSkyB gained 400,000 new subscribers, with the majority taking at least one premium channel as well, which helped BSkyB reach 3.5 million households by mid-1994. Michael Grade criticized the operations in front of the Select Committee on National Heritage, mainly for the lack of original programming on many of the new channels.", "BSkyB utilises the VideoGuard pay-TV scrambling system owned by NDS, a Cisco Systems company. There are tight controls over use of VideoGuard decoders; they are not available as stand-alone DVB CAMs (conditional-access modules). BSkyB has design authority over all digital satellite receivers capable of receiving their service. The receivers, though designed and built by different manufacturers, must conform to the same user interface look-and-feel as all the others. This extends to the Personal video recorder (PVR) offering (branded Sky+).", "BSkyB has no veto over the presence of channels on their EPG, with open access being an enforced part of their operating licence from Ofcom. Any channel which can get carriage on a suitable beam of a satellite at 28° East is entitled to access to BSkyB's EPG for a fee, ranging from £15–100,000. Third-party channels which opt for encryption receive discounts ranging from reduced price to free EPG entries, free carriage on a BSkyB leased transponder, or actual payment for being carried. However, even in this case, BSkyB does not carry any control over the channel's content or carriage issues such as picture quality."]</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -593,21 +548,6 @@
 As a result, by 1206 Temüjin had managed to unite or subdue the Merkits, Naimans, Mongols, Keraites, Tatars, Uyghurs, and other disparate smaller tribes under his rule. It was a monumental feat for the "Mongols" (as they became known collectively). At a Khuruldai, a council of Mongol chiefs, Temüjin was acknowledged as "Khan" of the consolidated tribes and took the new title "Genghis Khan". The title Khagan was not conferred on Genghis until after his death, when his son and successor, Ögedei, took the title for himself and extended it posthumously to his father (as he was also to be posthumously declared the founder of the Yuan dynasty). This unification of all confederations by Genghis Khan established peace between previously warring tribes and a single political and military force under Genghis Khan.</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>[803, 2, 569, 494, 668]</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>[0.8382490277290344, 0.8376836776733398, 0.8305801749229431, 0.8218026161193848, 0.8172245025634766]</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>["After the defeat of the Khwarezmian Empire in 1220, Genghis Khan gathered his forces in Persia and Armenia to return to the Mongolian steppes. Under the suggestion of Subutai, the Mongol army was split into two forces. Genghis Khan led the main army on a raid through Afghanistan and northern India towards Mongolia, while another 20,000 (two tumen) contingent marched through the Caucasus and into Russia under generals Jebe and Subutai. They pushed deep into Armenia and Azerbaijan. The Mongols destroyed the kingdom of Georgia, sacked the Genoese trade-fortress of Caffa in Crimea and overwintered near the Black Sea. Heading home, Subutai's forces attacked the allied forces of the Cuman–Kipchaks and the poorly coordinated 80,000 Kievan Rus' troops led by Mstislav the Bold of Halych and Mstislav III of Kiev who went out to stop the Mongols' actions in the area. Subutai sent emissaries to the Slavic princes calling for a separate peace, but the emissaries were executed. At the Battle of Kalka River in 1223, Subutai's forces defeated the larger Kievan force. They also may have fought against the neighboring Volga Bulgars. There is no historical record except a short account by the Arab historian Ibn al-Athir, writing in", "The invasions of Baghdad, Samarkand, Urgench, Kiev, Vladimir among others caused mass murders, such as when portions of southern Khuzestan were completely destroyed. His descendant Hulagu Khan destroyed much of Iran's northern part and sacked Baghdad although his forces were halted by the Mamluks of Egypt, but Hulagu's descendant Ghazan Khan would return to beat the Egyptian Mamluks right out of Levant, Palestine and even Gaza. According to the works of the Persian historian Rashid-al-Din Hamadani, the Mongols killed more than 70,000 people in Merv and more than 190,000 in Nishapur. In 1237 Batu Khan, a grandson of Genghis Khan, launched an invasion into Kievan Rus'. Over the course of three years, the Mongols destroyed and annihilated all of the major cities of Eastern Europe with the exceptions of Novgorod and Pskov.", "Genghis Khan united the Mongol and Turkic tribes of the steppes and became Great Khan in 1206. He and his successors expanded the Mongol empire across Asia. Under the reign of Genghis' third son, Ögedei Khan, the Mongols destroyed the weakened Jin dynasty in 1234, conquering most of northern China. Ögedei offered his nephew Kublai a position in Xingzhou, Hebei. Kublai was unable to read Chinese but had several Han Chinese teachers attached to him since his early years by his mother Sorghaghtani. He sought the counsel of Chinese Buddhist and Confucian advisers. Möngke Khan succeeded Ögedei's son, Güyük, as Great Khan in 1251. He granted his brother Kublai control over Mongol held territories in China. Kublai built schools for Confucian scholars, issued paper money, revived Chinese rituals, and endorsed policies that stimulated agricultural and commercial growth. He adopted as his capital city Kaiping in Inner Mongolia, later renamed Shangdu.", "With such a small force, the invading Mongols were forced to change strategies and resort to inciting internal revolt among Kuchlug's supporters, leaving the Qara Khitai more vulnerable to Mongol conquest. As a result, Kuchlug's army was defeated west of Kashgar. Kuchlug fled again, but was soon hunted down by Jebe's army and executed. By 1218, as a result of defeat of Qara Khitai, the Mongol Empire and its control extended as far west as Lake Balkhash, which bordered the Khwarezmia (Khwarezmid Empire), a Muslim state that reached the Caspian Sea to the west and Persian Gulf and the Arabian Sea to the south.", "As a result, by 1206 Temüjin had managed to unite or subdue the Merkits, Naimans, Mongols, Keraites, Tatars, Uyghurs, and other disparate smaller tribes under his rule. It was a monumental feat for the \"Mongols\" (as they became known collectively). At a Khuruldai, a council of Mongol chiefs, Temüjin was acknowledged as \"Khan\" of the consolidated tribes and took the new title \"Genghis Khan\". The title Khagan was not conferred on Genghis until after his death, when his son and successor, Ögedei, took the title for himself and extended it posthumously to his father (as he was also to be posthumously declared the founder of the Yuan dynasty). This unification of all confederations by Genghis Khan established peace between previously warring tribes and a single political and military force under Genghis Khan."]</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -639,21 +579,6 @@
 The popular neighborhood known as the Tower District is centered around the historic Tower Theatre, which is included on the National List of Historic Places. The theater was built in 1939 and is at Olive and Wishon Avenues in the heart of the Tower District. (The name of the theater refers to a well-known landmark water tower, which is actually in another nearby area). The Tower District neighborhood is just north of downtown Fresno proper, and one-half mile south of Fresno City College. Although the neighborhood was known as a residential area prior, the early commercial establishments of the Tower District began with small shops and services that flocked to the area shortly after World War II. The character of small local businesses largely remains today. To some extent, the businesses of the Tower District were developed due to the proximity of the original Fresno Normal School, (later renamed California State University at Fresno). In 1916 the college moved to what is now the site of Fresno City College one-half mile north of the Tower District.</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>[3, 166, 660, 717, 327]</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>[0.7375685572624207, 0.7267813086509705, 0.725538432598114, 0.6938217282295227, 0.6920809745788574]</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>["The university runs a number of academic institutions and programs apart from its undergraduate and postgraduate schools. It operates the University of Chicago Laboratory Schools (a private day school for K-12 students and day care), the Sonia Shankman Orthogenic School (a residential treatment program for those with behavioral and emotional problems), and four public charter schools on the South Side of Chicago administered by the university's Urban Education Institute. In addition, the Hyde Park Day School, a school for students with learning disabilities, maintains a location on the University of Chicago campus. Since 1983, the University of Chicago has maintained the University of Chicago School Mathematics Project, a mathematics program used in urban primary and secondary schools. The university runs a program called the Council on Advanced Studies in the Social Sciences and Humanities, which administers interdisciplinary workshops to provide a forum for graduate students, faculty, and visiting scholars to present scholarly work in progress. The university also operates the University of Chicago Press, the largest university press in the United States.", "There are eleven LEA-funded 11 to 18 schools and seven independent schools with sixth forms in Newcastle. There are a number of successful state schools, including Walker Technology College, Gosforth High School, Heaton Manor School, St Cuthbert's High School, St. Mary's Catholic Comprehensive School, Kenton School, George Stephenson High School, Sacred Heart and Benfield School. The largest co-ed independent school is the Royal Grammar School. The largest girls' independent school is Newcastle High School for Girls. Both schools are located on the same street in Jesmond. Newcastle School for Boys is the only independent boys' only school in the city and is situated in Gosforth. Newcastle College is the largest general further education college in the North East and is a beacon status college; there are two smaller colleges in the Newcastle area. St Cuthbert's High School and Sacred Heart are the two primary state-Catholic run high schools, and are both achieving results on par with the independent schools in Newcastle.", "Private schools are often Anglican, such as King's College and Diocesan School for Girls in Auckland, St Paul's Collegiate School in Hamilton, St Peter's School in Cambridge, Samuel Marsden Collegiate School in Wellington, and Christ's College and St Margaret's College in Christchurch; or Presbyterian, such as Saint Kentigern College and St Cuthbert's College in Auckland, Scots College and Queen Margaret College in Wellington, and St Andrew's College and Rangi Ruru Girls' School in Christchurch. Academic Colleges Group is a recent group of private schools run as a business, with schools throughout Auckland, including ACG Senior College in Auckland’s CBD, ACG Parnell College in Parnell, and international school ACG New Zealand International College. There are three private schools (including the secondary school, St Dominic's College) operated by the Catholic schismatic group, the Society of St Pius X in Wanganui.", "(later transferred to the Tate Gallery) and now used as the picture galleries and tapestry gallery respectively. The North and South Courts, were then built, both of which opened by June 1862. They now form the galleries for temporary exhibitions and are directly behind the Sheepshanks Gallery. On the very northern edge of the site is situated the Secretariat Wing, also built in 1862 this houses the offices and board room etc. and is not open to the public.", "The popular neighborhood known as the Tower District is centered around the historic Tower Theatre, which is included on the National List of Historic Places. The theater was built in 1939 and is at Olive and Wishon Avenues in the heart of the Tower District. (The name of the theater refers to a well-known landmark water tower, which is actually in another nearby area). The Tower District neighborhood is just north of downtown Fresno proper, and one-half mile south of Fresno City College. Although the neighborhood was known as a residential area prior, the early commercial establishments of the Tower District began with small shops and services that flocked to the area shortly after World War II. The character of small local businesses largely remains today. To some extent, the businesses of the Tower District were developed due to the proximity of the original Fresno Normal School, (later renamed California State University at Fresno). In 1916 the college moved to what is now the site of Fresno City College one-half mile north of the Tower District."]</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -685,21 +610,6 @@
 United States and Western Europe than in China (due to a greater tendency to take on debts).[unreliable source?][unreliable source?] Anthony Shorrocks, the lead author of the Credit Suisse report which is one of the sources of Oxfam's data, considers the criticism about debt to be a "silly argument" and "a non-issue . . . a diversion."</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>[4, 414, 765, 491, 827]</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>[0.8149519562721252, 0.7840211391448975, 0.7759851813316345, 0.773474395275116, 0.7363988161087036]</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>["The executive summary of the WG I Summary for Policymakers report says they are certain that emissions resulting from human activities are substantially increasing the atmospheric concentrations of the greenhouse gases, resulting on average in an additional warming of the Earth's surface. They calculate with confidence that CO2 has been responsible for over half the enhanced greenhouse effect. They predict that under a \"business as usual\" (BAU) scenario, global mean temperature will increase by about 0.3 °C per decade during the [21st] century. They judge that global mean surface air temperature has increased by 0.3 to 0.6 °C over the last 100 years, broadly consistent with prediction of climate models, but also of the same magnitude as natural climate variability. The unequivocal detection of the enhanced greenhouse effect is not likely for a decade or more.", "Michael Oppenheimer, a long-time participant in the IPCC and coordinating lead author of the Fifth Assessment Report conceded in Science Magazine's State of the Planet 2008-2009 some limitations of the IPCC consensus approach and asks for concurring, smaller assessments of special problems instead of the large scale approach as in the previous IPCC assessment reports. It has become more important to provide a broader exploration of uncertainties. Others see as well mixed blessings of the drive for consensus within the IPCC process and ask to include dissenting or minority positions or to improve statements about uncertainties.", "The IPCC process on climate change and its efficiency and success has been compared with dealings with other environmental challenges (compare Ozone depletion and global warming). In case of the Ozone depletion global regulation based on the Montreal Protocol has been successful, in case of Climate Change, the Kyoto Protocol failed. The Ozone case was used to assess the efficiency of the IPCC process. The lockstep situation of the IPCC is having built a broad science consensus while states and governments still follow different, if not opposing goals. The underlying linear model of policy-making of more knowledge we have, the better the political response will be is being doubted.", "According to Sheldon Ungar's comparison with global warming, the actors in the ozone depletion case had a better understanding of scientific ignorance and uncertainties. The ozone case communicated to lay persons \"with easy-to-understand bridging metaphors derived from the popular culture\" and related to \"immediate risks with everyday relevance\", while the public opinion on climate change sees no imminent danger. The stepwise mitigation of the ozone layer challenge was based as well on successfully reducing regional burden sharing conflicts. In case of the IPCC conclusions and the failure of the Kyoto Protocol, varying regional cost-benefit analysis and burden-sharing conflicts with regard to the distribution of emission reductions remain an unsolved problem. In the UK, a report for a House of Lords committee asked to urge the IPCC to involve better assessments of costs and benefits of climate change but the Stern Review ordered by the UK government made a stronger argument in favor to combat human-made climate change.", "United States and Western Europe than in China (due to a greater tendency to take on debts).[unreliable source?][unreliable source?] Anthony Shorrocks, the lead author of the Credit Suisse report which is one of the sources of Oxfam's data, considers the criticism about debt to be a \"silly argument\" and \"a non-issue . . . a diversion.\""]</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -731,21 +641,6 @@
 James Hutton is often viewed as the first modern geologist. In 1785 he presented a paper entitled Theory of the Earth to the Royal Society of Edinburgh. In his paper, he explained his theory that the Earth must be much older than had previously been supposed in order to allow enough time for mountains to be eroded and for sediments to form new rocks at the bottom of the sea, which in turn were raised up to become dry land. Hutton published a two-volume version of his ideas in 1795 (Vol. 1, Vol. 2).</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>[5, 555, 381, 490, 213]</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>[0.8118539452552795, 0.7626733183860779, 0.7505077123641968, 0.7479408383369446, 0.7418496608734131]</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>["The first European to travel the length of the Amazon River was Francisco de Orellana in 1542. The BBC's Unnatural Histories presents evidence that Orellana, rather than exaggerating his claims as previously thought, was correct in his observations that a complex civilization was flourishing along the Amazon in the 1540s. It is believed that the civilization was later devastated by the spread of diseases from Europe, such as smallpox. Since the 1970s, numerous geoglyphs have been discovered on deforested land dating between AD 0–1250, furthering claims about Pre-Columbian civilizations. Ondemar Dias is accredited with first discovering the geoglyphs in 1977 and Alceu Ranzi with furthering their discovery after flying over Acre. The BBC's Unnatural Histories presented evidence that the Amazon rainforest, rather than being a pristine wilderness, has been shaped by man for at least 11,000 years through practices such as forest gardening and terra preta.", "For a long time, it was thought that the Amazon rainforest was only ever sparsely populated, as it was impossible to sustain a large population through agriculture given the poor soil. Archeologist Betty Meggers was a prominent proponent of this idea, as described in her book Amazonia: Man and Culture in a Counterfeit Paradise. She claimed that a population density of 0.2 inhabitants per square kilometre (0.52/sq mi) is the maximum that can be sustained in the rainforest through hunting, with agriculture needed to host a larger population. However, recent anthropological findings have suggested that the region was actually densely populated. Some 5 million people may have lived in the Amazon region in AD 1500, divided between dense coastal settlements, such as that at Marajó, and inland dwellers. By 1900 the population had fallen to 1 million and by the early 1980s it was less than 200,000.", "Some modern scholars, such as Fielding H. Garrison, are of the opinion that the origin of the science of geology can be traced to Persia after the Muslim conquests had come to an end. Abu al-Rayhan al-Biruni (973–1048 CE) was one of the earliest Persian geologists, whose works included the earliest writings on the geology of India, hypothesizing that the Indian subcontinent was once a sea. Drawing from Greek and Indian scientific literature that were not destroyed by the Muslim conquests, the Persian scholar Ibn Sina (Avicenna, 981–1037) proposed detailed explanations for the formation of mountains, the origin of earthquakes, and other topics central to modern geology, which provided an essential foundation for the later development of the science. In China, the polymath Shen Kuo (1031–1095) formulated a hypothesis for the process of land formation: based on his observation of fossil animal shells in a geological stratum in a mountain hundreds of miles from the ocean, he inferred that the land was formed by erosion of the mountains and by deposition of silt.", "Fossils found in Kenya suggest that primates roamed the area more than 20 million years ago. Recent findings near Lake Turkana indicate that hominids such as Homo habilis (1.8 and 2.5 million years ago) and Homo erectus (1.8 million to 350,000 years ago) are possible direct ancestors of modern Homo sapiens, and lived in Kenya in the Pleistocene epoch. During excavations at Lake Turkana in 1984, paleoanthropologist Richard Leakey assisted by Kamoya Kimeu discovered the Turkana Boy, a 1.6-million-year-old fossil belonging to Homo erectus. Previous research on early hominids is particularly identified with Mary Leakey and Louis Leakey, who were responsible for the preliminary archaeological research at Olorgesailie and Hyrax Hill. Later work at the former site was undertaken by Glynn Isaac.", "James Hutton is often viewed as the first modern geologist. In 1785 he presented a paper entitled Theory of the Earth to the Royal Society of Edinburgh. In his paper, he explained his theory that the Earth must be much older than had previously been supposed in order to allow enough time for mountains to be eroded and for sediments to form new rocks at the bottom of the sea, which in turn were raised up to become dry land. Hutton published a two-volume version of his ideas in 1795 (Vol. 1, Vol. 2)."]</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -777,21 +672,6 @@
 Following their loss in the divisional round of the previous season's playoffs, the Denver Broncos underwent numerous coaching changes, including a mutual parting with head coach John Fox (who had won four divisional championships in his four years as Broncos head coach), and the hiring of Gary Kubiak as the new head coach. Under Kubiak, the Broncos planned to install a run-oriented offense with zone blocking to blend in with quarterback Peyton Manning's shotgun passing skills, but struggled with numerous changes and injuries to the offensive line, as well as Manning having his worst statistical season since his rookie year with the Indianapolis Colts in 1998, due to a plantar fasciitis injury in his heel that he had suffered since the summer, and the simple fact that Manning was getting old, as he turned 39 in the 2015 off-season. Although the team had a 7–0 start, Manning led the NFL in interceptions. In week 10, Manning suffered a partial tear of the plantar fasciitis in his left foot. He set the NFL's all-time record for career passing yards in this game, but was benched after throwing four interceptions in favor of backup quarterback Brock Osweiler, who took over as the</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>[6, 206, 29, 269, 205]</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>[0.8629498481750488, 0.826653778553009, 0.8123504519462585, 0.8079994916915894, 0.7905004024505615]</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>["The Broncos defeated the Pittsburgh Steelers in the divisional round, 23–16, by scoring 11 points in the final three minutes of the game. They then beat the defending Super Bowl XLIX champion New England Patriots in the AFC Championship Game, 20–18, by intercepting a pass on New England's 2-point conversion attempt with 17 seconds left on the clock. Despite Manning's problems with interceptions during the season, he didn't throw any in their two playoff games.", "in interceptions. In week 10, Manning suffered a partial tear of the plantar fasciitis in his left foot. He set the NFL's all-time record for career passing yards in this game, but was benched after throwing four interceptions in favor of backup quarterback Brock Osweiler, who took over as the starter for most of the remainder of the regular season. Osweiler was injured, however, leading to Manning's return during the Week 17 regular season finale, where the Broncos were losing 13–7 against the 4–11 San Diego Chargers, resulting in Manning re-claiming the starting quarterback position for the playoffs by leading the team to a key 27–20 win that enabled the team to clinch the number one overall AFC seed. Under defensive coordinator Wade Phillips, the Broncos' defense ranked number one in total yards allowed, passing yards allowed and sacks, and like the previous three seasons, the team has continued to set numerous individual, league and franchise records. With the defense carrying the team despite the issues with the offense, the Broncos finished the regular season with a 12–4 record and earned home-field advantage throughout the AFC playoffs.", "The Panthers finished the regular season with a 15–1 record, and quarterback Cam Newton was named the NFL Most Valuable Player (MVP). They defeated the Arizona Cardinals 49–15 in the NFC Championship Game and advanced to their second Super Bowl appearance since the franchise was founded in 1995. The Broncos finished the regular season with a 12–4 record, and denied the New England Patriots a chance to defend their title from Super Bowl XLIX by defeating them 20–18 in the AFC Championship Game. They joined the Patriots, Dallas Cowboys, and Pittsburgh Steelers as one of four teams that have made eight appearances in the Super Bowl.", "The Panthers beat the Seattle Seahawks in the divisional round, running up a 31–0 halftime lead and then holding off a furious second half comeback attempt to win 31–24, avenging their elimination from a year earlier. The Panthers then blew out the Arizona Cardinals in the NFC Championship Game, 49–15, racking up 487 yards and forcing seven turnovers.", "Following their loss in the divisional round of the previous season's playoffs, the Denver Broncos underwent numerous coaching changes, including a mutual parting with head coach John Fox (who had won four divisional championships in his four years as Broncos head coach), and the hiring of Gary Kubiak as the new head coach. Under Kubiak, the Broncos planned to install a run-oriented offense with zone blocking to blend in with quarterback Peyton Manning's shotgun passing skills, but struggled with numerous changes and injuries to the offensive line, as well as Manning having his worst statistical season since his rookie year with the Indianapolis Colts in 1998, due to a plantar fasciitis injury in his heel that he had suffered since the summer, and the simple fact that Manning was getting old, as he turned 39 in the 2015 off-season. Although the team had a 7–0 start, Manning led the NFL in interceptions. In week 10, Manning suffered a partial tear of the plantar fasciitis in his left foot. He set the NFL's all-time record for career passing yards in this game, but was benched after throwing four interceptions in favor of backup quarterback Brock Osweiler, who took over as the"]</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -823,21 +703,6 @@
 The success of the first two landings allowed the remaining missions to be crewed with a single veteran as Commander, with two rookies. Apollo 13 launched Lovell, Jack Swigert, and Fred Haise in April 1970, headed for the Fra Mauro formation. But two days out, a liquid oxygen tank exploded, disabling the Service Module and forcing the crew to use the LM as a "life boat" to return to Earth. Another NASA review board was convened to determine the cause, which turned out to be a combination of damage of the tank in the factory, and a subcontractor not making a tank component according to updated design specifications. Apollo was grounded again, for the remainder of 1970 while the oxygen tank was redesigned and an extra one was added.</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>[7, 815, 303, 319, 25]</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>[0.7849527597427368, 0.7791514992713928, 0.751289963722229, 0.7418358325958252, 0.7361841201782227]</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>["Seamans' establishment of an ad-hoc committee headed by his special technical assistant Nicholas E. Golovin in July 1961, to recommend a launch vehicle to be used in the Apollo program, represented a turning point in NASA's mission mode decision. This committee recognized that the chosen mode was an important part of the launch vehicle choice, and recommended in favor of a hybrid EOR-LOR mode. Its consideration of LOR —as well as Houbolt's ceaseless work— played an important role in publicizing the workability of the approach. In late 1961 and early 1962, members of the Manned Spacecraft Center began to come around to support LOR, including the newly hired deputy director of the Office of Manned Space Flight, Joseph Shea, who became a champion of LOR. The engineers at Marshall Space Flight Center (MSFC) took longer to become convinced of its merits, but their conversion was announced by Wernher von Braun at a briefing in June 1962.", "But even after NASA reached internal agreement, it was far from smooth sailing. Kennedy's science advisor Jerome Wiesner, who had expressed his opposition to manned spaceflight to Kennedy before the President took office, and had opposed the decision to land men on the Moon, hired Golovin, who had left NASA, to chair his own \"Space Vehicle Panel\", ostensibly to monitor, but actually to second-guess NASA's decisions on the Saturn V launch vehicle and LOR by forcing Shea, Seamans, and even Webb to defend themselves, delaying its formal announcement to the press on July 11, 1962, and forcing Webb to still hedge the decision as \"tentative\".", "Notable alumni in the field of government and politics include the founder of modern community organizing Saul Alinsky, Obama campaign advisor and top political advisor to President Bill Clinton David Axelrod, Attorney General and federal judge Robert Bork, Attorney General Ramsey Clark, Prohibition agent Eliot Ness, Supreme Court Justice John Paul Stevens, Prime Minister of Canada William Lyon Mackenzie King, 11th Prime Minister of Poland Marek Belka, Governor of the Bank of Japan Masaaki Shirakawa, the first female African-American Senator Carol Moseley Braun, United States Senator from Vermont and 2016 Democratic Presidential Candidate Bernie Sanders, and former World Bank President Paul Wolfowitz.", "In early 1961, direct ascent was generally the mission mode in favor at NASA. Many engineers feared that a rendezvous —let alone a docking— neither of which had been attempted even in Earth orbit, would be extremely difficult in lunar orbit. Dissenters including John Houbolt at Langley Research Center emphasized the important weight reductions that were offered by the LOR approach. Throughout 1960 and 1961, Houbolt campaigned for the recognition of LOR as a viable and practical option. Bypassing the NASA hierarchy, he sent a series of memos and reports on the issue to Associate Administrator Robert Seamans; while acknowledging that he spoke \"somewhat as a voice in the wilderness,\" Houbolt pleaded that LOR should not be discounted in studies of the question.", "The success of the first two landings allowed the remaining missions to be crewed with a single veteran as Commander, with two rookies. Apollo 13 launched Lovell, Jack Swigert, and Fred Haise in April 1970, headed for the Fra Mauro formation. But two days out, a liquid oxygen tank exploded, disabling the Service Module and forcing the crew to use the LM as a \"life boat\" to return to Earth. Another NASA review board was convened to determine the cause, which turned out to be a combination of damage of the tank in the factory, and a subcontractor not making a tank component according to updated design specifications. Apollo was grounded again, for the remainder of 1970 while the oxygen tank was redesigned and an extra one was added."]</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -869,21 +734,6 @@
 Where school class sizes are typically 40 to 50 students, maintaining order in the classroom can divert the teacher from instruction, leaving little opportunity for concentration and focus on what is being taught. In response, teachers may concentrate their attention on motivated students, ignoring attention-seeking and disruptive students. The result of this is that motivated students, facing demanding university entrance examinations, receive disproportionate resources. Given the emphasis on attainment of university places, administrators and governors may regard this policy as appropriate.</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>[8, 589, 338, 727, 705]</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>[0.7932546138763428, 0.77736896276474, 0.7633671760559082, 0.7482702732086182, 0.7449004054069519]</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>["Chris Keates, the general secretary of National Association of Schoolmasters Union of Women Teachers, said that teachers who have sex with pupils over the age of consent should not be placed on the sex offenders register and that prosecution for statutory rape \"is a real anomaly in the law that we are concerned about.\" This has led to outrage from child protection and parental rights groups. Fears of being labelled a pedophile or hebephile has led to several men who enjoy teaching avoiding the profession. This has in some jurisdictions reportedly led to a shortage of male teachers.", "In the United States especially, several high-profile cases such as Debra LaFave, Pamela Rogers, and Mary Kay Letourneau have caused increased scrutiny on teacher misconduct.", "In education, teachers facilitate student learning, often in a school or academy or perhaps in another environment such as outdoors. A teacher who teaches on an individual basis may be described as a tutor.", "Teachers are required to be registered with the Teaching Council; under Section 30 of the Teaching Council Act 2001, a person employed in any capacity in a recognised teaching post - who is not registered with the Teaching Council - may not be paid from Oireachtas funds.", "Where school class sizes are typically 40 to 50 students, maintaining order in the classroom can divert the teacher from instruction, leaving little opportunity for concentration and focus on what is being taught. In response, teachers may concentrate their attention on motivated students, ignoring attention-seeking and disruptive students. The result of this is that motivated students, facing demanding university entrance examinations, receive disproportionate resources. Given the emphasis on attainment of university places, administrators and governors may regard this policy as appropriate."]</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -913,21 +763,6 @@
 Luther's other major works on the Jews were his 60,000-word treatise Von den Juden und Ihren Lügen (On the Jews and Their Lies), and Vom Schem Hamphoras und vom Geschlecht Christi (On the Holy Name and the Lineage of Christ), both published in 1543, three years before his death. Luther argued that the Jews were no longer the chosen people but "the devil's people", and referred to them with violent, vile language. Citing Deuteronomy 13, wherein Moses commands the killing of idolaters and the burning of their cities and property as an offering to God, Luther called for a "scharfe Barmherzigkeit" ("sharp mercy") against the Jews "to see whether we might save at least a few from the glowing flames." Luther advocated setting synagogues on fire, destroying Jewish prayerbooks, forbidding rabbis from preaching, seizing Jews' property and money, and smashing up their homes, so that these "envenomed worms" would be forced into labour or expelled "for all time". In Robert Michael's view, Luther's words "We are at fault in not slaying them" amounted to a sanction for murder. "God's anger with them is so intense," Luther concluded, "that gentle mercy will only tend to make them worse, while sharp mercy
 His last sermon was delivered at Eisleben, his place of birth, on 15 February 1546, three days before his death. It was "entirely devoted to the obdurate Jews, whom it was a matter of great urgency to expel from all German territory," according to Léon Poliakov. James Mackinnon writes that it concluded with a "fiery summons to drive the Jews bag and baggage from their midst, unless they desisted from their calumny and their usury and became Christians." Luther said, "we want to practice Christian love toward them and pray that they convert," but also that they are "our public enemies ... and if they could kill us all, they would gladly do so. And so often they do."
 At the time of the Marburg Colloquy, Suleiman the Magnificent was besieging Vienna with a vast Ottoman army. Luther had argued against resisting the Turks in his 1518 Explanation of the Ninety-five Theses, provoking accusations of defeatism. He saw the Turks as a scourge sent to punish Christians by God, as agents of the Biblical apocalypse that would destroy the antichrist, whom Luther believed to be the papacy, and the Roman Church. He consistently rejected the idea of a Holy War, "as though our people were an army of Christians against the Turks, who were enemies of Christ. This is absolutely contrary to Christ's doctrine and name". On the other hand, in keeping with his doctrine of the two kingdoms, Luther did support non-religious war against the Turks. In 1526, he argued in Whether Soldiers can be in a State of Grace that national defence is reason for a just war. By 1529, in On War against the Turk, he was actively urging Emperor Charles V and the German people to fight a secular war against the Turks. He made clear, however, that the spiritual war against an alien faith was separate, to be waged through prayer and repentance. Around</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>[398, 179, 375, 9, 503]</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>[0.8531519770622253, 0.8479586243629456, 0.8420147895812988, 0.8375387191772461, 0.8305625319480896]</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>["Luther's rediscovery of \"Christ and His salvation\" was the first of two points that became the foundation for the Reformation. His railing against the sale of indulgences was based on it.", "The effect of Luther's intervention was immediate. After the sixth sermon, the Wittenberg jurist Jerome Schurf wrote to the elector: \"Oh, what joy has Dr. Martin's return spread among us! His words, through divine mercy, are bringing back every day misguided people into the way of the truth.\"", "Luther's other major works on the Jews were his 60,000-word treatise Von den Juden und Ihren Lügen (On the Jews and Their Lies), and Vom Schem Hamphoras und vom Geschlecht Christi (On the Holy Name and the Lineage of Christ), both published in 1543, three years before his death. Luther argued that the Jews were no longer the chosen people but \"the devil's people\", and referred to them with violent, vile language. Citing Deuteronomy 13, wherein Moses commands the killing of idolaters and the burning of their cities and property as an offering to God, Luther called for a \"scharfe Barmherzigkeit\" (\"sharp mercy\") against the Jews \"to see whether we might save at least a few from the glowing flames.\" Luther advocated setting synagogues on fire, destroying Jewish prayerbooks, forbidding rabbis from preaching, seizing Jews' property and money, and smashing up their homes, so that these \"envenomed worms\" would be forced into labour or expelled \"for all time\". In Robert Michael's view, Luther's words \"We are at fault in not slaying them\" amounted to a sanction for murder. \"God's anger with them is so intense,\" Luther concluded, \"that gentle mercy will only tend to make them worse, while sharp mercy", "His last sermon was delivered at Eisleben, his place of birth, on 15 February 1546, three days before his death. It was \"entirely devoted to the obdurate Jews, whom it was a matter of great urgency to expel from all German territory,\" according to Léon Poliakov. James Mackinnon writes that it concluded with a \"fiery summons to drive the Jews bag and baggage from their midst, unless they desisted from their calumny and their usury and became Christians.\" Luther said, \"we want to practice Christian love toward them and pray that they convert,\" but also that they are \"our public enemies ... and if they could kill us all, they would gladly do so. And so often they do.\"", "At the time of the Marburg Colloquy, Suleiman the Magnificent was besieging Vienna with a vast Ottoman army. Luther had argued against resisting the Turks in his 1518 Explanation of the Ninety-five Theses, provoking accusations of defeatism. He saw the Turks as a scourge sent to punish Christians by God, as agents of the Biblical apocalypse that would destroy the antichrist, whom Luther believed to be the papacy, and the Roman Church. He consistently rejected the idea of a Holy War, \"as though our people were an army of Christians against the Turks, who were enemies of Christ. This is absolutely contrary to Christ's doctrine and name\". On the other hand, in keeping with his doctrine of the two kingdoms, Luther did support non-religious war against the Turks. In 1526, he argued in Whether Soldiers can be in a State of Grace that national defence is reason for a just war. By 1529, in On War against the Turk, he was actively urging Emperor Charles V and the German people to fight a secular war against the Turks. He made clear, however, that the spiritual war against an alien faith was separate, to be waged through prayer and repentance. Around"]</t>
         </is>
       </c>
     </row>
@@ -974,21 +809,6 @@
 2 at only 6 m.</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>[10, 472, 0, 710, 86]</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>[0.8790021538734436, 0.7957876920700073, 0.7933358550071716, 0.7258614897727966, 0.71576988697052]</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>["Uptake of O\n2 from the air is the essential purpose of respiration, so oxygen supplementation is used in medicine. Treatment not only increases oxygen levels in the patient's blood, but has the secondary effect of decreasing resistance to blood flow in many types of diseased lungs, easing work load on the heart. Oxygen therapy is used to treat emphysema, pneumonia, some heart disorders (congestive heart failure), some disorders that cause increased pulmonary artery pressure, and any disease that impairs the body's ability to take up and use gaseous oxygen.", "Oxygen, as a supposed mild euphoric, has a history of recreational use in oxygen bars and in sports. Oxygen bars are establishments, found in Japan, California, and Las Vegas, Nevada since the late 1990s that offer higher than normal O\n2 exposure for a fee. Professional athletes, especially in American football, also sometimes go off field between plays to wear oxygen masks in order to get a \"boost\" in performance. The pharmacological effect is doubtful; a placebo effect is a more likely explanation. Available studies support a performance boost from enriched O\n2 mixtures only if they are breathed during aerobic exercise.", "Hyperbaric (high-pressure) medicine uses special oxygen chambers to increase the partial pressure of O\n2 around the patient and, when needed, the medical staff. Carbon monoxide poisoning, gas gangrene, and decompression sickness (the 'bends') are sometimes treated using these devices. Increased O\n2 concentration in the lungs helps to displace carbon monoxide from the heme group of hemoglobin. Oxygen gas is poisonous to the anaerobic bacteria that cause gas gangrene, so increasing its partial pressure helps kill them. Decompression sickness occurs in divers who decompress too quickly after a dive, resulting in bubbles of inert gas, mostly nitrogen and helium, forming in their blood. Increasing the pressure of O\n2 as soon as possible is part of the treatment.", "Oxygen gas (O\n2) can be toxic at elevated partial pressures, leading to convulsions and other health problems.[j] Oxygen toxicity usually begins to occur at partial pressures more than 50 kilopascals (kPa), equal to about 50% oxygen composition at standard pressure or 2.5 times the normal sea-level O\n2 partial pressure of about 21 kPa. This is not a problem except for patients on mechanical ventilators, since gas supplied through oxygen masks in medical applications is typically composed of only 30%–50% O\n2 by volume (about 30 kPa at standard pressure). (although this figure also is subject to wide variation, depending on type of mask).", "Oxygen toxicity to the lungs and central nervous system can also occur in deep scuba diving and surface supplied diving. Prolonged breathing of an air mixture with an O\n2 partial pressure more than 60 kPa can eventually lead to permanent pulmonary fibrosis. Exposure to a O\n2 partial pressures greater than 160 kPa (about 1.6 atm) may lead to convulsions (normally fatal for divers). Acute oxygen toxicity (causing seizures, its most feared effect for divers) can occur by breathing an air mixture with 21% O\n2 at 66 m or more of depth; the same thing can occur by breathing 100% O\n2 at only 6 m."]</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1020,21 +840,6 @@
 On 30 July 1891, at the age of 35, Tesla became a naturalized citizen of the United States, and established his South Fifth Avenue laboratory, and later another at 46 E. Houston Street, in New York. He lit electric lamps wirelessly at both locations, demonstrating the potential of wireless power transmission. In the same year, he patented the Tesla coil.</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>[11, 871, 791, 464, 761]</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>[0.736386775970459, 0.7358243465423584, 0.7357094287872314, 0.7340402007102966, 0.7311691641807556]</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>["Immigrants arrived from all over the world to search for gold, especially from Ireland and China. Many Chinese miners worked in Victoria, and their legacy is particularly strong in Bendigo and its environs. Although there was some racism directed at them, there was not the level of anti-Chinese violence that was seen at the Lambing Flat riots in New South Wales. However, there was a riot at Buckland Valley near Bright in 1857. Conditions on the gold fields were cramped and unsanitary; an outbreak of typhoid at Buckland Valley in 1854 killed over 1,000 miners.", "In the 19th century, shipbuilding and heavy engineering were central to the city's prosperity; and the city was a powerhouse of the Industrial Revolution. This revolution resulted in the urbanization of the city. In 1817 the Maling company, at one time the largest pottery company in the world, moved to the city. The Victorian industrial revolution brought industrial structures that included the 2 1⁄2-mile (4.0 km) Victoria Tunnelling, built in 1842, which provided underground wagon ways to the staithes. On 3 February 1879, Mosley Street in the city, was the first public road in the world to be lit up by the incandescent lightbulb. Newcastle was one of the first cities in the world to be lit up by electric lighting. Innovations in Newcastle and surrounding areas included the development of safety lamps, Stephenson's Rocket, Lord Armstrong's artillery, Be-Ro flour, Joseph Swan's electric light bulbs, and Charles Parsons' invention of the steam turbine, which led to the revolution of marine propulsion and the production of cheap electricity. In 1882, Newcastle became the seat of an Anglican diocese, with St. Nicholas' Church becoming its cathedral.", "In the Sandgate area, to the east of the city and beside the river, resided the close-knit community of keelmen and their families. They were so called because they worked on the keels, boats that were used to transfer coal from the river banks to the waiting colliers, for export to London and elsewhere. In the 1630s about 7,000 out of 20,000 inhabitants of Newcastle died of plague, more than one-third of the population. Specifically within the year 1636, it is roughly estimated with evidence held by the Society of Antiquaries that 47% of the then population of Newcastle died from the epidemic; this may also have been the most devastating loss in any British City in this period.", "On May 3, 1901, downtown Jacksonville was ravaged by a fire that started as a kitchen fire. Spanish moss at a nearby mattress factory was quickly engulfed in flames and enabling the fire to spread rapidly. In just eight hours, it swept through 146 city blocks, destroyed over 2,000 buildings, left about 10,000 homeless and killed 7 residents. The Confederate Monument in Hemming Park was one of the only landmarks to survive the fire. Governor Jennings declare martial law and sent the state militia to maintain order. On May 17 municipal authority resumed in Jacksonville. It is said the glow from the flames could be seen in Savannah, Georgia, and the smoke plumes seen in Raleigh, North Carolina. Known as the \"Great Fire of 1901\", it was one of the worst disasters in Florida history and the largest urban fire in the southeastern United States. Architect Henry John Klutho was a primary figure in the reconstruction of the city. The first multi-story structure built by Klutho was the Dyal-Upchurch Building in 1902. The St. James Building, built on the previous site of the St. James Hotel that burned down, was built in 1912 as Klutho's crowning achievement.", "On 30 July 1891, at the age of 35, Tesla became a naturalized citizen of the United States, and established his South Fifth Avenue laboratory, and later another at 46 E. Houston Street, in New York. He lit electric lamps wirelessly at both locations, demonstrating the potential of wireless power transmission. In the same year, he patented the Tesla coil."]</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1066,21 +871,6 @@
 Following their loss in the divisional round of the previous season's playoffs, the Denver Broncos underwent numerous coaching changes, including a mutual parting with head coach John Fox (who had won four divisional championships in his four years as Broncos head coach), and the hiring of Gary Kubiak as the new head coach. Under Kubiak, the Broncos planned to install a run-oriented offense with zone blocking to blend in with quarterback Peyton Manning's shotgun passing skills, but struggled with numerous changes and injuries to the offensive line, as well as Manning having his worst statistical season since his rookie year with the Indianapolis Colts in 1998, due to a plantar fasciitis injury in his heel that he had suffered since the summer, and the simple fact that Manning was getting old, as he turned 39 in the 2015 off-season. Although the team had a 7–0 start, Manning led the NFL in interceptions. In week 10, Manning suffered a partial tear of the plantar fasciitis in his left foot. He set the NFL's all-time record for career passing yards in this game, but was benched after throwing four interceptions in favor of backup quarterback Brock Osweiler, who took over as the</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>[12, 64, 206, 867, 205]</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>[0.8919463157653809, 0.8538646697998047, 0.8144341707229614, 0.8041219115257263, 0.8034545183181763]</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>["Peyton Manning became the first quarterback ever to lead two different teams to multiple Super Bowls. He is also the oldest quarterback ever to play in a Super Bowl at age 39. The past record was held by John Elway, who led the Broncos to victory in Super Bowl XXXIII at age 38 and is currently Denver's Executive Vice President of Football Operations and General Manager.", "This was the first Super Bowl to feature a quarterback on both teams who was the #1 pick in their draft classes. Manning was the #1 selection of the 1998 NFL draft, while Newton was picked first in 2011. The matchup also pits the top two picks of the 2011 draft against each other: Newton for Carolina and Von Miller for Denver. Manning and Newton also set the record for the largest age difference between opposing Super Bowl quarterbacks at 13 years and 48 days (Manning was 39, Newton was 26).", "in interceptions. In week 10, Manning suffered a partial tear of the plantar fasciitis in his left foot. He set the NFL's all-time record for career passing yards in this game, but was benched after throwing four interceptions in favor of backup quarterback Brock Osweiler, who took over as the starter for most of the remainder of the regular season. Osweiler was injured, however, leading to Manning's return during the Week 17 regular season finale, where the Broncos were losing 13–7 against the 4–11 San Diego Chargers, resulting in Manning re-claiming the starting quarterback position for the playoffs by leading the team to a key 27–20 win that enabled the team to clinch the number one overall AFC seed. Under defensive coordinator Wade Phillips, the Broncos' defense ranked number one in total yards allowed, passing yards allowed and sacks, and like the previous three seasons, the team has continued to set numerous individual, league and franchise records. With the defense carrying the team despite the issues with the offense, the Broncos finished the regular season with a 12–4 record and earned home-field advantage throughout the AFC playoffs.", "In honor of the 50th Super Bowl, the pregame ceremony featured the on-field introduction of 39 of the 43 previous Super Bowl Most Valuable Players. Bart Starr (MVP of Super Bowls I and II) and Chuck Howley (MVP of Super Bowl V) appeared via video, while Peyton Manning (MVP of Super Bowl XLI and current Broncos quarterback) was shown in the locker room preparing for the game. No plans were announced regarding the recognition of Harvey Martin, co-MVP of Super Bowl XII, who died in 2001.", "Following their loss in the divisional round of the previous season's playoffs, the Denver Broncos underwent numerous coaching changes, including a mutual parting with head coach John Fox (who had won four divisional championships in his four years as Broncos head coach), and the hiring of Gary Kubiak as the new head coach. Under Kubiak, the Broncos planned to install a run-oriented offense with zone blocking to blend in with quarterback Peyton Manning's shotgun passing skills, but struggled with numerous changes and injuries to the offensive line, as well as Manning having his worst statistical season since his rookie year with the Indianapolis Colts in 1998, due to a plantar fasciitis injury in his heel that he had suffered since the summer, and the simple fact that Manning was getting old, as he turned 39 in the 2015 off-season. Although the team had a 7–0 start, Manning led the NFL in interceptions. In week 10, Manning suffered a partial tear of the plantar fasciitis in his left foot. He set the NFL's all-time record for career passing yards in this game, but was benched after throwing four interceptions in favor of backup quarterback Brock Osweiler, who took over as the"]</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1112,21 +902,6 @@
 The Yuan undertook extensive public works. Among Kublai Khan's top engineers and scientists was the astronomer Guo Shoujing, who was tasked with many public works projects and helped the Yuan reform the lunisolar calendar to provide an accuracy of 365.2425 days of the year, which was only 26 seconds off the modern Gregorian calendar's measurement. Road and water communications were reorganized and improved. To provide against possible famines, granaries were ordered built throughout the empire. The city of Beijing was rebuilt with new palace grounds that included artificial lakes, hills and mountains, and parks. During the Yuan period, Beijing became the terminus of the Grand Canal of China, which was completely renovated. These commercially oriented improvements encouraged overland and maritime commerce throughout Asia and facilitated direct Chinese contacts with Europe. Chinese travelers to the West were able to provide assistance in such areas as hydraulic engineering. Contacts with the West also brought the introduction to China of a major food crop, sorghum, along with other foreign food products and methods of preparation.</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>[13, 78, 470, 390, 499]</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>[0.8261951804161072, 0.8082302808761597, 0.7382047772407532, 0.7239812612533569, 0.7189592123031616]</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>["The Chinese medical tradition of the Yuan had \"Four Great Schools\" that the Yuan inherited from the Jin dynasty. All four schools were based on the same intellectual foundation, but advocated different theoretical approaches toward medicine. Under the Mongols, the practice of Chinese medicine spread to other parts of the empire. Chinese physicians were brought along military campaigns by the Mongols as they expanded towards the west. Chinese medical techniques such as acupuncture, moxibustion, pulse diagnosis, and various herbal drugs and elixirs were transmitted westward to the Middle East and the rest of the empire. Several medical advances were made in the Yuan period. The physician Wei Yilin (1277–1347) invented a suspension method for reducing dislocated joints, which he performed using anesthetics. The Mongol physician Hu Sihui described the importance of a healthy diet in a 1330 medical treatise.", "Western medicine was also practiced in China by the Nestorian Christians of the Yuan court, where it was sometimes labeled as huihui or Muslim medicine. The Nestorian physician Jesus the Interpreter founded the Office of Western Medicine in 1263 during the reign of Kublai. Huihui doctors staffed at two imperial hospitals were responsible for treating the imperial family and members of the court. Chinese physicians opposed Western medicine because its humoral system contradicted the yin-yang and wuxing philosophy underlying traditional Chinese medicine. No Chinese translation of Western medical works is known, but it is possible that the Chinese had access to Avicenna's The Canon of Medicine.", "The physicians of the Yuan court came from diverse cultures. Healers were divided into non-Mongol physicians called otachi and traditional Mongol shamans. The Mongols characterized otachi doctors by their use of herbal remedies, which was distinguished from the spiritual cures of Mongol shamanism. Physicians received official support from the Yuan government and were given special legal privileges. Kublai created the Imperial Academy of Medicine to manage medical treatises and the education of new doctors. Confucian scholars were attracted to the medical profession because it ensured a high income and medical ethics were compatible with Confucian virtues.", "less than 700 preparations, their properties, modes of action, and their indications. He devoted in fact a whole volume to simple drugs in The Canon of Medicine. Of great impact were also the works by al-Maridini of Baghdad and Cairo, and Ibn al-Wafid (1008–1074), both of which were printed in Latin more than fifty times, appearing as De Medicinis universalibus et particularibus by 'Mesue' the younger, and the Medicamentis simplicibus by 'Abenguefit'. Peter of Abano (1250–1316) translated and added a supplement to the work of al-Maridini under the title De Veneris. Al-Muwaffaq’s contributions in the field are also pioneering. Living in the 10th century, he wrote The foundations of the true properties of Remedies, amongst others describing arsenious oxide, and being acquainted with silicic acid. He made clear distinction between sodium carbonate and potassium carbonate, and drew attention to the poisonous nature of copper compounds, especially copper vitriol, and also lead compounds. He also describes the distillation of sea-water for drinking.[verification needed]", "The Yuan undertook extensive public works. Among Kublai Khan's top engineers and scientists was the astronomer Guo Shoujing, who was tasked with many public works projects and helped the Yuan reform the lunisolar calendar to provide an accuracy of 365.2425 days of the year, which was only 26 seconds off the modern Gregorian calendar's measurement. Road and water communications were reorganized and improved. To provide against possible famines, granaries were ordered built throughout the empire. The city of Beijing was rebuilt with new palace grounds that included artificial lakes, hills and mountains, and parks. During the Yuan period, Beijing became the terminus of the Grand Canal of China, which was completely renovated. These commercially oriented improvements encouraged overland and maritime commerce throughout Asia and facilitated direct Chinese contacts with Europe. Chinese travelers to the West were able to provide assistance in such areas as hydraulic engineering. Contacts with the West also brought the introduction to China of a major food crop, sorghum, along with other foreign food products and methods of preparation."]</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1156,21 +931,6 @@
 A problem is regarded as inherently difficult if its solution requires significant resources, whatever the algorithm used. The theory formalizes this intuition, by introducing mathematical models of computation to study these problems and quantifying the amount of resources needed to solve them, such as time and storage. Other complexity measures are also used, such as the amount of communication (used in communication complexity), the number of gates in a circuit (used in circuit complexity) and the number of processors (used in parallel computing). One of the roles of computational complexity theory is to determine the practical limits on what computers can and cannot do.
 Many important complexity classes can be defined by bounding the time or space used by the algorithm. Some important complexity classes of decision problems defined in this manner are the following:
 The most commonly used reduction is a polynomial-time reduction. This means that the reduction process takes polynomial time. For example, the problem of squaring an integer can be reduced to the problem of multiplying two integers. This means an algorithm for multiplying two integers can be used to square an integer. Indeed, this can be done by giving the same input to both inputs of the multiplication algorithm. Thus we see that squaring is not more difficult than multiplication, since squaring can be reduced to multiplication.</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>[14, 784, 131, 475, 234]</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>[0.8678880333900452, 0.8372492790222168, 0.8150402903556824, 0.8126431703567505, 0.8120195269584656]</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>["The integer factorization problem is the computational problem of determining the prime factorization of a given integer. Phrased as a decision problem, it is the problem of deciding whether the input has a factor less than k. No efficient integer factorization algorithm is known, and this fact forms the basis of several modern cryptographic systems, such as the RSA algorithm. The integer factorization problem is in NP and in co-NP (and even in UP and co-UP). If the problem is NP-complete, the polynomial time hierarchy will collapse to its first level (i.e., NP will equal co-NP). The best known algorithm for integer factorization is the general number field sieve, which takes time O(e(64/9)1/3(n.log 2)1/3(log (n.log 2))2/3) to factor an n-bit integer. However, the best known quantum algorithm for this problem, Shor's algorithm, does run in polynomial time. Unfortunately, this fact doesn't say much about where the problem lies with respect to non-quantum complexity classes.", "It was shown by Ladner that if P ≠ NP then there exist problems in NP that are neither in P nor NP-complete. Such problems are called NP-intermediate problems. The graph isomorphism problem, the discrete logarithm problem and the integer factorization problem are examples of problems believed to be NP-intermediate. They are some of the very few NP problems not known to be in P or to be NP-complete.", "A problem is regarded as inherently difficult if its solution requires significant resources, whatever the algorithm used. The theory formalizes this intuition, by introducing mathematical models of computation to study these problems and quantifying the amount of resources needed to solve them, such as time and storage. Other complexity measures are also used, such as the amount of communication (used in communication complexity), the number of gates in a circuit (used in circuit complexity) and the number of processors (used in parallel computing). One of the roles of computational complexity theory is to determine the practical limits on what computers can and cannot do.", "Many important complexity classes can be defined by bounding the time or space used by the algorithm. Some important complexity classes of decision problems defined in this manner are the following:", "The most commonly used reduction is a polynomial-time reduction. This means that the reduction process takes polynomial time. For example, the problem of squaring an integer can be reduced to the problem of multiplying two integers. This means an algorithm for multiplying two integers can be used to square an integer. Indeed, this can be done by giving the same input to both inputs of the multiplication algorithm. Thus we see that squaring is not more difficult than multiplication, since squaring can be reduced to multiplication."]</t>
         </is>
       </c>
     </row>
@@ -1210,21 +970,6 @@
 3, in hematite and rust), and calcium carbonate (in limestone). The rest of the Earth's crust is also made of oxygen compounds, in particular various complex silicates (in silicate minerals). The Earth's mantle, of much larger mass than the crust, is largely composed of silicates of magnesium and iron.</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>[15, 254, 455, 590, 315]</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>[0.809039831161499, 0.7161040306091309, 0.715279221534729, 0.7046109437942505, 0.6988662481307983]</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>["For many geologic applications, isotope ratios of radioactive elements are measured in minerals that give the amount of time that has passed since a rock passed through its particular closure temperature, the point at which different radiometric isotopes stop diffusing into and out of the crystal lattice. These are used in geochronologic and thermochronologic studies. Common methods include uranium-lead dating, potassium-argon dating, argon-argon dating and uranium-thorium dating. These methods are used for a variety of applications. Dating of lava and volcanic ash layers found within a stratigraphic sequence can provide absolute age data for sedimentary rock units which do not contain radioactive isotopes and calibrate relative dating techniques. These methods can also be used to determine ages of pluton emplacement. Thermochemical techniques can be used to determine temperature profiles within the crust, the uplift of mountain ranges, and paleotopography.", "The principle of inclusions and components states that, with sedimentary rocks, if inclusions (or clasts) are found in a formation, then the inclusions must be older than the formation that contains them. For example, in sedimentary rocks, it is common for gravel from an older formation to be ripped up and included in a newer layer. A similar situation with igneous rocks occurs when xenoliths are found. These foreign bodies are picked up as magma or lava flows, and are incorporated, later to cool in the matrix. As a result, xenoliths are older than the rock which contains them.", "Highly combustible materials that leave little residue, such as wood or coal, were thought to be made mostly of phlogiston; whereas non-combustible substances that corrode, such as iron, contained very little. Air did not play a role in phlogiston theory, nor were any initial quantitative experiments conducted to test the idea; instead, it was based on observations of what happens when something burns, that most common objects appear to become lighter and seem to lose something in the process. The fact that a substance like wood gains overall weight in burning was hidden by the buoyancy of the gaseous combustion products. Indeed, one of the first clues that the phlogiston theory was incorrect was that metals, too, gain weight in rusting (when they were supposedly losing phlogiston).", "Among the most well-known experiments in structural geology are those involving orogenic wedges, which are zones in which mountains are built along convergent tectonic plate boundaries. In the analog versions of these experiments, horizontal layers of sand are pulled along a lower surface into a back stop, which results in realistic-looking patterns of faulting and the growth of a critically tapered (all angles remain the same) orogenic wedge. Numerical models work in the same way as these analog models, though they are often more sophisticated and can include patterns of erosion and uplift in the mountain belt. This helps to show the relationship between erosion and the shape of the mountain range. These studies can also give useful information about pathways for metamorphism through pressure, temperature, space, and time.", "Oxygen is present in the atmosphere in trace quantities in the form of carbon dioxide (CO\n2). The Earth's crustal rock is composed in large part of oxides of silicon (silica SiO\n2, as found in granite and quartz), aluminium (aluminium oxide Al\n2O\n3, in bauxite and corundum), iron (iron(III) oxide Fe\n2O\n3, in hematite and rust), and calcium carbonate (in limestone). The rest of the Earth's crust is also made of oxygen compounds, in particular various complex silicates (in silicate minerals). The Earth's mantle, of much larger mass than the crust, is largely composed of silicates of magnesium and iron."]</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1256,21 +1001,6 @@
 The Cestida ("belt animals") are ribbon-shaped planktonic animals, with the mouth and aboral organ aligned in the middle of opposite edges of the ribbon. There is a pair of comb-rows along each aboral edge, and tentilla emerging from a groove all along the oral edge, which stream back across most of the wing-like body surface. Cestids can swim by undulating their bodies as well as by the beating of their comb-rows. There are two known species, with worldwide distribution in warm, and warm-temperate waters: Cestum veneris ("Venus' girdle") is among the largest ctenophores – up to 1.5 meters (4.9 ft) long, and can undulate slowly or quite rapidly. Velamen parallelum, which is typically less than 20 centimeters (0.66 ft) long, can move much faster in what has been described as a "darting motion".</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>[61, 16, 847, 855, 840]</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>[0.7982907891273499, 0.7652561664581299, 0.7164751887321472, 0.7157790064811707, 0.7122554779052734]</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>["Almost all species are hermaphrodites, in other words they function as both males and females at the same time – except that in two species of the genus Ocryopsis individuals remain of the same single sex all their lives. The gonads are located in the parts of the internal canal network under the comb rows, and eggs and sperm are released via pores in the epidermis. Fertilization is external in most species, but platyctenids use internal fertilization and keep the eggs in brood chambers until they hatch. Self-fertilization has occasionally been seen in species of the genus Mnemiopsis, and it is thought that most of the hermaphroditic species are self-fertile.", "Most species are hermaphrodites—a single animal can produce both eggs and sperm, meaning it can fertilize its own egg, not needing a mate. Some are simultaneous hermaphrodites, which can produce both eggs and sperm at the same time. Others are sequential hermaphrodites, in which the eggs and sperm mature at different times. Fertilization is generally external, although platyctenids' eggs are fertilized inside their parents' bodies and kept there until they hatch. The young are generally planktonic and in most species look like miniature cydippids, gradually changing into their adult shapes as they grow. The exceptions are the beroids, whose young are miniature beroids with large mouths and no tentacles, and the platyctenids, whose young live as cydippid-like plankton until they reach near-adult size, but then sink to the bottom and rapidly metamorphose into the adult form. In at least some species, juveniles are capable of reproduction before reaching the adult size and shape. The combination of hermaphroditism and early reproduction enables small populations to grow at an explosive rate.", "Ranging from about 1 millimeter (0.039 in) to 1.5 meters (4.9 ft) in size, ctenophores are the largest non-colonial animals that use cilia (\"hairs\") as their main method of locomotion. Most species have eight strips, called comb rows, that run the length of their bodies and bear comb-like bands of cilia, called \"ctenes,\" stacked along the comb rows so that when the cilia beat, those of each comb touch the comb below. The name \"ctenophora\" means \"comb-bearing\", from the Greek κτείς (stem-form κτεν-) meaning \"comb\" and the Greek suffix -φορος meaning \"carrying\".", "body forms in a phylum with rather few species. The two-tentacled \"cydippid\" Lampea feeds exclusively on salps, close relatives of sea-squirts that form large chain-like floating colonies, and juveniles of Lampea attach themselves like parasites to salps that are too large for them to swallow. Members of the cydippid genus Pleurobrachia and the lobate Bolinopsis often reach high population densities at the same place and time because they specialize in different types of prey: Pleurobrachia's long tentacles mainly capture relatively strong swimmers such as adult copepods, while Bolinopsis generally feeds on smaller, weaker swimmers such as rotifers and mollusc and crustacean larvae.", "The Cestida (\"belt animals\") are ribbon-shaped planktonic animals, with the mouth and aboral organ aligned in the middle of opposite edges of the ribbon. There is a pair of comb-rows along each aboral edge, and tentilla emerging from a groove all along the oral edge, which stream back across most of the wing-like body surface. Cestids can swim by undulating their bodies as well as by the beating of their comb-rows. There are two known species, with worldwide distribution in warm, and warm-temperate waters: Cestum veneris (\"Venus' girdle\") is among the largest ctenophores – up to 1.5 meters (4.9 ft) long, and can undulate slowly or quite rapidly. Velamen parallelum, which is typically less than 20 centimeters (0.66 ft) long, can move much faster in what has been described as a \"darting motion\"."]</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1302,21 +1032,6 @@
 After the 1940s, the Gothic style on campus began to give way to modern styles. In 1955, Eero Saarinen was contracted to develop a second master plan, which led to the construction of buildings both north and south of the Midway, including the Laird Bell Law Quadrangle (a complex designed by Saarinen); a series of arts buildings; a building designed by Ludwig Mies van der Rohe for the university's School of Social Service Administration;, a building which is to become the home of the Harris School of Public Policy Studies by Edward Durrell Stone, and the Regenstein Library, the largest building on campus, a brutalist structure designed by Walter Netsch of the Chicago firm Skidmore, Owings &amp; Merrill. Another master plan, designed in 1999 and updated in 2004, produced the Gerald Ratner Athletics Center (2003), the Max Palevsky Residential Commons (2001), South Campus Residence Hall and dining commons (2009), a new children's hospital, and other construction, expansions, and restorations. In 2011, the university completed the glass dome-shaped Joe and Rika Mansueto Library, which provides a grand reading room for the university library and prevents the need for an off-campus book depository.</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>[17, 3, 442, 691, 138]</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>[0.8069320321083069, 0.7194464802742004, 0.7079836130142212, 0.6839126348495483, 0.6464253664016724]</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>["The university operates 12 research institutes and 113 research centers on campus. Among these are the Oriental Institute—a museum and research center for Near Eastern studies owned and operated by the university—and a number of National Resource Centers, including the Center for Middle Eastern Studies. Chicago also operates or is affiliated with a number of research institutions apart from the university proper. The university partially manages Argonne National Laboratory, part of the United States Department of Energy's national laboratory system, and has a joint stake in Fermilab, a nearby particle physics laboratory, as well as a stake in the Apache Point Observatory in Sunspot, New Mexico. Faculty and students at the adjacent Toyota Technological Institute at Chicago collaborate with the university, In 2013, the university announced that it was affiliating the formerly independent Marine Biological Laboratory in Woods Hole, Mass. Although formally unrelated, the National Opinion Research Center is located on Chicago's campus.", "The university runs a number of academic institutions and programs apart from its undergraduate and postgraduate schools. It operates the University of Chicago Laboratory Schools (a private day school for K-12 students and day care), the Sonia Shankman Orthogenic School (a residential treatment program for those with behavioral and emotional problems), and four public charter schools on the South Side of Chicago administered by the university's Urban Education Institute. In addition, the Hyde Park Day School, a school for students with learning disabilities, maintains a location on the University of Chicago campus. Since 1983, the University of Chicago has maintained the University of Chicago School Mathematics Project, a mathematics program used in urban primary and secondary schools. The university runs a program called the Council on Advanced Studies in the Social Sciences and Humanities, which administers interdisciplinary workshops to provide a forum for graduate students, faculty, and visiting scholars to present scholarly work in progress. The university also operates the University of Chicago Press, the largest university press in the United States.", "University of Chicago scholars have played a major role in the development of various academic disciplines, including: the Chicago school of economics, the Chicago school of sociology, the law and economics movement in legal analysis, the Chicago school of literary criticism, the Chicago school of religion, and the behavioralism school of political science. Chicago's physics department helped develop the world's first man-made, self-sustaining nuclear reaction beneath the university's Stagg Field. Chicago's research pursuits have been aided by unique affiliations with world-renowned institutions like the nearby Fermilab and Argonne National Laboratory, as well as the Marine Biological Laboratory. The university is also home to the University of Chicago Press, the largest university press in the United States. With an estimated completion date of 2020, the Barack Obama Presidential Center will be housed at the university and include both the Obama presidential library and offices of the Obama Foundation.", "From the mid-2000s, the university began a number of multimillion-dollar expansion projects. In 2008, the University of Chicago announced plans to establish the Milton Friedman Institute which attracted both support and controversy from faculty members and students. The institute will cost around $200 million and occupy the buildings of the Chicago Theological Seminary. During the same year, investor David G. Booth donated $300 million to the university's Booth School of Business, which is the largest gift in the university's history and the largest gift ever to any business school. In 2009, planning or construction on several new buildings, half of which cost $100 million or more, was underway. Since 2011, major construction projects have included the Jules and Gwen Knapp Center for Biomedical Discovery, a ten-story medical research center, and further additions to the medical campus of the University of Chicago Medical Center. In 2014 the University launched the public phase of a $4.5 billion fundraising campaign. In September 2015, the University received $100 million from The Pearson Family Foundation to establish The Pearson Institute for the Study and Resolution of Global Conflicts and The Pearson Global Forum at the Harris School of Public Policy Studies.", "After the 1940s, the Gothic style on campus began to give way to modern styles. In 1955, Eero Saarinen was contracted to develop a second master plan, which led to the construction of buildings both north and south of the Midway, including the Laird Bell Law Quadrangle (a complex designed by Saarinen); a series of arts buildings; a building designed by Ludwig Mies van der Rohe for the university's School of Social Service Administration;, a building which is to become the home of the Harris School of Public Policy Studies by Edward Durrell Stone, and the Regenstein Library, the largest building on campus, a brutalist structure designed by Walter Netsch of the Chicago firm Skidmore, Owings &amp; Merrill. Another master plan, designed in 1999 and updated in 2004, produced the Gerald Ratner Athletics Center (2003), the Max Palevsky Residential Commons (2001), South Campus Residence Hall and dining commons (2009), a new children's hospital, and other construction, expansions, and restorations. In 2011, the university completed the glass dome-shaped Joe and Rika Mansueto Library, which provides a grand reading room for the university library and prevents the need for an off-campus book depository."]</t>
-        </is>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1348,21 +1063,6 @@
 Historically, forces were first quantitatively investigated in conditions of static equilibrium where several forces canceled each other out. Such experiments demonstrate the crucial properties that forces are additive vector quantities: they have magnitude and direction. When two forces act on a point particle, the resulting force, the resultant (also called the net force), can be determined by following the parallelogram rule of vector addition: the addition of two vectors represented by sides of a parallelogram, gives an equivalent resultant vector that is equal in magnitude and direction to the transversal of the parallelogram. The magnitude of the resultant varies from the difference of the magnitudes of the two forces to their sum, depending on the angle between their lines of action. However, if the forces are acting on an extended body, their respective lines of application must also be specified in order to account for their effects on the motion of the body.</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>[18, 754, 436, 76, 650]</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>[0.8024594783782959, 0.7621064782142639, 0.7528319954872131, 0.7270205616950989, 0.7245141863822937]</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>["Tension forces can be modeled using ideal strings that are massless, frictionless, unbreakable, and unstretchable. They can be combined with ideal pulleys, which allow ideal strings to switch physical direction. Ideal strings transmit tension forces instantaneously in action-reaction pairs so that if two objects are connected by an ideal string, any force directed along the string by the first object is accompanied by a force directed along the string in the opposite direction by the second object. By connecting the same string multiple times to the same object through the use of a set-up that uses movable pulleys, the tension force on a load can be multiplied. For every string that acts on a load, another factor of the tension force in the string acts on the load. However, even though such machines allow for an increase in force, there is a corresponding increase in the length of string that must be displaced in order to move the load. These tandem effects result ultimately in the conservation of mechanical energy since the work done on the load is the same no matter how complicated the machine.", "Newton's laws and Newtonian mechanics in general were first developed to describe how forces affect idealized point particles rather than three-dimensional objects. However, in real life, matter has extended structure and forces that act on one part of an object might affect other parts of an object. For situations where lattice holding together the atoms in an object is able to flow, contract, expand, or otherwise change shape, the theories of continuum mechanics describe the way forces affect the material. For example, in extended fluids, differences in pressure result in forces being directed along the pressure gradients as follows:", "For certain physical scenarios, it is impossible to model forces as being due to gradient of potentials. This is often due to macrophysical considerations that yield forces as arising from a macroscopic statistical average of microstates. For example, friction is caused by the gradients of numerous electrostatic potentials between the atoms, but manifests as a force model that is independent of any macroscale position vector. Nonconservative forces other than friction include other contact forces, tension, compression, and drag. However, for any sufficiently detailed description, all these forces are the results of conservative ones since each of these macroscopic forces are the net results of the gradients of microscopic potentials.", "Since forces are perceived as pushes or pulls, this can provide an intuitive understanding for describing forces. As with other physical concepts (e.g. temperature), the intuitive understanding of forces is quantified using precise operational definitions that are consistent with direct observations and compared to a standard measurement scale. Through experimentation, it is determined that laboratory measurements of forces are fully consistent with the conceptual definition of force offered by Newtonian mechanics.", "Historically, forces were first quantitatively investigated in conditions of static equilibrium where several forces canceled each other out. Such experiments demonstrate the crucial properties that forces are additive vector quantities: they have magnitude and direction. When two forces act on a point particle, the resulting force, the resultant (also called the net force), can be determined by following the parallelogram rule of vector addition: the addition of two vectors represented by sides of a parallelogram, gives an equivalent resultant vector that is equal in magnitude and direction to the transversal of the parallelogram. The magnitude of the resultant varies from the difference of the magnitudes of the two forces to their sum, depending on the angle between their lines of action. However, if the forces are acting on an extended body, their respective lines of application must also be specified in order to account for their effects on the motion of the body."]</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1394,21 +1094,6 @@
 In cases where the criminalized behavior is pure speech, civil disobedience can consist simply of engaging in the forbidden speech. An example would be WBAI's broadcasting the track "Filthy Words" from a George Carlin comedy album, which eventually led to the 1978 Supreme Court case of FCC v. Pacifica Foundation. Threatening government officials is another classic way of expressing defiance toward the government and unwillingness to stand for its policies. For example, Joseph Haas was arrested for allegedly sending an email to the Lebanon, New Hampshire city councilors stating, "Wise up or die."</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>[602, 760, 182, 33, 514]</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>[0.7926405072212219, 0.7834293842315674, 0.7691366672515869, 0.7682362794876099, 0.7619557976722717]</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>["Some theories of civil disobedience hold that civil disobedience is only justified against governmental entities. Brownlee argues that disobedience in opposition to the decisions of non-governmental agencies such as trade unions, banks, and private universities can be justified if it reflects \"a larger challenge to the legal system that permits those decisions to be taken\". The same principle, she argues, applies to breaches of law in protest against international organizations and foreign governments.", "Some forms of civil disobedience, such as illegal boycotts, refusals to pay taxes, draft dodging, distributed denial-of-service attacks, and sit-ins, make it more difficult for a system to function. In this way, they might be considered coercive. Brownlee notes that \"although civil disobedients are constrained in their use of coercion by their conscientious aim to engage in moral dialogue, nevertheless they may find it necessary to employ limited coercion in order to get their issue onto the table.\" The Plowshares organization temporarily closed GCSB Waihopai by padlocking the gates and using sickles to deflate one of the large domes covering two satellite dishes.", "Civil disobedients have chosen a variety of different illegal acts. Bedau writes, \"There is a whole class of acts, undertaken in the name of civil disobedience, which, even if they were widely practiced, would in themselves constitute hardly more than a nuisance (e.g. trespassing at a nuclear-missile installation)...Such acts are often just a harassment and, at least to the bystander, somewhat inane...The remoteness of the connection between the disobedient act and the objectionable law lays such acts open to the charge of ineffectiveness and absurdity.\" Bedau also notes, though, that the very harmlessness of such entirely symbolic illegal protests toward public policy goals may serve a propaganda purpose. Some civil disobedients, such as the proprietors of illegal medical cannabis dispensaries and Voice in the Wilderness, which brought medicine to Iraq without the permission of the U.S. Government, directly achieve a desired social goal (such as the provision of medication to the sick) while openly breaking the law. Julia Butterfly Hill lived in Luna, a 180-foot (55 m)-tall, 600-year-old California Redwood tree for 738 days, successfully preventing it from being cut down.", "Courts have distinguished between two types of civil disobedience: \"Indirect civil disobedience involves violating a law which is not, itself, the object of protest, whereas direct civil disobedience involves protesting the existence of a particular law by breaking that law.\" During the Vietnam War, courts typically refused to excuse the perpetrators of illegal protests from punishment on the basis of their challenging the legality of the Vietnam War; the courts ruled it was a political question. The necessity defense has sometimes been used as a shadow defense by civil disobedients to deny guilt without denouncing their politically motivated acts, and to present their political beliefs in the courtroom. However, court cases such as U.S. v. Schoon have greatly curtailed the availability of the political necessity defense. Likewise, when Carter Wentworth was charged for his role in the Clamshell Alliance's 1977 illegal occupation of the Seabrook Station Nuclear Power Plant, the judge instructed the jury to disregard his competing harms defense, and he was found guilty. Fully Informed Jury Association activists have sometimes handed out educational leaflets inside courthouses despite admonitions not to; according to FIJA, many of them have escaped prosecution because \"prosecutors have reasoned (correctly) that if they arrest", "In cases where the criminalized behavior is pure speech, civil disobedience can consist simply of engaging in the forbidden speech. An example would be WBAI's broadcasting the track \"Filthy Words\" from a George Carlin comedy album, which eventually led to the 1978 Supreme Court case of FCC v. Pacifica Foundation. Threatening government officials is another classic way of expressing defiance toward the government and unwillingness to stand for its policies. For example, Joseph Haas was arrested for allegedly sending an email to the Lebanon, New Hampshire city councilors stating, \"Wise up or die.\""]</t>
-        </is>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1440,21 +1125,6 @@
 In addition to those actors who have headlined the series, others have portrayed versions of the Doctor in guest roles. Notably, in 2013, John Hurt guest-starred as a hitherto unknown incarnation of the Doctor known as the War Doctor in the run-up to the show's 50th anniversary special "The Day of the Doctor". He is shown in mini-episode "The Night of the Doctor" to have been retroactively inserted into the show's fictional chronology between McGann and Eccleston's Doctors, although his introduction was written so as not to disturb the established numerical naming of the Doctors. Another example is from the 1986 serial The Trial of a Time Lord, where Michael Jayston portrayed the Valeyard, who is described as an amalgamation of the darker sides of the Doctor's nature, somewhere between his twelfth and final incarnation.</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>[184, 20, 456, 185, 408]</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>[0.8198589086532593, 0.813040018081665, 0.8078722953796387, 0.804934561252594, 0.7978605031967163]</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>["Following the success of the 2005 series produced by Russell T Davies, the BBC commissioned Davies to produce a 13-part spin-off series titled Torchwood (an anagram of \"Doctor Who\"), set in modern-day Cardiff and investigating alien activities and crime. The series debuted on BBC Three on 22 October 2006. John Barrowman reprised his role of Jack Harkness from the 2005 series of Doctor Who. Two other actresses who appeared in Doctor Who also star in the series; Eve Myles as Gwen Cooper, who also played the similarly named servant girl Gwyneth in the 2005 Doctor Who episode \"The Unquiet Dead\", and Naoko Mori who reprised her role as Toshiko Sato first seen in \"Aliens of London\". A second series of Torchwood aired in 2008; for three episodes, the cast was joined by Freema Agyeman reprising her Doctor Who role of Martha Jones. A third series was broadcast from 6 to 10 July 2009, and consisted of a single five-part story called Children of Earth which was set largely in London. A fourth series, Torchwood: Miracle Day jointly produced by BBC Wales, BBC Worldwide and the American entertainment company Starz debuted in 2011. The series was predominantly set in the United", "With the show's 2005 revival, executive producer Russell T Davies stated his intention to reintroduce classic icons of Doctor Who one step at a time: the Autons with the Nestene Consciousness and Daleks in series 1, Cybermen in series 2, the Macra and the Master in series 3, the Sontarans and Davros in series 4, and the Time Lords (Rassilon) in the 2009–10 Specials. Davies' successor, Steven Moffat, has continued the trend by reviving the Silurians in series 5, Cybermats in series 6, the Great Intelligence and the Ice Warriors in Series 7, and Zygons in the 50th Anniversary Special. Since its 2005 return, the series has also introduced new recurring aliens: Slitheen (Raxacoricofallapatorian), Ood, Judoon, Weeping Angels and the Silence.", "Following the series revival in 2005, Derek Jacobi provided the character's re-introduction in the 2007 episode \"Utopia\". During that story the role was then assumed by John Simm who returned to the role multiple times through the Tenth Doctor's tenure. As of the 2014 episode \"Dark Water,\" it was revealed that the Master had become a female incarnation or \"Time Lady,\" going by the name of \"Missy\" (short for Mistress, the feminine equivalent of \"Master\"). This incarnation is played by Michelle Gomez.", "10 July 2009, and consisted of a single five-part story called Children of Earth which was set largely in London. A fourth series, Torchwood: Miracle Day jointly produced by BBC Wales, BBC Worldwide and the American entertainment company Starz debuted in 2011. The series was predominantly set in the United States, though Wales remained part of the show's setting.", "In addition to those actors who have headlined the series, others have portrayed versions of the Doctor in guest roles. Notably, in 2013, John Hurt guest-starred as a hitherto unknown incarnation of the Doctor known as the War Doctor in the run-up to the show's 50th anniversary special \"The Day of the Doctor\". He is shown in mini-episode \"The Night of the Doctor\" to have been retroactively inserted into the show's fictional chronology between McGann and Eccleston's Doctors, although his introduction was written so as not to disturb the established numerical naming of the Doctors. Another example is from the 1986 serial The Trial of a Time Lord, where Michael Jayston portrayed the Valeyard, who is described as an amalgamation of the darker sides of the Doctor's nature, somewhere between his twelfth and final incarnation."]</t>
-        </is>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1486,21 +1156,6 @@
 Legislative power in Warsaw is vested in a unicameral Warsaw City Council (Rada Miasta), which comprises 60 members. Council members are elected directly every four years. Like most legislative bodies, the City Council divides itself into committees which have the oversight of various functions of the city government. Bills passed by a simple majority are sent to the mayor (the President of Warsaw), who may sign them into law. If the mayor vetoes a bill, the Council has 30 days to override the veto by a two-thirds majority vote.</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>[21, 354, 796, 795, 580]</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>[0.7843536138534546, 0.7420654296875, 0.7181326150894165, 0.7136199474334717, 0.70298832654953]</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>["Bills can be introduced to Parliament in a number of ways; the Scottish Government can introduce new laws or amendments to existing laws as a bill; a committee of the Parliament can present a bill in one of the areas under its remit; a member of the Scottish Parliament can introduce a bill as a private member; or a private bill can be submitted to Parliament by an outside proposer. Most draft laws are government bills introduced by ministers in the governing party. Bills pass through Parliament in a number of stages:", "Immediately after Decision Time a \"Members Debate\" is held, which lasts for 45 minutes. Members Business is a debate on a motion proposed by an MSP who is not a Scottish minister. Such motions are on issues which may be of interest to a particular area such as a member's own constituency, an upcoming or past event or any other item which would otherwise not be accorded official parliamentary time. As well as the proposer, other members normally contribute to the debate. The relevant minister, whose department the debate and motion relate to \"winds up\" the debate by speaking after all other participants.", "in the legislative process still remains limited because no member can actually or pass legislation without the Commission and Council, meaning power (\"kratia\") is not in the hands of directly elected representatives of the people (\"demos\"): in the EU it is not yet true that \"the administration is in the hands of the many and not of the few.\"", "be the body representing member states - in the Parliament citizens of smaller member states have more voice than citizens in larger member states. MEPs divide, as they do in national Parliaments, along political party lines: the conservative European People's Party is currently the largest, and the Party of European Socialists leads the opposition. Parties do not receive public funds from the EU, as the Court of Justice held in Parti écologiste \"Les Verts\" v Parliament that this was entirely an issue to be regulated by the member states. The Parliament's powers include calling inquiries into maladministration or appoint an Ombudsman pending any court proceedings. It can require the Commission respond to questions and by a two-thirds majority can censure the whole Commission (as happened to the Santer Commission in 1999). In some cases, the Parliament has explicit consultation rights, which the Commission must genuinely follow. However its role participation in the legislative process still remains limited because no member can actually or pass legislation without the Commission and Council, meaning power (\"kratia\") is not in the hands of directly elected representatives of the people (\"demos\"): in the EU it is not yet true that \"the administration is in the", "Legislative power in Warsaw is vested in a unicameral Warsaw City Council (Rada Miasta), which comprises 60 members. Council members are elected directly every four years. Like most legislative bodies, the City Council divides itself into committees which have the oversight of various functions of the city government. Bills passed by a simple majority are sent to the mayor (the President of Warsaw), who may sign them into law. If the mayor vetoes a bill, the Council has 30 days to override the veto by a two-thirds majority vote."]</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1532,21 +1187,6 @@
 The university runs a number of academic institutions and programs apart from its undergraduate and postgraduate schools. It operates the University of Chicago Laboratory Schools (a private day school for K-12 students and day care), the Sonia Shankman Orthogenic School (a residential treatment program for those with behavioral and emotional problems), and four public charter schools on the South Side of Chicago administered by the university's Urban Education Institute. In addition, the Hyde Park Day School, a school for students with learning disabilities, maintains a location on the University of Chicago campus. Since 1983, the University of Chicago has maintained the University of Chicago School Mathematics Project, a mathematics program used in urban primary and secondary schools. The university runs a program called the Council on Advanced Studies in the Social Sciences and Humanities, which administers interdisciplinary workshops to provide a forum for graduate students, faculty, and visiting scholars to present scholarly work in progress. The university also operates the University of Chicago Press, the largest university press in the United States.</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>[22, 320, 524, 707, 3]</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>[0.7813141942024231, 0.7384185194969177, 0.735183835029602, 0.7256506085395813, 0.7206108570098877]</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>["Harvard has purchased tracts of land in Allston, a walk across the Charles River from Cambridge, with the intent of major expansion southward. The university now owns approximately fifty percent more land in Allston than in Cambridge. Proposals to connect the Cambridge campus with the new Allston campus include new and enlarged bridges, a shuttle service and/or a tram. Plans also call for sinking part of Storrow Drive (at Harvard's expense) for replacement with park land and pedestrian access to the Charles River, as well as the construction of bike paths, and buildings throughout the Allston campus. The institution asserts that such expansion will benefit not only the school, but surrounding community, pointing to such features as the enhanced transit infrastructure, possible shuttles open to the public, and park space which will also be publicly accessible.", "In terms of housing stock, the authority is one of few authorities to see the proportion of detached homes rise in the 2010 Census (to 7.8%), in this instance this was coupled with a similar rise in flats and waterside apartments to 25.6%, and the proportion of converted or shared houses in 2011 renders this dwelling type within the highest of the five colour-coded brackets at 5.9%, and on a par with Oxford and Reading, greater than Manchester and Liverpool and below a handful of historic densely occupied, arguably overinflated markets in the local authorities: Harrogate, Cheltenham, Bath, inner London, Hastings, Brighton and Tunbridge Wells.", "Private schools generally prefer to be called independent schools, because of their freedom to operate outside of government and local government control. Some of these are also known as public schools. Preparatory schools in the UK prepare pupils aged up to 13 years old to enter public schools. The name \"public school\" is based on the fact that the schools were open to pupils from anywhere, and not merely to those from a certain locality, and of any religion or occupation. According to The Good Schools Guide approximately 9 per cent of children being educated in the UK are doing so at fee-paying schools at GSCE level and 13 per cent at A-level.[citation needed] Many independent schools are single-sex (though this is becoming less common). Fees range from under £3,000 to £21,000 and above per year for day pupils, rising to £27,000+ per year for boarders. For details in Scotland, see \"Meeting the Cost\".", "spend $2.5 million to convert 20 acres (80,937 m2) of land in Hollywood into what would become The Prospect Studios, and construct a transmitter on Mount Wilson, in anticipation of the launch of KECA-TV, which was scheduled to begin operations on August 1 (but would not actually sign on until September 16).", "The university runs a number of academic institutions and programs apart from its undergraduate and postgraduate schools. It operates the University of Chicago Laboratory Schools (a private day school for K-12 students and day care), the Sonia Shankman Orthogenic School (a residential treatment program for those with behavioral and emotional problems), and four public charter schools on the South Side of Chicago administered by the university's Urban Education Institute. In addition, the Hyde Park Day School, a school for students with learning disabilities, maintains a location on the University of Chicago campus. Since 1983, the University of Chicago has maintained the University of Chicago School Mathematics Project, a mathematics program used in urban primary and secondary schools. The university runs a program called the Council on Advanced Studies in the Social Sciences and Humanities, which administers interdisciplinary workshops to provide a forum for graduate students, faculty, and visiting scholars to present scholarly work in progress. The university also operates the University of Chicago Press, the largest university press in the United States."]</t>
-        </is>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1578,21 +1218,6 @@
 These attacks resonated with conservative Muslims and the problem did not go away with Saddam's defeat either, since American troops remained stationed in the kingdom, and a de facto cooperation with the Palestinian-Israeli peace process developed. Saudi Arabia attempted to compensate for its loss of prestige among these groups by repressing those domestic Islamists who attacked it (bin Laden being a prime example), and increasing aid to Islamic groups (Islamist madrassas around the world and even aiding some violent Islamist groups) that did not, but its pre-war influence on behalf of moderation was greatly reduced. One result of this was a campaign of attacks on government officials and tourists in Egypt, a bloody civil war in Algeria and Osama bin Laden's terror attacks climaxing in the 9/11 attack.</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>[23, 27, 439, 493, 215]</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>[0.7477900981903076, 0.7268380522727966, 0.7168492674827576, 0.7089123725891113, 0.7085468173027039]</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>["During the 1970s and sometimes later, Western and pro-Western governments often supported sometimes fledgling Islamists and Islamist groups that later came to be seen as dangerous enemies. Islamists were considered by Western governments bulwarks against—what were thought to be at the time—more dangerous leftist/communist/nationalist insurgents/opposition, which Islamists were correctly seen as opposing. The US spent billions of dollars to aid the mujahideen Muslim Afghanistan enemies of the Soviet Union, and non-Afghan veterans of the war returned home with their prestige, \"experience, ideology, and weapons\", and had considerable impact.", "In 1979, the Soviet Union deployed its 40th Army into Afghanistan, attempting to suppress an Islamic rebellion against an allied Marxist regime in the Afghan Civil War. The conflict, pitting indigenous impoverished Muslims (mujahideen) against an anti-religious superpower, galvanized thousands of Muslims around the world to send aid and sometimes to go themselves to fight for their faith. Leading this pan-Islamic effort was Palestinian sheikh Abdullah Yusuf Azzam. While the military effectiveness of these \"Afghan Arabs\" was marginal, an estimated 16,000 to 35,000 Muslim volunteers came from around the world came to fight in Afghanistan.", "The central highlands were already home to over a million members of the Kikuyu people, most of whom had no land claims in European terms and lived as itinerant farmers. To protect their interests, the settlers banned the growing of coffee, introduced a hut tax, and the landless were granted less and less land in exchange for their labour. A massive exodus to the cities ensued as their ability to provide a living from the land dwindled. There were 80,000 white settlers living in Kenya in the 1950s.", "In 1874, Tesla evaded being drafted into the Austro-Hungarian Army in Smiljan by running away to Tomingaj, near Gračac. There, he explored the mountains in hunter's garb. Tesla said that this contact with nature made him stronger, both physically and mentally. He read many books while in Tomingaj, and later said that Mark Twain's works had helped him to miraculously recover from his earlier illness.", "These attacks resonated with conservative Muslims and the problem did not go away with Saddam's defeat either, since American troops remained stationed in the kingdom, and a de facto cooperation with the Palestinian-Israeli peace process developed. Saudi Arabia attempted to compensate for its loss of prestige among these groups by repressing those domestic Islamists who attacked it (bin Laden being a prime example), and increasing aid to Islamic groups (Islamist madrassas around the world and even aiding some violent Islamist groups) that did not, but its pre-war influence on behalf of moderation was greatly reduced. One result of this was a campaign of attacks on government officials and tourists in Egypt, a bloody civil war in Algeria and Osama bin Laden's terror attacks climaxing in the 9/11 attack."]</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1624,21 +1249,6 @@
 During the mid-Eocene, it is believed that the drainage basin of the Amazon was split along the middle of the continent by the Purus Arch. Water on the eastern side flowed toward the Atlantic, while to the west water flowed toward the Pacific across the Amazonas Basin. As the Andes Mountains rose, however, a large basin was created that enclosed a lake; now known as the Solimões Basin. Within the last 5–10 million years, this accumulating water broke through the Purus Arch, joining the easterly flow toward the Atlantic.</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>[24, 5, 555, 675, 565]</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>[0.857988715171814, 0.78989577293396, 0.7743000388145447, 0.7660484313964844, 0.7655718922615051]</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>["In 2010 the Amazon rainforest experienced another severe drought, in some ways more extreme than the 2005 drought. The affected region was approximate 1,160,000 square miles (3,000,000 km2) of rainforest, compared to 734,000 square miles (1,900,000 km2) in 2005. The 2010 drought had three epicenters where vegetation died off, whereas in 2005 the drought was focused on the southwestern part. The findings were published in the journal Science. In a typical year the Amazon absorbs 1.5 gigatons of carbon dioxide; during 2005 instead 5 gigatons were released and in 2010 8 gigatons were released.", "The first European to travel the length of the Amazon River was Francisco de Orellana in 1542. The BBC's Unnatural Histories presents evidence that Orellana, rather than exaggerating his claims as previously thought, was correct in his observations that a complex civilization was flourishing along the Amazon in the 1540s. It is believed that the civilization was later devastated by the spread of diseases from Europe, such as smallpox. Since the 1970s, numerous geoglyphs have been discovered on deforested land dating between AD 0–1250, furthering claims about Pre-Columbian civilizations. Ondemar Dias is accredited with first discovering the geoglyphs in 1977 and Alceu Ranzi with furthering their discovery after flying over Acre. The BBC's Unnatural Histories presented evidence that the Amazon rainforest, rather than being a pristine wilderness, has been shaped by man for at least 11,000 years through practices such as forest gardening and terra preta.", "For a long time, it was thought that the Amazon rainforest was only ever sparsely populated, as it was impossible to sustain a large population through agriculture given the poor soil. Archeologist Betty Meggers was a prominent proponent of this idea, as described in her book Amazonia: Man and Culture in a Counterfeit Paradise. She claimed that a population density of 0.2 inhabitants per square kilometre (0.52/sq mi) is the maximum that can be sustained in the rainforest through hunting, with agriculture needed to host a larger population. However, recent anthropological findings have suggested that the region was actually densely populated. Some 5 million people may have lived in the Amazon region in AD 1500, divided between dense coastal settlements, such as that at Marajó, and inland dwellers. By 1900 the population had fallen to 1 million and by the early 1980s it was less than 200,000.", "Between 1991 and 2000, the total area of forest lost in the Amazon rose from 415,000 to 587,000 square kilometres (160,000 to 227,000 sq mi), with most of the lost forest becoming pasture for cattle. Seventy percent of formerly forested land in the Amazon, and 91% of land deforested since 1970, is used for livestock pasture. Currently, Brazil is the second-largest global producer of soybeans after the United States. New research however, conducted by Leydimere Oliveira et al., has shown that the more rainforest is logged in the Amazon, the less precipitation reaches the area and so the lower the yield per hectare becomes. So despite the popular perception, there has been no economical advantage for Brazil from logging rainforest zones and converting these to pastoral fields.", "During the mid-Eocene, it is believed that the drainage basin of the Amazon was split along the middle of the continent by the Purus Arch. Water on the eastern side flowed toward the Atlantic, while to the west water flowed toward the Pacific across the Amazonas Basin. As the Andes Mountains rose, however, a large basin was created that enclosed a lake; now known as the Solimões Basin. Within the last 5–10 million years, this accumulating water broke through the Purus Arch, joining the easterly flow toward the Atlantic."]</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1670,21 +1280,6 @@
 Apollo 5 (AS-204) was the first unmanned test flight of LM in Earth orbit, launched from pad 37 on January 22, 1968, by the Saturn IB that would have been used for Apollo 1. The LM engines were successfully test-fired and restarted, despite a computer programming error which cut short the first descent stage firing. The ascent engine was fired in abort mode, known as a "fire-in-the-hole" test, where it was lit simultaneously with jettison of the descent stage. Although Grumman wanted a second unmanned test, George Low decided the next LM flight would be manned.</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>[308, 268, 770, 379, 429]</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>[0.7662948966026306, 0.7526673078536987, 0.7522671222686768, 0.7467450499534607, 0.739802360534668]</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>["Apollo ran from 1961 to 1972, and was supported by the two-man Gemini program which ran concurrently with it from 1962 to 1966. Gemini missions developed some of the space travel techniques that were necessary for the success of the Apollo missions. Apollo used Saturn family rockets as launch vehicles. Apollo/Saturn vehicles were also used for an Apollo Applications Program, which consisted of Skylab, a space station that supported three manned missions in 1973–74, and the Apollo–Soyuz Test Project, a joint Earth orbit mission with the Soviet Union in 1975.", "The crew of Apollo 8 sent the first live televised pictures of the Earth and the Moon back to Earth, and read from the creation story in the Book of Genesis, on Christmas Eve, 1968. An estimated one-quarter of the population of the world saw—either live or delayed—the Christmas Eve transmission during the ninth orbit of the Moon. The mission and Christmas provided an inspiring end to 1968, which had been a troubled year for the US, marked by Vietnam War protests, race riots, and the assassinations of civil rights leader Martin Luther King, Jr., and Senator Robert F. Kennedy.", "About the time of the first landing in 1969, it was decided to use an existing Saturn V to launch the Skylab orbital laboratory pre-built on the ground, replacing the original plan to construct it in orbit from several Saturn IB launches; this eliminated Apollo 20. NASA's yearly budget also began to shrink in light of the successful landing, and NASA also had to make funds available for the development of the upcoming Space Shuttle. By 1971, the decision was made to also cancel missions 18 and 19. The two unused Saturn Vs became museum exhibits at the John F. Kennedy Space Center on Merritt Island, Florida, George C. Marshall Space Center in Huntsville, Alabama, Michoud Assembly Facility in New Orleans, Louisiana, and Lyndon B. Johnson Space Center in Houston, Texas.", "In December 1966, the AS-205 mission was canceled, since the validation of the CSM would be accomplished on the 14-day first flight, and AS-205 would have been devoted to space experiments and contribute no new engineering knowledge about the spacecraft. Its Saturn IB was allocated to the dual mission, now redesignated AS-205/208 or AS-258, planned for August 1967. McDivitt, Scott and Schweickart were promoted to the prime AS-258 crew, and Schirra, Eisele and Cunningham were reassigned as the Apollo 1 backup crew.", "Apollo 5 (AS-204) was the first unmanned test flight of LM in Earth orbit, launched from pad 37 on January 22, 1968, by the Saturn IB that would have been used for Apollo 1. The LM engines were successfully test-fired and restarted, despite a computer programming error which cut short the first descent stage firing. The ascent engine was fired in abort mode, known as a \"fire-in-the-hole\" test, where it was lit simultaneously with jettison of the descent stage. Although Grumman wanted a second unmanned test, George Low decided the next LM flight would be manned."]</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1716,21 +1311,6 @@
 In 2012 the Economist Intelligence Unit ranked Warsaw as the 32nd most liveable city in the world. It was also ranked as one of the most liveable cities in Central Europe. Today Warsaw is considered an "Alpha–" global city, a major international tourist destination and a significant cultural, political and economic hub. Warsaw's economy, by a wide variety of industries, is characterised by FMCG manufacturing, metal processing, steel and electronic manufacturing and food processing. The city is a significant centre of research and development, BPO, ITO, as well as of the Polish media industry. The Warsaw Stock Exchange is one of the largest and most important in Central and Eastern Europe. Frontex, the European Union agency for external border security, has its headquarters in Warsaw. It has been said that Warsaw, together with Frankfurt, London, Paris and Barcelona is one of the cities with the highest number of skyscrapers in the European Union. Warsaw has also been called "Eastern Europe’s chic cultural capital with thriving art and club scenes and serious restaurants".</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>[337, 26, 396, 58, 35]</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>[0.8942301273345947, 0.8637393116950989, 0.8440546989440918, 0.813408374786377, 0.8107466101646423]</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>["Warsaw remained the capital of the Polish–Lithuanian Commonwealth until 1796, when it was annexed by the Kingdom of Prussia to become the capital of the province of South Prussia. Liberated by Napoleon's army in 1806, Warsaw was made the capital of the newly created Duchy of Warsaw. Following the Congress of Vienna of 1815, Warsaw became the centre of the Congress Poland, a constitutional monarchy under a personal union with Imperial Russia. The Royal University of Warsaw was established in 1816.", "In 1529, Warsaw for the first time became the seat of the General Sejm, permanent from 1569. In 1573 the city gave its name to the Warsaw Confederation, formally establishing religious freedom in the Polish–Lithuanian Commonwealth. Due to its central location between the Commonwealth's capitals of Kraków and Vilnius, Warsaw became the capital of the Commonwealth and the Crown of the Kingdom of Poland when King Sigismund III Vasa moved his court from Kraków to Warsaw in 1596. In the following years the town expanded towards the suburbs. Several private independent districts were established, the property of aristocrats and the gentry, which were ruled by their own laws. Three times between 1655–1658 the city was under siege and three times it was taken and pillaged by the Swedish, Brandenburgian and Transylvanian forces.", "Warsaw was occupied by Germany from 4 August 1915 until November 1918. The Allied Armistice terms required in Article 12 that Germany withdraw from areas controlled by Russia in 1914, which included Warsaw. Germany did so, and underground leader Piłsudski returned to Warsaw on 11 November and set up what became the Second Polish Republic, with Warsaw the capital. In the course of the Polish-Bolshevik War of 1920, the huge Battle of Warsaw was fought on the eastern outskirts of the city in which the capital was successfully defended and the Red Army defeated. Poland stopped by itself the full brunt of the Red Army and defeated an idea of the \"export of the revolution\".", "After World War II, under a Communist regime set up by the conquering Soviets, the \"Bricks for Warsaw\" campaign was initiated, and large prefabricated housing projects were erected in Warsaw to address the housing shortage, along with other typical buildings of an Eastern Bloc city, such as the Palace of Culture and Science, a gift from the Soviet Union. The city resumed its role as the capital of Poland and the country's centre of political and economic life. Many of the historic streets, buildings, and churches were restored to their original form. In 1980, Warsaw's historic Old Town was inscribed onto UNESCO's World Heritage list.", "In 2012 the Economist Intelligence Unit ranked Warsaw as the 32nd most liveable city in the world. It was also ranked as one of the most liveable cities in Central Europe. Today Warsaw is considered an \"Alpha–\" global city, a major international tourist destination and a significant cultural, political and economic hub. Warsaw's economy, by a wide variety of industries, is characterised by FMCG manufacturing, metal processing, steel and electronic manufacturing and food processing. The city is a significant centre of research and development, BPO, ITO, as well as of the Polish media industry. The Warsaw Stock Exchange is one of the largest and most important in Central and Eastern Europe. Frontex, the European Union agency for external border security, has its headquarters in Warsaw. It has been said that Warsaw, together with Frankfurt, London, Paris and Barcelona is one of the cities with the highest number of skyscrapers in the European Union. Warsaw has also been called \"Eastern Europe’s chic cultural capital with thriving art and club scenes and serious restaurants\"."]</t>
-        </is>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1762,21 +1342,6 @@
 The Taliban were spawned by the thousands of madrasahs the Deobandi movement established for impoverished Afghan refugees and supported by governmental and religious groups in neighboring Pakistan. The Taliban differed from other Islamist movements to the point where they might be more properly described as Islamic fundamentalist or neofundamentalist, interested in spreading "an idealized and systematized version of conservative tribal village customs" under the label of Sharia to an entire country. Their ideology was also described as being influenced by Wahhabism, and the extremist jihadism of their guest Osama bin Laden.</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>[27, 215, 23, 97, 258]</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>[0.8339310884475708, 0.7858116626739502, 0.7783777117729187, 0.760549783706665, 0.7567926645278931]</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>["In 1979, the Soviet Union deployed its 40th Army into Afghanistan, attempting to suppress an Islamic rebellion against an allied Marxist regime in the Afghan Civil War. The conflict, pitting indigenous impoverished Muslims (mujahideen) against an anti-religious superpower, galvanized thousands of Muslims around the world to send aid and sometimes to go themselves to fight for their faith. Leading this pan-Islamic effort was Palestinian sheikh Abdullah Yusuf Azzam. While the military effectiveness of these \"Afghan Arabs\" was marginal, an estimated 16,000 to 35,000 Muslim volunteers came from around the world came to fight in Afghanistan.", "These attacks resonated with conservative Muslims and the problem did not go away with Saddam's defeat either, since American troops remained stationed in the kingdom, and a de facto cooperation with the Palestinian-Israeli peace process developed. Saudi Arabia attempted to compensate for its loss of prestige among these groups by repressing those domestic Islamists who attacked it (bin Laden being a prime example), and increasing aid to Islamic groups (Islamist madrassas around the world and even aiding some violent Islamist groups) that did not, but its pre-war influence on behalf of moderation was greatly reduced. One result of this was a campaign of attacks on government officials and tourists in Egypt, a bloody civil war in Algeria and Osama bin Laden's terror attacks climaxing in the 9/11 attack.", "During the 1970s and sometimes later, Western and pro-Western governments often supported sometimes fledgling Islamists and Islamist groups that later came to be seen as dangerous enemies. Islamists were considered by Western governments bulwarks against—what were thought to be at the time—more dangerous leftist/communist/nationalist insurgents/opposition, which Islamists were correctly seen as opposing. The US spent billions of dollars to aid the mujahideen Muslim Afghanistan enemies of the Soviet Union, and non-Afghan veterans of the war returned home with their prestige, \"experience, ideology, and weapons\", and had considerable impact.", "\"The Islamic State\", formerly known as the \"Islamic State of Iraq and the Levant\" and before that as the \"Islamic State of Iraq\", (and called the acronym Daesh by its many detractors), is a Wahhabi/Salafi jihadist extremist militant group which is led by and mainly composed of Sunni Arabs from Iraq and Syria. In 2014, the group proclaimed itself a caliphate, with religious, political and military authority over all Muslims worldwide. As of March 2015[update], it had control over territory occupied by ten million people in Iraq and Syria, and has nominal control over small areas of Libya, Nigeria and Afghanistan. (While a self-described state, it lacks international recognition.) The group also operates or has affiliates in other parts of the world, including North Africa and South Asia.", "The Taliban were spawned by the thousands of madrasahs the Deobandi movement established for impoverished Afghan refugees and supported by governmental and religious groups in neighboring Pakistan. The Taliban differed from other Islamist movements to the point where they might be more properly described as Islamic fundamentalist or neofundamentalist, interested in spreading \"an idealized and systematized version of conservative tribal village customs\" under the label of Sharia to an entire country. Their ideology was also described as being influenced by Wahhabism, and the extremist jihadism of their guest Osama bin Laden."]</t>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1808,21 +1373,6 @@
 Colonel Monckton, in the sole British success that year, captured Fort Beauséjour in June 1755, cutting the French fortress at Louisbourg off from land-based reinforcements. To cut vital supplies to Louisbourg, Nova Scotia's Governor Charles Lawrence ordered the deportation of the French-speaking Acadian population from the area. Monckton's forces, including companies of Rogers' Rangers, forcibly removed thousands of Acadians, chasing down many who resisted, and sometimes committing atrocities. More than any other factor, the cutting off of supplies to Louisbourg led to its demise. The Acadian resistance, in concert with native allies, including the Mi'kmaq, was sometimes quite stiff, with ongoing frontier raids (against Dartmouth and Lunenburg among others). Other than the campaigns to expel the Acadians (ranging around the Bay of Fundy, on the Petitcodiac and St. John rivers, and Île Saint-Jean), the only clashes of any size were at Petitcodiac in 1755 and at Bloody Creek near Annapolis Royal in 1757.</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>[28, 654, 709, 535, 127]</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>[0.8130683898925781, 0.7950687408447266, 0.7834105491638184, 0.7723952531814575, 0.7721111178398132]</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>["Loudoun, a capable administrator but a cautious field commander, planned one major operation for 1757: an attack on New France's capital, Quebec. Leaving a sizable force at Fort William Henry to distract Montcalm, he began organizing for the expedition to Quebec. He was then ordered by William Pitt, the Secretary of State responsible for the colonies, to attack Louisbourg first. Beset by delays of all kinds, the expedition was finally ready to sail from Halifax, Nova Scotia in early August. In the meantime French ships had escaped the British blockade of the French coast, and a fleet outnumbering the British one awaited Loudoun at Louisbourg. Faced with this strength, Loudoun returned to New York amid news that a massacre had occurred at Fort William Henry.", "Braddock (with George Washington as one of his aides) led about 1,500 army troops and provincial militia on an expedition in June 1755 to take Fort Duquesne. The expedition was a disaster. It was attacked by French and Indian soldiers ambushing them from up in trees and behind logs. Braddock called for a retreat. He was killed. Approximately 1,000 British soldiers were killed or injured. The remaining 500 British troops, led by George Washington, retreated to Virginia. Two future opponents in the American Revolutionary War, Washington and Thomas Gage, played key roles in organizing the retreat.", "When Céloron's expedition arrived at Logstown, the Native Americans in the area informed Céloron that they owned the Ohio Country and that they would trade with the British regardless of the French. Céloron continued south until his expedition reached the confluence of the Ohio and the Miami rivers, which lay just south of the village of Pickawillany, the home of the Miami chief known as \"Old Briton\". Céloron threatened \"Old Briton\" with severe consequences if he continued to trade with the British. \"Old Briton\" ignored the warning. Disappointed, Céloron returned to Montreal in November 1749.", "On March 17, 1752, the Governor-General of New France, Marquis de la Jonquière, died and was temporarily replaced by Charles le Moyne de Longueuil. His permanent replacement, the Marquis Duquesne, did not arrive in New France until 1752 to take over the post. The continuing British activity in the Ohio territories prompted Longueuil to dispatch another expedition to the area under the command of Charles Michel de Langlade, an officer in the Troupes de la Marine. Langlade was given 300 men, including French-Canadians and warriors of the Ottawa. His objective was to punish the Miami people of Pickawillany for not following Céloron's orders to cease trading with the British. On June 21, the French war party attacked the trading centre at Pickawillany, capturing three traders and killing 14 people of the Miami nation, including Old Briton. He was reportedly ritually cannibalized by some aboriginal members of the expedition.", "Colonel Monckton, in the sole British success that year, captured Fort Beauséjour in June 1755, cutting the French fortress at Louisbourg off from land-based reinforcements. To cut vital supplies to Louisbourg, Nova Scotia's Governor Charles Lawrence ordered the deportation of the French-speaking Acadian population from the area. Monckton's forces, including companies of Rogers' Rangers, forcibly removed thousands of Acadians, chasing down many who resisted, and sometimes committing atrocities. More than any other factor, the cutting off of supplies to Louisbourg led to its demise. The Acadian resistance, in concert with native allies, including the Mi'kmaq, was sometimes quite stiff, with ongoing frontier raids (against Dartmouth and Lunenburg among others). Other than the campaigns to expel the Acadians (ranging around the Bay of Fundy, on the Petitcodiac and St. John rivers, and Île Saint-Jean), the only clashes of any size were at Petitcodiac in 1755 and at Bloody Creek near Annapolis Royal in 1757."]</t>
-        </is>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1854,21 +1404,6 @@
 in interceptions. In week 10, Manning suffered a partial tear of the plantar fasciitis in his left foot. He set the NFL's all-time record for career passing yards in this game, but was benched after throwing four interceptions in favor of backup quarterback Brock Osweiler, who took over as the starter for most of the remainder of the regular season. Osweiler was injured, however, leading to Manning's return during the Week 17 regular season finale, where the Broncos were losing 13–7 against the 4–11 San Diego Chargers, resulting in Manning re-claiming the starting quarterback position for the playoffs by leading the team to a key 27–20 win that enabled the team to clinch the number one overall AFC seed. Under defensive coordinator Wade Phillips, the Broncos' defense ranked number one in total yards allowed, passing yards allowed and sacks, and like the previous three seasons, the team has continued to set numerous individual, league and franchise records. With the defense carrying the team despite the issues with the offense, the Broncos finished the regular season with a 12–4 record and earned home-field advantage throughout the AFC playoffs.</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>[29, 269, 684, 6, 206]</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>[0.7968679666519165, 0.7960789799690247, 0.768484890460968, 0.7657801508903503, 0.7622981667518616]</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>["The Panthers finished the regular season with a 15–1 record, and quarterback Cam Newton was named the NFL Most Valuable Player (MVP). They defeated the Arizona Cardinals 49–15 in the NFC Championship Game and advanced to their second Super Bowl appearance since the franchise was founded in 1995. The Broncos finished the regular season with a 12–4 record, and denied the New England Patriots a chance to defend their title from Super Bowl XLIX by defeating them 20–18 in the AFC Championship Game. They joined the Patriots, Dallas Cowboys, and Pittsburgh Steelers as one of four teams that have made eight appearances in the Super Bowl.", "The Panthers beat the Seattle Seahawks in the divisional round, running up a 31–0 halftime lead and then holding off a furious second half comeback attempt to win 31–24, avenging their elimination from a year earlier. The Panthers then blew out the Arizona Cardinals in the NFC Championship Game, 49–15, racking up 487 yards and forcing seven turnovers.", "As the designated home team in the annual rotation between AFC and NFC teams, the Broncos elected to wear their road white jerseys with matching white pants. Elway stated, \"We've had Super Bowl success in our white uniforms.\" The Broncos last wore matching white jerseys and pants in the Super Bowl in Super Bowl XXXIII, Elway's last game as Denver QB, when they defeated the Atlanta Falcons 34–19. In their only other Super Bowl win in Super Bowl XXXII, Denver wore blue jerseys, which was their primary color at the time. They also lost Super Bowl XXI when they wore white jerseys, but they are 0-4 in Super Bowls when wearing orange jerseys, losing in Super Bowl XII, XXII, XXIV, and XLVIII. The only other AFC champion team to have worn white as the designated home team in the Super Bowl was the Pittsburgh Steelers; they defeated the Seattle Seahawks 21–10 in Super Bowl XL 10 seasons prior. The Broncos' decision to wear white meant the Panthers would wear their standard home uniform: black jerseys with silver pants.", "The Broncos defeated the Pittsburgh Steelers in the divisional round, 23–16, by scoring 11 points in the final three minutes of the game. They then beat the defending Super Bowl XLIX champion New England Patriots in the AFC Championship Game, 20–18, by intercepting a pass on New England's 2-point conversion attempt with 17 seconds left on the clock. Despite Manning's problems with interceptions during the season, he didn't throw any in their two playoff games.", "in interceptions. In week 10, Manning suffered a partial tear of the plantar fasciitis in his left foot. He set the NFL's all-time record for career passing yards in this game, but was benched after throwing four interceptions in favor of backup quarterback Brock Osweiler, who took over as the starter for most of the remainder of the regular season. Osweiler was injured, however, leading to Manning's return during the Week 17 regular season finale, where the Broncos were losing 13–7 against the 4–11 San Diego Chargers, resulting in Manning re-claiming the starting quarterback position for the playoffs by leading the team to a key 27–20 win that enabled the team to clinch the number one overall AFC seed. Under defensive coordinator Wade Phillips, the Broncos' defense ranked number one in total yards allowed, passing yards allowed and sacks, and like the previous three seasons, the team has continued to set numerous individual, league and franchise records. With the defense carrying the team despite the issues with the offense, the Broncos finished the regular season with a 12–4 record and earned home-field advantage throughout the AFC playoffs."]</t>
-        </is>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1900,21 +1435,6 @@
 Bethencourt took the title of King of the Canary Islands, as vassal to Henry III of Castile. In 1418, Jean's nephew Maciot de Bethencourt sold the rights to the islands to Enrique Pérez de Guzmán, 2nd Count de Niebla.</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>[535, 30, 28, 654, 842]</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>[0.822112500667572, 0.8051350116729736, 0.7790514230728149, 0.7744685411453247, 0.7568650245666504]</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>["On March 17, 1752, the Governor-General of New France, Marquis de la Jonquière, died and was temporarily replaced by Charles le Moyne de Longueuil. His permanent replacement, the Marquis Duquesne, did not arrive in New France until 1752 to take over the post. The continuing British activity in the Ohio territories prompted Longueuil to dispatch another expedition to the area under the command of Charles Michel de Langlade, an officer in the Troupes de la Marine. Langlade was given 300 men, including French-Canadians and warriors of the Ottawa. His objective was to punish the Miami people of Pickawillany for not following Céloron's orders to cease trading with the British. On June 21, the French war party attacked the trading centre at Pickawillany, capturing three traders and killing 14 people of the Miami nation, including Old Briton. He was reportedly ritually cannibalized by some aboriginal members of the expedition.", "Newcastle replaced him in January 1756 with Lord Loudoun, with Major General James Abercrombie as his second in command. Neither of these men had as much campaign experience as the trio of officers France sent to North America. French regular army reinforcements arrived in New France in May 1756, led by Major General Louis-Joseph de Montcalm and seconded by the Chevalier de Lévis and Colonel François-Charles de Bourlamaque, all experienced veterans from the War of the Austrian Succession. During that time in Europe, on May 18, 1756, England formally declared war on France, which expanded the war into Europe, which was later to be known as the Seven Years' War.", "Loudoun, a capable administrator but a cautious field commander, planned one major operation for 1757: an attack on New France's capital, Quebec. Leaving a sizable force at Fort William Henry to distract Montcalm, he began organizing for the expedition to Quebec. He was then ordered by William Pitt, the Secretary of State responsible for the colonies, to attack Louisbourg first. Beset by delays of all kinds, the expedition was finally ready to sail from Halifax, Nova Scotia in early August. In the meantime French ships had escaped the British blockade of the French coast, and a fleet outnumbering the British one awaited Loudoun at Louisbourg. Faced with this strength, Loudoun returned to New York amid news that a massacre had occurred at Fort William Henry.", "Braddock (with George Washington as one of his aides) led about 1,500 army troops and provincial militia on an expedition in June 1755 to take Fort Duquesne. The expedition was a disaster. It was attacked by French and Indian soldiers ambushing them from up in trees and behind logs. Braddock called for a retreat. He was killed. Approximately 1,000 British soldiers were killed or injured. The remaining 500 British troops, led by George Washington, retreated to Virginia. Two future opponents in the American Revolutionary War, Washington and Thomas Gage, played key roles in organizing the retreat.", "Bethencourt took the title of King of the Canary Islands, as vassal to Henry III of Castile. In 1418, Jean's nephew Maciot de Bethencourt sold the rights to the islands to Enrique Pérez de Guzmán, 2nd Count de Niebla."]</t>
-        </is>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1946,21 +1466,6 @@
 Spain ceded Florida to the British in 1763 after the French and Indian War, and the British soon constructed the King's Road connecting St. Augustine to Georgia. The road crossed the St. Johns River at a narrow point, which the Seminole called Wacca Pilatka and the British called the Cow Ford or Cowford; these names ostensibly reflect the fact that cattle were brought across the river there. The British introduced the cultivation of sugar cane, indigo and fruits as well the export of lumber. As a result, the northeastern Florida area prospered economically more than it had under the Spanish. Britain ceded control of the territory back to Spain in 1783, after its defeat in the American Revolutionary War, and the settlement at the Cow Ford continued to grow. After Spain ceded the Florida Territory to the United States in 1821, American settlers on the north side of the Cow Ford decided to plan a town, laying out the streets and plats. They soon named the town Jacksonville, after Andrew Jackson. Led by Isaiah D. Hart, residents wrote a charter for a town government, which was approved by the Florida Legislative Council on February 9, 1832.</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>[791, 725, 106, 761, 202]</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>[0.7653157114982605, 0.748794674873352, 0.7413872480392456, 0.7412694692611694, 0.7340927124023438]</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>["In the Sandgate area, to the east of the city and beside the river, resided the close-knit community of keelmen and their families. They were so called because they worked on the keels, boats that were used to transfer coal from the river banks to the waiting colliers, for export to London and elsewhere. In the 1630s about 7,000 out of 20,000 inhabitants of Newcastle died of plague, more than one-third of the population. Specifically within the year 1636, it is roughly estimated with evidence held by the Society of Antiquaries that 47% of the then population of Newcastle died from the epidemic; this may also have been the most devastating loss in any British City in this period.", "Huguenot immigrants did not disperse or settle in different parts of the country, but rather, formed three societies or congregations; one in the city of New York, another 21 miles north of New York in a town which they named New Rochelle, and a third further upstate in New Paltz. The \"Huguenot Street Historic District\" in New Paltz has been designated a National Historic Landmark site and contains the oldest street in the United States of America. A small group of Huguenots also settled on the south shore of Staten Island along the New York Harbor, for which the current neighborhood of Huguenot was named.", "In the early years, many Huguenots also settled in the area of present-day Charleston, South Carolina. In 1685, Rev. Elie Prioleau from the town of Pons in France, was among the first to settle there. He became pastor of the first Huguenot church in North America in that city. After the Revocation of the Edict of Nantes in 1685, several Huguenot families of Norman and Carolingian nobility and descent, including Edmund Bohun of Suffolk England from the Humphrey de Bohun line of French royalty descended from Charlemagne, Jean Postell of Dieppe France, Alexander Pepin, Antoine Poitevin of Orsement France, and Jacques de Bordeaux of Grenoble, immigrated to the Charleston Orange district. They were very successful at marriage and property speculation. After petitioning the British Crown in 1697 for the right to own land in the Baronies, they prospered as slave owners on the Cooper, Ashepoo, Ashley and Santee River plantations they purchased from the British Landgrave Edmund Bellinger. Some of their descendants moved into the Deep South and Texas, where they developed new plantations.", "On 30 July 1891, at the age of 35, Tesla became a naturalized citizen of the United States, and established his South Fifth Avenue laboratory, and later another at 46 E. Houston Street, in New York. He lit electric lamps wirelessly at both locations, demonstrating the potential of wireless power transmission. In the same year, he patented the Tesla coil.", "Spain ceded Florida to the British in 1763 after the French and Indian War, and the British soon constructed the King's Road connecting St. Augustine to Georgia. The road crossed the St. Johns River at a narrow point, which the Seminole called Wacca Pilatka and the British called the Cow Ford or Cowford; these names ostensibly reflect the fact that cattle were brought across the river there. The British introduced the cultivation of sugar cane, indigo and fruits as well the export of lumber. As a result, the northeastern Florida area prospered economically more than it had under the Spanish. Britain ceded control of the territory back to Spain in 1783, after its defeat in the American Revolutionary War, and the settlement at the Cow Ford continued to grow. After Spain ceded the Florida Territory to the United States in 1821, American settlers on the north side of the Cow Ford decided to plan a town, laying out the streets and plats. They soon named the town Jacksonville, after Andrew Jackson. Led by Isaiah D. Hart, residents wrote a charter for a town government, which was approved by the Florida Legislative Council on February 9, 1832."]</t>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1992,21 +1497,6 @@
 In general, there are three sectors of construction: buildings, infrastructure and industrial. Building construction is usually further divided into residential and non-residential (commercial/institutional). Infrastructure is often called heavy/highway, heavy civil or heavy engineering. It includes large public works, dams, bridges, highways, water/wastewater and utility distribution. Industrial includes refineries, process chemical, power generation, mills and manufacturing plants. There are other ways to break the industry into sectors or markets.</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>[211, 32, 35, 871, 730]</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>[0.7761452198028564, 0.7721577882766724, 0.7428798079490662, 0.7314518690109253, 0.7200450897216797]</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>["The city developed around the Roman settlement Pons Aelius and was named after the castle built in 1080 by Robert Curthose, William the Conqueror's eldest son. The city grew as an important centre for the wool trade in the 14th century, and later became a major coal mining area. The port developed in the 16th century and, along with the shipyards lower down the River Tyne, was amongst the world's largest shipbuilding and ship-repairing centres. Newcastle's economy includes corporate headquarters, learning, digital technology, retail, tourism and cultural centres, from which the city contributes £13 billion towards the United Kingdom's GVA. Among its icons are Newcastle Brown Ale; Newcastle United football club; and the Tyne Bridge. It has hosted the world's most popular half marathon, the Great North Run, since it began in 1981.", "The Swahili built Mombasa into a major port city and established trade links with other nearby city-states, as well as commercial centres in Persia, Arabia, and even India. By the 15th-century, Portuguese voyager Duarte Barbosa claimed that \"Mombasa is a place of great traffic and has a good harbour in which there are always moored small craft of many kinds and also great ships, both of which are bound from Sofala and others which come from Cambay and Melinde and others which sail to the island of Zanzibar.\"", "In 2012 the Economist Intelligence Unit ranked Warsaw as the 32nd most liveable city in the world. It was also ranked as one of the most liveable cities in Central Europe. Today Warsaw is considered an \"Alpha–\" global city, a major international tourist destination and a significant cultural, political and economic hub. Warsaw's economy, by a wide variety of industries, is characterised by FMCG manufacturing, metal processing, steel and electronic manufacturing and food processing. The city is a significant centre of research and development, BPO, ITO, as well as of the Polish media industry. The Warsaw Stock Exchange is one of the largest and most important in Central and Eastern Europe. Frontex, the European Union agency for external border security, has its headquarters in Warsaw. It has been said that Warsaw, together with Frankfurt, London, Paris and Barcelona is one of the cities with the highest number of skyscrapers in the European Union. Warsaw has also been called \"Eastern Europe’s chic cultural capital with thriving art and club scenes and serious restaurants\".", "In the 19th century, shipbuilding and heavy engineering were central to the city's prosperity; and the city was a powerhouse of the Industrial Revolution. This revolution resulted in the urbanization of the city. In 1817 the Maling company, at one time the largest pottery company in the world, moved to the city. The Victorian industrial revolution brought industrial structures that included the 2 1⁄2-mile (4.0 km) Victoria Tunnelling, built in 1842, which provided underground wagon ways to the staithes. On 3 February 1879, Mosley Street in the city, was the first public road in the world to be lit up by the incandescent lightbulb. Newcastle was one of the first cities in the world to be lit up by electric lighting. Innovations in Newcastle and surrounding areas included the development of safety lamps, Stephenson's Rocket, Lord Armstrong's artillery, Be-Ro flour, Joseph Swan's electric light bulbs, and Charles Parsons' invention of the steam turbine, which led to the revolution of marine propulsion and the production of cheap electricity. In 1882, Newcastle became the seat of an Anglican diocese, with St. Nicholas' Church becoming its cathedral.", "In general, there are three sectors of construction: buildings, infrastructure and industrial. Building construction is usually further divided into residential and non-residential (commercial/institutional). Infrastructure is often called heavy/highway, heavy civil or heavy engineering. It includes large public works, dams, bridges, highways, water/wastewater and utility distribution. Industrial includes refineries, process chemical, power generation, mills and manufacturing plants. There are other ways to break the industry into sectors or markets."]</t>
-        </is>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2038,21 +1528,6 @@
 Civil disobedients have chosen a variety of different illegal acts. Bedau writes, "There is a whole class of acts, undertaken in the name of civil disobedience, which, even if they were widely practiced, would in themselves constitute hardly more than a nuisance (e.g. trespassing at a nuclear-missile installation)...Such acts are often just a harassment and, at least to the bystander, somewhat inane...The remoteness of the connection between the disobedient act and the objectionable law lays such acts open to the charge of ineffectiveness and absurdity." Bedau also notes, though, that the very harmlessness of such entirely symbolic illegal protests toward public policy goals may serve a propaganda purpose. Some civil disobedients, such as the proprietors of illegal medical cannabis dispensaries and Voice in the Wilderness, which brought medicine to Iraq without the permission of the U.S. Government, directly achieve a desired social goal (such as the provision of medication to the sick) while openly breaking the law. Julia Butterfly Hill lived in Luna, a 180-foot (55 m)-tall, 600-year-old California Redwood tree for 738 days, successfully preventing it from being cut down.</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>[760, 33, 481, 686, 182]</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>[0.7954064607620239, 0.7757138013839722, 0.7689979672431946, 0.7567310333251953, 0.7506234645843506]</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>["Some forms of civil disobedience, such as illegal boycotts, refusals to pay taxes, draft dodging, distributed denial-of-service attacks, and sit-ins, make it more difficult for a system to function. In this way, they might be considered coercive. Brownlee notes that \"although civil disobedients are constrained in their use of coercion by their conscientious aim to engage in moral dialogue, nevertheless they may find it necessary to employ limited coercion in order to get their issue onto the table.\" The Plowshares organization temporarily closed GCSB Waihopai by padlocking the gates and using sickles to deflate one of the large domes covering two satellite dishes.", "Courts have distinguished between two types of civil disobedience: \"Indirect civil disobedience involves violating a law which is not, itself, the object of protest, whereas direct civil disobedience involves protesting the existence of a particular law by breaking that law.\" During the Vietnam War, courts typically refused to excuse the perpetrators of illegal protests from punishment on the basis of their challenging the legality of the Vietnam War; the courts ruled it was a political question. The necessity defense has sometimes been used as a shadow defense by civil disobedients to deny guilt without denouncing their politically motivated acts, and to present their political beliefs in the courtroom. However, court cases such as U.S. v. Schoon have greatly curtailed the availability of the political necessity defense. Likewise, when Carter Wentworth was charged for his role in the Clamshell Alliance's 1977 illegal occupation of the Seabrook Station Nuclear Power Plant, the judge instructed the jury to disregard his competing harms defense, and he was found guilty. Fully Informed Jury Association activists have sometimes handed out educational leaflets inside courthouses despite admonitions not to; according to FIJA, many of them have escaped prosecution because \"prosecutors have reasoned (correctly) that if they arrest", "Some civil disobedience defendants choose to make a defiant speech, or a speech explaining their actions, in allocution. In U.S. v. Burgos-Andujar, a defendant who was involved in a movement to stop military exercises by trespassing on U.S. Navy property argued to the court in allocution that \"the ones who are violating the greater law are the members of the Navy\". As a result, the judge increased her sentence from 40 to 60 days. This action was upheld because, according to the U.S. Court of Appeals for the First Circuit, her statement suggested a lack of remorse, an attempt to avoid responsibility for her actions, and even a likelihood of repeating her illegal actions. Some of the other allocution speeches given by the protesters complained about mistreatment from government officials.", "LeGrande writes that \"the formulation of a single all-encompassing definition of the term is extremely difficult, if not impossible. In reviewing the voluminous literature on the subject, the student of civil disobedience rapidly finds himself surrounded by a maze of semantical problems and grammatical niceties. Like Alice in Wonderland, he often finds that specific terminology has no more (or no less) meaning than the individual orator intends it to have.\" He encourages a distinction between lawful protest demonstration, nonviolent civil disobedience, and violent civil disobedience.", "Civil disobedients have chosen a variety of different illegal acts. Bedau writes, \"There is a whole class of acts, undertaken in the name of civil disobedience, which, even if they were widely practiced, would in themselves constitute hardly more than a nuisance (e.g. trespassing at a nuclear-missile installation)...Such acts are often just a harassment and, at least to the bystander, somewhat inane...The remoteness of the connection between the disobedient act and the objectionable law lays such acts open to the charge of ineffectiveness and absurdity.\" Bedau also notes, though, that the very harmlessness of such entirely symbolic illegal protests toward public policy goals may serve a propaganda purpose. Some civil disobedients, such as the proprietors of illegal medical cannabis dispensaries and Voice in the Wilderness, which brought medicine to Iraq without the permission of the U.S. Government, directly achieve a desired social goal (such as the provision of medication to the sick) while openly breaking the law. Julia Butterfly Hill lived in Luna, a 180-foot (55 m)-tall, 600-year-old California Redwood tree for 738 days, successfully preventing it from being cut down."]</t>
-        </is>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2084,21 +1559,6 @@
 Warsaw was occupied by Germany from 4 August 1915 until November 1918. The Allied Armistice terms required in Article 12 that Germany withdraw from areas controlled by Russia in 1914, which included Warsaw. Germany did so, and underground leader Piłsudski returned to Warsaw on 11 November and set up what became the Second Polish Republic, with Warsaw the capital. In the course of the Polish-Bolshevik War of 1920, the huge Battle of Warsaw was fought on the eastern outskirts of the city in which the capital was successfully defended and the Red Army defeated. Poland stopped by itself the full brunt of the Red Army and defeated an idea of the "export of the revolution".</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>[35, 41, 58, 26, 396]</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>[0.8750302195549011, 0.794160783290863, 0.7629186511039734, 0.7564669847488403, 0.7388185858726501]</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>["In 2012 the Economist Intelligence Unit ranked Warsaw as the 32nd most liveable city in the world. It was also ranked as one of the most liveable cities in Central Europe. Today Warsaw is considered an \"Alpha–\" global city, a major international tourist destination and a significant cultural, political and economic hub. Warsaw's economy, by a wide variety of industries, is characterised by FMCG manufacturing, metal processing, steel and electronic manufacturing and food processing. The city is a significant centre of research and development, BPO, ITO, as well as of the Polish media industry. The Warsaw Stock Exchange is one of the largest and most important in Central and Eastern Europe. Frontex, the European Union agency for external border security, has its headquarters in Warsaw. It has been said that Warsaw, together with Frankfurt, London, Paris and Barcelona is one of the cities with the highest number of skyscrapers in the European Union. Warsaw has also been called \"Eastern Europe’s chic cultural capital with thriving art and club scenes and serious restaurants\".", "In 1939, c. 1,300,000 people lived in Warsaw, but in 1945 – only 420,000. During the first years after the war, the population growth was c. 6%, so shortly the city started to suffer from the lack of flats and of areas for new houses. The first remedial measure was the Warsaw area enlargement (1951) – but the city authorities were still forced to introduce residency registration limitations: only the spouses and children of the permanent residents as well as some persons of public importance (like renowned specialists) were allowed to get the registration, hence halving the population growth in the following years. It also bolstered some kind of conviction among Poles that Varsovians thought of themselves as better only because they lived in the capital. Unfortunately this belief still lives on in Poland (although not as much as it used to be) – even though since 1990 there are no limitations to residency registration anymore.", "After World War II, under a Communist regime set up by the conquering Soviets, the \"Bricks for Warsaw\" campaign was initiated, and large prefabricated housing projects were erected in Warsaw to address the housing shortage, along with other typical buildings of an Eastern Bloc city, such as the Palace of Culture and Science, a gift from the Soviet Union. The city resumed its role as the capital of Poland and the country's centre of political and economic life. Many of the historic streets, buildings, and churches were restored to their original form. In 1980, Warsaw's historic Old Town was inscribed onto UNESCO's World Heritage list.", "In 1529, Warsaw for the first time became the seat of the General Sejm, permanent from 1569. In 1573 the city gave its name to the Warsaw Confederation, formally establishing religious freedom in the Polish–Lithuanian Commonwealth. Due to its central location between the Commonwealth's capitals of Kraków and Vilnius, Warsaw became the capital of the Commonwealth and the Crown of the Kingdom of Poland when King Sigismund III Vasa moved his court from Kraków to Warsaw in 1596. In the following years the town expanded towards the suburbs. Several private independent districts were established, the property of aristocrats and the gentry, which were ruled by their own laws. Three times between 1655–1658 the city was under siege and three times it was taken and pillaged by the Swedish, Brandenburgian and Transylvanian forces.", "Warsaw was occupied by Germany from 4 August 1915 until November 1918. The Allied Armistice terms required in Article 12 that Germany withdraw from areas controlled by Russia in 1914, which included Warsaw. Germany did so, and underground leader Piłsudski returned to Warsaw on 11 November and set up what became the Second Polish Republic, with Warsaw the capital. In the course of the Polish-Bolshevik War of 1920, the huge Battle of Warsaw was fought on the eastern outskirts of the city in which the capital was successfully defended and the Red Army defeated. Poland stopped by itself the full brunt of the Red Army and defeated an idea of the \"export of the revolution\"."]</t>
-        </is>
-      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2130,21 +1590,6 @@
 Seamans' establishment of an ad-hoc committee headed by his special technical assistant Nicholas E. Golovin in July 1961, to recommend a launch vehicle to be used in the Apollo program, represented a turning point in NASA's mission mode decision. This committee recognized that the chosen mode was an important part of the launch vehicle choice, and recommended in favor of a hybrid EOR-LOR mode. Its consideration of LOR —as well as Houbolt's ceaseless work— played an important role in publicizing the workability of the approach. In late 1961 and early 1962, members of the Manned Spacecraft Center began to come around to support LOR, including the newly hired deputy director of the Office of Manned Space Flight, Joseph Shea, who became a champion of LOR. The engineers at Marshall Space Flight Center (MSFC) took longer to become convinced of its merits, but their conversion was announced by Wernher von Braun at a briefing in June 1962.</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>[308, 770, 379, 25, 7]</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>[0.8559946417808533, 0.8445125818252563, 0.8210453987121582, 0.8199740648269653, 0.8122600317001343]</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>["Apollo ran from 1961 to 1972, and was supported by the two-man Gemini program which ran concurrently with it from 1962 to 1966. Gemini missions developed some of the space travel techniques that were necessary for the success of the Apollo missions. Apollo used Saturn family rockets as launch vehicles. Apollo/Saturn vehicles were also used for an Apollo Applications Program, which consisted of Skylab, a space station that supported three manned missions in 1973–74, and the Apollo–Soyuz Test Project, a joint Earth orbit mission with the Soviet Union in 1975.", "About the time of the first landing in 1969, it was decided to use an existing Saturn V to launch the Skylab orbital laboratory pre-built on the ground, replacing the original plan to construct it in orbit from several Saturn IB launches; this eliminated Apollo 20. NASA's yearly budget also began to shrink in light of the successful landing, and NASA also had to make funds available for the development of the upcoming Space Shuttle. By 1971, the decision was made to also cancel missions 18 and 19. The two unused Saturn Vs became museum exhibits at the John F. Kennedy Space Center on Merritt Island, Florida, George C. Marshall Space Center in Huntsville, Alabama, Michoud Assembly Facility in New Orleans, Louisiana, and Lyndon B. Johnson Space Center in Houston, Texas.", "In December 1966, the AS-205 mission was canceled, since the validation of the CSM would be accomplished on the 14-day first flight, and AS-205 would have been devoted to space experiments and contribute no new engineering knowledge about the spacecraft. Its Saturn IB was allocated to the dual mission, now redesignated AS-205/208 or AS-258, planned for August 1967. McDivitt, Scott and Schweickart were promoted to the prime AS-258 crew, and Schirra, Eisele and Cunningham were reassigned as the Apollo 1 backup crew.", "The success of the first two landings allowed the remaining missions to be crewed with a single veteran as Commander, with two rookies. Apollo 13 launched Lovell, Jack Swigert, and Fred Haise in April 1970, headed for the Fra Mauro formation. But two days out, a liquid oxygen tank exploded, disabling the Service Module and forcing the crew to use the LM as a \"life boat\" to return to Earth. Another NASA review board was convened to determine the cause, which turned out to be a combination of damage of the tank in the factory, and a subcontractor not making a tank component according to updated design specifications. Apollo was grounded again, for the remainder of 1970 while the oxygen tank was redesigned and an extra one was added.", "Seamans' establishment of an ad-hoc committee headed by his special technical assistant Nicholas E. Golovin in July 1961, to recommend a launch vehicle to be used in the Apollo program, represented a turning point in NASA's mission mode decision. This committee recognized that the chosen mode was an important part of the launch vehicle choice, and recommended in favor of a hybrid EOR-LOR mode. Its consideration of LOR —as well as Houbolt's ceaseless work— played an important role in publicizing the workability of the approach. In late 1961 and early 1962, members of the Manned Spacecraft Center began to come around to support LOR, including the newly hired deputy director of the Office of Manned Space Flight, Joseph Shea, who became a champion of LOR. The engineers at Marshall Space Flight Center (MSFC) took longer to become convinced of its merits, but their conversion was announced by Wernher von Braun at a briefing in June 1962."]</t>
-        </is>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2176,21 +1621,6 @@
 Pink Floyd, the Australian string ensemble Fourplay, New Zealand punk band Blam Blam Blam, The Pogues, Thin Lizzy, Dub Syndicate, and the comedians Bill Bailey and Mitch Benn. Both the theme and obsessive fans were satirised on The Chaser's War on Everything. The theme tune has also appeared on many compilation CDs, and has made its way into mobile-phone ringtones. Fans have also produced and distributed their own remixes of the theme. In January 2011 the Mankind version was released as a digital download on the album Gallifrey And Beyond.</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>[37, 36, 332, 664, 563]</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>[0.8143310546875, 0.7523804903030396, 0.7188303470611572, 0.7167617678642273, 0.7140572667121887]</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>["stopped with its 1998–2002 four-note jingles for promotions and production company vanity cards following the closing credits of most of its programs over seventeen years, now it have a different and adventure-type music (with the drums of the network's four-note signature in the ending). The old four-note theme tune is still used by ABC on Demand to the beginning of the ABC show.", "In 1998, the network began using a minimalist graphical identity, designed by Pittard Sullivan, featuring a small black-and-white \"ABC Circle\" logo on a yellow background (promotions during this time also featured a sequence of still photos of the stars of its programs during the timeslot card as well as the schedule sequence that began each night's prime time lineup). A new four-note theme tune was introduced alongside the package, based around the network's \"We Love TV\" image campaign introduced that year, creating an audio signature on par with the NBC chimes, CBS' various three-note soundmarks (including the current version used since 2000) and the Fox Fanfare. The four-note signature has been updated with every television season thereafter (though variants of it used since the 1998–99 season remain in use during the production company vanity cards shown following the closing credits of most programs). In the fall of 2015, ABC is stopped with its 1998–2002 four-note jingles for promotions and production company vanity cards following the closing credits of most of its programs over seventeen years, now it have a different and adventure-type music (with the drums of the network's four-note signature in the ending). The old four-note theme tune is", "In 1962, graphic designer Paul Rand redesigned the ABC logo into its best-known (and current) form, with the lowercase letters \"abc\" enclosed in a single black circle. The new logo debuted on-air for ABC's promos at the start of the 1963–64 season. The letters are strongly reminiscent of the Bauhaus typeface designed by Herbert Bayer in the 1920s, but also share similarities with several other fonts, such as ITC Avant Garde and Horatio, and most closely resembling Chalet. The logo's simplicity made it easier to redesign and duplicate, which conferred a benefit for ABC (mostly before the advent of computer graphics).", "The 1970s and 1980s saw the emergence of many graphical imaging packages for the network in which based the logo's setting mainly on special lighting effects then under development including white, blue, pink, rainbow neon and glittering dotted lines. Among the \"ABC Circle\" logo's many variants was a 1977 ID sequence that featured a bubble on a black background representing the circle with glossy gold letters, and as such, was the first ABC identification card to have a three-dimensional appearance.", "Pink Floyd, the Australian string ensemble Fourplay, New Zealand punk band Blam Blam Blam, The Pogues, Thin Lizzy, Dub Syndicate, and the comedians Bill Bailey and Mitch Benn. Both the theme and obsessive fans were satirised on The Chaser's War on Everything. The theme tune has also appeared on many compilation CDs, and has made its way into mobile-phone ringtones. Fans have also produced and distributed their own remixes of the theme. In January 2011 the Mankind version was released as a digital download on the album Gallifrey And Beyond."]</t>
-        </is>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2222,21 +1652,6 @@
 The 1970s and 1980s saw the emergence of many graphical imaging packages for the network in which based the logo's setting mainly on special lighting effects then under development including white, blue, pink, rainbow neon and glittering dotted lines. Among the "ABC Circle" logo's many variants was a 1977 ID sequence that featured a bubble on a black background representing the circle with glossy gold letters, and as such, was the first ABC identification card to have a three-dimensional appearance.</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>[631, 64, 516, 709, 664]</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>[0.681933581829071, 0.6812793016433716, 0.6617340445518494, 0.6606945395469666, 0.660497784614563]</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>["Westwood One will carry the game throughout North America, with Kevin Harlan as play-by-play announcer, Boomer Esiason and Dan Fouts as color analysts, and James Lofton and Mark Malone as sideline reporters. Jim Gray will anchor the pre-game and halftime coverage.", "This was the first Super Bowl to feature a quarterback on both teams who was the #1 pick in their draft classes. Manning was the #1 selection of the 1998 NFL draft, while Newton was picked first in 2011. The matchup also pits the top two picks of the 2011 draft against each other: Newton for Carolina and Von Miller for Denver. Manning and Newton also set the record for the largest age difference between opposing Super Bowl quarterbacks at 13 years and 48 days (Manning was 39, Newton was 26).", "Carolina suffered a major setback when Thomas Davis, an 11-year veteran who had already overcome three ACL tears in his career, went down with a broken arm in the NFC Championship Game. Despite this, he insisted he would still find a way to play in the Super Bowl. His prediction turned out to be accurate.", "When Céloron's expedition arrived at Logstown, the Native Americans in the area informed Céloron that they owned the Ohio Country and that they would trade with the British regardless of the French. Céloron continued south until his expedition reached the confluence of the Ohio and the Miami rivers, which lay just south of the village of Pickawillany, the home of the Miami chief known as \"Old Briton\". Céloron threatened \"Old Briton\" with severe consequences if he continued to trade with the British. \"Old Briton\" ignored the warning. Disappointed, Céloron returned to Montreal in November 1749.", "The 1970s and 1980s saw the emergence of many graphical imaging packages for the network in which based the logo's setting mainly on special lighting effects then under development including white, blue, pink, rainbow neon and glittering dotted lines. Among the \"ABC Circle\" logo's many variants was a 1977 ID sequence that featured a bubble on a black background representing the circle with glossy gold letters, and as such, was the first ABC identification card to have a three-dimensional appearance."]</t>
-        </is>
-      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2268,21 +1683,6 @@
 As opposed to broadcasts of primetime series, CBS broadcast special episodes of its late night talk shows as its lead-out programs for Super Bowl 50, beginning with a special episode of The Late Show with Stephen Colbert following the game. Following a break for late local programming, CBS also aired a special episode of The Late Late Show with James Corden.</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>[39, 666, 867, 263, 160]</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>[0.8560473918914795, 0.8526903390884399, 0.7796630263328552, 0.7579885721206665, 0.7371344566345215]</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>["CBS broadcast Super Bowl 50 in the U.S., and charged an average of $5 million for a 30-second commercial during the game. The Super Bowl 50 halftime show was headlined by the British rock group Coldplay with special guest performers Beyoncé and Bruno Mars, who headlined the Super Bowl XLVII and Super Bowl XLVIII halftime shows, respectively. It was the third-most watched U.S. broadcast ever.", "In late November 2015, reports surfaced stating that \"multiple acts\" would perform during the halftime show. On December 3, the league confirmed that the show would be headlined by the British rock group Coldplay. On January 7, 2016, Pepsi confirmed to the Associated Press that Beyoncé, who headlined the Super Bowl XLVII halftime show and collaborated with Coldplay on the single \"Hymn for the Weekend\", would be making an appearance. Bruno Mars, who headlined the Super Bowl XLVIII halftime show, and Mark Ronson also performed.", "In honor of the 50th Super Bowl, the pregame ceremony featured the on-field introduction of 39 of the 43 previous Super Bowl Most Valuable Players. Bart Starr (MVP of Super Bowls I and II) and Chuck Howley (MVP of Super Bowl V) appeared via video, while Peyton Manning (MVP of Super Bowl XLI and current Broncos quarterback) was shown in the locker room preparing for the game. No plans were announced regarding the recognition of Harvey Martin, co-MVP of Super Bowl XII, who died in 2001.", "Super Bowl 50 was an American football game to determine the champion of the National Football League (NFL) for the 2015 season. The American Football Conference (AFC) champion Denver Broncos defeated the National Football Conference (NFC) champion Carolina Panthers 24–10 to earn their third Super Bowl title. The game was played on February 7, 2016, at Levi's Stadium in the San Francisco Bay Area at Santa Clara, California. As this was the 50th Super Bowl, the league emphasized the \"golden anniversary\" with various gold-themed initiatives, as well as temporarily suspending the tradition of naming each Super Bowl game with Roman numerals (under which the game would have been known as \"Super Bowl L\"), so that the logo could prominently feature the Arabic numerals 50.", "As opposed to broadcasts of primetime series, CBS broadcast special episodes of its late night talk shows as its lead-out programs for Super Bowl 50, beginning with a special episode of The Late Show with Stephen Colbert following the game. Following a break for late local programming, CBS also aired a special episode of The Late Late Show with James Corden."]</t>
-        </is>
-      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2314,21 +1714,6 @@
 Other predecessors of the Reformed church included the pro-reform and Gallican Roman Catholics, such as Jacques Lefevre (c. 1455–1536). The Gallicans briefly achieved independence for the French church, on the principle that the religion of France could not be controlled by the Bishop of Rome, a foreign power. During the Protestant Reformation, Lefevre, a professor at the University of Paris, published his French translation of the New Testament in 1523, followed by the whole Bible in the French language in 1530. William Farel was a student of Lefevre who went on to become a leader of the Swiss Reformation, establishing a Protestant government in Geneva. Jean Cauvin (John Calvin), another student at the University of Paris, also converted to Protestantism. Long after the sect was suppressed by Francis I, the remaining French Waldensians, then mostly in the Luberon region, sought to join William Farel, Calvin and the Reformation, and Olivetan published a French Bible for them. The French Confession of 1559 shows a decidedly Calvinistic influence. Sometime between 1550 and 1580, members of the Reformed church in France came to be commonly known as Huguenots.[citation needed]</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>[40, 106, 343, 489, 306]</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>[0.8322597146034241, 0.8021693825721741, 0.790977418422699, 0.7751494646072388, 0.7727789878845215]</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>["In 1735, John and Charles Wesley went to America to teach the gospel to the American Indians in the colony of Georgia. In less than two years, the \"Holy Club\" disbanded. John Wesley returned to England and met with a group of clergy he respected. He said \"they appeared to be of one heart, as well as of one judgment, resolved to be Bible-Christians at all events; and, wherever they were, to preach with all their might plain, old, Bible Christianity\". The ministers retained their membership in the Church of England. Though not always emphasized or appreciated in the Anglican churches of their day, their teaching emphasized salvation by God's grace, acquired through faith in Christ. Three teachings they saw as the foundation of Christian faith were:", "In the early years, many Huguenots also settled in the area of present-day Charleston, South Carolina. In 1685, Rev. Elie Prioleau from the town of Pons in France, was among the first to settle there. He became pastor of the first Huguenot church in North America in that city. After the Revocation of the Edict of Nantes in 1685, several Huguenot families of Norman and Carolingian nobility and descent, including Edmund Bohun of Suffolk England from the Humphrey de Bohun line of French royalty descended from Charlemagne, Jean Postell of Dieppe France, Alexander Pepin, Antoine Poitevin of Orsement France, and Jacques de Bordeaux of Grenoble, immigrated to the Charleston Orange district. They were very successful at marriage and property speculation. After petitioning the British Crown in 1697 for the right to own land in the Baronies, they prospered as slave owners on the Cooper, Ashepoo, Ashley and Santee River plantations they purchased from the British Landgrave Edmund Bellinger. Some of their descendants moved into the Deep South and Texas, where they developed new plantations.", "Richard Allen and Absalom Jones became the first African Americans ordained by the Methodist Church. They were licensed by St. George's Church in 1784. Three years later, protesting racial segregation in the worship services, Allen led most of the black members out of St. George's; eventually they founded the Mother Bethel A.M.E. Church and the African Methodist Episcopal denomination. Absalom Jones became an Episcopal priest. In 1836, the church's basement was excavated to make room for a Sunday School. In the 1920s a court case saved the church from being demolished to make way for the Benjamin Franklin Bridge. The case resulted in the bridge being relocated. Historic St Georges welcomes visitors and is home to archives and a museum on Methodism.", "Both before and after the 1708 passage of the Foreign Protestants Naturalization Act, an estimated 50,000 Protestant Walloons and Huguenots fled to England, with many moving on to Ireland and elsewhere. In relative terms, this was one of the largest waves of immigration ever of a single ethnic community to Britain. Andrew Lortie (born André Lortie), a leading Huguenot theologian and writer who led the exiled community in London, became known for articulating their criticism of the Pope and the doctrine of transubstantiation during Mass.", "Other predecessors of the Reformed church included the pro-reform and Gallican Roman Catholics, such as Jacques Lefevre (c. 1455–1536). The Gallicans briefly achieved independence for the French church, on the principle that the religion of France could not be controlled by the Bishop of Rome, a foreign power. During the Protestant Reformation, Lefevre, a professor at the University of Paris, published his French translation of the New Testament in 1523, followed by the whole Bible in the French language in 1530. William Farel was a student of Lefevre who went on to become a leader of the Swiss Reformation, establishing a Protestant government in Geneva. Jean Cauvin (John Calvin), another student at the University of Paris, also converted to Protestantism. Long after the sect was suppressed by Francis I, the remaining French Waldensians, then mostly in the Luberon region, sought to join William Farel, Calvin and the Reformation, and Olivetan published a French Bible for them. The French Confession of 1559 shows a decidedly Calvinistic influence. Sometime between 1550 and 1580, members of the Reformed church in France came to be commonly known as Huguenots.[citation needed]"]</t>
-        </is>
-      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2360,21 +1745,6 @@
 In 1529, Warsaw for the first time became the seat of the General Sejm, permanent from 1569. In 1573 the city gave its name to the Warsaw Confederation, formally establishing religious freedom in the Polish–Lithuanian Commonwealth. Due to its central location between the Commonwealth's capitals of Kraków and Vilnius, Warsaw became the capital of the Commonwealth and the Crown of the Kingdom of Poland when King Sigismund III Vasa moved his court from Kraków to Warsaw in 1596. In the following years the town expanded towards the suburbs. Several private independent districts were established, the property of aristocrats and the gentry, which were ruled by their own laws. Three times between 1655–1658 the city was under siege and three times it was taken and pillaged by the Swedish, Brandenburgian and Transylvanian forces.</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>[41, 58, 35, 396, 26]</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>[0.9029138088226318, 0.7995834946632385, 0.7837378978729248, 0.7743574380874634, 0.7735847234725952]</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>["In 1939, c. 1,300,000 people lived in Warsaw, but in 1945 – only 420,000. During the first years after the war, the population growth was c. 6%, so shortly the city started to suffer from the lack of flats and of areas for new houses. The first remedial measure was the Warsaw area enlargement (1951) – but the city authorities were still forced to introduce residency registration limitations: only the spouses and children of the permanent residents as well as some persons of public importance (like renowned specialists) were allowed to get the registration, hence halving the population growth in the following years. It also bolstered some kind of conviction among Poles that Varsovians thought of themselves as better only because they lived in the capital. Unfortunately this belief still lives on in Poland (although not as much as it used to be) – even though since 1990 there are no limitations to residency registration anymore.", "After World War II, under a Communist regime set up by the conquering Soviets, the \"Bricks for Warsaw\" campaign was initiated, and large prefabricated housing projects were erected in Warsaw to address the housing shortage, along with other typical buildings of an Eastern Bloc city, such as the Palace of Culture and Science, a gift from the Soviet Union. The city resumed its role as the capital of Poland and the country's centre of political and economic life. Many of the historic streets, buildings, and churches were restored to their original form. In 1980, Warsaw's historic Old Town was inscribed onto UNESCO's World Heritage list.", "In 2012 the Economist Intelligence Unit ranked Warsaw as the 32nd most liveable city in the world. It was also ranked as one of the most liveable cities in Central Europe. Today Warsaw is considered an \"Alpha–\" global city, a major international tourist destination and a significant cultural, political and economic hub. Warsaw's economy, by a wide variety of industries, is characterised by FMCG manufacturing, metal processing, steel and electronic manufacturing and food processing. The city is a significant centre of research and development, BPO, ITO, as well as of the Polish media industry. The Warsaw Stock Exchange is one of the largest and most important in Central and Eastern Europe. Frontex, the European Union agency for external border security, has its headquarters in Warsaw. It has been said that Warsaw, together with Frankfurt, London, Paris and Barcelona is one of the cities with the highest number of skyscrapers in the European Union. Warsaw has also been called \"Eastern Europe’s chic cultural capital with thriving art and club scenes and serious restaurants\".", "Warsaw was occupied by Germany from 4 August 1915 until November 1918. The Allied Armistice terms required in Article 12 that Germany withdraw from areas controlled by Russia in 1914, which included Warsaw. Germany did so, and underground leader Piłsudski returned to Warsaw on 11 November and set up what became the Second Polish Republic, with Warsaw the capital. In the course of the Polish-Bolshevik War of 1920, the huge Battle of Warsaw was fought on the eastern outskirts of the city in which the capital was successfully defended and the Red Army defeated. Poland stopped by itself the full brunt of the Red Army and defeated an idea of the \"export of the revolution\".", "In 1529, Warsaw for the first time became the seat of the General Sejm, permanent from 1569. In 1573 the city gave its name to the Warsaw Confederation, formally establishing religious freedom in the Polish–Lithuanian Commonwealth. Due to its central location between the Commonwealth's capitals of Kraków and Vilnius, Warsaw became the capital of the Commonwealth and the Crown of the Kingdom of Poland when King Sigismund III Vasa moved his court from Kraków to Warsaw in 1596. In the following years the town expanded towards the suburbs. Several private independent districts were established, the property of aristocrats and the gentry, which were ruled by their own laws. Three times between 1655–1658 the city was under siege and three times it was taken and pillaged by the Swedish, Brandenburgian and Transylvanian forces."]</t>
-        </is>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2406,21 +1776,6 @@
 One key figure in the plans for what would come to be known as American Empire, was a geographer named Isiah Bowman. Bowman was the director of the American Geographical Society in 1914. Three years later in 1917, he was appointed to then President Woodrow Wilson's inquiry in 1917. The inquiry was the idea of President Wilson and the American delegation from the Paris Peace Conference. The point of this inquiry was to build a premise that would allow for U.S authorship of a 'new world' which was to be characterized by geographical order. As a result of his role in the inquiry, Isiah Bowman would come to be known as Wilson's geographer.</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>[42, 303, 631, 104, 38]</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>[0.7898745536804199, 0.7757090926170349, 0.750375509262085, 0.7465083003044128, 0.7240219116210938]</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>["Edward John Noble, the owner of Life Savers candy, drugstore chain Rexall and New York City radio station WMCA, purchased the network for $8 million. Due to FCC ownership rules, the transaction, which was to include the purchase of three RCA stations by Noble, would require him to resell his station with the FCC's approval. The Commission authorized the transaction on October 12, 1943. Soon afterward, the Blue Network was purchased by the new company Noble founded, the American Broadcasting System. Noble subsequently acquired the rights to the \"American Broadcasting Company\" name from George B. Storer in 1944; its parent company adopted the corporate name American Broadcasting Companies, Inc. Woods retained his position as president and CEO of ABC until December 1949, and was subsequently promoted to vice-chairman of the board before leaving ABC altogether on June 30, 1951.", "Notable alumni in the field of government and politics include the founder of modern community organizing Saul Alinsky, Obama campaign advisor and top political advisor to President Bill Clinton David Axelrod, Attorney General and federal judge Robert Bork, Attorney General Ramsey Clark, Prohibition agent Eliot Ness, Supreme Court Justice John Paul Stevens, Prime Minister of Canada William Lyon Mackenzie King, 11th Prime Minister of Poland Marek Belka, Governor of the Bank of Japan Masaaki Shirakawa, the first female African-American Senator Carol Moseley Braun, United States Senator from Vermont and 2016 Democratic Presidential Candidate Bernie Sanders, and former World Bank President Paul Wolfowitz.", "Westwood One will carry the game throughout North America, with Kevin Harlan as play-by-play announcer, Boomer Esiason and Dan Fouts as color analysts, and James Lofton and Mark Malone as sideline reporters. Jim Gray will anchor the pre-game and halftime coverage.", "the merger, Thomas S. Murphy left ABC with Robert Iger taking his place as president and CEO. Around the time of the merger, Disney's television production units had already produced series for the network such as Home Improvement and Boy Meets World, while the deal also allowed ABC access to Disney's children's programming library for its Saturday morning block. In 1998, ABC premiered the Aaron Sorkin-created sitcom Sports Night, centering on the travails of the staff of a SportsCenter-style sports news program; despite earning critical praise and multiple Emmy Awards, the series was cancelled in 2000 after two seasons.", "One key figure in the plans for what would come to be known as American Empire, was a geographer named Isiah Bowman. Bowman was the director of the American Geographical Society in 1914. Three years later in 1917, he was appointed to then President Woodrow Wilson's inquiry in 1917. The inquiry was the idea of President Wilson and the American delegation from the Paris Peace Conference. The point of this inquiry was to build a premise that would allow for U.S authorship of a 'new world' which was to be characterized by geographical order. As a result of his role in the inquiry, Isiah Bowman would come to be known as Wilson's geographer."]</t>
-        </is>
-      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2452,21 +1807,6 @@
 The Upper Rhine region was changed significantly by a Rhine straightening program in the 19th Century. The rate of flow was increased and the ground water level fell significantly. Dead branches dried up and the amount of forests on the flood plains decreased sharply. On the French side, the Grand Canal d'Alsace was dug, which carries a significant part of the river water, and all of the traffic. In some places, there are large compensation pools, for example the huge Bassin de compensation de Plobsheim in Alsace.</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>[77, 612, 758, 43, 345]</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>[0.8362835645675659, 0.8325671553611755, 0.8321154713630676, 0.8317866325378418, 0.8236998915672302]</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>["Most of the Rhine's current course was not under the ice during the last Ice Age; although, its source must still have been a glacier. A tundra, with Ice Age flora and fauna, stretched across middle Europe, from Asia to the Atlantic Ocean. Such was the case during the Last Glacial Maximum, ca. 22,000–14,000 yr BP, when ice-sheets covered Scandinavia, the Baltics, Scotland and the Alps, but left the space between as open tundra. The loess or wind-blown dust over that tundra, settled in and around the Rhine Valley, contributing to its current agricultural usefulness.", "The name Rijn, from here on, is used only for smaller streams farther to the north, which together formed the main river Rhine in Roman times. Though they retained the name, these streams no longer carry water from the Rhine, but are used for draining the surrounding land and polders. From Wijk bij Duurstede, the old north branch of the Rhine is called Kromme Rijn (\"Bent Rhine\") past Utrecht, first Leidse Rijn (\"Rhine of Leiden\") and then, Oude Rijn (\"Old Rhine\"). The latter flows west into a sluice at Katwijk, where its waters can be discharged into the North Sea. This branch once formed the line along which the Limes Germanicus were built. During periods of lower sea levels within the various ice ages, the Rhine took a left turn, creating the Channel River, the course of which now lies below the English Channel.", "The Rhine emerges from Lake Constance, flows generally westward, as the Hochrhein, passes the Rhine Falls, and is joined by its major tributary, the river Aare. The Aare more than doubles the Rhine's water discharge, to an average of nearly 1,000 m3/s (35,000 cu ft/s), and provides more than a fifth of the discharge at the Dutch border. The Aare also contains the waters from the 4,274 m (14,022 ft) summit of Finsteraarhorn, the highest point of the Rhine basin. The Rhine roughly forms the German-Swiss border from Lake Constance with the exceptions of the canton of Schaffhausen and parts of the cantons of Zürich and Basel-Stadt, until it turns north at the so-called Rhine knee at Basel, leaving Switzerland.", "At the begin of the Holocene (~11,700 years ago), the Rhine occupied its Late-Glacial valley. As a meandering river, it reworked its ice-age braidplain. As sea-level continued to rise in the Netherlands, the formation of the Holocene Rhine-Meuse delta began (~8,000 years ago). Coeval absolute sea-level rise and tectonic subsidence have strongly influenced delta evolution. Other factors of importance to the shape of the delta are the local tectonic activities of the Peel Boundary Fault, the substrate and geomorphology, as inherited from the Last Glacial and the coastal-marine dynamics, such as barrier and tidal inlet formations.", "The Upper Rhine region was changed significantly by a Rhine straightening program in the 19th Century. The rate of flow was increased and the ground water level fell significantly. Dead branches dried up and the amount of forests on the flood plains decreased sharply. On the French side, the Grand Canal d'Alsace was dug, which carries a significant part of the river water, and all of the traffic. In some places, there are large compensation pools, for example the huge Bassin de compensation de Plobsheim in Alsace."]</t>
-        </is>
-      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2498,21 +1838,6 @@
 With such a small force, the invading Mongols were forced to change strategies and resort to inciting internal revolt among Kuchlug's supporters, leaving the Qara Khitai more vulnerable to Mongol conquest. As a result, Kuchlug's army was defeated west of Kashgar. Kuchlug fled again, but was soon hunted down by Jebe's army and executed. By 1218, as a result of defeat of Qara Khitai, the Mongol Empire and its control extended as far west as Lake Balkhash, which bordered the Khwarezmia (Khwarezmid Empire), a Muslim state that reached the Caspian Sea to the west and Persian Gulf and the Arabian Sea to the south.</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>[45, 44, 803, 80, 494]</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>[0.871289074420929, 0.8599246740341187, 0.8598129749298096, 0.8486800789833069, 0.8436545133590698]</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>["seen as an affront and insult to Genghis Khan. Outraged, Genghis Khan planned one of his largest invasion campaigns by organizing together around 100,000 soldiers (10 tumens), his most capable generals and some of his sons. He left a commander and number of troops in China, designated his successors to be his family members and likely appointed Ögedei to be his immediate successor and then went out to Khwarezmia.", "In the early 13th century, the Khwarazmian dynasty was governed by Shah Ala ad-Din Muhammad. Genghis Khan saw the potential advantage in Khwarezmia as a commercial trading partner using the Silk Road, and he initially sent a 500-man caravan to establish official trade ties with the empire. However, Inalchuq, the governor of the Khwarezmian city of Otrar, attacked the caravan that came from Mongolia, claiming that the caravan contained spies and therefore was a conspiracy against Khwarezmia. The situation became further complicated because the governor later refused to make repayments for the looting of the caravans and handing over the perpetrators. Genghis Khan then sent again a second group of three ambassadors (two Mongols and a Muslim) to meet the Shah himself instead of the governor Inalchuq. The Shah had all the men shaved and the Muslim beheaded and sent his head back with the two remaining ambassadors. This was seen as an affront and insult to Genghis Khan. Outraged, Genghis Khan planned one of his largest invasion campaigns by organizing together around 100,000 soldiers (10 tumens), his most capable generals and some of his sons. He left a commander and number of troops in China, designated his successors to", "After the defeat of the Khwarezmian Empire in 1220, Genghis Khan gathered his forces in Persia and Armenia to return to the Mongolian steppes. Under the suggestion of Subutai, the Mongol army was split into two forces. Genghis Khan led the main army on a raid through Afghanistan and northern India towards Mongolia, while another 20,000 (two tumen) contingent marched through the Caucasus and into Russia under generals Jebe and Subutai. They pushed deep into Armenia and Azerbaijan. The Mongols destroyed the kingdom of Georgia, sacked the Genoese trade-fortress of Caffa in Crimea and overwintered near the Black Sea. Heading home, Subutai's forces attacked the allied forces of the Cuman–Kipchaks and the poorly coordinated 80,000 Kievan Rus' troops led by Mstislav the Bold of Halych and Mstislav III of Kiev who went out to stop the Mongols' actions in the area. Subutai sent emissaries to the Slavic princes calling for a separate peace, but the emissaries were executed. At the Battle of Kalka River in 1223, Subutai's forces defeated the larger Kievan force. They also may have fought against the neighboring Volga Bulgars. There is no historical record except a short account by the Arab historian Ibn al-Athir, writing in", "The Shah's army was split by diverse internecine feuds and by the Shah's decision to divide his army into small groups concentrated in various cities. This fragmentation was decisive in Khwarezmia's defeats, as it allowed the Mongols, although exhausted from the long journey, to immediately set about defeating small fractions of the Khwarzemi forces instead of facing a unified defense. The Mongol army quickly seized the town of Otrar, relying on superior strategy and tactics. Genghis Khan ordered the wholesale massacre of many of the civilians, enslaved the rest of the population and executed Inalchuq by pouring molten silver into his ears and eyes, as retribution for his actions. Near the end of the battle the Shah fled rather than surrender. Genghis Khan ordered Subutai and Jebe to hunt him down, giving them 20,000 men and two years to do this. The Shah died under mysterious circumstances on a small island within his empire.", "With such a small force, the invading Mongols were forced to change strategies and resort to inciting internal revolt among Kuchlug's supporters, leaving the Qara Khitai more vulnerable to Mongol conquest. As a result, Kuchlug's army was defeated west of Kashgar. Kuchlug fled again, but was soon hunted down by Jebe's army and executed. By 1218, as a result of defeat of Qara Khitai, the Mongol Empire and its control extended as far west as Lake Balkhash, which bordered the Khwarezmia (Khwarezmid Empire), a Muslim state that reached the Caspian Sea to the west and Persian Gulf and the Arabian Sea to the south."]</t>
-        </is>
-      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2544,21 +1869,6 @@
 Economist Joseph Stiglitz presented evidence in 2009 that both global inequality and inequality within countries prevent growth by limiting aggregate demand. Economist Branko Milanovic, wrote in 2001 that, "The view that income inequality harms growth – or that improved equality can help sustain growth – has become more widely held in recent years. ... The main reason for this shift is the increasing importance of human capital in development. When physical capital mattered most, savings and investments were key. Then it was important to have a large contingent of rich people who could save a greater proportion of their income than the poor and invest it in physical capital. But now that human capital is scarcer than machines, widespread education has become the secret to growth."</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>[46, 549, 438, 407, 115]</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>[0.8433719277381897, 0.8426294326782227, 0.7560001015663147, 0.7488906383514404, 0.7465800046920776]</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>["According to economists David Castells-Quintana and Vicente Royuela, increasing inequality harms economic growth. High and persistent unemployment, in which inequality increases, has a negative effect on subsequent long-run economic growth. Unemployment can harm growth not only because it is a waste of resources, but also because it generates redistributive pressures and subsequent distortions, drives people to poverty, constrains liquidity limiting labor mobility, and erodes self-esteem promoting social dislocation, unrest and conflict. Policies aiming at controlling unemployment and in particular at reducing its inequality-associated effects support economic growth.", "2013 Economics Nobel prize winner Robert J. Shiller said that rising inequality in the United States and elsewhere is the most important problem. Increasing inequality harms economic growth. High and persistent unemployment, in which inequality increases, has a negative effect on subsequent long-run economic growth. Unemployment can harm growth not only because it is a waste of resources, but also because it generates redistributive pressures and subsequent distortions, drives people to poverty, constrains liquidity limiting labor mobility, and erodes self-esteem promoting social dislocation, unrest and conflict. Policies aiming at controlling unemployment and in particular at reducing its inequality-associated effects support economic growth.", "When a person’s capabilities are lowered, they are in some way deprived of earning as much income as they would otherwise. An old, ill man cannot earn as much as a healthy young man; gender roles and customs may prevent a woman from receiving an education or working outside the home. There may be an epidemic that causes widespread panic, or there could be rampant violence in the area that prevents people from going to work for fear of their lives. As a result, income and economic inequality increases, and it becomes more difficult to reduce the gap without additional aid. To prevent such inequality, this approach believes it’s important to have political freedom, economic facilities, social opportunities, transparency guarantees, and protective security to ensure that people aren’t denied their functionings, capabilities, and agency and can thus work towards a better relevant income.", "wages due to the nature of the job, since there is a relative shortage of workers for the particular position. Professional and labor organizations may limit the supply of workers which results in higher demand and greater incomes for members. Members may also receive higher wages through collective bargaining, political influence, or corruption.", "Economist Joseph Stiglitz presented evidence in 2009 that both global inequality and inequality within countries prevent growth by limiting aggregate demand. Economist Branko Milanovic, wrote in 2001 that, \"The view that income inequality harms growth – or that improved equality can help sustain growth – has become more widely held in recent years. ... The main reason for this shift is the increasing importance of human capital in development. When physical capital mattered most, savings and investments were key. Then it was important to have a large contingent of rich people who could save a greater proportion of their income than the poor and invest it in physical capital. But now that human capital is scarcer than machines, widespread education has become the secret to growth.\""]</t>
-        </is>
-      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2590,21 +1900,6 @@
 members of the Reformed Church) involved in the Amboise plot of 1560: a foiled attempt to wrest power in France from the influential House of Guise. The move would have had the side effect of fostering relations with the Swiss. Thus, Hugues plus Eidgenosse by way of Huisgenoten supposedly became Huguenot, a nickname associating the Protestant cause with politics unpopular in France.[citation needed]</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>[504, 487, 145, 30, 502]</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>[0.7845924496650696, 0.7790302634239197, 0.7559201121330261, 0.7481638789176941, 0.7435165047645569]</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>["war. By 1529, in On War against the Turk, he was actively urging Emperor Charles V and the German people to fight a secular war against the Turks. He made clear, however, that the spiritual war against an alien faith was separate, to be waged through prayer and repentance. Around the time of the Siege of Vienna, Luther wrote a prayer for national deliverance from the Turks, asking God to \"give to our emperor perpetual victory over our enemies\".", "The War of the Austrian Succession (whose North American theater is known as King George's War) formally ended in 1748 with the signing of the Treaty of Aix-la-Chapelle. The treaty was primarily focused on resolving issues in Europe. The issues of conflicting territorial claims between British and French colonies in North America were turned over to a commission to resolve, but it reached no decision. Frontiers from between Nova Scotia and Acadia in the north, to the Ohio Country in the south, were claimed by both sides. The disputes also extended into the Atlantic Ocean, where both powers wanted access to the rich fisheries of the Grand Banks off Newfoundland.", "The British, for their part, were happy to take New France, as defence of their North American colonies would no longer be an issue and also because they already had ample places from which to obtain sugar. Spain, which traded Florida to Britain to regain Cuba, also gained Louisiana, including New Orleans, from France in compensation for its losses. Great Britain and Spain also agreed that navigation on the Mississippi River was to be open to vessels of all nations.", "Newcastle replaced him in January 1756 with Lord Loudoun, with Major General James Abercrombie as his second in command. Neither of these men had as much campaign experience as the trio of officers France sent to North America. French regular army reinforcements arrived in New France in May 1756, led by Major General Louis-Joseph de Montcalm and seconded by the Chevalier de Lévis and Colonel François-Charles de Bourlamaque, all experienced veterans from the War of the Austrian Succession. During that time in Europe, on May 18, 1756, England formally declared war on France, which expanded the war into Europe, which was later to be known as the Seven Years' War.", "members of the Reformed Church) involved in the Amboise plot of 1560: a foiled attempt to wrest power in France from the influential House of Guise. The move would have had the side effect of fostering relations with the Swiss. Thus, Hugues plus Eidgenosse by way of Huisgenoten supposedly became Huguenot, a nickname associating the Protestant cause with politics unpopular in France.[citation needed]"]</t>
-        </is>
-      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2636,21 +1931,6 @@
 The Yuan undertook extensive public works. Among Kublai Khan's top engineers and scientists was the astronomer Guo Shoujing, who was tasked with many public works projects and helped the Yuan reform the lunisolar calendar to provide an accuracy of 365.2425 days of the year, which was only 26 seconds off the modern Gregorian calendar's measurement. Road and water communications were reorganized and improved. To provide against possible famines, granaries were ordered built throughout the empire. The city of Beijing was rebuilt with new palace grounds that included artificial lakes, hills and mountains, and parks. During the Yuan period, Beijing became the terminus of the Grand Canal of China, which was completely renovated. These commercially oriented improvements encouraged overland and maritime commerce throughout Asia and facilitated direct Chinese contacts with Europe. Chinese travelers to the West were able to provide assistance in such areas as hydraulic engineering. Contacts with the West also brought the introduction to China of a major food crop, sorghum, along with other foreign food products and methods of preparation.</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>[678, 49, 852, 390, 499]</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>[0.753781795501709, 0.7508062124252319, 0.7440353035926819, 0.7338786721229553, 0.7323763966560364]</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>["Gasquet (1908) claimed that the Latin name atra mors (Black Death) for the 14th-century epidemic first appeared in modern times in 1631 in a book on Danish history by J.I. Pontanus: \"Vulgo &amp; ab effectu atram mortem vocatibant. (\"Commonly and from its effects, they called it the black death\"). The name spread through Scandinavia and then Germany, gradually becoming attached to the mid 14th-century epidemic as a proper name. In England, it was not until 1823 that the medieval epidemic was first called the Black Death.", "Guo Shoujing applied mathematics to the construction of calendars. He was one of the first mathematicians in China to work on spherical trigonometry. Gou derived a cubic interpolation formula for his astronomical calculations. His calendar, the Shoushi Li (授時暦) or Calendar for Fixing the Seasons, was disseminated in 1281 as the official calendar of the Yuan dynasty. The calendar may have been influenced solely by the work of Song dynasty astronomer Shen Kuo or possibly by the work of Arab astronomers. There are no explicit signs of Muslim influences in the Shoushi calendar, but Mongol rulers were known to be interested in Muslim calendars. Mathematical knowledge from the Middle East was introduced to China under the Mongols, and Muslim astronomers brought Arabic numerals to China in the 13th century.", "In this last connection, the name could suggest the derogatory inference of superstitious worship; popular fancy held that Huguon, the gate of King Hugo, was haunted by the ghost of le roi Huguet (regarded by Roman Catholics as an infamous scoundrel) and other spirits, who instead of being in Purgatory came back to harm the living at night. It was in this place in Tours that the prétendus réformés (\"these supposedly 'reformed'\") habitually gathered at night, both for political purposes, and for prayer and singing psalms. Such explanations have been traced to the contemporary, Reguier de la Plancha (d. 1560), who in De l'Estat de France offered the following account as to the origin of the name, as cited by The Cape Monthly:", "less than 700 preparations, their properties, modes of action, and their indications. He devoted in fact a whole volume to simple drugs in The Canon of Medicine. Of great impact were also the works by al-Maridini of Baghdad and Cairo, and Ibn al-Wafid (1008–1074), both of which were printed in Latin more than fifty times, appearing as De Medicinis universalibus et particularibus by 'Mesue' the younger, and the Medicamentis simplicibus by 'Abenguefit'. Peter of Abano (1250–1316) translated and added a supplement to the work of al-Maridini under the title De Veneris. Al-Muwaffaq’s contributions in the field are also pioneering. Living in the 10th century, he wrote The foundations of the true properties of Remedies, amongst others describing arsenious oxide, and being acquainted with silicic acid. He made clear distinction between sodium carbonate and potassium carbonate, and drew attention to the poisonous nature of copper compounds, especially copper vitriol, and also lead compounds. He also describes the distillation of sea-water for drinking.[verification needed]", "The Yuan undertook extensive public works. Among Kublai Khan's top engineers and scientists was the astronomer Guo Shoujing, who was tasked with many public works projects and helped the Yuan reform the lunisolar calendar to provide an accuracy of 365.2425 days of the year, which was only 26 seconds off the modern Gregorian calendar's measurement. Road and water communications were reorganized and improved. To provide against possible famines, granaries were ordered built throughout the empire. The city of Beijing was rebuilt with new palace grounds that included artificial lakes, hills and mountains, and parks. During the Yuan period, Beijing became the terminus of the Grand Canal of China, which was completely renovated. These commercially oriented improvements encouraged overland and maritime commerce throughout Asia and facilitated direct Chinese contacts with Europe. Chinese travelers to the West were able to provide assistance in such areas as hydraulic engineering. Contacts with the West also brought the introduction to China of a major food crop, sorghum, along with other foreign food products and methods of preparation."]</t>
-        </is>
-      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2682,21 +1962,6 @@
 texture every episode, with the texture relating to some aspect of the story. The logo for the Twelfth Doctor had the "DW" TARDIS insignia removed and the font was subtly altered, as well as made slightly larger. As of 2014, the logo used for the Third and Eighth Doctors is the primary logo used on all media and merchandise relating to past Doctors, and the current Doctor Who logo is used for all merchandise relating to the current Doctor.</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>[50, 686, 558, 807, 511]</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>[0.7594755291938782, 0.7525122165679932, 0.7484481334686279, 0.7470220327377319, 0.7443040609359741]</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>["Producers introduced the concept of regeneration to permit the recasting of the main character. This was first prompted by original star William Hartnell's poor health. The actual term \"regeneration\" was not initially conceived of until the Doctor's third on-screen regeneration however; Hartnell's Doctor had merely described undergoing a \"renewal,\" and the Second Doctor underwent a \"change of appearance\".[citation needed] The device has allowed for the recasting of the actor various times in the show's history, as well as the depiction of alternative Doctors either from the Doctor's relative past or future.[citation needed]", "LeGrande writes that \"the formulation of a single all-encompassing definition of the term is extremely difficult, if not impossible. In reviewing the voluminous literature on the subject, the student of civil disobedience rapidly finds himself surrounded by a maze of semantical problems and grammatical niceties. Like Alice in Wonderland, he often finds that specific terminology has no more (or no less) meaning than the individual orator intends it to have.\" He encourages a distinction between lawful protest demonstration, nonviolent civil disobedience, and violent civil disobedience.", "to further the story by requesting exposition from the Doctor and manufacturing peril for the Doctor to resolve. The Doctor regularly gains new companions and loses old ones; sometimes they return home or find new causes — or loves — on worlds they have visited. Some have died during the course of the series. Companions are usually human, or humanoid aliens.", "Doctor clarified he was the product of the twelfth regeneration, due to a previous incarnation which he chose not to count and one other aborted regeneration. The name Eleventh is still used for this incarnation; the same episode depicts the prophesied \"Fall of the Eleventh\" which had been trailed throughout the series.", "texture every episode, with the texture relating to some aspect of the story. The logo for the Twelfth Doctor had the \"DW\" TARDIS insignia removed and the font was subtly altered, as well as made slightly larger. As of 2014, the logo used for the Third and Eighth Doctors is the primary logo used on all media and merchandise relating to past Doctors, and the current Doctor Who logo is used for all merchandise relating to the current Doctor."]</t>
-        </is>
-      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2728,21 +1993,6 @@
 In September 1967, Mueller approved a sequence of mission types which had to be successfully accomplished in order to achieve the manned lunar landing. Each step had to be successfully accomplished before the next ones could be performed, and it was unknown how many tries of each mission would be necessary; therefore letters were used instead of numbers. The A missions were unmanned Saturn V validation; B was unmanned LM validation using the Saturn IB; C was manned CSM Earth orbit validation using the Saturn IB; D was the first manned CSM/LM flight (this replaced AS-258, using a single Saturn V launch); E would be a higher Earth orbit CSM/LM flight; F would be the first lunar mission, testing the LM in lunar orbit but without landing (a "dress rehearsal"); and G would be the first manned landing. The list of types covered follow-on lunar exploration to include H lunar landings, I for lunar orbital survey missions, and J for extended-stay lunar landings.</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>[51, 478, 770, 225, 817]</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>[0.8825985193252563, 0.7858784794807434, 0.7719290852546692, 0.7713872194290161, 0.768706202507019]</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>["In 2008, Japan Aerospace Exploration Agency's SELENE probe observed evidence of the halo surrounding the Apollo 15 Lunar Module blast crater while orbiting above the lunar surface. In 2009, NASA's robotic Lunar Reconnaissance Orbiter, while orbiting 50 kilometers (31 mi) above the Moon, began photographing the remnants of the Apollo program left on the lunar surface, and photographed each site where manned Apollo flights landed. All of the U. S. flags left on the Moon during the Apollo missions were found to still be standing, with the exception of the one left during the Apollo 11 mission, which was blown over during that mission's lift-off from the lunar surface and return to the mission Command Module in lunar orbit; the degree to which these flags retain their original colors remains unknown.", "The Apollo astronauts were chosen from the Project Mercury and Gemini veterans, plus from two later astronaut groups. All missions were commanded by Gemini or Mercury veterans. Crews on all development flights (except the Earth orbit CSM development flights) through the first two landings on Apollo 11 and Apollo 12, included at least two (sometimes three) Gemini veterans. Dr. Harrison Schmitt, a geologist, was the first NASA scientist astronaut to fly in space, and landed on the Moon on the last mission, Apollo 17. Schmitt participated in the lunar geology training of all of the Apollo landing crews.", "About the time of the first landing in 1969, it was decided to use an existing Saturn V to launch the Skylab orbital laboratory pre-built on the ground, replacing the original plan to construct it in orbit from several Saturn IB launches; this eliminated Apollo 20. NASA's yearly budget also began to shrink in light of the successful landing, and NASA also had to make funds available for the development of the upcoming Space Shuttle. By 1971, the decision was made to also cancel missions 18 and 19. The two unused Saturn Vs became museum exhibits at the John F. Kennedy Space Center on Merritt Island, Florida, George C. Marshall Space Center in Huntsville, Alabama, Michoud Assembly Facility in New Orleans, Louisiana, and Lyndon B. Johnson Space Center in Houston, Texas.", "The Moon landing data was recorded by a special Apollo TV camera which recorded in a format incompatible with broadcast TV. This resulted in lunar footage that had to be converted for the live television broadcast and stored on magnetic telemetry tapes. During the following years, a magnetic tape shortage prompted NASA to remove massive numbers of magnetic tapes from the National Archives and Records Administration to be recorded over with newer satellite data. Stan Lebar, who led the team that designed and built the lunar television camera at Westinghouse Electric Corporation, also worked with Nafzger to try to locate the missing tapes.", "In September 1967, Mueller approved a sequence of mission types which had to be successfully accomplished in order to achieve the manned lunar landing. Each step had to be successfully accomplished before the next ones could be performed, and it was unknown how many tries of each mission would be necessary; therefore letters were used instead of numbers. The A missions were unmanned Saturn V validation; B was unmanned LM validation using the Saturn IB; C was manned CSM Earth orbit validation using the Saturn IB; D was the first manned CSM/LM flight (this replaced AS-258, using a single Saturn V launch); E would be a higher Earth orbit CSM/LM flight; F would be the first lunar mission, testing the LM in lunar orbit but without landing (a \"dress rehearsal\"); and G would be the first manned landing. The list of types covered follow-on lunar exploration to include H lunar landings, I for lunar orbital survey missions, and J for extended-stay lunar landings."]</t>
-        </is>
-      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2774,21 +2024,6 @@
 The popular neighborhood known as the Tower District is centered around the historic Tower Theatre, which is included on the National List of Historic Places. The theater was built in 1939 and is at Olive and Wishon Avenues in the heart of the Tower District. (The name of the theater refers to a well-known landmark water tower, which is actually in another nearby area). The Tower District neighborhood is just north of downtown Fresno proper, and one-half mile south of Fresno City College. Although the neighborhood was known as a residential area prior, the early commercial establishments of the Tower District began with small shops and services that flocked to the area shortly after World War II. The character of small local businesses largely remains today. To some extent, the businesses of the Tower District were developed due to the proximity of the original Fresno Normal School, (later renamed California State University at Fresno). In 1916 the college moved to what is now the site of Fresno City College one-half mile north of the Tower District.</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>[52, 297, 717, 534, 327]</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>[0.7780028581619263, 0.7530316114425659, 0.6900136470794678, 0.6887408494949341, 0.6856423616409302]</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>["Nearby, in Ogród Saski (the Saxon Garden), the Summer Theatre was in operation from 1870 to 1939, and in the inter-war period, the theatre complex also included Momus, Warsaw's first literary cabaret, and Leon Schiller's musical theatre Melodram. The Wojciech Bogusławski Theatre (1922–26), was the best example of \"Polish monumental theatre\". From the mid-1930s, the Great Theatre building housed the Upati Institute of Dramatic Arts – the first state-run academy of dramatic art, with an acting department and a stage directing department.", "The city still contains many theatres. The largest, the Theatre Royal on Grey Street, first opened in 1837, designed by John and Benjamin Green. It has hosted a season of performances from the Royal Shakespeare Company for over 25 years, as well as touring productions of West End musicals. The Mill Volvo Tyne Theatre hosts smaller touring productions, whilst other venues feature local talent. Northern Stage, formally known as the Newcastle Playhouse and Gulbenkian Studio, hosts various local, national and international productions in addition to those produced by the Northern Stage company. Other theatres in the city include the Live Theatre, the People's Theatre and the Jubilee Theatre. NewcastleGateshead was voted in 2006 as the arts capital of the UK in a survey conducted by the Artsworld TV channel.", "(later transferred to the Tate Gallery) and now used as the picture galleries and tapestry gallery respectively. The North and South Courts, were then built, both of which opened by June 1862. They now form the galleries for temporary exhibitions and are directly behind the Sheepshanks Gallery. On the very northern edge of the site is situated the Secretariat Wing, also built in 1862 this houses the offices and board room etc. and is not open to the public.", "Every May since 1987, the University of Chicago has held the University of Chicago Scavenger Hunt, in which large teams of students compete to obtain notoriously esoteric items from a list. Since 1963, the Festival of the Arts (FOTA) takes over campus for 7–10 days of exhibitions and interactive artistic endeavors. Every January, the university holds a week-long winter festival, Kuviasungnerk/Kangeiko, which include early morning exercise routines and fitness workshops. The university also annually holds a summer carnival and concert called Summer Breeze that hosts outside musicians, and is home to Doc Films, a student film society founded in 1932 that screens films nightly at the university. Since 1946, the university has organized the Latke-Hamantash Debate, which involves humorous discussions about the relative merits and meanings of latkes and hamantashen.", "The popular neighborhood known as the Tower District is centered around the historic Tower Theatre, which is included on the National List of Historic Places. The theater was built in 1939 and is at Olive and Wishon Avenues in the heart of the Tower District. (The name of the theater refers to a well-known landmark water tower, which is actually in another nearby area). The Tower District neighborhood is just north of downtown Fresno proper, and one-half mile south of Fresno City College. Although the neighborhood was known as a residential area prior, the early commercial establishments of the Tower District began with small shops and services that flocked to the area shortly after World War II. The character of small local businesses largely remains today. To some extent, the businesses of the Tower District were developed due to the proximity of the original Fresno Normal School, (later renamed California State University at Fresno). In 1916 the college moved to what is now the site of Fresno City College one-half mile north of the Tower District."]</t>
-        </is>
-      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2820,21 +2055,6 @@
 Luther dedicated himself to the Augustinian order, devoting himself to fasting, long hours in prayer, pilgrimage, and frequent confession. Luther described this period of his life as one of deep spiritual despair. He said, "I lost touch with Christ the Savior and Comforter, and made of him the jailer and hangman of my poor soul." Johann von Staupitz, his superior, pointed Luther's mind away from continual reflection upon his sins toward the merits of Christ. He taught that true repentance does not involve self-inflicted penances and punishments but rather a change of heart.</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>[53, 150, 65, 305, 81]</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>[0.8145040273666382, 0.7665321826934814, 0.7523845434188843, 0.7443422079086304, 0.7431483864784241]</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>["Sanctifying Grace is that grace of God which sustains the believers in the journey toward Christian Perfection: a genuine love of God with heart, soul, mind, and strength, and a genuine love of our neighbors as ourselves. Sanctifying grace enables us to respond to God by leading a Spirit-filled and Christ-like life aimed toward love. Wesley never claimed this state of perfection for himself but instead insisted the attainment of perfection was possible for all Christians. Here the English Reformer parted company with both Luther and Calvin, who denied that a man would ever reach a state in this life in which he could not fall into sin. Such a man can lose all inclination to evil and can gain perfection in this life.", "was \"as though I had been born again.\" His entry into Paradise, no less, was a discovery about \"the righteousness of God\" – a discovery that \"the just person\" of whom the Bible speaks (as in Romans 1:17) lives by faith. He explained his concept of \"justification\" in the Smalcald Articles:", "Justifying Grace or Accepting Grace is that grace, offered by God to all people, that we receive by faith and trust in Christ, through which God pardons the believer of sin. It is in justifying grace we are received by God, in spite of our sin. In this reception, we are forgiven through the atoning work of Jesus Christ on the cross. The justifying grace cancels our guilt and empowers us to resist the power of sin and to fully love God and neighbor. Today, justifying grace is also known as conversion, \"accepting Jesus as your personal Lord and Savior,\" or being \"born again\". John Wesley originally called this experience the New Birth. This experience can occur in different ways; it can be one transforming moment, such as an altar call experience, or it may involve a series of decisions across a period of time.", "In his theses and disputations against the antinomians, Luther reviews and reaffirms, on the one hand, what has been called the \"second use of the law,\" that is, the law as the Holy Spirit's tool to work sorrow over sin in man's heart, thus preparing him for Christ's fulfillment of the law offered in the gospel. Luther states that everything that is used to work sorrow over sin is called the law, even if it is Christ's life, Christ's death for sin, or God's goodness experienced in creation. Simply refusing to preach the Ten Commandments among Christians – thereby, as it were, removing the three letters l-a-w from the church – does not eliminate the accusing law. Claiming that the law – in any form – should not be preached to Christians anymore would be tantamount to asserting that Christians are no longer sinners in themselves and that the church consists only of essentially holy people.", "Luther dedicated himself to the Augustinian order, devoting himself to fasting, long hours in prayer, pilgrimage, and frequent confession. Luther described this period of his life as one of deep spiritual despair. He said, \"I lost touch with Christ the Savior and Comforter, and made of him the jailer and hangman of my poor soul.\" Johann von Staupitz, his superior, pointed Luther's mind away from continual reflection upon his sins toward the merits of Christ. He taught that true repentance does not involve self-inflicted penances and punishments but rather a change of heart."]</t>
-        </is>
-      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2866,21 +2086,6 @@
 When rock units are placed under horizontal compression, they shorten and become thicker. Because rock units, other than muds, do not significantly change in volume, this is accomplished in two primary ways: through faulting and folding. In the shallow crust, where brittle deformation can occur, thrust faults form, which cause deeper rock to move on top of shallower rock. Because deeper rock is often older, as noted by the principle of superposition, this can result in older rocks moving on top of younger ones. Movement along faults can result in folding, either because the faults are not planar or because rock layers are dragged along, forming drag folds as slip occurs along the fault. Deeper in the Earth, rocks behave plastically, and fold instead of faulting. These folds can either be those where the material in the center of the fold buckles upwards, creating "antiforms", or where it buckles downwards, creating "synforms". If the tops of the rock units within the folds remain pointing upwards, they are called anticlines and synclines, respectively. If some of the units in the fold are facing downward, the structure is called an overturned anticline or syncline, and if all of the rock units are</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>[218, 54, 590, 657, 217]</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>[0.7301808595657349, 0.7056863903999329, 0.7028726935386658, 0.6762965321540833, 0.671741783618927]</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>["creating \"synforms\". If the tops of the rock units within the folds remain pointing upwards, they are called anticlines and synclines, respectively. If some of the units in the fold are facing downward, the structure is called an overturned anticline or syncline, and if all of the rock units are overturned or the correct up-direction is unknown, they are simply called by the most general terms, antiforms and synforms.", "The chloroplasts of some hornworts and algae contain structures called pyrenoids. They are not found in higher plants. Pyrenoids are roughly spherical and highly refractive bodies which are a site of starch accumulation in plants that contain them. They consist of a matrix opaque to electrons, surrounded by two hemispherical starch plates. The starch is accumulated as the pyrenoids mature. In algae with carbon concentrating mechanisms, the enzyme rubisco is found in the pyrenoids. Starch can also accumulate around the pyrenoids when CO2 is scarce. Pyrenoids can divide to form new pyrenoids, or be produced \"de novo\".", "Among the most well-known experiments in structural geology are those involving orogenic wedges, which are zones in which mountains are built along convergent tectonic plate boundaries. In the analog versions of these experiments, horizontal layers of sand are pulled along a lower surface into a back stop, which results in realistic-looking patterns of faulting and the growth of a critically tapered (all angles remain the same) orogenic wedge. Numerical models work in the same way as these analog models, though they are often more sophisticated and can include patterns of erosion and uplift in the mountain belt. This helps to show the relationship between erosion and the shape of the mountain range. These studies can also give useful information about pathways for metamorphism through pressure, temperature, space, and time.", "Warsaw is located on two main geomorphologic formations: the plain moraine plateau and the Vistula Valley with its asymmetrical pattern of different terraces. The Vistula River is the specific axis of Warsaw, which divides the city into two parts, left and right. The left one is situated both on the moraine plateau (10 to 25 m (32.8 to 82.0 ft) above Vistula level) and on the Vistula terraces (max. 6.5 m (21.3 ft) above Vistula level). The significant element of the relief, in this part of Warsaw, is the edge of moraine plateau called Warsaw Escarpment. It is 20 to 25 m (65.6 to 82.0 ft) high in the Old Town and Central district and about 10 m (32.8 ft) in the north and south of Warsaw. It goes through the city and plays an important role as a landmark.", "When rock units are placed under horizontal compression, they shorten and become thicker. Because rock units, other than muds, do not significantly change in volume, this is accomplished in two primary ways: through faulting and folding. In the shallow crust, where brittle deformation can occur, thrust faults form, which cause deeper rock to move on top of shallower rock. Because deeper rock is often older, as noted by the principle of superposition, this can result in older rocks moving on top of younger ones. Movement along faults can result in folding, either because the faults are not planar or because rock layers are dragged along, forming drag folds as slip occurs along the fault. Deeper in the Earth, rocks behave plastically, and fold instead of faulting. These folds can either be those where the material in the center of the fold buckles upwards, creating \"antiforms\", or where it buckles downwards, creating \"synforms\". If the tops of the rock units within the folds remain pointing upwards, they are called anticlines and synclines, respectively. If some of the units in the fold are facing downward, the structure is called an overturned anticline or syncline, and if all of the rock units are"]</t>
-        </is>
-      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2912,21 +2117,6 @@
 Kenya has a warm and humid tropical climate on its Indian Ocean coastline. The climate is cooler in the savannah grasslands around the capital city, Nairobi, and especially closer to Mount Kenya, which has snow permanently on its peaks. Further inland, in the Nyanza region, there is a hot and dry climate which becomes humid around Lake Victoria, the largest tropical fresh-water lake in the world. This gives way to temperate and forested hilly areas in the neighboring western region. The north-eastern regions along the border with Somalia and Ethiopia are arid and semi-arid areas with near-desert landscapes. Kenya is known for its safaris, diverse climate and geography, and expansive wildlife reserves and national parks such as the East and West Tsavo National Park, the Maasai Mara, Lake Nakuru National Park, and Aberdares National Park. Kenya has several world heritage sites such as Lamu and numerous beaches, including in Diani, Bamburi and Kilifi, where international yachting competitions are held every year.</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>[55, 145, 565, 144, 813]</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>[0.7489407062530518, 0.688716471195221, 0.6798688769340515, 0.669360876083374, 0.6660453677177429]</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>["Between 1402 and 1405, the expedition led by the Norman noble Jean de Bethencourt and the Poitevine Gadifer de la Salle conquered the Canarian islands of Lanzarote, Fuerteventura and El Hierro off the Atlantic coast of Africa. Their troops were gathered in Normandy, Gascony and were later reinforced by Castilian colonists.", "The British, for their part, were happy to take New France, as defence of their North American colonies would no longer be an issue and also because they already had ample places from which to obtain sugar. Spain, which traded Florida to Britain to regain Cuba, also gained Louisiana, including New Orleans, from France in compensation for its losses. Great Britain and Spain also agreed that navigation on the Mississippi River was to be open to vessels of all nations.", "During the mid-Eocene, it is believed that the drainage basin of the Amazon was split along the middle of the continent by the Purus Arch. Water on the eastern side flowed toward the Atlantic, while to the west water flowed toward the Pacific across the Amazonas Basin. As the Andes Mountains rose, however, a large basin was created that enclosed a lake; now known as the Solimões Basin. Within the last 5–10 million years, this accumulating water broke through the Purus Arch, joining the easterly flow toward the Atlantic.", "The war in North America officially ended with the signing of the Treaty of Paris on 10 February 1763, and war in the European theatre of the Seven Years' War was settled by the Treaty of Hubertusburg on 15 February 1763. The British offered France the choice of surrendering either its continental North American possessions east of the Mississippi or the Caribbean islands of Guadeloupe and Martinique, which had been occupied by the British. France chose to cede the former, but was able to negotiate the retention of Saint Pierre and Miquelon, two small islands in the Gulf of St. Lawrence, along with fishing rights in the area. They viewed the economic value of the Caribbean islands' sugar cane to be greater and easier to defend than the furs from the continent. The contemporaneous French philosopher Voltaire referred to Canada disparagingly as nothing more than a few acres of snow. The British, for their part, were happy to take New France, as defence of their North American colonies would no longer be an issue and also because they already had ample places from which to obtain sugar. Spain, which traded Florida to Britain to regain Cuba, also gained Louisiana, including", "Kenya has a warm and humid tropical climate on its Indian Ocean coastline. The climate is cooler in the savannah grasslands around the capital city, Nairobi, and especially closer to Mount Kenya, which has snow permanently on its peaks. Further inland, in the Nyanza region, there is a hot and dry climate which becomes humid around Lake Victoria, the largest tropical fresh-water lake in the world. This gives way to temperate and forested hilly areas in the neighboring western region. The north-eastern regions along the border with Somalia and Ethiopia are arid and semi-arid areas with near-desert landscapes. Kenya is known for its safaris, diverse climate and geography, and expansive wildlife reserves and national parks such as the East and West Tsavo National Park, the Maasai Mara, Lake Nakuru National Park, and Aberdares National Park. Kenya has several world heritage sites such as Lamu and numerous beaches, including in Diani, Bamburi and Kilifi, where international yachting competitions are held every year."]</t>
-        </is>
-      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2958,21 +2148,6 @@
 In the late 17th century, Robert Boyle proved that air is necessary for combustion. English chemist John Mayow (1641–1679) refined this work by showing that fire requires only a part of air that he called spiritus nitroaereus or just nitroaereus. In one experiment he found that placing either a mouse or a lit candle in a closed container over water caused the water to rise and replace one-fourteenth of the air's volume before extinguishing the subjects. From this he surmised that nitroaereus is consumed in both respiration and combustion.</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>[56, 847, 840, 664, 428]</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>[0.7142725586891174, 0.6865575909614563, 0.6851338148117065, 0.6786825060844421, 0.6647255420684814]</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>["The Lobata have a pair of lobes, which are muscular, cuplike extensions of the body that project beyond the mouth. Their inconspicuous tentacles originate from the corners of the mouth, running in convoluted grooves and spreading out over the inner surface of the lobes (rather than trailing far behind, as in the Cydippida). Between the lobes on either side of the mouth, many species of lobates have four auricles, gelatinous projections edged with cilia that produce water currents that help direct microscopic prey toward the mouth. This combination of structures enables lobates to feed continuously on suspended planktonic prey.", "Ranging from about 1 millimeter (0.039 in) to 1.5 meters (4.9 ft) in size, ctenophores are the largest non-colonial animals that use cilia (\"hairs\") as their main method of locomotion. Most species have eight strips, called comb rows, that run the length of their bodies and bear comb-like bands of cilia, called \"ctenes,\" stacked along the comb rows so that when the cilia beat, those of each comb touch the comb below. The name \"ctenophora\" means \"comb-bearing\", from the Greek κτείς (stem-form κτεν-) meaning \"comb\" and the Greek suffix -φορος meaning \"carrying\".", "The Cestida (\"belt animals\") are ribbon-shaped planktonic animals, with the mouth and aboral organ aligned in the middle of opposite edges of the ribbon. There is a pair of comb-rows along each aboral edge, and tentilla emerging from a groove all along the oral edge, which stream back across most of the wing-like body surface. Cestids can swim by undulating their bodies as well as by the beating of their comb-rows. There are two known species, with worldwide distribution in warm, and warm-temperate waters: Cestum veneris (\"Venus' girdle\") is among the largest ctenophores – up to 1.5 meters (4.9 ft) long, and can undulate slowly or quite rapidly. Velamen parallelum, which is typically less than 20 centimeters (0.66 ft) long, can move much faster in what has been described as a \"darting motion\".", "The 1970s and 1980s saw the emergence of many graphical imaging packages for the network in which based the logo's setting mainly on special lighting effects then under development including white, blue, pink, rainbow neon and glittering dotted lines. Among the \"ABC Circle\" logo's many variants was a 1977 ID sequence that featured a bubble on a black background representing the circle with glossy gold letters, and as such, was the first ABC identification card to have a three-dimensional appearance.", "In the late 17th century, Robert Boyle proved that air is necessary for combustion. English chemist John Mayow (1641–1679) refined this work by showing that fire requires only a part of air that he called spiritus nitroaereus or just nitroaereus. In one experiment he found that placing either a mouse or a lit candle in a closed container over water caused the water to rise and replace one-fourteenth of the air's volume before extinguishing the subjects. From this he surmised that nitroaereus is consumed in both respiration and combustion."]</t>
-        </is>
-      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3004,21 +2179,6 @@
 Free movement of goods within the European Union is achieved by a customs union, and the principle of non-discrimination. The EU manages imports from non-member states, duties between member states are prohibited, and imports circulate freely. In addition under the Treaty on the Functioning of the European Union article 34, ‘Quantitative restrictions on imports and all measures having equivalent effect shall be prohibited between Member States’. In Procureur du Roi v Dassonville the Court of Justice held that this rule meant all "trading rules" that are "enacted by Member States" which could hinder trade "directly or indirectly, actually or potentially" would be caught by article 34. This meant that a Belgian law requiring Scotch whisky imports to have a certificate of origin was unlikely to be lawful. It discriminated against parallel importers like Mr Dassonville, who could not get certificates from authorities in France, where they bought the Scotch. This "wide test", to determine what could potentially be an unlawful restriction on trade, applies equally to actions by quasi-government bodies, such as the former "Buy Irish" company that had government appointees. It also means states can be responsible for private actors. For instance, in Commission v France French farmer vigilantes</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>[287, 838, 837, 876, 836]</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>[0.8189836144447327, 0.8185984492301941, 0.8156924247741699, 0.8144097924232483, 0.8043364882469177]</t>
-        </is>
-      </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>["While the Treaties and Regulations will have direct effect (if clear, unconditional and immediate), Directives do not generally give citizens (as opposed to the member state) standing to sue other citizens. In theory, this is because TFEU article 288 says Directives are addressed to the member states and usually \"leave to the national authorities the choice of form and methods\" to implement. In part this reflects that directives often create minimum standards, leaving member states to apply higher standards. For example, the Working Time Directive requires that every worker has at least 4 weeks paid holidays each year, but most member states require more than 28 days in national law. However, on the current position adopted by the Court of Justice, citizens have standing to make claims based on national laws that implement Directives, but not from Directives themselves. Directives do not have so called \"horizontal\" direct effect (i.e. between non-state parties). This view was instantly controversial, and in the early 1990s three Advocate Generals persuasively argued that Directives should create rights and duties for all citizens. The Court of Justice refused, but there are five large exceptions.", "justify restrictions on trade as an overriding requirement derived from TFEU article 11. More generally, it has been increasingly acknowledged that fundamental human rights should take priority over all trade rules. So, in Schmidberger v Austria the Court of Justice held that Austria did not infringe article 34 by failing to ban a protest that blocked heavy traffic passing over the A13, Brenner Autobahn, en route to Italy. Although many companies, including Mr Schmidberger's German undertaking, were prevented from trading, the Court of Justice reasoned that freedom of association is one of the ‘fundamental pillars of a democratic society’, against which the free movement of goods had to be balanced, and was probably subordinate. If a member state does appeal to the article 36 justification, the measures it takes have to be applied proportionately. This means the rule must be pursue a legitimate aim and (1) be suitable to achieve the aim, (2) be necessary, so that a less restrictive measure could not achieve the same result, and (3) be reasonable in balancing the interests of free trade with interests in article 36.", "\"wide test\", to determine what could potentially be an unlawful restriction on trade, applies equally to actions by quasi-government bodies, such as the former \"Buy Irish\" company that had government appointees. It also means states can be responsible for private actors. For instance, in Commission v France French farmer vigilantes were continually sabotaging shipments of Spanish strawberries, and even Belgian tomato imports. France was liable for these hindrances to trade because the authorities ‘manifestly and persistently abstained' from preventing the sabotage. Generally speaking, if a member state has laws or practices that directly discriminate against imports (or exports under TFEU article 35) then it must be justified under article 36. The justifications include public morality, policy or security, \"protection of health and life of humans, animals or plants\", \"national treasures\" of \"artistic, historic or archaeological value\" and \"industrial and commercial property.\" In addition, although not clearly listed, environmental protection can justify restrictions on trade as an overriding requirement derived from TFEU article 11. More generally, it has been increasingly acknowledged that fundamental human rights should take priority over all trade rules. So, in Schmidberger v Austria the Court of Justice held that Austria did not infringe article 34 by failing", "domestic legal provisions, however framed... without the legal basis of the community itself being called into question.\" This meant any \"subsequent unilateral act\" of the member state inapplicable. Similarly, in Amministrazione delle Finanze v Simmenthal SpA, a company, Simmenthal SpA, claimed that a public health inspection fee under an Italian law of 1970 for importing beef from France to Italy was contrary to two Regulations from 1964 and 1968. In \"accordance with the principle of the precedence of Community law,\" said the Court of Justice, the \"directly applicable measures of the institutions\" (such as the Regulations in the case) \"render automatically inapplicable any conflicting provision of current national law\". This was necessary to prevent a \"corresponding denial\" of Treaty \"obligations undertaken unconditionally and irrevocably by member states\", that could \"imperil the very foundations of the\" EU. But despite the views of the Court of Justice, the national courts of member states have not accepted the same analysis.", "Free movement of goods within the European Union is achieved by a customs union, and the principle of non-discrimination. The EU manages imports from non-member states, duties between member states are prohibited, and imports circulate freely. In addition under the Treaty on the Functioning of the European Union article 34, ‘Quantitative restrictions on imports and all measures having equivalent effect shall be prohibited between Member States’. In Procureur du Roi v Dassonville the Court of Justice held that this rule meant all \"trading rules\" that are \"enacted by Member States\" which could hinder trade \"directly or indirectly, actually or potentially\" would be caught by article 34. This meant that a Belgian law requiring Scotch whisky imports to have a certificate of origin was unlikely to be lawful. It discriminated against parallel importers like Mr Dassonville, who could not get certificates from authorities in France, where they bought the Scotch. This \"wide test\", to determine what could potentially be an unlawful restriction on trade, applies equally to actions by quasi-government bodies, such as the former \"Buy Irish\" company that had government appointees. It also means states can be responsible for private actors. For instance, in Commission v France French farmer vigilantes"]</t>
-        </is>
-      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3050,21 +2210,6 @@
 Continuing the style of the earlier buildings, various designers were responsible for the decoration, the terracotta embellishments were again the work of Godfrey Sykes, although sgraffito was used to decorate the east side of the building designed by F. W. Moody, a final embellishment were the wrought iron gates made as late as 1885 designed by Starkie Gardner, these lead to a passage through the building. Scott also designed the two Cast Courts 1870–73 to the southeast of the garden (the site of the "Brompton Boilers"), these vast spaces have ceilings 70 feet (21 m) in height to accommodate the plaster casts of parts of famous buildings, including Trajan's Column (in two separate pieces). The final part of the museum designed by Scott was the Art Library and what is now the sculpture gallery on the south side of the garden, built 1877–83, the exterior mosaic panels in the parapet were designed by Reuben Townroe who also designed the plaster work in the library, Sir John Taylor designed the book shelves and cases, also this was the first part of the museum to have electric lighting. This completed the northern half of the site, creating a quadrangle with the garden</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>[58, 588, 138, 716, 587]</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>[0.7848709225654602, 0.7783191800117493, 0.7746615409851074, 0.7651125192642212, 0.7606277465820312]</t>
-        </is>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>["After World War II, under a Communist regime set up by the conquering Soviets, the \"Bricks for Warsaw\" campaign was initiated, and large prefabricated housing projects were erected in Warsaw to address the housing shortage, along with other typical buildings of an Eastern Bloc city, such as the Palace of Culture and Science, a gift from the Soviet Union. The city resumed its role as the capital of Poland and the country's centre of political and economic life. Many of the historic streets, buildings, and churches were restored to their original form. In 1980, Warsaw's historic Old Town was inscribed onto UNESCO's World Heritage list.", "were designed by Reuben Townroe who also designed the plaster work in the library, Sir John Taylor designed the book shelves and cases, also this was the first part of the museum to have electric lighting. This completed the northern half of the site, creating a quadrangle with the garden at its centre, but left the museum without a proper façade. In 1890 the government launched a competition to design new buildings for the museum, with architect Alfred Waterhouse as one of the judges; this would give the museum a new imposing front entrance.", "After the 1940s, the Gothic style on campus began to give way to modern styles. In 1955, Eero Saarinen was contracted to develop a second master plan, which led to the construction of buildings both north and south of the Midway, including the Laird Bell Law Quadrangle (a complex designed by Saarinen); a series of arts buildings; a building designed by Ludwig Mies van der Rohe for the university's School of Social Service Administration;, a building which is to become the home of the Harris School of Public Policy Studies by Edward Durrell Stone, and the Regenstein Library, the largest building on campus, a brutalist structure designed by Walter Netsch of the Chicago firm Skidmore, Owings &amp; Merrill. Another master plan, designed in 1999 and updated in 2004, produced the Gerald Ratner Athletics Center (2003), the Max Palevsky Residential Commons (2001), South Campus Residence Hall and dining commons (2009), a new children's hospital, and other construction, expansions, and restorations. In 2011, the university completed the glass dome-shaped Joe and Rika Mansueto Library, which provides a grand reading room for the university library and prevents the need for an off-campus book depository.", "The Victorian parts of the building have a complex history, with piecemeal additions by different architects. Founded in May 1852, it was not until 1857 that the museum moved to the present site. This area of London was known as Brompton but had been renamed South Kensington. The land was occupied by Brompton Park House, which was extended, most notably by the \"Brompton Boilers\", which were starkly utilitarian iron galleries with a temporary look and were later dismantled and used to build the V&amp;A Museum of Childhood. The first building to be erected that still forms part of the museum was the Sheepshanks Gallery in 1857 on the eastern side of the garden. Its architect was civil engineer Captain Francis Fowke, Royal Engineers, who was appointed by Cole. The next major expansions were designed by the same architect, the Turner and Vernon galleries built 1858-9 to house the eponymous collections (later transferred to the Tate Gallery) and now used as the picture galleries and tapestry gallery respectively. The North and South Courts, were then built, both of which opened by June 1862. They now form the galleries for temporary exhibitions and are directly behind the Sheepshanks Gallery. On the very", "Continuing the style of the earlier buildings, various designers were responsible for the decoration, the terracotta embellishments were again the work of Godfrey Sykes, although sgraffito was used to decorate the east side of the building designed by F. W. Moody, a final embellishment were the wrought iron gates made as late as 1885 designed by Starkie Gardner, these lead to a passage through the building. Scott also designed the two Cast Courts 1870–73 to the southeast of the garden (the site of the \"Brompton Boilers\"), these vast spaces have ceilings 70 feet (21 m) in height to accommodate the plaster casts of parts of famous buildings, including Trajan's Column (in two separate pieces). The final part of the museum designed by Scott was the Art Library and what is now the sculpture gallery on the south side of the garden, built 1877–83, the exterior mosaic panels in the parapet were designed by Reuben Townroe who also designed the plaster work in the library, Sir John Taylor designed the book shelves and cases, also this was the first part of the museum to have electric lighting. This completed the northern half of the site, creating a quadrangle with the garden"]</t>
-        </is>
-      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3096,21 +2241,6 @@
 the merger, Thomas S. Murphy left ABC with Robert Iger taking his place as president and CEO. Around the time of the merger, Disney's television production units had already produced series for the network such as Home Improvement and Boy Meets World, while the deal also allowed ABC access to Disney's children's programming library for its Saturday morning block. In 1998, ABC premiered the Aaron Sorkin-created sitcom Sports Night, centering on the travails of the staff of a SportsCenter-style sports news program; despite earning critical praise and multiple Emmy Awards, the series was cancelled in 2000 after two seasons.</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>[60, 59, 155, 857, 104]</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>[0.8094450235366821, 0.7514116168022156, 0.7370472550392151, 0.7303920388221741, 0.7290820479393005]</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>["telecasts are scheduled, usually airing between 4:00 and 6:00 p.m. Eastern and Pacific Time. During the summer, ABC airs ESPN-produced highlight compilation programs for The Open Championship golf and The Wimbledon tennis tournaments to provide some presence for both events on American broadcast television. ABC also carries various X Games weekend events not broadcast by ESPN. ABC airs NBA games on Sundays, normally starting in January as \"NBA Sunday Showcase\" during the regular season, and shows Christmas Day games, regularly between 2–7 PM ET, and NBA playoff games during the weekends, and exclusive rights to the NBA Finals.", "Sports programming is also provided on some weekend afternoons at any time from 12:00 to 6:00 p.m. Eastern Time (9:00 a.m. to 3:00 p.m. Pacific) and, during college football season, during prime time on Saturday nights as part of the Saturday Night Football package. Due to the erratic and (outside of college football season) highly inconsistent scheduling of sports programming on weekend afternoons since ESPN took over responsibilities for ABC's sports division in 2006, ABC carries the ESPN Sports Saturday block on Saturday late afternoons (featuring various ESPN-produced documentaries), and on Sundays either encores of primetime reality series, cancelled series being burned off that had no room on the primetime schedule, occasional theatrical films which were acquired by the network in the early to mid-2000s that no longer have a primetime slot to air in or more recently, figure skating and gymnastics specials supplied by Disson Skating, when no sports telecasts are scheduled, usually airing between 4:00 and 6:00 p.m. Eastern and Pacific Time. During the summer, ABC airs ESPN-produced highlight compilation programs for The Open Championship golf and The Wimbledon tennis tournaments to provide some presence for both events on American broadcast television. ABC also carries various X Games", "In May 2013, ABC launched \"WATCH ABC\", a revamp of its traditional multi-platform streaming services encompassing the network's existing streaming portal at ABC.com and a mobile app for smartphones and tablet computers; in addition to providing full-length episodes of ABC programs, the service allows live programming streams of local ABC affiliates in select markets (the first such offering by a U.S. broadcast network). Similar to sister network ESPN's WatchESPN service (which originated the \"WATCH\" brand used by the streaming services of Disney's television networks), live streams of ABC stations are only available to authenticated subscribers of participating pay television providers in certain markets. New York City O&amp;O WABC-TV and Philadelphia O&amp;O WPVI-TV were the first stations to offer streams of their programming on the service (with a free preview for non-subscribers through June 2013), with the six remaining ABC O&amp;Os offering streams by the start of the 2013–14 season. Hearst Television also reached a deal to offer streams of its ABC affiliates (including stations in Boston, Kansas City, Milwaukee and West Palm Beach) on the service.", "Always in search of new programs that would help it compete with NBC and CBS, ABC's management believed that sports could be a major catalyst in improving the network's market share. On April 29, 1961, ABC debuted Wide World of Sports, an anthology series created by Edgar Scherick through his company Sports Programs, Inc. and produced by a young Roone Arledge which featured a different sporting event each broadcast. ABC purchased Sports Programs, Inc. in exchange for shares in the company, leading it to become the future core of ABC Sports, with Arledge as the executive producer of that division's shows. Wide World of Sports, in particular, was not merely devoted to a single sport, but rather to generally all sporting events.", "the merger, Thomas S. Murphy left ABC with Robert Iger taking his place as president and CEO. Around the time of the merger, Disney's television production units had already produced series for the network such as Home Improvement and Boy Meets World, while the deal also allowed ABC access to Disney's children's programming library for its Saturday morning block. In 1998, ABC premiered the Aaron Sorkin-created sitcom Sports Night, centering on the travails of the staff of a SportsCenter-style sports news program; despite earning critical praise and multiple Emmy Awards, the series was cancelled in 2000 after two seasons."]</t>
-        </is>
-      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3142,21 +2272,6 @@
 Newborn infants have no prior exposure to microbes and are particularly vulnerable to infection. Several layers of passive protection are provided by the mother. During pregnancy, a particular type of antibody, called IgG, is transported from mother to baby directly across the placenta, so human babies have high levels of antibodies even at birth, with the same range of antigen specificities as their mother. Breast milk or colostrum also contains antibodies that are transferred to the gut of the infant and protect against bacterial infections until the newborn can synthesize its own antibodies. This is passive immunity because the fetus does not actually make any memory cells or antibodies—it only borrows them. This passive immunity is usually short-term, lasting from a few days up to several months. In medicine, protective passive immunity can also be transferred artificially from one individual to another via antibody-rich serum.</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>[61, 16, 360, 428, 700]</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>[0.7584619522094727, 0.755547285079956, 0.6412495970726013, 0.6383759379386902, 0.6378107666969299]</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>["Almost all species are hermaphrodites, in other words they function as both males and females at the same time – except that in two species of the genus Ocryopsis individuals remain of the same single sex all their lives. The gonads are located in the parts of the internal canal network under the comb rows, and eggs and sperm are released via pores in the epidermis. Fertilization is external in most species, but platyctenids use internal fertilization and keep the eggs in brood chambers until they hatch. Self-fertilization has occasionally been seen in species of the genus Mnemiopsis, and it is thought that most of the hermaphroditic species are self-fertile.", "Most species are hermaphrodites—a single animal can produce both eggs and sperm, meaning it can fertilize its own egg, not needing a mate. Some are simultaneous hermaphrodites, which can produce both eggs and sperm at the same time. Others are sequential hermaphrodites, in which the eggs and sperm mature at different times. Fertilization is generally external, although platyctenids' eggs are fertilized inside their parents' bodies and kept there until they hatch. The young are generally planktonic and in most species look like miniature cydippids, gradually changing into their adult shapes as they grow. The exceptions are the beroids, whose young are miniature beroids with large mouths and no tentacles, and the platyctenids, whose young live as cydippid-like plankton until they reach near-adult size, but then sink to the bottom and rapidly metamorphose into the adult form. In at least some species, juveniles are capable of reproduction before reaching the adult size and shape. The combination of hermaphroditism and early reproduction enables small populations to grow at an explosive rate.", "Chloroplasts' main role is to conduct photosynthesis, where the photosynthetic pigment chlorophyll captures the energy from sunlight and converts it and stores it in the energy-storage molecules ATP and NADPH while freeing oxygen from water. They then use the ATP and NADPH to make organic molecules from carbon dioxide in a process known as the Calvin cycle. Chloroplasts carry out a number of other functions, including fatty acid synthesis, much amino acid synthesis, and the immune response in plants. The number of chloroplasts per cell varies from 1 in algae up to 100 in plants like Arabidopsis and wheat.", "In the late 17th century, Robert Boyle proved that air is necessary for combustion. English chemist John Mayow (1641–1679) refined this work by showing that fire requires only a part of air that he called spiritus nitroaereus or just nitroaereus. In one experiment he found that placing either a mouse or a lit candle in a closed container over water caused the water to rise and replace one-fourteenth of the air's volume before extinguishing the subjects. From this he surmised that nitroaereus is consumed in both respiration and combustion.", "Newborn infants have no prior exposure to microbes and are particularly vulnerable to infection. Several layers of passive protection are provided by the mother. During pregnancy, a particular type of antibody, called IgG, is transported from mother to baby directly across the placenta, so human babies have high levels of antibodies even at birth, with the same range of antigen specificities as their mother. Breast milk or colostrum also contains antibodies that are transferred to the gut of the infant and protect against bacterial infections until the newborn can synthesize its own antibodies. This is passive immunity because the fetus does not actually make any memory cells or antibodies—it only borrows them. This passive immunity is usually short-term, lasting from a few days up to several months. In medicine, protective passive immunity can also be transferred artificially from one individual to another via antibody-rich serum."]</t>
-        </is>
-      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3188,21 +2303,6 @@
 From their original homelands in Scandinavia and northern Europe, Germanic tribes expanded throughout northern and western Europe in the middle period of classical antiquity; southern Europe in late antiquity, conquering Celtic and other peoples; and by 800 CE, forming the Holy Roman Empire, the first German Empire. However, there was no real systemic continuity from the Western Roman Empire to its German successor which was famously described as "not holy, not Roman, and not an empire", as a great number of small states and principalities existed in the loosely autonomous confederation. Although by 1000 CE, the Germanic conquest of central, western, and southern Europe (west of and including Italy) was complete, excluding only Muslim Iberia. There was, however, little cultural integration or national identity, and "Germany" remained largely a conceptual term referring to an amorphous area of central Europe.</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>[62, 403, 91, 141, 546]</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>[0.8420627117156982, 0.7350544333457947, 0.7284502983093262, 0.6961082220077515, 0.6925464868545532]</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>["The Ottoman Empire was an imperial state that lasted from 1299 to 1923. During the 16th and 17th centuries, in particular at the height of its power under the reign of Suleiman the Magnificent, the Ottoman Empire was a powerful multinational, multilingual empire controlling much of Southeast Europe, Western Asia, the Caucasus, North Africa, and the Horn of Africa. At the beginning of the 17th century the empire contained 32 provinces and numerous vassal states. Some of these were later absorbed into the empire, while others were granted various types of autonomy during the course of centuries.", "\"The word ‘empire’ comes from the Latin word imperium; for which the closest modern English equivalent would perhaps be ‘sovereignty’, or simply ‘rule’\". The greatest distinction of an empire is through the amount of land that a nation has conquered and expanded. Political power grew from conquering land, however cultural and economic aspects flourished through sea and trade routes. A distinction about empires is \"that although political empires were built mostly by expansion overland, economic and cultural influences spread at least as much by sea\". Some of the main aspects of trade that went overseas consisted of animals and plant products. European empires in Asia and Africa \"have come to be seen as the classic forms of imperialism: and indeed most books on the subject confine themselves to the European seaborne empires\". European expansion caused the world to be divided by how developed and developing nation are portrayed through the world systems theory. The two main regions are the core and the periphery. The core consists of high areas of income and profit; the periphery is on the opposing side of the spectrum consisting of areas of low income and profit. These critical theories of Geo-politics have led to increased", "The plague struck various countries in the Middle East during the pandemic, leading to serious depopulation and permanent change in both economic and social structures. As it spread to western Europe, the disease entered the region from southern Russia also. By autumn 1347, the plague reached Alexandria in Egypt, probably through the port's trade with Constantinople, and ports on the Black Sea. During 1347, the disease travelled eastward to Gaza, and north along the eastern coast to cities in Lebanon, Syria and Palestine, including Ashkelon, Acre, Jerusalem, Sidon, Damascus, Homs, and Aleppo. In 1348–49, the disease reached Antioch. The city's residents fled to the north, most of them dying during the journey, but the infection had been spread to the people of Asia Minor.[citation needed]", "The African Great Lakes region, which Kenya is a part of, has been inhabited by humans since the Lower Paleolithic period. By the first millennium AD, the Bantu expansion had reached the area from West-Central Africa. The borders of the modern state consequently comprise the crossroads of the Niger-Congo, Nilo-Saharan and Afroasiatic areas of the continent, representing most major ethnolinguistic groups found in Africa. Bantu and Nilotic populations together constitute around 97% of the nation's residents. European and Arab presence in coastal Mombasa dates to the Early Modern period; European exploration of the interior began in the 19th century. The British Empire established the East Africa Protectorate in 1895, which starting in 1920 gave way to the Kenya Colony. Kenya obtained independence in December 1963. Following a referendum in August 2010 and adoption of a new constitution, Kenya is now divided into 47 semi-autonomous counties, governed by elected governors.", "From their original homelands in Scandinavia and northern Europe, Germanic tribes expanded throughout northern and western Europe in the middle period of classical antiquity; southern Europe in late antiquity, conquering Celtic and other peoples; and by 800 CE, forming the Holy Roman Empire, the first German Empire. However, there was no real systemic continuity from the Western Roman Empire to its German successor which was famously described as \"not holy, not Roman, and not an empire\", as a great number of small states and principalities existed in the loosely autonomous confederation. Although by 1000 CE, the Germanic conquest of central, western, and southern Europe (west of and including Italy) was complete, excluding only Muslim Iberia. There was, however, little cultural integration or national identity, and \"Germany\" remained largely a conceptual term referring to an amorphous area of central Europe."]</t>
-        </is>
-      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3234,21 +2334,6 @@
 stopped with its 1998–2002 four-note jingles for promotions and production company vanity cards following the closing credits of most of its programs over seventeen years, now it have a different and adventure-type music (with the drums of the network's four-note signature in the ending). The old four-note theme tune is still used by ABC on Demand to the beginning of the ABC show.</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>[469, 219, 201, 245, 37]</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>[0.7242060899734497, 0.7143369317054749, 0.7084680795669556, 0.7071031928062439, 0.7040810585021973]</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>["The Social Charter was subsequently adopted in 1989 by 11 of the then 12 member states. The UK refused to sign the Social Charter and was exempt from the legislation covering Social Charter issues unless it agreed to be bound by the legislation. The UK subsequently was the only member state to veto the Social Charter being included as the \"Social Chapter\" of the 1992 Maastricht Treaty - instead, an Agreement on Social Policy was added as a protocol. Again, the UK was exempt from legislation arising from the protocol, unless it agreed to be bound by it. The protocol was to become known as \"Social Chapter\", despite not actually being a chapter of the Maastricht Treaty. To achieve aims of the Agreement on Social Policy the European Union was to \"support and complement\" the policies of member states. The aims of the Agreement on Social Policy are:", "Decisions in-between the four-year meetings are made by the Mission Council (usually consisting of church bishops). One of the most high profile decisions in recent years by one of the councils was a decision by the Mission Council of the South Central Jurisdiction which in March 2007 approved a 99-year lease of 36 acres (150,000 m2) at Southern Methodist University for the George W. Bush Presidential Library. The decision generated controversy in light of Bush's support of the Iraq War which the church bishops have criticized. A debate over whether the decision should or could be submitted for approval by the Southern Jurisdictional Conference at its July 2008 meeting in Dallas, Texas, remains unresolved.", "In December 2014, President Uhuru Kenyatta signed a Security Laws Amendment Bill, which supporters of the law suggested was necessary to guard against armed groups. Opposition politicians, human rights groups, and nine Western countries criticised the security bill, arguing that it infringed on democratic freedoms. The governments of the United States, Britain, Germany and France also collectively issued a press statement cautioning about the law's potential impact. Through the Jubillee Coalition, the Bill was later passed on 19 December in the National Assembly under acrimonious circumstances.", "The principal Treaties that form the European Union began with common rules for coal and steel, and then atomic energy, but more complete and formal institutions were established through the Treaty of Rome 1957 and the Maastricht Treaty 1992 (now: TFEU). Minor amendments were made during the 1960s and 1970s. Major amending treaties were signed to complete the development of a single, internal market in the Single European Act 1986, to further the development of a more social Europe in the Treaty of Amsterdam 1997, and to make minor amendments to the relative power of member states in the EU institutions in the Treaty of Nice 2001 and the Treaty of Lisbon 2007. Since its establishment, more member states have joined through a series of accession treaties, from the UK, Ireland, Denmark and Norway in 1972 (though Norway did not end up joining), Greece in 1979, Spain and Portugal 1985, Austria, Finland, Norway and Sweden in 1994 (though again Norway failed to join, because of lack of support in the referendum), the Czech Republic, Cyprus, Estonia, Hungary, Latvia, Lithuania, Malta, Poland, Slovakia and Slovenia in 2004, Romania and Bulgaria in 2007 and Croatia in 2013. Greenland signed a Treaty in", "stopped with its 1998–2002 four-note jingles for promotions and production company vanity cards following the closing credits of most of its programs over seventeen years, now it have a different and adventure-type music (with the drums of the network's four-note signature in the ending). The old four-note theme tune is still used by ABC on Demand to the beginning of the ABC show."]</t>
-        </is>
-      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3280,21 +2365,6 @@
 The Broncos' defense ranked first in the NFL yards allowed (4,530) for the first time in franchise history, and fourth in points allowed (296). Defensive ends Derek Wolfe and Malik Jackson each had 5½ sacks. Pro Bowl linebacker Von Miller led the team with 11 sacks, forced four fumbles, and recovered three. Linebacker DeMarcus Ware was selected to play in the Pro Bowl for the ninth time in his career, ranking second on the team with 7½ sacks. Linebacker Brandon Marshall led the team in total tackles with 109, while Danny Trevathan ranked second with 102. Cornerbacks Aqib Talib (three interceptions) and Chris Harris, Jr. (two interceptions) were the other two Pro Bowl selections from the defense.</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>[64, 867, 418, 12, 523]</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>[0.8645331859588623, 0.7592966556549072, 0.7352710962295532, 0.7349357604980469, 0.7341500520706177]</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>["This was the first Super Bowl to feature a quarterback on both teams who was the #1 pick in their draft classes. Manning was the #1 selection of the 1998 NFL draft, while Newton was picked first in 2011. The matchup also pits the top two picks of the 2011 draft against each other: Newton for Carolina and Von Miller for Denver. Manning and Newton also set the record for the largest age difference between opposing Super Bowl quarterbacks at 13 years and 48 days (Manning was 39, Newton was 26).", "In honor of the 50th Super Bowl, the pregame ceremony featured the on-field introduction of 39 of the 43 previous Super Bowl Most Valuable Players. Bart Starr (MVP of Super Bowls I and II) and Chuck Howley (MVP of Super Bowl V) appeared via video, while Peyton Manning (MVP of Super Bowl XLI and current Broncos quarterback) was shown in the locker room preparing for the game. No plans were announced regarding the recognition of Harvey Martin, co-MVP of Super Bowl XII, who died in 2001.", "In early 2012, NFL Commissioner Roger Goodell stated that the league planned to make the 50th Super Bowl \"spectacular\" and that it would be \"an important game for us as a league\".", "Peyton Manning became the first quarterback ever to lead two different teams to multiple Super Bowls. He is also the oldest quarterback ever to play in a Super Bowl at age 39. The past record was held by John Elway, who led the Broncos to victory in Super Bowl XXXIII at age 38 and is currently Denver's Executive Vice President of Football Operations and General Manager.", "The Broncos' defense ranked first in the NFL yards allowed (4,530) for the first time in franchise history, and fourth in points allowed (296). Defensive ends Derek Wolfe and Malik Jackson each had 5½ sacks. Pro Bowl linebacker Von Miller led the team with 11 sacks, forced four fumbles, and recovered three. Linebacker DeMarcus Ware was selected to play in the Pro Bowl for the ninth time in his career, ranking second on the team with 7½ sacks. Linebacker Brandon Marshall led the team in total tackles with 109, while Danny Trevathan ranked second with 102. Cornerbacks Aqib Talib (three interceptions) and Chris Harris, Jr. (two interceptions) were the other two Pro Bowl selections from the defense."]</t>
-        </is>
-      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3326,21 +2396,6 @@
 Sanctifying Grace is that grace of God which sustains the believers in the journey toward Christian Perfection: a genuine love of God with heart, soul, mind, and strength, and a genuine love of our neighbors as ourselves. Sanctifying grace enables us to respond to God by leading a Spirit-filled and Christ-like life aimed toward love. Wesley never claimed this state of perfection for himself but instead insisted the attainment of perfection was possible for all Christians. Here the English Reformer parted company with both Luther and Calvin, who denied that a man would ever reach a state in this life in which he could not fall into sin. Such a man can lose all inclination to evil and can gain perfection in this life.</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>[40, 150, 398, 446, 53]</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>[0.8305776715278625, 0.7937824726104736, 0.7859063148498535, 0.7809157967567444, 0.7754032015800476]</t>
-        </is>
-      </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>["In 1735, John and Charles Wesley went to America to teach the gospel to the American Indians in the colony of Georgia. In less than two years, the \"Holy Club\" disbanded. John Wesley returned to England and met with a group of clergy he respected. He said \"they appeared to be of one heart, as well as of one judgment, resolved to be Bible-Christians at all events; and, wherever they were, to preach with all their might plain, old, Bible Christianity\". The ministers retained their membership in the Church of England. Though not always emphasized or appreciated in the Anglican churches of their day, their teaching emphasized salvation by God's grace, acquired through faith in Christ. Three teachings they saw as the foundation of Christian faith were:", "was \"as though I had been born again.\" His entry into Paradise, no less, was a discovery about \"the righteousness of God\" – a discovery that \"the just person\" of whom the Bible speaks (as in Romans 1:17) lives by faith. He explained his concept of \"justification\" in the Smalcald Articles:", "Luther's rediscovery of \"Christ and His salvation\" was the first of two points that became the foundation for the Reformation. His railing against the sale of indulgences was based on it.", "The movement which would become The United Methodist Church began in the mid-18th century within the Church of England. A small group of students, including John Wesley, Charles Wesley and George Whitefield, met on the Oxford University campus. They focused on Bible study, methodical study of scripture and living a holy life. Other students mocked them, saying they were the \"Holy Club\" and \"the Methodists\", being methodical and exceptionally detailed in their Bible study, opinions and disciplined lifestyle. Eventually, the so-called Methodists started individual societies or classes for members of the Church of England who wanted to live a more religious life.", "Sanctifying Grace is that grace of God which sustains the believers in the journey toward Christian Perfection: a genuine love of God with heart, soul, mind, and strength, and a genuine love of our neighbors as ourselves. Sanctifying grace enables us to respond to God by leading a Spirit-filled and Christ-like life aimed toward love. Wesley never claimed this state of perfection for himself but instead insisted the attainment of perfection was possible for all Christians. Here the English Reformer parted company with both Luther and Calvin, who denied that a man would ever reach a state in this life in which he could not fall into sin. Such a man can lose all inclination to evil and can gain perfection in this life."]</t>
-        </is>
-      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3372,21 +2427,6 @@
 in interceptions. In week 10, Manning suffered a partial tear of the plantar fasciitis in his left foot. He set the NFL's all-time record for career passing yards in this game, but was benched after throwing four interceptions in favor of backup quarterback Brock Osweiler, who took over as the starter for most of the remainder of the regular season. Osweiler was injured, however, leading to Manning's return during the Week 17 regular season finale, where the Broncos were losing 13–7 against the 4–11 San Diego Chargers, resulting in Manning re-claiming the starting quarterback position for the playoffs by leading the team to a key 27–20 win that enabled the team to clinch the number one overall AFC seed. Under defensive coordinator Wade Phillips, the Broncos' defense ranked number one in total yards allowed, passing yards allowed and sacks, and like the previous three seasons, the team has continued to set numerous individual, league and franchise records. With the defense carrying the team despite the issues with the offense, the Broncos finished the regular season with a 12–4 record and earned home-field advantage throughout the AFC playoffs.</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>[64, 867, 12, 205, 206]</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>[0.8205466866493225, 0.8067194819450378, 0.8025323152542114, 0.7732101082801819, 0.7730382680892944]</t>
-        </is>
-      </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>["This was the first Super Bowl to feature a quarterback on both teams who was the #1 pick in their draft classes. Manning was the #1 selection of the 1998 NFL draft, while Newton was picked first in 2011. The matchup also pits the top two picks of the 2011 draft against each other: Newton for Carolina and Von Miller for Denver. Manning and Newton also set the record for the largest age difference between opposing Super Bowl quarterbacks at 13 years and 48 days (Manning was 39, Newton was 26).", "In honor of the 50th Super Bowl, the pregame ceremony featured the on-field introduction of 39 of the 43 previous Super Bowl Most Valuable Players. Bart Starr (MVP of Super Bowls I and II) and Chuck Howley (MVP of Super Bowl V) appeared via video, while Peyton Manning (MVP of Super Bowl XLI and current Broncos quarterback) was shown in the locker room preparing for the game. No plans were announced regarding the recognition of Harvey Martin, co-MVP of Super Bowl XII, who died in 2001.", "Peyton Manning became the first quarterback ever to lead two different teams to multiple Super Bowls. He is also the oldest quarterback ever to play in a Super Bowl at age 39. The past record was held by John Elway, who led the Broncos to victory in Super Bowl XXXIII at age 38 and is currently Denver's Executive Vice President of Football Operations and General Manager.", "Following their loss in the divisional round of the previous season's playoffs, the Denver Broncos underwent numerous coaching changes, including a mutual parting with head coach John Fox (who had won four divisional championships in his four years as Broncos head coach), and the hiring of Gary Kubiak as the new head coach. Under Kubiak, the Broncos planned to install a run-oriented offense with zone blocking to blend in with quarterback Peyton Manning's shotgun passing skills, but struggled with numerous changes and injuries to the offensive line, as well as Manning having his worst statistical season since his rookie year with the Indianapolis Colts in 1998, due to a plantar fasciitis injury in his heel that he had suffered since the summer, and the simple fact that Manning was getting old, as he turned 39 in the 2015 off-season. Although the team had a 7–0 start, Manning led the NFL in interceptions. In week 10, Manning suffered a partial tear of the plantar fasciitis in his left foot. He set the NFL's all-time record for career passing yards in this game, but was benched after throwing four interceptions in favor of backup quarterback Brock Osweiler, who took over as the", "in interceptions. In week 10, Manning suffered a partial tear of the plantar fasciitis in his left foot. He set the NFL's all-time record for career passing yards in this game, but was benched after throwing four interceptions in favor of backup quarterback Brock Osweiler, who took over as the starter for most of the remainder of the regular season. Osweiler was injured, however, leading to Manning's return during the Week 17 regular season finale, where the Broncos were losing 13–7 against the 4–11 San Diego Chargers, resulting in Manning re-claiming the starting quarterback position for the playoffs by leading the team to a key 27–20 win that enabled the team to clinch the number one overall AFC seed. Under defensive coordinator Wade Phillips, the Broncos' defense ranked number one in total yards allowed, passing yards allowed and sacks, and like the previous three seasons, the team has continued to set numerous individual, league and franchise records. With the defense carrying the team despite the issues with the offense, the Broncos finished the regular season with a 12–4 record and earned home-field advantage throughout the AFC playoffs."]</t>
-        </is>
-      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3418,21 +2458,6 @@
 In 1968, ABC took advantage of new FCC ownership regulations that allowed broadcasting companies to own a maximum of seven radio stations nationwide in order to purchase Houston radio stations KXYZ and KXYZ-FM for $1 million in shares and $1.5 million in bonds. That year, Roone Arledge was named president of ABC Sports; the company also founded ABC Pictures, a film production company which released its first picture that year, the Ralph Nelson-directed Charly. It was renamed ABC Motion Pictures in 1979; the unit was dissolved in 1985. The studio also operated two subsidiaries, Palomar Pictures International and Selmur Pictures. In July 1968, ABC continued its acquisitions in the amusement parks sector with the opening of ABC Marine World in Redwood City, California; that park was sold in 1972 and demolished in 1986, with the land that occupied the park later becoming home to the headquarters of Oracle Corporation.</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>[66, 689, 584, 104, 462]</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>[0.8404031991958618, 0.7827366590499878, 0.781259298324585, 0.766303300857544, 0.7590834498405457]</t>
-        </is>
-      </c>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>["On the television side, in September 1969, ABC launched the Movie of the Week, a weekly showcase aimed at capitalizing on the growing success of made-for-TV movies since the early 1960s. The Movie of the Week broadcast feature-length dramatic films directed by such talented filmmakers as Aaron Spelling, David Wolper and Steven Spielberg (the latter of whom gained early success through the showcase for his 1971 film Duel) that were produced on an average budget of $400,000–$450,000. Hits for the television network during the late 1960s and early 1970s included The Courtship of Eddie's Father, The Brady Bunch and The Partridge Family.", "Due to pressure from film studios wanting to increase their production, as the major networks began airing theatrically released films, ABC joined CBS and NBC in broadcasting films on Sunday nights in 1962, with the launch of the ABC Sunday Night Movie, which debuted a year behind its competitors and was initially presented in black-and-white. Despite a significant increase in viewership (with its audience share having increased to 33% from the 15% share it had in 1953), ABC remained in third place; the company had a total revenue of $15.5 million, a third of the revenue pulled in by CBS at the same period. To catch up, ABC followed up The Flintstones with another animated series from Hanna-Barbera, The Jetsons, which debuted on September 23, 1962 as the first television series to be broadcast in color on the network. On April 1, 1963, ABC debuted the soap opera General Hospital, which would go on to become the television network's long-running entertainment program. That year also saw the premiere of The Fugitive (on September 17), a drama series centering on a man on the run after being accused of committing a murder he did not commit.", "At the same time he made attempts to help grow ABC, Goldenson had been trying since mid-1953 to provide content for the network by contacting his old acquaintances in Hollywood, with whom he had worked when UPT was a subsidiary of Paramount Pictures. ABC's merger with UPT led to the creation of relationships with Hollywood's film production studios, breaking a quarantine that had existed at that time between film and television, the latter of which had previously been more connected to radio. ABC's flagship productions at the time were The Lone Ranger, based on the radio program of the same title, and The Adventures of Ozzie and Harriet, the latter of which (at 13 seasons, running from 1952 to 1965) held the record for the longest-running prime time comedy in U.S. television history, until it was surpassed by The Simpsons in 2002.", "the merger, Thomas S. Murphy left ABC with Robert Iger taking his place as president and CEO. Around the time of the merger, Disney's television production units had already produced series for the network such as Home Improvement and Boy Meets World, while the deal also allowed ABC access to Disney's children's programming library for its Saturday morning block. In 1998, ABC premiered the Aaron Sorkin-created sitcom Sports Night, centering on the travails of the staff of a SportsCenter-style sports news program; despite earning critical praise and multiple Emmy Awards, the series was cancelled in 2000 after two seasons.", "In 1968, ABC took advantage of new FCC ownership regulations that allowed broadcasting companies to own a maximum of seven radio stations nationwide in order to purchase Houston radio stations KXYZ and KXYZ-FM for $1 million in shares and $1.5 million in bonds. That year, Roone Arledge was named president of ABC Sports; the company also founded ABC Pictures, a film production company which released its first picture that year, the Ralph Nelson-directed Charly. It was renamed ABC Motion Pictures in 1979; the unit was dissolved in 1985. The studio also operated two subsidiaries, Palomar Pictures International and Selmur Pictures. In July 1968, ABC continued its acquisitions in the amusement parks sector with the opening of ABC Marine World in Redwood City, California; that park was sold in 1972 and demolished in 1986, with the land that occupied the park later becoming home to the headquarters of Oracle Corporation."]</t>
-        </is>
-      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3464,21 +2489,6 @@
 While experimenting, Tesla inadvertently faulted a power station generator, causing a power outage. In August 1917, Tesla explained what had happened in The Electrical Experimenter: "As an example of what has been done with several hundred kilowatts of high frequency energy liberated, it was found that the dynamos in a power house six miles away were repeatedly burned out, due to the powerful high frequency currents set up in them, and which caused heavy sparks to jump through the windings and destroy the insulation!"</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>[67, 664, 312, 379, 785]</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>[0.7696036696434021, 0.729641854763031, 0.7260945439338684, 0.7244550585746765, 0.7242887020111084]</t>
-        </is>
-      </c>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>["Grissom, White, and Chaffee decided to name their flight Apollo 1 as a motivational focus on the first manned flight. They trained and conducted tests of their spacecraft at North American, and in the altitude chamber at the Kennedy Space Center. A \"plugs-out\" test was planned for January, which would simulate a launch countdown on LC-34 with the spacecraft transferring from pad-supplied to internal power. If successful, this would be followed by a more rigorous countdown simulation test closer to the February 21 launch, with both spacecraft and launch vehicle fueled.", "The 1970s and 1980s saw the emergence of many graphical imaging packages for the network in which based the logo's setting mainly on special lighting effects then under development including white, blue, pink, rainbow neon and glittering dotted lines. Among the \"ABC Circle\" logo's many variants was a 1977 ID sequence that featured a bubble on a black background representing the circle with glossy gold letters, and as such, was the first ABC identification card to have a three-dimensional appearance.", "The delay in the CSM caused by the fire enabled NASA to catch up on man-rating the LM and Saturn V. Apollo 4 (AS-501) was the first unmanned flight of the Saturn V, carrying a Block I CSM on November 9, 1967. The capability of the Command Module's heat shield to survive a trans-lunar reentry was demonstrated by using the Service Module engine to ram it into the atmosphere at higher than the usual Earth-orbital reentry speed. This was followed on April 4, 1968, by Apollo 6 (AS-502) which carried a CSM and a LM Test Article as ballast. The intent of this mission was to achieve trans-lunar injection, followed closely by a simulated direct-return abort, using the Service Module engine to achieve another high-speed reentry. The Saturn V experienced pogo oscillation, a problem caused by non-steady engine combustion, which damaged fuel lines in the second and third stages. Two S-II engines shut down prematurely, but the remaining engines were able to compensate. The damage to the third stage engine was more severe, preventing it from restarting for trans-lunar injection. Mission controllers were able to use the Service Module engine to essentially repeat the flight profile of Apollo 4. Based", "In December 1966, the AS-205 mission was canceled, since the validation of the CSM would be accomplished on the 14-day first flight, and AS-205 would have been devoted to space experiments and contribute no new engineering knowledge about the spacecraft. Its Saturn IB was allocated to the dual mission, now redesignated AS-205/208 or AS-258, planned for August 1967. McDivitt, Scott and Schweickart were promoted to the prime AS-258 crew, and Schirra, Eisele and Cunningham were reassigned as the Apollo 1 backup crew.", "While experimenting, Tesla inadvertently faulted a power station generator, causing a power outage. In August 1917, Tesla explained what had happened in The Electrical Experimenter: \"As an example of what has been done with several hundred kilowatts of high frequency energy liberated, it was found that the dynamos in a power house six miles away were repeatedly burned out, due to the powerful high frequency currents set up in them, and which caused heavy sparks to jump through the windings and destroy the insulation!\""]</t>
-        </is>
-      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3510,21 +2520,6 @@
 The mouth of the Rhine into Lake Constance forms an inland delta. The delta is delimited in the West by the Alter Rhein ("Old Rhine") and in the East by a modern canalized section. Most of the delta is a nature reserve and bird sanctuary. It includes the Austrian towns of Gaißau, Höchst and Fußach. The natural Rhine originally branched into at least two arms and formed small islands by precipitating sediments. In the local Alemannic dialect, the singular is pronounced "Isel" and this is also the local pronunciation of Esel ("Donkey"). Many local fields have an official name containing this element.</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>[109, 345, 68, 612, 747]</t>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>[0.7853541374206543, 0.7779421210289001, 0.7717975378036499, 0.7613059878349304, 0.7561031579971313]</t>
-        </is>
-      </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>["A regulation of the Rhine was called for, with an upper canal near Diepoldsau and a lower canal at Fußach, in order to counteract the constant flooding and strong sedimentation in the western Rhine Delta. The Dornbirner Ach had to be diverted, too, and it now flows parallel to the canalized Rhine into the lake. Its water has a darker color than the Rhine; the latter's lighter suspended load comes from higher up the mountains. It is expected that the continuous input of sediment into the lake will silt up the lake. This has already happened to the former Lake Tuggenersee.", "The Upper Rhine region was changed significantly by a Rhine straightening program in the 19th Century. The rate of flow was increased and the ground water level fell significantly. Dead branches dried up and the amount of forests on the flood plains decreased sharply. On the French side, the Grand Canal d'Alsace was dug, which carries a significant part of the river water, and all of the traffic. In some places, there are large compensation pools, for example the huge Bassin de compensation de Plobsheim in Alsace.", "The hydrography of the current delta is characterized by the delta's main arms, disconnected arms (Hollandse IJssel, Linge, Vecht, etc.) and smaller rivers and streams. Many rivers have been closed (\"dammed\") and now serve as drainage channels for the numerous polders. The construction of Delta Works changed the Delta in the second half of the 20th Century fundamentally. Currently Rhine water runs into the sea, or into former marine bays now separated from the sea, in five places, namely at the mouths of the Nieuwe Merwede, Nieuwe Waterway (Nieuwe Maas), Dordtse Kil, Spui and IJssel.", "The name Rijn, from here on, is used only for smaller streams farther to the north, which together formed the main river Rhine in Roman times. Though they retained the name, these streams no longer carry water from the Rhine, but are used for draining the surrounding land and polders. From Wijk bij Duurstede, the old north branch of the Rhine is called Kromme Rijn (\"Bent Rhine\") past Utrecht, first Leidse Rijn (\"Rhine of Leiden\") and then, Oude Rijn (\"Old Rhine\"). The latter flows west into a sluice at Katwijk, where its waters can be discharged into the North Sea. This branch once formed the line along which the Limes Germanicus were built. During periods of lower sea levels within the various ice ages, the Rhine took a left turn, creating the Channel River, the course of which now lies below the English Channel.", "The mouth of the Rhine into Lake Constance forms an inland delta. The delta is delimited in the West by the Alter Rhein (\"Old Rhine\") and in the East by a modern canalized section. Most of the delta is a nature reserve and bird sanctuary. It includes the Austrian towns of Gaißau, Höchst and Fußach. The natural Rhine originally branched into at least two arms and formed small islands by precipitating sediments. In the local Alemannic dialect, the singular is pronounced \"Isel\" and this is also the local pronunciation of Esel (\"Donkey\"). Many local fields have an official name containing this element."]</t>
-        </is>
-      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3556,21 +2551,6 @@
 As of the census of 2000, there were 427,652 people, 140,079 households, and 97,915 families residing in the city. The population density was 4,097.9 people per square mile (1,582.2/km²). There were 149,025 housing units at an average density of 1,427.9 square miles (3,698 km2). The racial makeup of the city was 50.2% White, 8.4% Black or African American, 1.6% Native American, 11.2% Asian (about a third of which is Hmong), 0.1% Pacific Islander, 23.4% from other races, and 5.2% from two or more races. Hispanic or Latino of any race were 39.9% of the population.</t>
         </is>
       </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>[530, 740, 726, 69, 626]</t>
-        </is>
-      </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>[0.7884246110916138, 0.7812803983688354, 0.7637519836425781, 0.739832878112793, 0.7341710329055786]</t>
-        </is>
-      </c>
-      <c r="H68" t="inlineStr">
-        <is>
-          <t>["Jacksonville, like most large cities in the United States, suffered from negative effects of rapid urban sprawl after World War II. The construction of highways led residents to move to newer housing in the suburbs. After World War II, the government of the city of Jacksonville began to increase spending to fund new public building projects in the boom that occurred after the war. Mayor W. Haydon Burns' Jacksonville Story resulted in the construction of a new city hall, civic auditorium, public library and other projects that created a dynamic sense of civic pride. However, the development of suburbs and a subsequent wave of middle class \"white flight\" left Jacksonville with a much poorer population than before. The city's most populous ethnic group, non-Hispanic white, declined from 75.8% in 1970 to 55.1% by 2010.", "Jacksonville is the largest city by population in the U.S. state of Florida, and the largest city by area in the contiguous United States. It is the county seat of Duval County, with which the city government consolidated in 1968. Consolidation gave Jacksonville its great size and placed most of its metropolitan population within the city limits; with an estimated population of 853,382 in 2014, it is the most populous city proper in Florida and the Southeast, and the 12th most populous in the United States. Jacksonville is the principal city in the Jacksonville metropolitan area, with a population of 1,345,596 in 2010.", "Much of the city's tax base dissipated, leading to problems with funding education, sanitation, and traffic control within the city limits. In addition, residents in unincorporated suburbs had difficulty obtaining municipal services, such as sewage and building code enforcement. In 1958, a study recommended that the city of Jacksonville begin annexing outlying communities in order to create the needed tax base to improve services throughout the county. Voters outside the city limits rejected annexation plans in six referendums between 1960 and 1965.", "As of 2010[update], there were 366,273 households out of which 11.8% were vacant. 23.9% of households had children under the age of 18 living with them, 43.8% were married couples, 15.2% had a female householder with no husband present, and 36.4% were non-families. 29.7% of all households were made up of individuals and 7.9% had someone living alone who was 65 years of age or older. The average household size was 2.55 and the average family size was 3.21. In the city, the population was spread out with 23.9% under the age of 18, 10.5% from 18 to 24, 28.5% from 25 to 44, 26.2% from 45 to 64, and 10.9% who were 65 years of age or older. The median age was 35.5 years. For every 100 females there were 94.1 males. For every 100 females age 18 and over, there were 91.3 males.", "As of the census of 2000, there were 427,652 people, 140,079 households, and 97,915 families residing in the city. The population density was 4,097.9 people per square mile (1,582.2/km²). There were 149,025 housing units at an average density of 1,427.9 square miles (3,698 km2). The racial makeup of the city was 50.2% White, 8.4% Black or African American, 1.6% Native American, 11.2% Asian (about a third of which is Hmong), 0.1% Pacific Islander, 23.4% from other races, and 5.2% from two or more races. Hispanic or Latino of any race were 39.9% of the population."]</t>
-        </is>
-      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3602,21 +2582,6 @@
 The principle of inclusions and components states that, with sedimentary rocks, if inclusions (or clasts) are found in a formation, then the inclusions must be older than the formation that contains them. For example, in sedimentary rocks, it is common for gravel from an older formation to be ripped up and included in a newer layer. A similar situation with igneous rocks occurs when xenoliths are found. These foreign bodies are picked up as magma or lava flows, and are incorporated, later to cool in the matrix. As a result, xenoliths are older than the rock which contains them.</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>[15, 139, 590, 307, 254]</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>[0.857639729976654, 0.8067424297332764, 0.7553637623786926, 0.7061424255371094, 0.7048064470291138]</t>
-        </is>
-      </c>
-      <c r="H69" t="inlineStr">
-        <is>
-          <t>["For many geologic applications, isotope ratios of radioactive elements are measured in minerals that give the amount of time that has passed since a rock passed through its particular closure temperature, the point at which different radiometric isotopes stop diffusing into and out of the crystal lattice. These are used in geochronologic and thermochronologic studies. Common methods include uranium-lead dating, potassium-argon dating, argon-argon dating and uranium-thorium dating. These methods are used for a variety of applications. Dating of lava and volcanic ash layers found within a stratigraphic sequence can provide absolute age data for sedimentary rock units which do not contain radioactive isotopes and calibrate relative dating techniques. These methods can also be used to determine ages of pluton emplacement. Thermochemical techniques can be used to determine temperature profiles within the crust, the uplift of mountain ranges, and paleotopography.", "In the laboratory, biostratigraphers analyze rock samples from outcrop and drill cores for the fossils found in them. These fossils help scientists to date the core and to understand the depositional environment in which the rock units formed. Geochronologists precisely date rocks within the stratigraphic section in order to provide better absolute bounds on the timing and rates of deposition. Magnetic stratigraphers look for signs of magnetic reversals in igneous rock units within the drill cores. Other scientists perform stable isotope studies on the rocks to gain information about past climate.", "Among the most well-known experiments in structural geology are those involving orogenic wedges, which are zones in which mountains are built along convergent tectonic plate boundaries. In the analog versions of these experiments, horizontal layers of sand are pulled along a lower surface into a back stop, which results in realistic-looking patterns of faulting and the growth of a critically tapered (all angles remain the same) orogenic wedge. Numerical models work in the same way as these analog models, though they are often more sophisticated and can include patterns of erosion and uplift in the mountain belt. This helps to show the relationship between erosion and the shape of the mountain range. These studies can also give useful information about pathways for metamorphism through pressure, temperature, space, and time.", "The rocks collected from the Moon are extremely old compared to rocks found on Earth, as measured by radiometric dating techniques. They range in age from about 3.2 billion years for the basaltic samples derived from the lunar maria, to about 4.6 billion years for samples derived from the highlands crust. As such, they represent samples from a very early period in the development of the Solar System, that are largely absent on Earth. One important rock found during the Apollo Program is dubbed the Genesis Rock, retrieved by astronauts David Scott and James Irwin during the Apollo 15 mission. This anorthosite rock is composed almost exclusively of the calcium-rich feldspar mineral anorthite, and is believed to be representative of the highland crust. A geochemical component called KREEP was discovered, which has no known terrestrial counterpart. KREEP and the anorthositic samples have been used to infer that the outer portion of the Moon was once completely molten (see lunar magma ocean).", "The principle of inclusions and components states that, with sedimentary rocks, if inclusions (or clasts) are found in a formation, then the inclusions must be older than the formation that contains them. For example, in sedimentary rocks, it is common for gravel from an older formation to be ripped up and included in a newer layer. A similar situation with igneous rocks occurs when xenoliths are found. These foreign bodies are picked up as magma or lava flows, and are incorporated, later to cool in the matrix. As a result, xenoliths are older than the rock which contains them."]</t>
-        </is>
-      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3648,21 +2613,6 @@
 There are infinitely many primes, as demonstrated by Euclid around 300 BC. There is no known simple formula that separates prime numbers from composite numbers. However, the distribution of primes, that is to say, the statistical behaviour of primes in the large, can be modelled. The first result in that direction is the prime number theorem, proven at the end of the 19th century, which says that the probability that a given, randomly chosen number n is prime is inversely proportional to its number of digits, or to the logarithm of n.</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>[70, 766, 762, 391, 551]</t>
-        </is>
-      </c>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t>[0.889678955078125, 0.779110312461853, 0.7586722373962402, 0.758024275302887, 0.7436473369598389]</t>
-        </is>
-      </c>
-      <c r="H70" t="inlineStr">
-        <is>
-          <t>["The following table gives the largest known primes of the mentioned types. Some of these primes have been found using distributed computing. In 2009, the Great Internet Mersenne Prime Search project was awarded a US$100,000 prize for first discovering a prime with at least 10 million digits. The Electronic Frontier Foundation also offers $150,000 and $250,000 for primes with at least 100 million digits and 1 billion digits, respectively. Some of the largest primes not known to have any particular form (that is, no simple formula such as that of Mersenne primes) have been found by taking a piece of semi-random binary data, converting it to a number n, multiplying it by 256k for some positive integer k, and searching for possible primes within the interval [256kn + 1, 256k(n + 1) − 1].[citation needed]", "For a long time, number theory in general, and the study of prime numbers in particular, was seen as the canonical example of pure mathematics, with no applications outside of the self-interest of studying the topic with the exception of use of prime numbered gear teeth to distribute wear evenly. In particular, number theorists such as British mathematician G. H. Hardy prided themselves on doing work that had absolutely no military significance. However, this vision was shattered in the 1970s, when it was publicly announced that prime numbers could be used as the basis for the creation of public key cryptography algorithms. Prime numbers are also used for hash tables and pseudorandom number generators.", "Most early Greeks did not even consider 1 to be a number, so they could not consider it to be a prime. By the Middle Ages and Renaissance many mathematicians included 1 as the first prime number. In the mid-18th century Christian Goldbach listed 1 as the first prime in his famous correspondence with Leonhard Euler -- who did not agree. In the 19th century many mathematicians still considered the number 1 to be a prime. For example, Derrick Norman Lehmer's list of primes up to 10,006,721, reprinted as late as 1956, started with 1 as its first prime. Henri Lebesgue is said to be the last professional mathematician to call 1 prime. By the early 20th century, mathematicians began to accept that 1 is not a prime number, but rather forms its own special category as a \"unit\".", "Many questions regarding prime numbers remain open, such as Goldbach's conjecture (that every even integer greater than 2 can be expressed as the sum of two primes), and the twin prime conjecture (that there are infinitely many pairs of primes whose difference is 2). Such questions spurred the development of various branches of number theory, focusing on analytic or algebraic aspects of numbers. Primes are used in several routines in information technology, such as public-key cryptography, which makes use of properties such as the difficulty of factoring large numbers into their prime factors. Prime numbers give rise to various generalizations in other mathematical domains, mainly algebra, such as prime elements and prime ideals.", "There are infinitely many primes, as demonstrated by Euclid around 300 BC. There is no known simple formula that separates prime numbers from composite numbers. However, the distribution of primes, that is to say, the statistical behaviour of primes in the large, can be modelled. The first result in that direction is the prime number theorem, proven at the end of the 19th century, which says that the probability that a given, randomly chosen number n is prime is inversely proportional to its number of digits, or to the logarithm of n."]</t>
-        </is>
-      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3692,21 +2642,6 @@
 When considering computational problems, a problem instance is a string over an alphabet. Usually, the alphabet is taken to be the binary alphabet (i.e., the set {0,1}), and thus the strings are bitstrings. As in a real-world computer, mathematical objects other than bitstrings must be suitably encoded. For example, integers can be represented in binary notation, and graphs can be encoded directly via their adjacency matrices, or by encoding their adjacency lists in binary.
 run for about 4 × 1010 years, which is the same order of magnitude as the age of the universe. Even with a much faster computer, the program would only be useful for very small instances and in that sense the intractability of a problem is somewhat independent of technological progress. Nevertheless, a polynomial time algorithm is not always practical. If its running time is, say, n15, it is unreasonable to consider it efficient and it is still useless except on small instances.
 The most commonly used reduction is a polynomial-time reduction. This means that the reduction process takes polynomial time. For example, the problem of squaring an integer can be reduced to the problem of multiplying two integers. This means an algorithm for multiplying two integers can be used to square an integer. Indeed, this can be done by giving the same input to both inputs of the multiplication algorithm. Thus we see that squaring is not more difficult than multiplication, since squaring can be reduced to multiplication.</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>[71, 152, 741, 605, 234]</t>
-        </is>
-      </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>[0.8279779553413391, 0.7975757718086243, 0.7921947240829468, 0.7873315811157227, 0.7778883576393127]</t>
-        </is>
-      </c>
-      <c r="H71" t="inlineStr">
-        <is>
-          <t>["A computational problem can be viewed as an infinite collection of instances together with a solution for every instance. The input string for a computational problem is referred to as a problem instance, and should not be confused with the problem itself. In computational complexity theory, a problem refers to the abstract question to be solved. In contrast, an instance of this problem is a rather concrete utterance, which can serve as the input for a decision problem. For example, consider the problem of primality testing. The instance is a number (e.g. 15) and the solution is \"yes\" if the number is prime and \"no\" otherwise (in this case \"no\"). Stated another way, the instance is a particular input to the problem, and the solution is the output corresponding to the given input.", "A function problem is a computational problem where a single output (of a total function) is expected for every input, but the output is more complex than that of a decision problem, that is, it isn't just yes or no. Notable examples include the traveling salesman problem and the integer factorization problem.", "When considering computational problems, a problem instance is a string over an alphabet. Usually, the alphabet is taken to be the binary alphabet (i.e., the set {0,1}), and thus the strings are bitstrings. As in a real-world computer, mathematical objects other than bitstrings must be suitably encoded. For example, integers can be represented in binary notation, and graphs can be encoded directly via their adjacency matrices, or by encoding their adjacency lists in binary.", "run for about 4 × 1010 years, which is the same order of magnitude as the age of the universe. Even with a much faster computer, the program would only be useful for very small instances and in that sense the intractability of a problem is somewhat independent of technological progress. Nevertheless, a polynomial time algorithm is not always practical. If its running time is, say, n15, it is unreasonable to consider it efficient and it is still useless except on small instances.", "The most commonly used reduction is a polynomial-time reduction. This means that the reduction process takes polynomial time. For example, the problem of squaring an integer can be reduced to the problem of multiplying two integers. This means an algorithm for multiplying two integers can be used to square an integer. Indeed, this can be done by giving the same input to both inputs of the multiplication algorithm. Thus we see that squaring is not more difficult than multiplication, since squaring can be reduced to multiplication."]</t>
         </is>
       </c>
     </row>
@@ -3741,21 +2676,6 @@
 In a few species like Cyanidioschyzon merolæ, chloroplasts have a third plastid-dividing ring located in the chloroplast's intermembrane space.</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>[786, 459, 649, 623, 603]</t>
-        </is>
-      </c>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>[0.8423106074333191, 0.8417642712593079, 0.840059220790863, 0.8353739380836487, 0.8329559564590454]</t>
-        </is>
-      </c>
-      <c r="H72" t="inlineStr">
-        <is>
-          <t>["The chloroplastidan chloroplasts, or green chloroplasts, are another large, highly diverse primary chloroplast lineage. Their host organisms are commonly known as the green algae and land plants. They differ from glaucophyte and red algal chloroplasts in that they have lost their phycobilisomes, and contain chlorophyll b instead. Most green chloroplasts are (obviously) green, though some aren't, like some forms of Hæmatococcus pluvialis, due to accessory pigments that override the chlorophylls' green colors. Chloroplastidan chloroplasts have lost the peptidoglycan wall between their double membrane, and have replaced it with an intermembrane space. Some plants seem to have kept the genes for the synthesis of the peptidoglycan layer, though they've been repurposed for use in chloroplast division instead.", "Cryptophytes, or cryptomonads are a group of algae that contain a red-algal derived chloroplast. Cryptophyte chloroplasts contain a nucleomorph that superficially resembles that of the chlorarachniophytes. Cryptophyte chloroplasts have four membranes, the outermost of which is continuous with the rough endoplasmic reticulum. They synthesize ordinary starch, which is stored in granules found in the periplastid space—outside the original double membrane, in the place that corresponds to the red alga's cytoplasm. Inside cryptophyte chloroplasts is a pyrenoid and thylakoids in stacks of two.", "Some chloroplasts contain a structure called the chloroplast peripheral reticulum. It is often found in the chloroplasts of C4 plants, though it has also been found in some C3 angiosperms, and even some gymnosperms. The chloroplast peripheral reticulum consists of a maze of membranous tubes and vesicles continuous with the inner chloroplast membrane that extends into the internal stromal fluid of the chloroplast. Its purpose is thought to be to increase the chloroplast's surface area for cross-membrane transport between its stroma and the cell cytoplasm. The small vesicles sometimes observed may serve as transport vesicles to shuttle stuff between the thylakoids and intermembrane space.", "The chloroplast membranes sometimes protrude out into the cytoplasm, forming a stromule, or stroma-containing tubule. Stromules are very rare in chloroplasts, and are much more common in other plastids like chromoplasts and amyloplasts in petals and roots, respectively. They may exist to increase the chloroplast's surface area for cross-membrane transport, because they are often branched and tangled with the endoplasmic reticulum. When they were first observed in 1962, some plant biologists dismissed the structures as artifactual, claiming that stromules were just oddly shaped chloroplasts with constricted regions or dividing chloroplasts. However, there is a growing body of evidence that stromules are functional, integral features of plant cell plastids, not merely artifacts.", "Next, the two plastid-dividing rings, or PD rings form. The inner plastid-dividing ring is located in the inner side of the chloroplast's inner membrane, and is formed first. The outer plastid-dividing ring is found wrapped around the outer chloroplast membrane. It consists of filaments about 5 nanometers across, arranged in rows 6.4 nanometers apart, and shrinks to squeeze the chloroplast. This is when chloroplast constriction begins.\nIn a few species like Cyanidioschyzon merolæ, chloroplasts have a third plastid-dividing ring located in the chloroplast's intermembrane space."]</t>
-        </is>
-      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3787,21 +2707,6 @@
 in interceptions. In week 10, Manning suffered a partial tear of the plantar fasciitis in his left foot. He set the NFL's all-time record for career passing yards in this game, but was benched after throwing four interceptions in favor of backup quarterback Brock Osweiler, who took over as the starter for most of the remainder of the regular season. Osweiler was injured, however, leading to Manning's return during the Week 17 regular season finale, where the Broncos were losing 13–7 against the 4–11 San Diego Chargers, resulting in Manning re-claiming the starting quarterback position for the playoffs by leading the team to a key 27–20 win that enabled the team to clinch the number one overall AFC seed. Under defensive coordinator Wade Phillips, the Broncos' defense ranked number one in total yards allowed, passing yards allowed and sacks, and like the previous three seasons, the team has continued to set numerous individual, league and franchise records. With the defense carrying the team despite the issues with the offense, the Broncos finished the regular season with a 12–4 record and earned home-field advantage throughout the AFC playoffs.</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>[12, 64, 867, 205, 206]</t>
-        </is>
-      </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>[0.8894465565681458, 0.8635738492012024, 0.8324222564697266, 0.8183662295341492, 0.816746711730957]</t>
-        </is>
-      </c>
-      <c r="H73" t="inlineStr">
-        <is>
-          <t>["Peyton Manning became the first quarterback ever to lead two different teams to multiple Super Bowls. He is also the oldest quarterback ever to play in a Super Bowl at age 39. The past record was held by John Elway, who led the Broncos to victory in Super Bowl XXXIII at age 38 and is currently Denver's Executive Vice President of Football Operations and General Manager.", "This was the first Super Bowl to feature a quarterback on both teams who was the #1 pick in their draft classes. Manning was the #1 selection of the 1998 NFL draft, while Newton was picked first in 2011. The matchup also pits the top two picks of the 2011 draft against each other: Newton for Carolina and Von Miller for Denver. Manning and Newton also set the record for the largest age difference between opposing Super Bowl quarterbacks at 13 years and 48 days (Manning was 39, Newton was 26).", "In honor of the 50th Super Bowl, the pregame ceremony featured the on-field introduction of 39 of the 43 previous Super Bowl Most Valuable Players. Bart Starr (MVP of Super Bowls I and II) and Chuck Howley (MVP of Super Bowl V) appeared via video, while Peyton Manning (MVP of Super Bowl XLI and current Broncos quarterback) was shown in the locker room preparing for the game. No plans were announced regarding the recognition of Harvey Martin, co-MVP of Super Bowl XII, who died in 2001.", "Following their loss in the divisional round of the previous season's playoffs, the Denver Broncos underwent numerous coaching changes, including a mutual parting with head coach John Fox (who had won four divisional championships in his four years as Broncos head coach), and the hiring of Gary Kubiak as the new head coach. Under Kubiak, the Broncos planned to install a run-oriented offense with zone blocking to blend in with quarterback Peyton Manning's shotgun passing skills, but struggled with numerous changes and injuries to the offensive line, as well as Manning having his worst statistical season since his rookie year with the Indianapolis Colts in 1998, due to a plantar fasciitis injury in his heel that he had suffered since the summer, and the simple fact that Manning was getting old, as he turned 39 in the 2015 off-season. Although the team had a 7–0 start, Manning led the NFL in interceptions. In week 10, Manning suffered a partial tear of the plantar fasciitis in his left foot. He set the NFL's all-time record for career passing yards in this game, but was benched after throwing four interceptions in favor of backup quarterback Brock Osweiler, who took over as the", "in interceptions. In week 10, Manning suffered a partial tear of the plantar fasciitis in his left foot. He set the NFL's all-time record for career passing yards in this game, but was benched after throwing four interceptions in favor of backup quarterback Brock Osweiler, who took over as the starter for most of the remainder of the regular season. Osweiler was injured, however, leading to Manning's return during the Week 17 regular season finale, where the Broncos were losing 13–7 against the 4–11 San Diego Chargers, resulting in Manning re-claiming the starting quarterback position for the playoffs by leading the team to a key 27–20 win that enabled the team to clinch the number one overall AFC seed. Under defensive coordinator Wade Phillips, the Broncos' defense ranked number one in total yards allowed, passing yards allowed and sacks, and like the previous three seasons, the team has continued to set numerous individual, league and franchise records. With the defense carrying the team despite the issues with the offense, the Broncos finished the regular season with a 12–4 record and earned home-field advantage throughout the AFC playoffs."]</t>
-        </is>
-      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3833,21 +2738,6 @@
 The alga Cyanophora, a glaucophyte, is thought to be one of the first organisms to contain a chloroplast. The glaucophyte chloroplast group is the smallest of the three primary chloroplast lineages, being found in only 13 species, and is thought to be the one that branched off the earliest. Glaucophytes have chloroplasts that retain a peptidoglycan wall between their double membranes, like their cyanobacterial parent. For this reason, glaucophyte chloroplasts are also known as muroplasts. Glaucophyte chloroplasts also contain concentric unstacked thylakoids, which surround a carboxysome - an icosahedral structure that glaucophyte chloroplasts and cyanobacteria keep their carbon fixation enzyme rubisco in. The starch that they synthesize collects outside the chloroplast. Like cyanobacteria, glaucophyte chloroplast thylakoids are studded with light collecting structures called phycobilisomes. For these reasons, glaucophyte chloroplasts are considered a primitive intermediate between cyanobacteria and the more evolved chloroplasts in red algae and plants.</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>[73, 459, 471, 378, 778]</t>
-        </is>
-      </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>[0.8497679233551025, 0.810733437538147, 0.798054575920105, 0.7973419427871704, 0.7786021828651428]</t>
-        </is>
-      </c>
-      <c r="H74" t="inlineStr">
-        <is>
-          <t>["Some dinophytes, like Kryptoperidinium and Durinskia have a diatom (heterokontophyte) derived chloroplast. These chloroplasts are bounded by up to five membranes, (depending on whether you count the entire diatom endosymbiont as the chloroplast, or just the red algal derived chloroplast inside it). The diatom endosymbiont has been reduced relatively little—it still retains its original mitochondria, and has endoplasmic reticulum, ribosomes, a nucleus, and of course, red algal derived chloroplasts—practically a complete cell, all inside the host's endoplasmic reticulum lumen. However the diatom endosymbiont can't store its own food—its starch is found in granules in the dinophyte host's cytoplasm instead. The diatom endosymbiont's nucleus is present, but it probably can't be called a nucleomorph because it shows no sign of genome reduction, and might have even been expanded. Diatoms have been engulfed by dinoflagellates at least three times.", "Cryptophytes, or cryptomonads are a group of algae that contain a red-algal derived chloroplast. Cryptophyte chloroplasts contain a nucleomorph that superficially resembles that of the chlorarachniophytes. Cryptophyte chloroplasts have four membranes, the outermost of which is continuous with the rough endoplasmic reticulum. They synthesize ordinary starch, which is stored in granules found in the periplastid space—outside the original double membrane, in the place that corresponds to the red alga's cytoplasm. Inside cryptophyte chloroplasts is a pyrenoid and thylakoids in stacks of two.", "Apicomplexans are another group of chromalveolates. Like the helicosproidia, they're parasitic, and have a nonphotosynthetic chloroplast. They were once thought to be related to the helicosproidia, but it is now known that the helicosproida are green algae rather than chromalveolates. The apicomplexans include Plasmodium, the malaria parasite. Many apicomplexans keep a vestigial red algal derived chloroplast called an apicoplast, which they inherited from their ancestors. Other apicomplexans like Cryptosporidium have lost the chloroplast completely. Apicomplexans store their energy in amylopectin starch granules that are located in their cytoplasm, even though they are nonphotosynthetic.", "Lepidodinium viride and its close relatives are dinophytes that lost their original peridinin chloroplast and replaced it with a green algal derived chloroplast (more specifically, a prasinophyte). Lepidodinium is the only dinophyte that has a chloroplast that's not from the rhodoplast lineage. The chloroplast is surrounded by two membranes and has no nucleomorph—all the nucleomorph genes have been transferred to the dinophyte nucleus. The endosymbiotic event that led to this chloroplast was serial secondary endosymbiosis rather than tertiary endosymbiosis—the endosymbiont was a green alga containing a primary chloroplast (making a secondary chloroplast).", "The alga Cyanophora, a glaucophyte, is thought to be one of the first organisms to contain a chloroplast. The glaucophyte chloroplast group is the smallest of the three primary chloroplast lineages, being found in only 13 species, and is thought to be the one that branched off the earliest. Glaucophytes have chloroplasts that retain a peptidoglycan wall between their double membranes, like their cyanobacterial parent. For this reason, glaucophyte chloroplasts are also known as muroplasts. Glaucophyte chloroplasts also contain concentric unstacked thylakoids, which surround a carboxysome - an icosahedral structure that glaucophyte chloroplasts and cyanobacteria keep their carbon fixation enzyme rubisco in. The starch that they synthesize collects outside the chloroplast. Like cyanobacteria, glaucophyte chloroplast thylakoids are studded with light collecting structures called phycobilisomes. For these reasons, glaucophyte chloroplasts are considered a primitive intermediate between cyanobacteria and the more evolved chloroplasts in red algae and plants."]</t>
-        </is>
-      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3879,21 +2769,6 @@
 BSkyB utilises the VideoGuard pay-TV scrambling system owned by NDS, a Cisco Systems company. There are tight controls over use of VideoGuard decoders; they are not available as stand-alone DVB CAMs (conditional-access modules). BSkyB has design authority over all digital satellite receivers capable of receiving their service. The receivers, though designed and built by different manufacturers, must conform to the same user interface look-and-feel as all the others. This extends to the Personal video recorder (PVR) offering (branded Sky+).</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr">
-        <is>
-          <t>[74, 155, 658, 541, 624]</t>
-        </is>
-      </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>[0.8356844782829285, 0.7582891583442688, 0.7561945915222168, 0.7386825680732727, 0.7321329116821289]</t>
-        </is>
-      </c>
-      <c r="H75" t="inlineStr">
-        <is>
-          <t>["CBS provided digital streams of the game via CBSSports.com, and the CBS Sports apps on tablets, Windows 10, Xbox One and other digital media players (such as Chromecast and Roku). Due to Verizon Communications exclusivity, streaming on smartphones was only provided to Verizon Wireless customers via the NFL Mobile service. The ESPN Deportes Spanish broadcast was made available through WatchESPN.", "In May 2013, ABC launched \"WATCH ABC\", a revamp of its traditional multi-platform streaming services encompassing the network's existing streaming portal at ABC.com and a mobile app for smartphones and tablet computers; in addition to providing full-length episodes of ABC programs, the service allows live programming streams of local ABC affiliates in select markets (the first such offering by a U.S. broadcast network). Similar to sister network ESPN's WatchESPN service (which originated the \"WATCH\" brand used by the streaming services of Disney's television networks), live streams of ABC stations are only available to authenticated subscribers of participating pay television providers in certain markets. New York City O&amp;O WABC-TV and Philadelphia O&amp;O WPVI-TV were the first stations to offer streams of their programming on the service (with a free preview for non-subscribers through June 2013), with the six remaining ABC O&amp;Os offering streams by the start of the 2013–14 season. Hearst Television also reached a deal to offer streams of its ABC affiliates (including stations in Boston, Kansas City, Milwaukee and West Palm Beach) on the service.", "Provided is a universal Ku band LNB (9.75/10.600 GHz) which is fitted at the end of the dish and pointed at the correct satellite constellation; most digital receivers will receive the free to air channels. Some broadcasts are free-to-air and unencrypted, some are encrypted but do not require a monthly subscription (known as free-to-view), some are encrypted and require a monthly subscription, and some are pay-per-view services. To view the encrypted content a VideoGuard UK equipped receiver (all of which are dedicated to the Sky service, and cannot be used to decrypt other services) needs to be used. Unofficial CAMs are now available to view the service, although use of them breaks the user's contract with Sky and invalidates the user's rights to use the card.", "The service started on 1 September 1993 based on the idea from the then chief executive officer, Sam Chisholm and Rupert Murdoch, of converting the company business strategy to an entirely fee-based concept. The new package included four channels formerly available free-to-air, broadcasting on Astra's satellites, as well as introducing new channels. The service continued until the closure of BSkyB's analogue service on 27 September 2001, due to the launch and expansion of the Sky Digital platform. Some of the channels did broadcast either in the clear or soft encrypted (whereby a Videocrypt decoder was required to decode, without a subscription card) prior to their addition to the Sky Multichannels package. Within two months of the launch, BSkyB gained 400,000 new subscribers, with the majority taking at least one premium channel as well, which helped BSkyB reach 3.5 million households by mid-1994. Michael Grade criticized the operations in front of the Select Committee on National Heritage, mainly for the lack of original programming on many of the new channels.", "BSkyB utilises the VideoGuard pay-TV scrambling system owned by NDS, a Cisco Systems company. There are tight controls over use of VideoGuard decoders; they are not available as stand-alone DVB CAMs (conditional-access modules). BSkyB has design authority over all digital satellite receivers capable of receiving their service. The receivers, though designed and built by different manufacturers, must conform to the same user interface look-and-feel as all the others. This extends to the Personal video recorder (PVR) offering (branded Sky+)."]</t>
-        </is>
-      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3925,21 +2800,6 @@
 Following the success of the 2005 series produced by Russell T Davies, the BBC commissioned Davies to produce a 13-part spin-off series titled Torchwood (an anagram of "Doctor Who"), set in modern-day Cardiff and investigating alien activities and crime. The series debuted on BBC Three on 22 October 2006. John Barrowman reprised his role of Jack Harkness from the 2005 series of Doctor Who. Two other actresses who appeared in Doctor Who also star in the series; Eve Myles as Gwen Cooper, who also played the similarly named servant girl Gwyneth in the 2005 Doctor Who episode "The Unquiet Dead", and Naoko Mori who reprised her role as Toshiko Sato first seen in "Aliens of London". A second series of Torchwood aired in 2008; for three episodes, the cast was joined by Freema Agyeman reprising her Doctor Who role of Martha Jones. A third series was broadcast from 6 to 10 July 2009, and consisted of a single five-part story called Children of Earth which was set largely in London. A fourth series, Torchwood: Miracle Day jointly produced by BBC Wales, BBC Worldwide and the American entertainment company Starz debuted in 2011. The series was predominantly set in the United</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t>[492, 75, 185, 209, 184]</t>
-        </is>
-      </c>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>[0.8117756843566895, 0.7897528409957886, 0.7485792636871338, 0.7400177121162415, 0.7391876578330994]</t>
-        </is>
-      </c>
-      <c r="H76" t="inlineStr">
-        <is>
-          <t>["Doctor Who books have been published from the mid-sixties through to the present day. From 1965 to 1991 the books published were primarily novelised adaptations of broadcast episodes; beginning in 1991 an extensive line of original fiction was launched, the Virgin New Adventures and Virgin Missing Adventures. Since the relaunch of the programme in 2005, a new range of novels have been published by BBC Books. Numerous non-fiction books about the series, including guidebooks and critical studies, have also been published, and a dedicated Doctor Who Magazine with newsstand circulation has been published regularly since 1979. This is published by Panini, as is the Doctor Who Adventures magazine for younger fans.", "In 1975, Season 11 of the series won a Writers' Guild of Great Britain award for Best Writing in a Children's Serial. In 1996, BBC television held the \"Auntie Awards\" as the culmination of their \"TV60\" series, celebrating 60 years of BBC television broadcasting, where Doctor Who was voted as the \"Best Popular Drama\" the corporation had ever produced, ahead of such ratings heavyweights as EastEnders and Casualty. In 2000, Doctor Who was ranked third in a list of the 100 Greatest British Television Programmes of the 20th century, produced by the British Film Institute and voted on by industry professionals. In 2005, the series came first in a survey by SFX magazine of \"The Greatest UK Science Fiction and Fantasy Television Series Ever\". Also, in the 100 Greatest Kids' TV shows (a Channel 4 countdown in 2001), the 1963–1989 run was placed at number eight.", "10 July 2009, and consisted of a single five-part story called Children of Earth which was set largely in London. A fourth series, Torchwood: Miracle Day jointly produced by BBC Wales, BBC Worldwide and the American entertainment company Starz debuted in 2011. The series was predominantly set in the United States, though Wales remained part of the show's setting.", "The 2005 version of Doctor Who is a direct plot continuation of the original 1963–1989 series[note 2] and the 1996 telefilm. This is similar to the 1988 continuation of Mission Impossible, but differs from most other series relaunches which have either been reboots (for example, Battlestar Galactica and Bionic Woman[citation needed]) or set in the same universe as the original but in a different time period and with different characters (for example, Star Trek: The Next Generation and spin-offs[citation needed]).", "Following the success of the 2005 series produced by Russell T Davies, the BBC commissioned Davies to produce a 13-part spin-off series titled Torchwood (an anagram of \"Doctor Who\"), set in modern-day Cardiff and investigating alien activities and crime. The series debuted on BBC Three on 22 October 2006. John Barrowman reprised his role of Jack Harkness from the 2005 series of Doctor Who. Two other actresses who appeared in Doctor Who also star in the series; Eve Myles as Gwen Cooper, who also played the similarly named servant girl Gwyneth in the 2005 Doctor Who episode \"The Unquiet Dead\", and Naoko Mori who reprised her role as Toshiko Sato first seen in \"Aliens of London\". A second series of Torchwood aired in 2008; for three episodes, the cast was joined by Freema Agyeman reprising her Doctor Who role of Martha Jones. A third series was broadcast from 6 to 10 July 2009, and consisted of a single five-part story called Children of Earth which was set largely in London. A fourth series, Torchwood: Miracle Day jointly produced by BBC Wales, BBC Worldwide and the American entertainment company Starz debuted in 2011. The series was predominantly set in the United"]</t>
-        </is>
-      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3971,21 +2831,6 @@
 Aristotle provided a philosophical discussion of the concept of a force as an integral part of Aristotelian cosmology. In Aristotle's view, the terrestrial sphere contained four elements that come to rest at different "natural places" therein. Aristotle believed that motionless objects on Earth, those composed mostly of the elements earth and water, to be in their natural place on the ground and that they will stay that way if left alone. He distinguished between the innate tendency of objects to find their "natural place" (e.g., for heavy bodies to fall), which led to "natural motion", and unnatural or forced motion, which required continued application of a force. This theory, based on the everyday experience of how objects move, such as the constant application of a force needed to keep a cart moving, had conceptual trouble accounting for the behavior of projectiles, such as the flight of arrows. The place where the archer moves the projectile was at the start of the flight, and while the projectile sailed through the air, no discernible efficient cause acts on it. Aristotle was aware of this problem and proposed that the air displaced through the projectile's path carries the projectile to its target. This</t>
         </is>
       </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>[76, 686, 436, 650, 621]</t>
-        </is>
-      </c>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t>[0.7946696877479553, 0.7762023210525513, 0.7435693144798279, 0.7359496355056763, 0.7352085709571838]</t>
-        </is>
-      </c>
-      <c r="H77" t="inlineStr">
-        <is>
-          <t>["Since forces are perceived as pushes or pulls, this can provide an intuitive understanding for describing forces. As with other physical concepts (e.g. temperature), the intuitive understanding of forces is quantified using precise operational definitions that are consistent with direct observations and compared to a standard measurement scale. Through experimentation, it is determined that laboratory measurements of forces are fully consistent with the conceptual definition of force offered by Newtonian mechanics.", "LeGrande writes that \"the formulation of a single all-encompassing definition of the term is extremely difficult, if not impossible. In reviewing the voluminous literature on the subject, the student of civil disobedience rapidly finds himself surrounded by a maze of semantical problems and grammatical niceties. Like Alice in Wonderland, he often finds that specific terminology has no more (or no less) meaning than the individual orator intends it to have.\" He encourages a distinction between lawful protest demonstration, nonviolent civil disobedience, and violent civil disobedience.", "For certain physical scenarios, it is impossible to model forces as being due to gradient of potentials. This is often due to macrophysical considerations that yield forces as arising from a macroscopic statistical average of microstates. For example, friction is caused by the gradients of numerous electrostatic potentials between the atoms, but manifests as a force model that is independent of any macroscale position vector. Nonconservative forces other than friction include other contact forces, tension, compression, and drag. However, for any sufficiently detailed description, all these forces are the results of conservative ones since each of these macroscopic forces are the net results of the gradients of microscopic potentials.", "Historically, forces were first quantitatively investigated in conditions of static equilibrium where several forces canceled each other out. Such experiments demonstrate the crucial properties that forces are additive vector quantities: they have magnitude and direction. When two forces act on a point particle, the resulting force, the resultant (also called the net force), can be determined by following the parallelogram rule of vector addition: the addition of two vectors represented by sides of a parallelogram, gives an equivalent resultant vector that is equal in magnitude and direction to the transversal of the parallelogram. The magnitude of the resultant varies from the difference of the magnitudes of the two forces to their sum, depending on the angle between their lines of action. However, if the forces are acting on an extended body, their respective lines of application must also be specified in order to account for their effects on the motion of the body.", "Aristotle provided a philosophical discussion of the concept of a force as an integral part of Aristotelian cosmology. In Aristotle's view, the terrestrial sphere contained four elements that come to rest at different \"natural places\" therein. Aristotle believed that motionless objects on Earth, those composed mostly of the elements earth and water, to be in their natural place on the ground and that they will stay that way if left alone. He distinguished between the innate tendency of objects to find their \"natural place\" (e.g., for heavy bodies to fall), which led to \"natural motion\", and unnatural or forced motion, which required continued application of a force. This theory, based on the everyday experience of how objects move, such as the constant application of a force needed to keep a cart moving, had conceptual trouble accounting for the behavior of projectiles, such as the flight of arrows. The place where the archer moves the projectile was at the start of the flight, and while the projectile sailed through the air, no discernible efficient cause acts on it. Aristotle was aware of this problem and proposed that the air displaced through the projectile's path carries the projectile to its target. This"]</t>
-        </is>
-      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -4017,21 +2862,6 @@
 During the mid-Eocene, it is believed that the drainage basin of the Amazon was split along the middle of the continent by the Purus Arch. Water on the eastern side flowed toward the Atlantic, while to the west water flowed toward the Pacific across the Amazonas Basin. As the Andes Mountains rose, however, a large basin was created that enclosed a lake; now known as the Solimões Basin. Within the last 5–10 million years, this accumulating water broke through the Purus Arch, joining the easterly flow toward the Atlantic.</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr">
-        <is>
-          <t>[77, 546, 43, 594, 565]</t>
-        </is>
-      </c>
-      <c r="G78" t="inlineStr">
-        <is>
-          <t>[0.8585054874420166, 0.7811861038208008, 0.7702623009681702, 0.7651633024215698, 0.7582635283470154]</t>
-        </is>
-      </c>
-      <c r="H78" t="inlineStr">
-        <is>
-          <t>["Most of the Rhine's current course was not under the ice during the last Ice Age; although, its source must still have been a glacier. A tundra, with Ice Age flora and fauna, stretched across middle Europe, from Asia to the Atlantic Ocean. Such was the case during the Last Glacial Maximum, ca. 22,000–14,000 yr BP, when ice-sheets covered Scandinavia, the Baltics, Scotland and the Alps, but left the space between as open tundra. The loess or wind-blown dust over that tundra, settled in and around the Rhine Valley, contributing to its current agricultural usefulness.", "From their original homelands in Scandinavia and northern Europe, Germanic tribes expanded throughout northern and western Europe in the middle period of classical antiquity; southern Europe in late antiquity, conquering Celtic and other peoples; and by 800 CE, forming the Holy Roman Empire, the first German Empire. However, there was no real systemic continuity from the Western Roman Empire to its German successor which was famously described as \"not holy, not Roman, and not an empire\", as a great number of small states and principalities existed in the loosely autonomous confederation. Although by 1000 CE, the Germanic conquest of central, western, and southern Europe (west of and including Italy) was complete, excluding only Muslim Iberia. There was, however, little cultural integration or national identity, and \"Germany\" remained largely a conceptual term referring to an amorphous area of central Europe.", "At the begin of the Holocene (~11,700 years ago), the Rhine occupied its Late-Glacial valley. As a meandering river, it reworked its ice-age braidplain. As sea-level continued to rise in the Netherlands, the formation of the Holocene Rhine-Meuse delta began (~8,000 years ago). Coeval absolute sea-level rise and tectonic subsidence have strongly influenced delta evolution. Other factors of importance to the shape of the delta are the local tectonic activities of the Peel Boundary Fault, the substrate and geomorphology, as inherited from the Last Glacial and the coastal-marine dynamics, such as barrier and tidal inlet formations.", "Following the Cretaceous–Paleogene extinction event, the extinction of the dinosaurs and the wetter climate may have allowed the tropical rainforest to spread out across the continent. From 66–34 Mya, the rainforest extended as far south as 45°. Climate fluctuations during the last 34 million years have allowed savanna regions to expand into the tropics. During the Oligocene, for example, the rainforest spanned a relatively narrow band. It expanded again during the Middle Miocene, then retracted to a mostly inland formation at the last glacial maximum. However, the rainforest still managed to thrive during these glacial periods, allowing for the survival and evolution of a broad diversity of species.", "During the mid-Eocene, it is believed that the drainage basin of the Amazon was split along the middle of the continent by the Purus Arch. Water on the eastern side flowed toward the Atlantic, while to the west water flowed toward the Pacific across the Amazonas Basin. As the Andes Mountains rose, however, a large basin was created that enclosed a lake; now known as the Solimões Basin. Within the last 5–10 million years, this accumulating water broke through the Purus Arch, joining the easterly flow toward the Atlantic."]</t>
-        </is>
-      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -4063,21 +2893,6 @@
 United States and Western Europe than in China (due to a greater tendency to take on debts).[unreliable source?][unreliable source?] Anthony Shorrocks, the lead author of the Credit Suisse report which is one of the sources of Oxfam's data, considers the criticism about debt to be a "silly argument" and "a non-issue . . . a diversion."</t>
         </is>
       </c>
-      <c r="F79" t="inlineStr">
-        <is>
-          <t>[302, 664, 747, 92, 827]</t>
-        </is>
-      </c>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>[0.6491631865501404, 0.6466248035430908, 0.6362127065658569, 0.635114848613739, 0.6349173188209534]</t>
-        </is>
-      </c>
-      <c r="H79" t="inlineStr">
-        <is>
-          <t>["recorded in central England in 2007. The MBH99 finding was supported by cited reconstructions by Jones et al. 1998, Pollack, Huang &amp; Shen 1998, Crowley &amp; Lowery 2000 and Briffa 2000, using differing data and methods. The Jones et al. and Briffa reconstructions were overlaid with the MBH99 reconstruction in Figure 2.21 of the IPCC report.", "The 1970s and 1980s saw the emergence of many graphical imaging packages for the network in which based the logo's setting mainly on special lighting effects then under development including white, blue, pink, rainbow neon and glittering dotted lines. Among the \"ABC Circle\" logo's many variants was a 1977 ID sequence that featured a bubble on a black background representing the circle with glossy gold letters, and as such, was the first ABC identification card to have a three-dimensional appearance.", "The mouth of the Rhine into Lake Constance forms an inland delta. The delta is delimited in the West by the Alter Rhein (\"Old Rhine\") and in the East by a modern canalized section. Most of the delta is a nature reserve and bird sanctuary. It includes the Austrian towns of Gaißau, Höchst and Fußach. The natural Rhine originally branched into at least two arms and formed small islands by precipitating sediments. In the local Alemannic dialect, the singular is pronounced \"Isel\" and this is also the local pronunciation of Esel (\"Donkey\"). Many local fields have an official name containing this element.", "Genghis Khan, the title is spelled in variety of ways in different languages such as Mongolian Chinggis Khaan, English Chinghiz, Chinghis, and Chingiz, Chinese: 成吉思汗; pinyin: Chéngjísī Hán, Turkic: Cengiz Han, Çingiz Xan, Çingiz Han, Chingizxon, Çıñğız Xan, Chengez Khan, Chinggis Khan, Chinggis Xaan, Chingis Khan, Jenghis Khan, Chinggis Qan, Djingis Kahn, Russian: Чингисхан (Čingiskhan) or Чингиз-хан (Čingiz-khan), etc. Temüjin is written in Chinese as simplified Chinese: 铁木真; traditional Chinese: 鐵木眞; pinyin: Tiěmùzhēn.", "United States and Western Europe than in China (due to a greater tendency to take on debts).[unreliable source?][unreliable source?] Anthony Shorrocks, the lead author of the Credit Suisse report which is one of the sources of Oxfam's data, considers the criticism about debt to be a \"silly argument\" and \"a non-issue . . . a diversion.\""]</t>
-        </is>
-      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -4109,21 +2924,6 @@
 Continuing the style of the earlier buildings, various designers were responsible for the decoration, the terracotta embellishments were again the work of Godfrey Sykes, although sgraffito was used to decorate the east side of the building designed by F. W. Moody, a final embellishment were the wrought iron gates made as late as 1885 designed by Starkie Gardner, these lead to a passage through the building. Scott also designed the two Cast Courts 1870–73 to the southeast of the garden (the site of the "Brompton Boilers"), these vast spaces have ceilings 70 feet (21 m) in height to accommodate the plaster casts of parts of famous buildings, including Trajan's Column (in two separate pieces). The final part of the museum designed by Scott was the Art Library and what is now the sculpture gallery on the south side of the garden, built 1877–83, the exterior mosaic panels in the parapet were designed by Reuben Townroe who also designed the plaster work in the library, Sir John Taylor designed the book shelves and cases, also this was the first part of the museum to have electric lighting. This completed the northern half of the site, creating a quadrangle with the garden</t>
         </is>
       </c>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t>[79, 540, 186, 588, 587]</t>
-        </is>
-      </c>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>[0.8927464485168457, 0.7699087858200073, 0.7599356770515442, 0.7547442317008972, 0.7336236834526062]</t>
-        </is>
-      </c>
-      <c r="H80" t="inlineStr">
-        <is>
-          <t>["In 2004, the V&amp;A alongside Royal Institute of British Architects opened the first permanent gallery in the UK covering the history of architecture with displays using models, photographs, elements from buildings and original drawings. With the opening of the new gallery, the RIBA Drawings and Archives Collection has been transferred to the museum, joining the already extensive collection held by the V&amp;A. With over 600,000 drawings, over 750,000 papers and paraphernalia, and over 700,000 photographs from around the world, together they form the world's most comprehensive architectural resource.", "As interesting examples of expositions the most notable are: the world's first Museum of Posters boasting one of the largest collections of art posters in the world, Museum of Hunting and Riding and the Railway Museum. From among Warsaw's 60 museums, the most prestigious ones are National Museum with a collection of works whose origin ranges in time from antiquity till the present epoch as well as one of the best collections of paintings in the country including some paintings from Adolf Hitler's private collection, and Museum of the Polish Army whose set portrays the history of arms.", "The Victoria and Albert Museum’s Word and Image Department was under the same pressure being felt in archives around the world, to digitize their collection. A large scale digitization project began in 2007 in that department. That project was entitled the Factory Project to reference Andy Warhol and to create a factory to completely digitize the collection. The first step of the Factory Project was to take photographs utilizing digital cameras. The Word and Image Department had a collection of old photos but they were in black and white and in variant conditions, so new photos were shot. Those new photographs will be accessible to researchers to the Victoria and Albert Museum web-site. 15,000 images were taken during the first year of the Factory Project, including drawings, watercolors, computer-generated art, photographs, posters, and woodcuts. The second step of the Factory Project is to catalog everything. The third step of the Factory Project is to audit the collection. All of those items which were photographed and cataloged, must be audited to make sure everything listed as being in the collection was physically found during the creation of the Factory Project. The fourth goal of the Factory Project is conservation, which means", "were designed by Reuben Townroe who also designed the plaster work in the library, Sir John Taylor designed the book shelves and cases, also this was the first part of the museum to have electric lighting. This completed the northern half of the site, creating a quadrangle with the garden at its centre, but left the museum without a proper façade. In 1890 the government launched a competition to design new buildings for the museum, with architect Alfred Waterhouse as one of the judges; this would give the museum a new imposing front entrance.", "Continuing the style of the earlier buildings, various designers were responsible for the decoration, the terracotta embellishments were again the work of Godfrey Sykes, although sgraffito was used to decorate the east side of the building designed by F. W. Moody, a final embellishment were the wrought iron gates made as late as 1885 designed by Starkie Gardner, these lead to a passage through the building. Scott also designed the two Cast Courts 1870–73 to the southeast of the garden (the site of the \"Brompton Boilers\"), these vast spaces have ceilings 70 feet (21 m) in height to accommodate the plaster casts of parts of famous buildings, including Trajan's Column (in two separate pieces). The final part of the museum designed by Scott was the Art Library and what is now the sculpture gallery on the south side of the garden, built 1877–83, the exterior mosaic panels in the parapet were designed by Reuben Townroe who also designed the plaster work in the library, Sir John Taylor designed the book shelves and cases, also this was the first part of the museum to have electric lighting. This completed the northern half of the site, creating a quadrangle with the garden"]</t>
-        </is>
-      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -4155,21 +2955,6 @@
 After each team punted, Panthers quarterback Cam Newton appeared to complete a 24-yard pass Jerricho Cotchery, but the call was ruled an incompletion and upheld after a replay challenge. CBS analyst and retired referee Mike Carey stated he disagreed with the call and felt the review clearly showed the pass was complete. A few plays later, on 3rd-and-10 from the 15-yard line, linebacker Von Miller knocked the ball out of Newton's hands while sacking him, and Malik Jackson recovered it in the end zone for a Broncos touchdown, giving the team a 10–0 lead. This was the first fumble return touchdown in a Super Bowl since Super Bowl XXVIII at the end of the 1993 season.</t>
         </is>
       </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>[29, 269, 6, 206, 608]</t>
-        </is>
-      </c>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>[0.8762896656990051, 0.8621740341186523, 0.8313350677490234, 0.7921356558799744, 0.7917261719703674]</t>
-        </is>
-      </c>
-      <c r="H81" t="inlineStr">
-        <is>
-          <t>["The Panthers finished the regular season with a 15–1 record, and quarterback Cam Newton was named the NFL Most Valuable Player (MVP). They defeated the Arizona Cardinals 49–15 in the NFC Championship Game and advanced to their second Super Bowl appearance since the franchise was founded in 1995. The Broncos finished the regular season with a 12–4 record, and denied the New England Patriots a chance to defend their title from Super Bowl XLIX by defeating them 20–18 in the AFC Championship Game. They joined the Patriots, Dallas Cowboys, and Pittsburgh Steelers as one of four teams that have made eight appearances in the Super Bowl.", "The Panthers beat the Seattle Seahawks in the divisional round, running up a 31–0 halftime lead and then holding off a furious second half comeback attempt to win 31–24, avenging their elimination from a year earlier. The Panthers then blew out the Arizona Cardinals in the NFC Championship Game, 49–15, racking up 487 yards and forcing seven turnovers.", "The Broncos defeated the Pittsburgh Steelers in the divisional round, 23–16, by scoring 11 points in the final three minutes of the game. They then beat the defending Super Bowl XLIX champion New England Patriots in the AFC Championship Game, 20–18, by intercepting a pass on New England's 2-point conversion attempt with 17 seconds left on the clock. Despite Manning's problems with interceptions during the season, he didn't throw any in their two playoff games.", "in interceptions. In week 10, Manning suffered a partial tear of the plantar fasciitis in his left foot. He set the NFL's all-time record for career passing yards in this game, but was benched after throwing four interceptions in favor of backup quarterback Brock Osweiler, who took over as the starter for most of the remainder of the regular season. Osweiler was injured, however, leading to Manning's return during the Week 17 regular season finale, where the Broncos were losing 13–7 against the 4–11 San Diego Chargers, resulting in Manning re-claiming the starting quarterback position for the playoffs by leading the team to a key 27–20 win that enabled the team to clinch the number one overall AFC seed. Under defensive coordinator Wade Phillips, the Broncos' defense ranked number one in total yards allowed, passing yards allowed and sacks, and like the previous three seasons, the team has continued to set numerous individual, league and franchise records. With the defense carrying the team despite the issues with the offense, the Broncos finished the regular season with a 12–4 record and earned home-field advantage throughout the AFC playoffs.", "After each team punted, Panthers quarterback Cam Newton appeared to complete a 24-yard pass Jerricho Cotchery, but the call was ruled an incompletion and upheld after a replay challenge. CBS analyst and retired referee Mike Carey stated he disagreed with the call and felt the review clearly showed the pass was complete. A few plays later, on 3rd-and-10 from the 15-yard line, linebacker Von Miller knocked the ball out of Newton's hands while sacking him, and Malik Jackson recovered it in the end zone for a Broncos touchdown, giving the team a 10–0 lead. This was the first fumble return touchdown in a Super Bowl since Super Bowl XXVIII at the end of the 1993 season."]</t>
-        </is>
-      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4201,21 +2986,6 @@
 a separate peace, but the emissaries were executed. At the Battle of Kalka River in 1223, Subutai's forces defeated the larger Kievan force. They also may have fought against the neighboring Volga Bulgars. There is no historical record except a short account by the Arab historian Ibn al-Athir, writing in Mosul some 1100 miles away from the event. Various historical secondary sources - Morgan, Chambers, Grousset - state that the Mongols actually defeated the Bulgars, Chambers even going so far as to say that the Bulgars had made up stories to tell the (recently crushed) Russians that they had beaten the Mongols and driven them from their territory. The Russian princes then sued for peace. Subutai agreed but was in no mood to pardon the princes. As was customary in Mongol society for nobility, the Russian princes were given a bloodless death. Subutai had a large wooden platform constructed on which he ate his meals along with his other generals. Six Russian princes, including Mstislav III of Kiev, were put under this platform and crushed to death.</t>
         </is>
       </c>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t>[80, 2, 44, 45, 804]</t>
-        </is>
-      </c>
-      <c r="G82" t="inlineStr">
-        <is>
-          <t>[0.8581974506378174, 0.8428511619567871, 0.8284873962402344, 0.8164754509925842, 0.8136602640151978]</t>
-        </is>
-      </c>
-      <c r="H82" t="inlineStr">
-        <is>
-          <t>["The Shah's army was split by diverse internecine feuds and by the Shah's decision to divide his army into small groups concentrated in various cities. This fragmentation was decisive in Khwarezmia's defeats, as it allowed the Mongols, although exhausted from the long journey, to immediately set about defeating small fractions of the Khwarzemi forces instead of facing a unified defense. The Mongol army quickly seized the town of Otrar, relying on superior strategy and tactics. Genghis Khan ordered the wholesale massacre of many of the civilians, enslaved the rest of the population and executed Inalchuq by pouring molten silver into his ears and eyes, as retribution for his actions. Near the end of the battle the Shah fled rather than surrender. Genghis Khan ordered Subutai and Jebe to hunt him down, giving them 20,000 men and two years to do this. The Shah died under mysterious circumstances on a small island within his empire.", "The invasions of Baghdad, Samarkand, Urgench, Kiev, Vladimir among others caused mass murders, such as when portions of southern Khuzestan were completely destroyed. His descendant Hulagu Khan destroyed much of Iran's northern part and sacked Baghdad although his forces were halted by the Mamluks of Egypt, but Hulagu's descendant Ghazan Khan would return to beat the Egyptian Mamluks right out of Levant, Palestine and even Gaza. According to the works of the Persian historian Rashid-al-Din Hamadani, the Mongols killed more than 70,000 people in Merv and more than 190,000 in Nishapur. In 1237 Batu Khan, a grandson of Genghis Khan, launched an invasion into Kievan Rus'. Over the course of three years, the Mongols destroyed and annihilated all of the major cities of Eastern Europe with the exceptions of Novgorod and Pskov.", "In the early 13th century, the Khwarazmian dynasty was governed by Shah Ala ad-Din Muhammad. Genghis Khan saw the potential advantage in Khwarezmia as a commercial trading partner using the Silk Road, and he initially sent a 500-man caravan to establish official trade ties with the empire. However, Inalchuq, the governor of the Khwarezmian city of Otrar, attacked the caravan that came from Mongolia, claiming that the caravan contained spies and therefore was a conspiracy against Khwarezmia. The situation became further complicated because the governor later refused to make repayments for the looting of the caravans and handing over the perpetrators. Genghis Khan then sent again a second group of three ambassadors (two Mongols and a Muslim) to meet the Shah himself instead of the governor Inalchuq. The Shah had all the men shaved and the Muslim beheaded and sent his head back with the two remaining ambassadors. This was seen as an affront and insult to Genghis Khan. Outraged, Genghis Khan planned one of his largest invasion campaigns by organizing together around 100,000 soldiers (10 tumens), his most capable generals and some of his sons. He left a commander and number of troops in China, designated his successors to", "seen as an affront and insult to Genghis Khan. Outraged, Genghis Khan planned one of his largest invasion campaigns by organizing together around 100,000 soldiers (10 tumens), his most capable generals and some of his sons. He left a commander and number of troops in China, designated his successors to be his family members and likely appointed Ögedei to be his immediate successor and then went out to Khwarezmia.", "a separate peace, but the emissaries were executed. At the Battle of Kalka River in 1223, Subutai's forces defeated the larger Kievan force. They also may have fought against the neighboring Volga Bulgars. There is no historical record except a short account by the Arab historian Ibn al-Athir, writing in Mosul some 1100 miles away from the event. Various historical secondary sources - Morgan, Chambers, Grousset - state that the Mongols actually defeated the Bulgars, Chambers even going so far as to say that the Bulgars had made up stories to tell the (recently crushed) Russians that they had beaten the Mongols and driven them from their territory. The Russian princes then sued for peace. Subutai agreed but was in no mood to pardon the princes. As was customary in Mongol society for nobility, the Russian princes were given a bloodless death. Subutai had a large wooden platform constructed on which he ate his meals along with his other generals. Six Russian princes, including Mstislav III of Kiev, were put under this platform and crushed to death."]</t>
-        </is>
-      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4247,21 +3017,6 @@
 Luther's rediscovery of "Christ and His salvation" was the first of two points that became the foundation for the Reformation. His railing against the sale of indulgences was based on it.</t>
         </is>
       </c>
-      <c r="F83" t="inlineStr">
-        <is>
-          <t>[572, 179, 412, 81, 398]</t>
-        </is>
-      </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>[0.8453444242477417, 0.8165795803070068, 0.8059324026107788, 0.7969955801963806, 0.7968401908874512]</t>
-        </is>
-      </c>
-      <c r="H83" t="inlineStr">
-        <is>
-          <t>["(1528), drafted by Melanchthon with Luther's approval, stressed the role of repentance in the forgiveness of sins, despite Luther's position that faith alone ensures justification. The Eisleben reformer Johannes Agricola challenged this compromise, and Luther condemned him for teaching that faith is separate from works. The Instruction is a problematic document for those seeking a consistent evolution in Luther's thought and practice.", "The effect of Luther's intervention was immediate. After the sixth sermon, the Wittenberg jurist Jerome Schurf wrote to the elector: \"Oh, what joy has Dr. Martin's return spread among us! His words, through divine mercy, are bringing back every day misguided people into the way of the truth.\"", "The Lutheran theologian Franz Pieper observed that Luther's teaching about the state of the Christian's soul after death differed from the later Lutheran theologians such as Johann Gerhard. Lessing (1755) had earlier reached the same conclusion in his analysis of Lutheran orthodoxy on this issue.", "Luther dedicated himself to the Augustinian order, devoting himself to fasting, long hours in prayer, pilgrimage, and frequent confession. Luther described this period of his life as one of deep spiritual despair. He said, \"I lost touch with Christ the Savior and Comforter, and made of him the jailer and hangman of my poor soul.\" Johann von Staupitz, his superior, pointed Luther's mind away from continual reflection upon his sins toward the merits of Christ. He taught that true repentance does not involve self-inflicted penances and punishments but rather a change of heart.", "Luther's rediscovery of \"Christ and His salvation\" was the first of two points that became the foundation for the Reformation. His railing against the sale of indulgences was based on it."]</t>
-        </is>
-      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4293,21 +3048,6 @@
 In 1882, Tesla began working for the Continental Edison Company in France, designing and making improvements to electrical equipment. In June 1884, he relocated to New York City:57–60 where he was hired by Thomas Edison to work at his Edison Machine Works on Manhattan's lower east side. Tesla's work for Edison began with simple electrical engineering and quickly progressed to solving more difficult problems.</t>
         </is>
       </c>
-      <c r="F84" t="inlineStr">
-        <is>
-          <t>[606, 82, 48, 473, 757]</t>
-        </is>
-      </c>
-      <c r="G84" t="inlineStr">
-        <is>
-          <t>[0.7607412934303284, 0.7540321350097656, 0.694690465927124, 0.6914713978767395, 0.6898600459098816]</t>
-        </is>
-      </c>
-      <c r="H84" t="inlineStr">
-        <is>
-          <t>["Many of Tesla's writings are freely available on the web, including the article \"The Problem of Increasing Human Energy,\" published in The Century Magazine in 1900, and the article \"Experiments With Alternate Currents Of High Potential And High Frequency,\" published in his book Inventions, Researches and Writings of Nikola Tesla.", "In 1888, the editor of Electrical World magazine, Thomas Commerford Martin (a friend and publicist), arranged for Tesla to demonstrate his alternating current system, including his induction motor, at the American Institute of Electrical Engineers (now IEEE). Engineers working for the Westinghouse Electric &amp; Manufacturing Company reported to George Westinghouse that Tesla had a viable AC motor and related power system — something for which Westinghouse had been trying to secure patents. Westinghouse looked into getting a patent on a similar commutator-less, rotating magnetic field-based induction motor presented in a paper in March 1888 by the Italian physicist Galileo Ferraris, but decided Tesla's patent would probably control the market.", "Tesla's motor had to be put on hold for a while. The competition resulted in Edison Machine Works pursuing AC development in 1890 and by 1892 Thomas Edison was no longer in control of his own company, which was consolidated into the conglomerate General Electric and converting to an AC delivery system at that point.", "Tesla gained experience in telephony and electrical engineering before emigrating to the United States in 1884 to work for Thomas Edison in New York City. He soon struck out on his own with financial backers, setting up laboratories and companies to develop a range of electrical devices. His patented AC induction motor and transformer were licensed by George Westinghouse, who also hired Tesla for a short time as a consultant. His work in the formative years of electric power development was involved in a corporate alternating current/direct current \"War of Currents\" as well as various patent battles.", "In 1882, Tesla began working for the Continental Edison Company in France, designing and making improvements to electrical equipment. In June 1884, he relocated to New York City:57–60 where he was hired by Thomas Edison to work at his Edison Machine Works on Manhattan's lower east side. Tesla's work for Edison began with simple electrical engineering and quickly progressed to solving more difficult problems."]</t>
-        </is>
-      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -4339,21 +3079,6 @@
 The War of the Austrian Succession (whose North American theater is known as King George's War) formally ended in 1748 with the signing of the Treaty of Aix-la-Chapelle. The treaty was primarily focused on resolving issues in Europe. The issues of conflicting territorial claims between British and French colonies in North America were turned over to a commission to resolve, but it reached no decision. Frontiers from between Nova Scotia and Acadia in the north, to the Ohio Country in the south, were claimed by both sides. The disputes also extended into the Atlantic Ocean, where both powers wanted access to the rich fisheries of the Grand Banks off Newfoundland.</t>
         </is>
       </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t>[83, 709, 260, 679, 487]</t>
-        </is>
-      </c>
-      <c r="G85" t="inlineStr">
-        <is>
-          <t>[0.8484999537467957, 0.7721326351165771, 0.7494194507598877, 0.7322988510131836, 0.7231785655021667]</t>
-        </is>
-      </c>
-      <c r="H85" t="inlineStr">
-        <is>
-          <t>["In between the French and the British, large areas were dominated by native tribes. To the north, the Mi'kmaq and the Abenaki were engaged in Father Le Loutre's War and still held sway in parts of Nova Scotia, Acadia, and the eastern portions of the province of Canada, as well as much of present-day Maine. The Iroquois Confederation dominated much of present-day Upstate New York and the Ohio Country, although the latter also included Algonquian-speaking populations of Delaware and Shawnee, as well as Iroquoian-speaking Mingo. These tribes were formally under Iroquois rule, and were limited by them in authority to make agreements.", "When Céloron's expedition arrived at Logstown, the Native Americans in the area informed Céloron that they owned the Ohio Country and that they would trade with the British regardless of the French. Céloron continued south until his expedition reached the confluence of the Ohio and the Miami rivers, which lay just south of the village of Pickawillany, the home of the Miami chief known as \"Old Briton\". Céloron threatened \"Old Briton\" with severe consequences if he continued to trade with the British. \"Old Briton\" ignored the warning. Disappointed, Céloron returned to Montreal in November 1749.", "For many native populations, the elimination of French power in North America meant the disappearance of a strong ally and counterweight to British expansion, leading to their ultimate dispossession. The Ohio Country was particularly vulnerable to legal and illegal settlement due to the construction of military roads to the area by Braddock and Forbes. Although the Spanish takeover of the Louisiana territory (which was not completed until 1769) had modest repercussions, the British takeover of Spanish Florida resulted in the westward migration of tribes that did not want to do business with the British, and a rise in tensions between the Choctaw and the Creek, historic enemies whose divisions the British at times exploited. The change of control in Florida also prompted most of its Spanish Catholic population to leave. Most went to Cuba, including the entire governmental records from St. Augustine, although some Christianized Yamasee were resettled to the coast of Mexico.", "British settlers outnumbered the French 20 to 1 with a population of about 1.5 million ranged along the eastern coast of the continent, from Nova Scotia and Newfoundland in the north, to Georgia in the south. Many of the older colonies had land claims that extended arbitrarily far to the west, as the extent of the continent was unknown at the time their provincial charters were granted. While their population centers were along the coast, the settlements were growing into the interior. Nova Scotia, which had been captured from France in 1713, still had a significant French-speaking population. Britain also claimed Rupert's Land, where the Hudson's Bay Company traded for furs with local tribes.", "The War of the Austrian Succession (whose North American theater is known as King George's War) formally ended in 1748 with the signing of the Treaty of Aix-la-Chapelle. The treaty was primarily focused on resolving issues in Europe. The issues of conflicting territorial claims between British and French colonies in North America were turned over to a commission to resolve, but it reached no decision. Frontiers from between Nova Scotia and Acadia in the north, to the Ohio Country in the south, were claimed by both sides. The disputes also extended into the Atlantic Ocean, where both powers wanted access to the rich fisheries of the Grand Banks off Newfoundland."]</t>
-        </is>
-      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4385,21 +3110,6 @@
 Luther's rediscovery of "Christ and His salvation" was the first of two points that became the foundation for the Reformation. His railing against the sale of indulgences was based on it.</t>
         </is>
       </c>
-      <c r="F86" t="inlineStr">
-        <is>
-          <t>[480, 179, 84, 412, 398]</t>
-        </is>
-      </c>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>[0.838001549243927, 0.8260897397994995, 0.8251415491104126, 0.8191632032394409, 0.8172340393066406]</t>
-        </is>
-      </c>
-      <c r="H86" t="inlineStr">
-        <is>
-          <t>["was one of the worst mistakes Luther made, and, next to the landgrave himself, who was directly responsible for it, history chiefly holds Luther accountable\". Brecht argues that Luther's mistake was not that he gave private pastoral advice, but that he miscalculated the political implications. The affair caused lasting damage to Luther's reputation.", "The effect of Luther's intervention was immediate. After the sixth sermon, the Wittenberg jurist Jerome Schurf wrote to the elector: \"Oh, what joy has Dr. Martin's return spread among us! His words, through divine mercy, are bringing back every day misguided people into the way of the truth.\"", "His poor physical health made him short-tempered and even harsher in his writings and comments. His wife Katharina was overheard saying, \"Dear husband, you are too rude,\" and he responded, \"They are teaching me to be rude.\" In 1545 and 1546 Luther preached three times in the Market Church in Halle, staying with his friend Justus Jonas during Christmas.", "The Lutheran theologian Franz Pieper observed that Luther's teaching about the state of the Christian's soul after death differed from the later Lutheran theologians such as Johann Gerhard. Lessing (1755) had earlier reached the same conclusion in his analysis of Lutheran orthodoxy on this issue.", "Luther's rediscovery of \"Christ and His salvation\" was the first of two points that became the foundation for the Reformation. His railing against the sale of indulgences was based on it."]</t>
-        </is>
-      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4429,21 +3139,6 @@
 Kenya has a warm and humid tropical climate on its Indian Ocean coastline. The climate is cooler in the savannah grasslands around the capital city, Nairobi, and especially closer to Mount Kenya, which has snow permanently on its peaks. Further inland, in the Nyanza region, there is a hot and dry climate which becomes humid around Lake Victoria, the largest tropical fresh-water lake in the world. This gives way to temperate and forested hilly areas in the neighboring western region. The north-eastern regions along the border with Somalia and Ethiopia are arid and semi-arid areas with near-desert landscapes. Kenya is known for its safaris, diverse climate and geography, and expansive wildlife reserves and national parks such as the East and West Tsavo National Park, the Maasai Mara, Lake Nakuru National Park, and Aberdares National Park. Kenya has several world heritage sites such as Lamu and numerous beaches, including in Diani, Bamburi and Kilifi, where international yachting competitions are held every year.
 The city developed around the Roman settlement Pons Aelius and was named after the castle built in 1080 by Robert Curthose, William the Conqueror's eldest son. The city grew as an important centre for the wool trade in the 14th century, and later became a major coal mining area. The port developed in the 16th century and, along with the shipyards lower down the River Tyne, was amongst the world's largest shipbuilding and ship-repairing centres. Newcastle's economy includes corporate headquarters, learning, digital technology, retail, tourism and cultural centres, from which the city contributes £13 billion towards the United Kingdom's GVA. Among its icons are Newcastle Brown Ale; Newcastle United football club; and the Tyne Bridge. It has hosted the world's most popular half marathon, the Great North Run, since it began in 1981.
 The Tyneside flat was the dominant housing form constructed at the time when the industrial centres on Tyneside were growing most rapidly. They can still be found in areas such as South Heaton in Newcastle but once dominated the streetscape on both sides of the Tyne. Tyneside flats were built as terraces, one of each pair of doors led to an upstairs flat while the other led into the ground-floor flat, each of two or three rooms. A new development in the Ouseburn valley has recreated them; Architects Cany Ash and Robert Sakula were attracted by the possibilities of high density without building high and getting rid of common areas.</t>
-        </is>
-      </c>
-      <c r="F87" t="inlineStr">
-        <is>
-          <t>[85, 228, 813, 211, 316]</t>
-        </is>
-      </c>
-      <c r="G87" t="inlineStr">
-        <is>
-          <t>[0.8372297286987305, 0.7439129948616028, 0.7246624827384949, 0.6986282467842102, 0.6902270317077637]</t>
-        </is>
-      </c>
-      <c r="H87" t="inlineStr">
-        <is>
-          <t>["The climate in Newcastle is oceanic (Köppen Cfb) and significantly milder than some other locations in the world at a similar latitude, due to the warming influence of the Gulf Stream (via the North Atlantic Drift). Being in the rain shadow of the North Pennines, it is among the driest cities in the UK. Temperature extremes recorded at Newcastle Weather Centre include 32.5 °C (90.5 °F) during August 1990 down to −12.6 °C (9.3 °F) during January 1982. In contrast to other areas influenced by the Gulf Stream, such as inland Scandinavia, Newcastle has milder winters and cooler summers, similar to the remainder of the British Isles.", "Like much of the south Atlantic region of the United States, Jacksonville has a humid subtropical climate (Köppen Cfa), with mild weather during winters and hot and humid weather during summers. Seasonal rainfall is concentrated in the warmest months from May through September, while the driest months are from November through April. Due to Jacksonville's low latitude and coastal location, the city sees very little cold weather, and winters are typically mild and sunny. Summers can be hot and wet, and summer thunderstorms with torrential but brief downpours are common.", "Kenya has a warm and humid tropical climate on its Indian Ocean coastline. The climate is cooler in the savannah grasslands around the capital city, Nairobi, and especially closer to Mount Kenya, which has snow permanently on its peaks. Further inland, in the Nyanza region, there is a hot and dry climate which becomes humid around Lake Victoria, the largest tropical fresh-water lake in the world. This gives way to temperate and forested hilly areas in the neighboring western region. The north-eastern regions along the border with Somalia and Ethiopia are arid and semi-arid areas with near-desert landscapes. Kenya is known for its safaris, diverse climate and geography, and expansive wildlife reserves and national parks such as the East and West Tsavo National Park, the Maasai Mara, Lake Nakuru National Park, and Aberdares National Park. Kenya has several world heritage sites such as Lamu and numerous beaches, including in Diani, Bamburi and Kilifi, where international yachting competitions are held every year.", "The city developed around the Roman settlement Pons Aelius and was named after the castle built in 1080 by Robert Curthose, William the Conqueror's eldest son. The city grew as an important centre for the wool trade in the 14th century, and later became a major coal mining area. The port developed in the 16th century and, along with the shipyards lower down the River Tyne, was amongst the world's largest shipbuilding and ship-repairing centres. Newcastle's economy includes corporate headquarters, learning, digital technology, retail, tourism and cultural centres, from which the city contributes £13 billion towards the United Kingdom's GVA. Among its icons are Newcastle Brown Ale; Newcastle United football club; and the Tyne Bridge. It has hosted the world's most popular half marathon, the Great North Run, since it began in 1981.", "The Tyneside flat was the dominant housing form constructed at the time when the industrial centres on Tyneside were growing most rapidly. They can still be found in areas such as South Heaton in Newcastle but once dominated the streetscape on both sides of the Tyne. Tyneside flats were built as terraces, one of each pair of doors led to an upstairs flat while the other led into the ground-floor flat, each of two or three rooms. A new development in the Ouseburn valley has recreated them; Architects Cany Ash and Robert Sakula were attracted by the possibilities of high density without building high and getting rid of common areas."]</t>
         </is>
       </c>
     </row>
@@ -4486,21 +3181,6 @@
 2 mixtures only if they are breathed during aerobic exercise.</t>
         </is>
       </c>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t>[0, 86, 607, 558, 472]</t>
-        </is>
-      </c>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t>[0.707305908203125, 0.7016441226005554, 0.7014697194099426, 0.6943860054016113, 0.6770566701889038]</t>
-        </is>
-      </c>
-      <c r="H88" t="inlineStr">
-        <is>
-          <t>["Hyperbaric (high-pressure) medicine uses special oxygen chambers to increase the partial pressure of O\n2 around the patient and, when needed, the medical staff. Carbon monoxide poisoning, gas gangrene, and decompression sickness (the 'bends') are sometimes treated using these devices. Increased O\n2 concentration in the lungs helps to displace carbon monoxide from the heme group of hemoglobin. Oxygen gas is poisonous to the anaerobic bacteria that cause gas gangrene, so increasing its partial pressure helps kill them. Decompression sickness occurs in divers who decompress too quickly after a dive, resulting in bubbles of inert gas, mostly nitrogen and helium, forming in their blood. Increasing the pressure of O\n2 as soon as possible is part of the treatment.", "Oxygen toxicity to the lungs and central nervous system can also occur in deep scuba diving and surface supplied diving. Prolonged breathing of an air mixture with an O\n2 partial pressure more than 60 kPa can eventually lead to permanent pulmonary fibrosis. Exposure to a O\n2 partial pressures greater than 160 kPa (about 1.6 atm) may lead to convulsions (normally fatal for divers). Acute oxygen toxicity (causing seizures, its most feared effect for divers) can occur by breathing an air mixture with 21% O\n2 at 66 m or more of depth; the same thing can occur by breathing 100% O\n2 at only 6 m.", "The reason for the majority rule is the high risk of a conflict of interest and/or the avoidance of absolute powers. Otherwise, the physician has a financial self-interest in \"diagnosing\" as many conditions as possible, and in exaggerating their seriousness, because he or she can then sell more medications to the patient. Such self-interest directly conflicts with the patient's interest in obtaining cost-effective medication and avoiding the unnecessary use of medication that may have side-effects. This system reflects much similarity to the checks and balances system of the U.S. and many other governments.[citation needed]", "to further the story by requesting exposition from the Doctor and manufacturing peril for the Doctor to resolve. The Doctor regularly gains new companions and loses old ones; sometimes they return home or find new causes — or loves — on worlds they have visited. Some have died during the course of the series. Companions are usually human, or humanoid aliens.", "Oxygen, as a supposed mild euphoric, has a history of recreational use in oxygen bars and in sports. Oxygen bars are establishments, found in Japan, California, and Las Vegas, Nevada since the late 1990s that offer higher than normal O\n2 exposure for a fee. Professional athletes, especially in American football, also sometimes go off field between plays to wear oxygen masks in order to get a \"boost\" in performance. The pharmacological effect is doubtful; a placebo effect is a more likely explanation. Available studies support a performance boost from enriched O\n2 mixtures only if they are breathed during aerobic exercise."]</t>
-        </is>
-      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4532,21 +3212,6 @@
 manpower in such a way that necessitated colonial expansion. This conception of imperialism as a structural feature of capitalism is echoed by later Marxist theoreticians. Many theoreticians on the left have followed in emphasizing the structural or systemic character of "imperialism". Such writers have expanded the time period associated with the term so that it now designates neither a policy, nor a short space of decades in the late 19th century, but a world system extending over a period of centuries, often going back to Christopher Columbus and, in some accounts, to the Crusades. As the application of the term has expanded, its meaning has shifted along five distinct but often parallel axes: the moral, the economic, the systemic, the cultural, and the temporal. Those changes reflect - among other shifts in sensibility - a growing unease, even squeamishness, with the fact of power, specifically, Western power.</t>
         </is>
       </c>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t>[87, 686, 532, 827, 615]</t>
-        </is>
-      </c>
-      <c r="G89" t="inlineStr">
-        <is>
-          <t>[0.7324826121330261, 0.7218717336654663, 0.6867578625679016, 0.6812943816184998, 0.6784130334854126]</t>
-        </is>
-      </c>
-      <c r="H89" t="inlineStr">
-        <is>
-          <t>["Some disagree with such double or triple non-French linguistic origins, arguing that for the word to have spread into common use in France, it must have originated in the French language. The \"Hugues hypothesis\" argues that the name was derived by association with Hugues Capet, king of France, who reigned long before the Reformation. He was regarded by the Gallicans and Protestants as a noble man who respected people's dignity and lives. Janet Gray and other supporters of the hypothesis suggest that the name huguenote would be roughly equivalent to little Hugos, or those who want Hugo.", "LeGrande writes that \"the formulation of a single all-encompassing definition of the term is extremely difficult, if not impossible. In reviewing the voluminous literature on the subject, the student of civil disobedience rapidly finds himself surrounded by a maze of semantical problems and grammatical niceties. Like Alice in Wonderland, he often finds that specific terminology has no more (or no less) meaning than the individual orator intends it to have.\" He encourages a distinction between lawful protest demonstration, nonviolent civil disobedience, and violent civil disobedience.", "\"Bairn\" and \"hyem\", meaning \"child\" and \"home\", respectively, are examples of Geordie words with origins in Scandinavia; barn and hjem are the corresponding modern Norwegian and Danish words. Some words used in the Geordie dialect are used elsewhere in the Northern United Kingdom. The words \"bonny\" (meaning \"pretty\"), \"howay\" (\"come on\"), \"stot\" (\"bounce\") and \"hadaway\" (\"go away\" or \"you're kidding\"), all appear to be used in Scots; \"aye\" (\"yes\") and \"nowt\" (IPA://naʊt/, rhymes with out,\"nothing\") are used elsewhere in Northern England. Many words, however, appear to be used exclusively in Newcastle and the surrounding area, such as \"Canny\" (a versatile word meaning \"good\", \"nice\" or \"very\"), \"hacky\" (\"dirty\"), \"netty\" (\"toilet\"), \"hoy\" (\"throw\", from the Dutch gooien, via West Frisian), \"hockle\" (\"spit\").", "United States and Western Europe than in China (due to a greater tendency to take on debts).[unreliable source?][unreliable source?] Anthony Shorrocks, the lead author of the Credit Suisse report which is one of the sources of Oxfam's data, considers the criticism about debt to be a \"silly argument\" and \"a non-issue . . . a diversion.\"", "manpower in such a way that necessitated colonial expansion. This conception of imperialism as a structural feature of capitalism is echoed by later Marxist theoreticians. Many theoreticians on the left have followed in emphasizing the structural or systemic character of \"imperialism\". Such writers have expanded the time period associated with the term so that it now designates neither a policy, nor a short space of decades in the late 19th century, but a world system extending over a period of centuries, often going back to Christopher Columbus and, in some accounts, to the Crusades. As the application of the term has expanded, its meaning has shifted along five distinct but often parallel axes: the moral, the economic, the systemic, the cultural, and the temporal. Those changes reflect - among other shifts in sensibility - a growing unease, even squeamishness, with the fact of power, specifically, Western power."]</t>
-        </is>
-      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4578,21 +3243,6 @@
 Southern California consists of one Combined Statistical Area, eight Metropolitan Statistical Areas, one international metropolitan area, and multiple metropolitan divisions. The region is home to two extended metropolitan areas that exceed five million in population. These are the Greater Los Angeles Area at 17,786,419, and San Diego–Tijuana at 5,105,768. Of these metropolitan areas, the Los Angeles-Long Beach-Santa Ana metropolitan area, Riverside-San Bernardino-Ontario metropolitan area, and Oxnard-Thousand Oaks-Ventura metropolitan area form Greater Los Angeles; while the El Centro metropolitan area and San Diego-Carlsbad-San Marcos metropolitan area form the Southern Border Region. North of Greater Los Angeles are the Santa Barbara, San Luis Obispo, and Bakersfield metropolitan areas.</t>
         </is>
       </c>
-      <c r="F90" t="inlineStr">
-        <is>
-          <t>[88, 643, 293, 597, 250]</t>
-        </is>
-      </c>
-      <c r="G90" t="inlineStr">
-        <is>
-          <t>[0.9077863097190857, 0.8016424775123596, 0.8009201288223267, 0.8001531958580017, 0.795451819896698]</t>
-        </is>
-      </c>
-      <c r="H90" t="inlineStr">
-        <is>
-          <t>["Los Angeles (at 3.7 million people) and San Diego (at 1.3 million people), both in southern California, are the two largest cities in all of California (and two of the eight largest cities in the United States). In southern California there are also twelve cities with more than 200,000 residents and 34 cities over 100,000 in population. Many of southern California's most developed cities lie along or in close proximity to the coast, with the exception of San Bernardino and Riverside.", "Fresno (/ˈfrɛznoʊ/ FREZ-noh), the county seat of Fresno County, is a city in the U.S. state of California. As of 2015, the city's population was 520,159, making it the fifth-largest city in California, the largest inland city in California and the 34th-largest in the nation. Fresno is in the center of the San Joaquin Valley and is the largest city in the Central Valley, which contains the San Joaquin Valley. It is approximately 220 miles (350 km) northwest of Los Angeles, 170 miles (270 km) south of the state capital, Sacramento, or 185 miles (300 km) south of San Francisco. The name Fresno means \"ash tree\" in Spanish, and an ash leaf is featured on the city's flag.", "Southern California consists of a heavily developed urban environment, home to some of the largest urban areas in the state, along with vast areas that have been left undeveloped. It is the third most populated megalopolis in the United States, after the Great Lakes Megalopolis and the Northeastern megalopolis. Much of southern California is famous for its large, spread-out, suburban communities and use of automobiles and highways. The dominant areas are Los Angeles, Orange County, San Diego, and Riverside-San Bernardino, each of which is the center of its respective metropolitan area, composed of numerous smaller cities and communities. The urban area is also host to an international metropolitan region in the form of San Diego–Tijuana, created by the urban area spilling over into Baja California.", "Its counties of Los Angeles, Orange, San Diego, San Bernardino, and Riverside are the five most populous in the state and all are in the top 15 most populous counties in the United States.", "Southern California consists of one Combined Statistical Area, eight Metropolitan Statistical Areas, one international metropolitan area, and multiple metropolitan divisions. The region is home to two extended metropolitan areas that exceed five million in population. These are the Greater Los Angeles Area at 17,786,419, and San Diego–Tijuana at 5,105,768. Of these metropolitan areas, the Los Angeles-Long Beach-Santa Ana metropolitan area, Riverside-San Bernardino-Ontario metropolitan area, and Oxnard-Thousand Oaks-Ventura metropolitan area form Greater Los Angeles; while the El Centro metropolitan area and San Diego-Carlsbad-San Marcos metropolitan area form the Southern Border Region. North of Greater Los Angeles are the Santa Barbara, San Luis Obispo, and Bakersfield metropolitan areas."]</t>
-        </is>
-      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4624,21 +3274,6 @@
 On April 14, 2011, ABC canceled the long-running soap operas All My Children and One Life to Live after 41 and 43 years on the air, respectively (following backlash from fans, ABC sold the rights to both shows to Prospect Park, which eventually revived the soaps on Hulu for one additional season in 2013 and with both companies suing one another for allegations of interference with the process of reviving the shows, failure to pay licensing fees and issues over ABC's use of certain characters from One Live to Live on General Hospital during the transition). The talk/lifestyle show that replaced One Life to Live, The Revolution, failed to generate satisfactory ratings and was in turn canceled after only seven months. The 2011–12 season saw ABC drop to fourth place in the 18–49 demographic despite renewing a handful of new shows (including freshmen dramas Scandal, Revenge and Once Upon a Time) for second seasons.</t>
         </is>
       </c>
-      <c r="F91" t="inlineStr">
-        <is>
-          <t>[89, 810, 584, 689, 356]</t>
-        </is>
-      </c>
-      <c r="G91" t="inlineStr">
-        <is>
-          <t>[0.8695352077484131, 0.8568935990333557, 0.8418570160865784, 0.8208155035972595, 0.8123363852500916]</t>
-        </is>
-      </c>
-      <c r="H91" t="inlineStr">
-        <is>
-          <t>["It was not until the late 1950s that the ABC network became a serious contender to NBC and CBS, and this was in large part due to the diverse range of programming that met the expectations of the public, such as westerns and detective series. Despite an almost 500% increase in advertising revenues between 1953 and 1958, the network only had a national reach of between 10% and 18% of the total U.S. population, as it still had relatively fewer affiliates than NBC and CBS. In 1957, ABC Entertainment president Ollie Treiz discovered that the locally produced variety show Bandstand had pulled very strong ratings in the Philadelphia market on WFIL-TV; Treiz ultimately negotiated a deal to take the show national, under the revised title American Bandstand; the show quickly became a social phenomenon by presenting new musical talent and dances to America's youth and helped make a star out of its host, Dick Clark.", "ABC dominated the American television landscape during the 1970s and early 1980s (by 1980, the three major networks represented 90% of all prime-time television viewership in the U.S.). Several flagship series debuted on the network during this time including Dynasty, an opulent drama from Aaron Spelling that became a hit when it premiered as a midseason series in 1981, five months before Spelling's other ABC hit Charlie's Angels ended its run. The network was also propelled during the early 1980s by the continued successes of Happy Days, Three's Company, Laverne &amp; Shirley and Fantasy Island, and gained new hits in Too Close for Comfort, Soap spinoff Benson and Happy Days spinoff Mork &amp; Mindy. In 1981, ABC (through its ABC Video Services division) launched the Alpha Repertory Television Service (ARTS), a cable channel operated as a joint venture with the Hearst Corporation offering cultural and arts programming, which aired as a nighttime service over the channel space of Nickelodeon.", "At the same time he made attempts to help grow ABC, Goldenson had been trying since mid-1953 to provide content for the network by contacting his old acquaintances in Hollywood, with whom he had worked when UPT was a subsidiary of Paramount Pictures. ABC's merger with UPT led to the creation of relationships with Hollywood's film production studios, breaking a quarantine that had existed at that time between film and television, the latter of which had previously been more connected to radio. ABC's flagship productions at the time were The Lone Ranger, based on the radio program of the same title, and The Adventures of Ozzie and Harriet, the latter of which (at 13 seasons, running from 1952 to 1965) held the record for the longest-running prime time comedy in U.S. television history, until it was surpassed by The Simpsons in 2002.", "Due to pressure from film studios wanting to increase their production, as the major networks began airing theatrically released films, ABC joined CBS and NBC in broadcasting films on Sunday nights in 1962, with the launch of the ABC Sunday Night Movie, which debuted a year behind its competitors and was initially presented in black-and-white. Despite a significant increase in viewership (with its audience share having increased to 33% from the 15% share it had in 1953), ABC remained in third place; the company had a total revenue of $15.5 million, a third of the revenue pulled in by CBS at the same period. To catch up, ABC followed up The Flintstones with another animated series from Hanna-Barbera, The Jetsons, which debuted on September 23, 1962 as the first television series to be broadcast in color on the network. On April 1, 1963, ABC debuted the soap opera General Hospital, which would go on to become the television network's long-running entertainment program. That year also saw the premiere of The Fugitive (on September 17), a drama series centering on a man on the run after being accused of committing a murder he did not commit.", "On April 14, 2011, ABC canceled the long-running soap operas All My Children and One Life to Live after 41 and 43 years on the air, respectively (following backlash from fans, ABC sold the rights to both shows to Prospect Park, which eventually revived the soaps on Hulu for one additional season in 2013 and with both companies suing one another for allegations of interference with the process of reviving the shows, failure to pay licensing fees and issues over ABC's use of certain characters from One Live to Live on General Hospital during the transition). The talk/lifestyle show that replaced One Life to Live, The Revolution, failed to generate satisfactory ratings and was in turn canceled after only seven months. The 2011–12 season saw ABC drop to fourth place in the 18–49 demographic despite renewing a handful of new shows (including freshmen dramas Scandal, Revenge and Once Upon a Time) for second seasons."]</t>
-        </is>
-      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -4670,21 +3305,6 @@
 Highly combustible materials that leave little residue, such as wood or coal, were thought to be made mostly of phlogiston; whereas non-combustible substances that corrode, such as iron, contained very little. Air did not play a role in phlogiston theory, nor were any initial quantitative experiments conducted to test the idea; instead, it was based on observations of what happens when something burns, that most common objects appear to become lighter and seem to lose something in the process. The fact that a substance like wood gains overall weight in burning was hidden by the buoyancy of the gaseous combustion products. Indeed, one of the first clues that the phlogiston theory was incorrect was that metals, too, gain weight in rusting (when they were supposedly losing phlogiston).</t>
         </is>
       </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>[90, 360, 326, 164, 455]</t>
-        </is>
-      </c>
-      <c r="G92" t="inlineStr">
-        <is>
-          <t>[0.8251729607582092, 0.782328724861145, 0.7658107280731201, 0.7274931073188782, 0.7237328886985779]</t>
-        </is>
-      </c>
-      <c r="H92" t="inlineStr">
-        <is>
-          <t>["One of the main functions of the chloroplast is its role in photosynthesis, the process by which light is transformed into chemical energy, to subsequently produce food in the form of sugars. Water (H2O) and carbon dioxide (CO2) are used in photosynthesis, and sugar and oxygen (O2) is made, using light energy. Photosynthesis is divided into two stages—the light reactions, where water is split to produce oxygen, and the dark reactions, or Calvin cycle, which builds sugar molecules from carbon dioxide. The two phases are linked by the energy carriers adenosine triphosphate (ATP) and nicotinamide adenine dinucleotide phosphate (NADP+).", "Chloroplasts' main role is to conduct photosynthesis, where the photosynthetic pigment chlorophyll captures the energy from sunlight and converts it and stores it in the energy-storage molecules ATP and NADPH while freeing oxygen from water. They then use the ATP and NADPH to make organic molecules from carbon dioxide in a process known as the Calvin cycle. Chloroplasts carry out a number of other functions, including fatty acid synthesis, much amino acid synthesis, and the immune response in plants. The number of chloroplasts per cell varies from 1 in algae up to 100 in plants like Arabidopsis and wheat.", "To fix carbon dioxide into sugar molecules in the process of photosynthesis, chloroplasts use an enzyme called rubisco. Rubisco has a problem—it has trouble distinguishing between carbon dioxide and oxygen, so at high oxygen concentrations, rubisco starts accidentally adding oxygen to sugar precursors. This has the end result of ATP energy being wasted and CO2 being released, all with no sugar being produced. This is a big problem, since O2 is produced by the initial light reactions of photosynthesis, causing issues down the line in the Calvin cycle which uses rubisco.", "Photorespiration can occur when the oxygen concentration is too high. Rubisco cannot distinguish between oxygen and carbon dioxide very well, so it can accidentally add O2 instead of CO2 to RuBP. This process reduces the efficiency of photosynthesis—it consumes ATP and oxygen, releases CO2, and produces no sugar. It can waste up to half the carbon fixed by the Calvin cycle. Several mechanisms have evolved in different lineages that raise the carbon dioxide concentration relative to oxygen within the chloroplast, increasing the efficiency of photosynthesis. These mechanisms are called carbon dioxide concentrating mechanisms, or CCMs. These include Crassulacean acid metabolism, C4 carbon fixation, and pyrenoids. Chloroplasts in C4 plants are notable as they exhibit a distinct chloroplast dimorphism.", "Highly combustible materials that leave little residue, such as wood or coal, were thought to be made mostly of phlogiston; whereas non-combustible substances that corrode, such as iron, contained very little. Air did not play a role in phlogiston theory, nor were any initial quantitative experiments conducted to test the idea; instead, it was based on observations of what happens when something burns, that most common objects appear to become lighter and seem to lose something in the process. The fact that a substance like wood gains overall weight in burning was hidden by the buoyancy of the gaseous combustion products. Indeed, one of the first clues that the phlogiston theory was incorrect was that metals, too, gain weight in rusting (when they were supposedly losing phlogiston)."]</t>
-        </is>
-      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -4716,21 +3336,6 @@
 In the first half of the 17th century, a plague claimed some 1.7 million victims in Italy, or about 14% of the population. In 1656, the plague killed about half of Naples' 300,000 inhabitants. More than 1.25 million deaths resulted from the extreme incidence of plague in 17th-century Spain. The plague of 1649 probably reduced the population of Seville by half. In 1709–13, a plague epidemic that followed the Great Northern War (1700–21, Sweden v. Russia and allies) killed about 100,000 in Sweden, and 300,000 in Prussia. The plague killed two-thirds of the inhabitants of Helsinki, and claimed a third of Stockholm's population. Europe's last major epidemic occurred in 1720 in Marseille.</t>
         </is>
       </c>
-      <c r="F93" t="inlineStr">
-        <is>
-          <t>[91, 715, 522, 678, 427]</t>
-        </is>
-      </c>
-      <c r="G93" t="inlineStr">
-        <is>
-          <t>[0.845255434513092, 0.8265877366065979, 0.8164545297622681, 0.7883668541908264, 0.7800713181495667]</t>
-        </is>
-      </c>
-      <c r="H93" t="inlineStr">
-        <is>
-          <t>["The plague struck various countries in the Middle East during the pandemic, leading to serious depopulation and permanent change in both economic and social structures. As it spread to western Europe, the disease entered the region from southern Russia also. By autumn 1347, the plague reached Alexandria in Egypt, probably through the port's trade with Constantinople, and ports on the Black Sea. During 1347, the disease travelled eastward to Gaza, and north along the eastern coast to cities in Lebanon, Syria and Palestine, including Ashkelon, Acre, Jerusalem, Sidon, Damascus, Homs, and Aleppo. In 1348–49, the disease reached Antioch. The city's residents fled to the north, most of them dying during the journey, but the infection had been spread to the people of Asia Minor.[citation needed]", "The historian Francis Aidan Gasquet wrote about the 'Great Pestilence' in 1893 and suggested that \"it would appear to be some form of the ordinary Eastern or bubonic plague\". He was able to adopt the epidemiology of the bubonic plague for the Black Death for the second edition in 1908, implicating rats and fleas in the process, and his interpretation was widely accepted for other ancient and medieval epidemics, such as the Justinian plague that was prevalent in the Eastern Roman Empire from 541 to 700 CE.", "The plague disease, caused by Yersinia pestis, is enzootic (commonly present) in populations of fleas carried by ground rodents, including marmots, in various areas including Central Asia, Kurdistan, Western Asia, Northern India and Uganda. Nestorian graves dating to 1338–39 near Lake Issyk Kul in Kyrgyzstan have inscriptions referring to plague and are thought by many epidemiologists to mark the outbreak of the epidemic, from which it could easily have spread to China and India. In October 2010, medical geneticists suggested that all three of the great waves of the plague originated in China. In China, the 13th century Mongol conquest caused a decline in farming and trading. However, economic recovery had been observed at the beginning of the 14th century. In the 1330s a large number of natural disasters and plagues led to widespread famine, starting in 1331, with a deadly plague arriving soon after. Epidemics that may have included plague killed an estimated 25 million Chinese and other Asians during the 15 years before it reached Constantinople in 1347.", "Gasquet (1908) claimed that the Latin name atra mors (Black Death) for the 14th-century epidemic first appeared in modern times in 1631 in a book on Danish history by J.I. Pontanus: \"Vulgo &amp; ab effectu atram mortem vocatibant. (\"Commonly and from its effects, they called it the black death\"). The name spread through Scandinavia and then Germany, gradually becoming attached to the mid 14th-century epidemic as a proper name. In England, it was not until 1823 that the medieval epidemic was first called the Black Death.", "In the first half of the 17th century, a plague claimed some 1.7 million victims in Italy, or about 14% of the population. In 1656, the plague killed about half of Naples' 300,000 inhabitants. More than 1.25 million deaths resulted from the extreme incidence of plague in 17th-century Spain. The plague of 1649 probably reduced the population of Seville by half. In 1709–13, a plague epidemic that followed the Great Northern War (1700–21, Sweden v. Russia and allies) killed about 100,000 in Sweden, and 300,000 in Prussia. The plague killed two-thirds of the inhabitants of Helsinki, and claimed a third of Stockholm's population. Europe's last major epidemic occurred in 1720 in Marseille."]</t>
-        </is>
-      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -4762,21 +3367,6 @@
 LeGrande writes that "the formulation of a single all-encompassing definition of the term is extremely difficult, if not impossible. In reviewing the voluminous literature on the subject, the student of civil disobedience rapidly finds himself surrounded by a maze of semantical problems and grammatical niceties. Like Alice in Wonderland, he often finds that specific terminology has no more (or no less) meaning than the individual orator intends it to have." He encourages a distinction between lawful protest demonstration, nonviolent civil disobedience, and violent civil disobedience.</t>
         </is>
       </c>
-      <c r="F94" t="inlineStr">
-        <is>
-          <t>[92, 532, 87, 668, 686]</t>
-        </is>
-      </c>
-      <c r="G94" t="inlineStr">
-        <is>
-          <t>[0.7389503121376038, 0.7092235088348389, 0.6972635388374329, 0.6868628859519958, 0.685661792755127]</t>
-        </is>
-      </c>
-      <c r="H94" t="inlineStr">
-        <is>
-          <t>["Genghis Khan, the title is spelled in variety of ways in different languages such as Mongolian Chinggis Khaan, English Chinghiz, Chinghis, and Chingiz, Chinese: 成吉思汗; pinyin: Chéngjísī Hán, Turkic: Cengiz Han, Çingiz Xan, Çingiz Han, Chingizxon, Çıñğız Xan, Chengez Khan, Chinggis Khan, Chinggis Xaan, Chingis Khan, Jenghis Khan, Chinggis Qan, Djingis Kahn, Russian: Чингисхан (Čingiskhan) or Чингиз-хан (Čingiz-khan), etc. Temüjin is written in Chinese as simplified Chinese: 铁木真; traditional Chinese: 鐵木眞; pinyin: Tiěmùzhēn.", "\"Bairn\" and \"hyem\", meaning \"child\" and \"home\", respectively, are examples of Geordie words with origins in Scandinavia; barn and hjem are the corresponding modern Norwegian and Danish words. Some words used in the Geordie dialect are used elsewhere in the Northern United Kingdom. The words \"bonny\" (meaning \"pretty\"), \"howay\" (\"come on\"), \"stot\" (\"bounce\") and \"hadaway\" (\"go away\" or \"you're kidding\"), all appear to be used in Scots; \"aye\" (\"yes\") and \"nowt\" (IPA://naʊt/, rhymes with out,\"nothing\") are used elsewhere in Northern England. Many words, however, appear to be used exclusively in Newcastle and the surrounding area, such as \"Canny\" (a versatile word meaning \"good\", \"nice\" or \"very\"), \"hacky\" (\"dirty\"), \"netty\" (\"toilet\"), \"hoy\" (\"throw\", from the Dutch gooien, via West Frisian), \"hockle\" (\"spit\").", "Some disagree with such double or triple non-French linguistic origins, arguing that for the word to have spread into common use in France, it must have originated in the French language. The \"Hugues hypothesis\" argues that the name was derived by association with Hugues Capet, king of France, who reigned long before the Reformation. He was regarded by the Gallicans and Protestants as a noble man who respected people's dignity and lives. Janet Gray and other supporters of the hypothesis suggest that the name huguenote would be roughly equivalent to little Hugos, or those who want Hugo.", "As a result, by 1206 Temüjin had managed to unite or subdue the Merkits, Naimans, Mongols, Keraites, Tatars, Uyghurs, and other disparate smaller tribes under his rule. It was a monumental feat for the \"Mongols\" (as they became known collectively). At a Khuruldai, a council of Mongol chiefs, Temüjin was acknowledged as \"Khan\" of the consolidated tribes and took the new title \"Genghis Khan\". The title Khagan was not conferred on Genghis until after his death, when his son and successor, Ögedei, took the title for himself and extended it posthumously to his father (as he was also to be posthumously declared the founder of the Yuan dynasty). This unification of all confederations by Genghis Khan established peace between previously warring tribes and a single political and military force under Genghis Khan.", "LeGrande writes that \"the formulation of a single all-encompassing definition of the term is extremely difficult, if not impossible. In reviewing the voluminous literature on the subject, the student of civil disobedience rapidly finds himself surrounded by a maze of semantical problems and grammatical niceties. Like Alice in Wonderland, he often finds that specific terminology has no more (or no less) meaning than the individual orator intends it to have.\" He encourages a distinction between lawful protest demonstration, nonviolent civil disobedience, and violent civil disobedience."]</t>
-        </is>
-      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -4808,21 +3398,6 @@
 In 2014, economists with the Standard &amp; Poor's rating agency concluded that the widening disparity between the U.S.'s wealthiest citizens and the rest of the nation had slowed its recovery from the 2008-2009 recession and made it more prone to boom-and-bust cycles. To partially remedy the wealth gap and the resulting slow growth, S&amp;P recommended increasing access to education. It estimated that if the average United States worker had completed just one more year of school, it would add an additional $105 billion in growth to the country's economy over five years.</t>
         </is>
       </c>
-      <c r="F95" t="inlineStr">
-        <is>
-          <t>[407, 93, 736, 115, 743]</t>
-        </is>
-      </c>
-      <c r="G95" t="inlineStr">
-        <is>
-          <t>[0.8059675693511963, 0.798097550868988, 0.7812707424163818, 0.7772154211997986, 0.7746075391769409]</t>
-        </is>
-      </c>
-      <c r="H95" t="inlineStr">
-        <is>
-          <t>["wages due to the nature of the job, since there is a relative shortage of workers for the particular position. Professional and labor organizations may limit the supply of workers which results in higher demand and greater incomes for members. Members may also receive higher wages through collective bargaining, political influence, or corruption.", "During the mass high school education movement from 1910–1940, there was an increase in skilled workers, which led to a decrease in the price of skilled labor. High school education during the period was designed to equip students with necessary skill sets to be able to perform at work. In fact, it differs from the present high school education, which is regarded as a stepping-stone to acquire college and advanced degrees. This decrease in wages caused a period of compression and decreased inequality between skilled and unskilled workers. Education is very important for the growth of the economy, however educational inequality in gender also influence towards the economy. Lagerlof and Galor stated that gender inequality in education can result to low economic growth, and continued gender inequality in education, thus creating a poverty trap. It is suggested that a large gap in male and female education may indicate backwardness and so may be associated with lower economic growth, which can explain why there is economic inequality between countries.", "Since the 1920s, motion pictures, petroleum and aircraft manufacturing have been major industries. In one of the richest agricultural regions in the U.S., cattle and citrus were major industries until farmlands were turned into suburbs. Although military spending cutbacks have had an impact, aerospace continues to be a major factor.", "Economist Joseph Stiglitz presented evidence in 2009 that both global inequality and inequality within countries prevent growth by limiting aggregate demand. Economist Branko Milanovic, wrote in 2001 that, \"The view that income inequality harms growth – or that improved equality can help sustain growth – has become more widely held in recent years. ... The main reason for this shift is the increasing importance of human capital in development. When physical capital mattered most, savings and investments were key. Then it was important to have a large contingent of rich people who could save a greater proportion of their income than the poor and invest it in physical capital. But now that human capital is scarcer than machines, widespread education has become the secret to growth.\"", "In 2014, economists with the Standard &amp; Poor's rating agency concluded that the widening disparity between the U.S.'s wealthiest citizens and the rest of the nation had slowed its recovery from the 2008-2009 recession and made it more prone to boom-and-bust cycles. To partially remedy the wealth gap and the resulting slow growth, S&amp;P recommended increasing access to education. It estimated that if the average United States worker had completed just one more year of school, it would add an additional $105 billion in growth to the country's economy over five years."]</t>
-        </is>
-      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -4854,21 +3429,6 @@
 Southern California is divided culturally, politically, and economically into distinctive regions, each containing its own culture and atmosphere, anchored usually by a city with both national and sometimes global recognition, which are often the hub of economic activity for its respective region and being home to many tourist destinations. Each region is further divided into many culturally distinct areas but as a whole combine to create the southern California atmosphere.</t>
         </is>
       </c>
-      <c r="F96" t="inlineStr">
-        <is>
-          <t>[94, 88, 293, 181, 687]</t>
-        </is>
-      </c>
-      <c r="G96" t="inlineStr">
-        <is>
-          <t>[0.8827776908874512, 0.7870879173278809, 0.7725933194160461, 0.7627499103546143, 0.7599688172340393]</t>
-        </is>
-      </c>
-      <c r="H96" t="inlineStr">
-        <is>
-          <t>["Many locals and tourists frequent the southern California coast for its popular beaches, and the desert city of Palm Springs is popular for its resort feel and nearby open spaces.", "Los Angeles (at 3.7 million people) and San Diego (at 1.3 million people), both in southern California, are the two largest cities in all of California (and two of the eight largest cities in the United States). In southern California there are also twelve cities with more than 200,000 residents and 34 cities over 100,000 in population. Many of southern California's most developed cities lie along or in close proximity to the coast, with the exception of San Bernardino and Riverside.", "Southern California consists of a heavily developed urban environment, home to some of the largest urban areas in the state, along with vast areas that have been left undeveloped. It is the third most populated megalopolis in the United States, after the Great Lakes Megalopolis and the Northeastern megalopolis. Much of southern California is famous for its large, spread-out, suburban communities and use of automobiles and highways. The dominant areas are Los Angeles, Orange County, San Diego, and Riverside-San Bernardino, each of which is the center of its respective metropolitan area, composed of numerous smaller cities and communities. The urban area is also host to an international metropolitan region in the form of San Diego–Tijuana, created by the urban area spilling over into Baja California.", "Southern California's economy is diverse and one of the largest in the United States. It is dominated and heavily dependent upon abundance of petroleum, as opposed to other regions where automobiles not nearly as dominant, the vast majority of transport runs on this fuel. Southern California is famous for tourism and Hollywood (film, television, and music). Other industries include software, automotive, ports, finance, tourism, biomedical, and regional logistics. The region was a leader in the housing bubble 2001–2007, and has been heavily impacted by the housing crash.", "Southern California is divided culturally, politically, and economically into distinctive regions, each containing its own culture and atmosphere, anchored usually by a city with both national and sometimes global recognition, which are often the hub of economic activity for its respective region and being home to many tourist destinations. Each region is further divided into many culturally distinct areas but as a whole combine to create the southern California atmosphere."]</t>
-        </is>
-      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -4900,21 +3460,6 @@
 The mouth of the Rhine into Lake Constance forms an inland delta. The delta is delimited in the West by the Alter Rhein ("Old Rhine") and in the East by a modern canalized section. Most of the delta is a nature reserve and bird sanctuary. It includes the Austrian towns of Gaißau, Höchst and Fußach. The natural Rhine originally branched into at least two arms and formed small islands by precipitating sediments. In the local Alemannic dialect, the singular is pronounced "Isel" and this is also the local pronunciation of Esel ("Donkey"). Many local fields have an official name containing this element.</t>
         </is>
       </c>
-      <c r="F97" t="inlineStr">
-        <is>
-          <t>[95, 35, 657, 253, 747]</t>
-        </is>
-      </c>
-      <c r="G97" t="inlineStr">
-        <is>
-          <t>[0.7769045233726501, 0.7591420412063599, 0.7545980215072632, 0.7507529854774475, 0.7336955070495605]</t>
-        </is>
-      </c>
-      <c r="H97" t="inlineStr">
-        <is>
-          <t>["Warsaw lies in east-central Poland about 300 km (190 mi) from the Carpathian Mountains and about 260 km (160 mi) from the Baltic Sea, 523 km (325 mi) east of Berlin, Germany. The city straddles the Vistula River. It is located in the heartland of the Masovian Plain, and its average elevation is 100 metres (330 ft) above sea level. The highest point on the left side of the city lies at a height of 115.7 metres (379.6 ft) (\"Redutowa\" bus depot, district of Wola), on the right side – 122.1 metres (400.6 ft) (\"Groszówka\" estate, district of Wesoła, by the eastern border). The lowest point lies at a height 75.6 metres (248.0 ft) (at the right bank of the Vistula, by the eastern border of Warsaw). There are some hills (mostly artificial) located within the confines of the city – e.g. Warsaw Uprising Hill (121 metres (397.0 ft)), Szczęśliwice hill (138 metres (452.8 ft) – the highest point of Warsaw in general).", "In 2012 the Economist Intelligence Unit ranked Warsaw as the 32nd most liveable city in the world. It was also ranked as one of the most liveable cities in Central Europe. Today Warsaw is considered an \"Alpha–\" global city, a major international tourist destination and a significant cultural, political and economic hub. Warsaw's economy, by a wide variety of industries, is characterised by FMCG manufacturing, metal processing, steel and electronic manufacturing and food processing. The city is a significant centre of research and development, BPO, ITO, as well as of the Polish media industry. The Warsaw Stock Exchange is one of the largest and most important in Central and Eastern Europe. Frontex, the European Union agency for external border security, has its headquarters in Warsaw. It has been said that Warsaw, together with Frankfurt, London, Paris and Barcelona is one of the cities with the highest number of skyscrapers in the European Union. Warsaw has also been called \"Eastern Europe’s chic cultural capital with thriving art and club scenes and serious restaurants\".", "Warsaw is located on two main geomorphologic formations: the plain moraine plateau and the Vistula Valley with its asymmetrical pattern of different terraces. The Vistula River is the specific axis of Warsaw, which divides the city into two parts, left and right. The left one is situated both on the moraine plateau (10 to 25 m (32.8 to 82.0 ft) above Vistula level) and on the Vistula terraces (max. 6.5 m (21.3 ft) above Vistula level). The significant element of the relief, in this part of Warsaw, is the edge of moraine plateau called Warsaw Escarpment. It is 20 to 25 m (65.6 to 82.0 ft) high in the Old Town and Central district and about 10 m (32.8 ft) in the north and south of Warsaw. It goes through the city and plays an important role as a landmark.", "The Lower Rhine flows through North Rhine-Westphalia. Its banks are usually heavily populated and industrialized, in particular the agglomerations Cologne, Düsseldorf and Ruhr area. Here the Rhine flows through the largest conurbation in Germany, the Rhine-Ruhr region. One of the most important cities in this region is Duisburg with the largest river port in Europe (Duisport). The region downstream of Duisburg is more agricultural. In Wesel, 30 km downstream of Duisburg, is located the western end of the second east-west shipping route, the Wesel-Datteln Canal, which runs parallel to the Lippe. Between Emmerich and Cleves the Emmerich Rhine Bridge, the longest suspension bridge in Germany, crosses the 400 m wide river. Near Krefeld, the river crosses the Uerdingen line, the line which separates the areas where Low German and High German are spoken.", "The mouth of the Rhine into Lake Constance forms an inland delta. The delta is delimited in the West by the Alter Rhein (\"Old Rhine\") and in the East by a modern canalized section. Most of the delta is a nature reserve and bird sanctuary. It includes the Austrian towns of Gaißau, Höchst and Fußach. The natural Rhine originally branched into at least two arms and formed small islands by precipitating sediments. In the local Alemannic dialect, the singular is pronounced \"Isel\" and this is also the local pronunciation of Esel (\"Donkey\"). Many local fields have an official name containing this element."]</t>
-        </is>
-      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -4946,21 +3491,6 @@
 When B cells and T cells are activated and begin to replicate, some of their offspring become long-lived memory cells. Throughout the lifetime of an animal, these memory cells remember each specific pathogen encountered and can mount a strong response if the pathogen is detected again. This is "adaptive" because it occurs during the lifetime of an individual as an adaptation to infection with that pathogen and prepares the immune system for future challenges. Immunological memory can be in the form of either passive short-term memory or active long-term memory.</t>
         </is>
       </c>
-      <c r="F98" t="inlineStr">
-        <is>
-          <t>[96, 676, 350, 529, 548]</t>
-        </is>
-      </c>
-      <c r="G98" t="inlineStr">
-        <is>
-          <t>[0.8403216004371643, 0.8295778036117554, 0.7448256611824036, 0.7416180372238159, 0.7193408608436584]</t>
-        </is>
-      </c>
-      <c r="H98" t="inlineStr">
-        <is>
-          <t>["The main response of the immune system to tumors is to destroy the abnormal cells using killer T cells, sometimes with the assistance of helper T cells. Tumor antigens are presented on MHC class I molecules in a similar way to viral antigens. This allows killer T cells to recognize the tumor cell as abnormal. NK cells also kill tumorous cells in a similar way, especially if the tumor cells have fewer MHC class I molecules on their surface than normal; this is a common phenomenon with tumors. Sometimes antibodies are generated against tumor cells allowing for their destruction by the complement system.", "Clearly, some tumors evade the immune system and go on to become cancers. Tumor cells often have a reduced number of MHC class I molecules on their surface, thus avoiding detection by killer T cells. Some tumor cells also release products that inhibit the immune response; for example by secreting the cytokine TGF-β, which suppresses the activity of macrophages and lymphocytes. In addition, immunological tolerance may develop against tumor antigens, so the immune system no longer attacks the tumor cells.", "Neutrophils and macrophages are phagocytes that travel throughout the body in pursuit of invading pathogens. Neutrophils are normally found in the bloodstream and are the most abundant type of phagocyte, normally representing 50% to 60% of the total circulating leukocytes. During the acute phase of inflammation, particularly as a result of bacterial infection, neutrophils migrate toward the site of inflammation in a process called chemotaxis, and are usually the first cells to arrive at the scene of infection. Macrophages are versatile cells that reside within tissues and produce a wide array of chemicals including enzymes, complement proteins, and regulatory factors such as interleukin 1. Macrophages also act as scavengers, ridding the body of worn-out cells and other debris, and as antigen-presenting cells that activate the adaptive immune system.", "Overactive immune responses comprise the other end of immune dysfunction, particularly the autoimmune disorders. Here, the immune system fails to properly distinguish between self and non-self, and attacks part of the body. Under normal circumstances, many T cells and antibodies react with \"self\" peptides. One of the functions of specialized cells (located in the thymus and bone marrow) is to present young lymphocytes with self antigens produced throughout the body and to eliminate those cells that recognize self-antigens, preventing autoimmunity.", "When B cells and T cells are activated and begin to replicate, some of their offspring become long-lived memory cells. Throughout the lifetime of an animal, these memory cells remember each specific pathogen encountered and can mount a strong response if the pathogen is detected again. This is \"adaptive\" because it occurs during the lifetime of an individual as an adaptation to infection with that pathogen and prepares the immune system for future challenges. Immunological memory can be in the form of either passive short-term memory or active long-term memory."]</t>
-        </is>
-      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -4992,21 +3522,6 @@
 During the 1970s and sometimes later, Western and pro-Western governments often supported sometimes fledgling Islamists and Islamist groups that later came to be seen as dangerous enemies. Islamists were considered by Western governments bulwarks against—what were thought to be at the time—more dangerous leftist/communist/nationalist insurgents/opposition, which Islamists were correctly seen as opposing. The US spent billions of dollars to aid the mujahideen Muslim Afghanistan enemies of the Soviet Union, and non-Afghan veterans of the war returned home with their prestige, "experience, ideology, and weapons", and had considerable impact.</t>
         </is>
       </c>
-      <c r="F99" t="inlineStr">
-        <is>
-          <t>[97, 153, 751, 386, 23]</t>
-        </is>
-      </c>
-      <c r="G99" t="inlineStr">
-        <is>
-          <t>[0.810435950756073, 0.7721166014671326, 0.7680274248123169, 0.763443112373352, 0.761938214302063]</t>
-        </is>
-      </c>
-      <c r="H99" t="inlineStr">
-        <is>
-          <t>["\"The Islamic State\", formerly known as the \"Islamic State of Iraq and the Levant\" and before that as the \"Islamic State of Iraq\", (and called the acronym Daesh by its many detractors), is a Wahhabi/Salafi jihadist extremist militant group which is led by and mainly composed of Sunni Arabs from Iraq and Syria. In 2014, the group proclaimed itself a caliphate, with religious, political and military authority over all Muslims worldwide. As of March 2015[update], it had control over territory occupied by ten million people in Iraq and Syria, and has nominal control over small areas of Libya, Nigeria and Afghanistan. (While a self-described state, it lacks international recognition.) The group also operates or has affiliates in other parts of the world, including North Africa and South Asia.", "Islamism is a controversial concept not just because it posits a political role for Islam but also because its supporters believe their views merely reflect Islam, while the contrary idea that Islam is, or can be, apolitical is an error. Scholars and observers who do not believe that Islam is merely a political ideology include Fred Halliday, John Esposito and Muslim intellectuals like Javed Ahmad Ghamidi. Hayri Abaza argues the failure to distinguish between Islam and Islamism leads many in the West to support illiberal Islamic regimes, to the detriment of progressive moderates who seek to separate religion from politics.", "Sunni Muslim nation headed by a near absolutist monarchy. In the wake of the Iranian revolution the Saudis were forced to deal with the prospect of internal destabilization via the radicalism of Islamism, a reality which would quickly be revealed in the seizure of the Grand Mosque in Mecca by Wahhabi extremists during November 1979 and a Shiite revolt in the oil rich Al-Hasa region of Saudi Arabia in December of the same year. In November 2010, Wikileaks leaked confidential diplomatic cables pertaining to the United States and its allies which revealed that the late Saudi King Abdullah urged the United States to attack Iran in order to destroy its potential nuclear weapons program, describing Iran as \"a snake whose head should be cut off without any procrastination.\"", "The views of Ali Shariati, ideologue of the Iranian Revolution, had resemblance with Mohammad Iqbal, ideological father of the State of Pakistan, but Khomeini's beliefs is perceived to be placed somewhere between beliefs of Sunni Islamic thinkers like Mawdudi and Qutb. He believed that complete imitation of the Prophet Mohammad and his successors such as Ali for restoration of Sharia law was essential to Islam, that many secular, Westernizing Muslims were actually agents of the West serving Western interests, and that the acts such as \"plundering\" of Muslim lands was part of a long-term conspiracy against Islam by the Western governments.", "During the 1970s and sometimes later, Western and pro-Western governments often supported sometimes fledgling Islamists and Islamist groups that later came to be seen as dangerous enemies. Islamists were considered by Western governments bulwarks against—what were thought to be at the time—more dangerous leftist/communist/nationalist insurgents/opposition, which Islamists were correctly seen as opposing. The US spent billions of dollars to aid the mujahideen Muslim Afghanistan enemies of the Soviet Union, and non-Afghan veterans of the war returned home with their prestige, \"experience, ideology, and weapons\", and had considerable impact."]</t>
-        </is>
-      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -5038,21 +3553,6 @@
 The invasions of Baghdad, Samarkand, Urgench, Kiev, Vladimir among others caused mass murders, such as when portions of southern Khuzestan were completely destroyed. His descendant Hulagu Khan destroyed much of Iran's northern part and sacked Baghdad although his forces were halted by the Mamluks of Egypt, but Hulagu's descendant Ghazan Khan would return to beat the Egyptian Mamluks right out of Levant, Palestine and even Gaza. According to the works of the Persian historian Rashid-al-Din Hamadani, the Mongols killed more than 70,000 people in Merv and more than 190,000 in Nishapur. In 1237 Batu Khan, a grandson of Genghis Khan, launched an invasion into Kievan Rus'. Over the course of three years, the Mongols destroyed and annihilated all of the major cities of Eastern Europe with the exceptions of Novgorod and Pskov.</t>
         </is>
       </c>
-      <c r="F100" t="inlineStr">
-        <is>
-          <t>[98, 311, 552, 494, 2]</t>
-        </is>
-      </c>
-      <c r="G100" t="inlineStr">
-        <is>
-          <t>[0.7752463221549988, 0.7471147775650024, 0.7229059338569641, 0.7203985452651978, 0.7163239121437073]</t>
-        </is>
-      </c>
-      <c r="H100" t="inlineStr">
-        <is>
-          <t>["After al-Nimeiry was overthrown in 1985 the party did poorly in national elections, but in 1989 it was able to overthrow the elected post-al-Nimeiry government with the help of the military. Turabi was noted for proclaiming his support for the democratic process and a liberal government before coming to power, but strict application of sharia law, torture and mass imprisonment of the opposition, and an intensification of the long-running war in southern Sudan, once in power. The NIF regime also harbored Osama bin Laden for a time (before 9/11), and worked to unify Islamist opposition to the American attack on Iraq in the 1991 Gulf War.", "The next direct threat to Temüjin was the Naimans (Naiman Mongols), with whom Jamukha and his followers took refuge. The Naimans did not surrender, although enough sectors again voluntarily sided with Temüjin. In 1201, a khuruldai elected Jamukha as Gür Khan, \"universal ruler\", a title used by the rulers of the Qara Khitai. Jamukha's assumption of this title was the final breach with Temüjin, and Jamukha formed a coalition of tribes to oppose him. Before the conflict, however, several generals abandoned Jamukha, including Subutai, Jelme's well-known younger brother. After several battles, Jamukha was finally turned over to Temüjin by his own men in 1206.", "From the late 1340s onwards, people in the countryside suffered from frequent natural disasters such as droughts, floods and the resulting famines, and the government's lack of effective policy led to a loss of popular support. In 1351, the Red Turban Rebellion started and grew into a nationwide uprising. In 1354, when Toghtogha led a large army to crush the Red Turban rebels, Toghun Temür suddenly dismissed him for fear of betrayal. This resulted in Toghun Temür's restoration of power on the one hand and a rapid weakening of the central government on the other. He had no choice but to rely on local warlords' military power, and gradually lost his interest in politics and ceased to intervene in political struggles. He fled north to Shangdu from Khanbaliq (present-day Beijing) in 1368 after the approach of the forces of the Míng dynasty (1368–1644), founded by Zhu Yuanzhang in the south. He had tried to regain Khanbaliq, which eventually failed; he died in Yingchang (located in present-day Inner Mongolia) two years later (1370). Yingchang was seized by the Ming shortly after his death. Some royal family members still lived in Henan today.", "With such a small force, the invading Mongols were forced to change strategies and resort to inciting internal revolt among Kuchlug's supporters, leaving the Qara Khitai more vulnerable to Mongol conquest. As a result, Kuchlug's army was defeated west of Kashgar. Kuchlug fled again, but was soon hunted down by Jebe's army and executed. By 1218, as a result of defeat of Qara Khitai, the Mongol Empire and its control extended as far west as Lake Balkhash, which bordered the Khwarezmia (Khwarezmid Empire), a Muslim state that reached the Caspian Sea to the west and Persian Gulf and the Arabian Sea to the south.", "The invasions of Baghdad, Samarkand, Urgench, Kiev, Vladimir among others caused mass murders, such as when portions of southern Khuzestan were completely destroyed. His descendant Hulagu Khan destroyed much of Iran's northern part and sacked Baghdad although his forces were halted by the Mamluks of Egypt, but Hulagu's descendant Ghazan Khan would return to beat the Egyptian Mamluks right out of Levant, Palestine and even Gaza. According to the works of the Persian historian Rashid-al-Din Hamadani, the Mongols killed more than 70,000 people in Merv and more than 190,000 in Nishapur. In 1237 Batu Khan, a grandson of Genghis Khan, launched an invasion into Kievan Rus'. Over the course of three years, the Mongols destroyed and annihilated all of the major cities of Eastern Europe with the exceptions of Novgorod and Pskov."]</t>
-        </is>
-      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -5084,21 +3584,6 @@
 Many questions regarding prime numbers remain open, such as Goldbach's conjecture (that every even integer greater than 2 can be expressed as the sum of two primes), and the twin prime conjecture (that there are infinitely many pairs of primes whose difference is 2). Such questions spurred the development of various branches of number theory, focusing on analytic or algebraic aspects of numbers. Primes are used in several routines in information technology, such as public-key cryptography, which makes use of properties such as the difficulty of factoring large numbers into their prime factors. Prime numbers give rise to various generalizations in other mathematical domains, mainly algebra, such as prime elements and prime ideals.</t>
         </is>
       </c>
-      <c r="F101" t="inlineStr">
-        <is>
-          <t>[70, 99, 272, 405, 391]</t>
-        </is>
-      </c>
-      <c r="G101" t="inlineStr">
-        <is>
-          <t>[0.7964144349098206, 0.7960580587387085, 0.7890852689743042, 0.7684698104858398, 0.7637836933135986]</t>
-        </is>
-      </c>
-      <c r="H101" t="inlineStr">
-        <is>
-          <t>["The following table gives the largest known primes of the mentioned types. Some of these primes have been found using distributed computing. In 2009, the Great Internet Mersenne Prime Search project was awarded a US$100,000 prize for first discovering a prime with at least 10 million digits. The Electronic Frontier Foundation also offers $150,000 and $250,000 for primes with at least 100 million digits and 1 billion digits, respectively. Some of the largest primes not known to have any particular form (that is, no simple formula such as that of Mersenne primes) have been found by taking a piece of semi-random binary data, converting it to a number n, multiplying it by 256k for some positive integer k, and searching for possible primes within the interval [256kn + 1, 256k(n + 1) − 1].[citation needed]", "The most basic method of checking the primality of a given integer n is called trial division. This routine consists of dividing n by each integer m that is greater than 1 and less than or equal to the square root of n. If the result of any of these divisions is an integer, then n is not a prime, otherwise it is a prime. Indeed, if  is composite (with a and b ≠ 1) then one of the factors a or b is necessarily at most . For example, for , the trial divisions are by m = 2, 3, 4, 5, and 6. None of these numbers divides 37, so 37 is prime. This routine can be implemented more efficiently if a complete list of primes up to  is known—then trial divisions need to be checked only for those m that are prime. For example, to check the primality of 37, only three divisions are necessary (m = 2, 3, and 5), given that 4 and 6 are composite.", "After the Greeks, little happened with the study of prime numbers until the 17th century. In 1640 Pierre de Fermat stated (without proof) Fermat's little theorem (later proved by Leibniz and Euler). Fermat also conjectured that all numbers of the form 22n + 1 are prime (they are called Fermat numbers) and he verified this up to n = 4 (or 216 + 1). However, the very next Fermat number 232 + 1 is composite (one of its prime factors is 641), as Euler discovered later, and in fact no further Fermat numbers are known to be prime. The French monk Marin Mersenne looked at primes of the form 2p − 1, with p a prime. They are called Mersenne primes in his honor.", "can have infinitely many primes only when a and q are coprime, i.e., their greatest common divisor is one. If this necessary condition is satisfied, Dirichlet's theorem on arithmetic progressions asserts that the progression contains infinitely many primes. The picture below illustrates this with q = 9: the numbers are \"wrapped around\" as soon as a multiple of 9 is passed. Primes are highlighted in red. The rows (=progressions) starting with a = 3, 6, or 9 contain at most one prime number. In all other rows (a = 1, 2, 4, 5, 7, and 8) there are infinitely many prime numbers. What is more, the primes are distributed equally among those rows in the long run—the density of all primes congruent a modulo 9 is 1/6.", "Many questions regarding prime numbers remain open, such as Goldbach's conjecture (that every even integer greater than 2 can be expressed as the sum of two primes), and the twin prime conjecture (that there are infinitely many pairs of primes whose difference is 2). Such questions spurred the development of various branches of number theory, focusing on analytic or algebraic aspects of numbers. Primes are used in several routines in information technology, such as public-key cryptography, which makes use of properties such as the difficulty of factoring large numbers into their prime factors. Prime numbers give rise to various generalizations in other mathematical domains, mainly algebra, such as prime elements and prime ideals."]</t>
-        </is>
-      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -5130,21 +3615,6 @@
 In 1952, when the release of the FCC's Sixth Report and Order announced the end of its freeze on new station license applications, among the issues the Commission was slated to address was whether to approve the UPT-ABC merger. One FCC Commissioner saw the possibility of ABC, funded by UPT, becoming a viable and competitive third television network. On February 9, 1953, the FCC approved UPT's purchase of ABC in exchange for $25 million in shares. The merged company, renamed American Broadcasting-Paramount Theatres, Inc. and headquartered in the Paramount Building at 1501 Broadway in Manhattan, owned six AM and several FM radio stations, five television stations and 644 cinemas in 300 U.S. cities. To comply with FCC ownership restrictions in effect at the time that barred common ownership of two television stations in the same market, UPT sold its Chicago television station, WBKB-TV, to CBS (which subsequently changed the station's call letters to WBBM-TV) for $6 million, while it kept ABC's existing Chicago station, WENR-TV. The merged company acquired the WBKB call letters for channel 7, which would eventually become WLS-TV. Goldenson began to sell some of the older theaters to help finance the new television network.</t>
         </is>
       </c>
-      <c r="F102" t="inlineStr">
-        <is>
-          <t>[100, 585, 89, 382, 277]</t>
-        </is>
-      </c>
-      <c r="G102" t="inlineStr">
-        <is>
-          <t>[0.8322247266769409, 0.8072770833969116, 0.7805702090263367, 0.7805342078208923, 0.7763429284095764]</t>
-        </is>
-      </c>
-      <c r="H102" t="inlineStr">
-        <is>
-          <t>["The Sinclair Broadcast Group is the largest operator of ABC stations by numerical total, owning or providing services to 28 ABC affiliates and two additional subchannel-only affiliates; Sinclair owns the largest ABC subchannel affiliate by market size, WABM-DT2/WDBB-DT2 in the Birmingham market, which serve as repeaters of WBMA-LD (the largest low-power \"Big Four\" affiliate by market size, which itself is also simulcast on a subchannel of former WBMA satellite WGWW, owned by Sinclair partner company Howard Stirk Holdings). The E. W. Scripps Company is the largest operator of ABC stations in terms of overall market reach, owning 15 ABC-affiliated stations (including affiliates in larger markets such as Cleveland, Phoenix, Detroit and Denver), and through its ownership of Phoenix affiliate KNXV, Las Vegas affiliate KTNV-TV and Tucson affiliate KGUN-TV, the only provider of ABC programming for the majority of Arizona (outside of the Yuma-El Centro market) and Southern Nevada.", "Since its inception, ABC has had many affiliated stations, which include WABC-TV and WPVI-TV, the first two stations to carry the network's programming. As of March 2015[update], ABC has eight owned-and-operated stations, and current and pending affiliation agreements with 235 additional television stations encompassing 49 states, the District of Columbia, four U.S. possessions, Bermuda and Saba; this makes ABC the largest U.S. broadcast television network by total number of affiliates. The network has an estimated national reach of 96.26% of all households in the United States (or 300,794,157 Americans with at least one television set).", "It was not until the late 1950s that the ABC network became a serious contender to NBC and CBS, and this was in large part due to the diverse range of programming that met the expectations of the public, such as westerns and detective series. Despite an almost 500% increase in advertising revenues between 1953 and 1958, the network only had a national reach of between 10% and 18% of the total U.S. population, as it still had relatively fewer affiliates than NBC and CBS. In 1957, ABC Entertainment president Ollie Treiz discovered that the locally produced variety show Bandstand had pulled very strong ratings in the Philadelphia market on WFIL-TV; Treiz ultimately negotiated a deal to take the show national, under the revised title American Bandstand; the show quickly became a social phenomenon by presenting new musical talent and dances to America's youth and helped make a star out of its host, Dick Clark.", "On April 30, 2000, as a result of a carriage dispute with ABC, Time Warner Cable removed ABC owned-and-operated stations from the cable provider's systems in four markets (WABC-TV in New York City, KABC-TV in Los Angeles, KTRK in Houston and WTVD in Raleigh-Durham). The network had earlier reached an eleventh-hour deal to renew its carriage agreement with the provider on December 31, 1999. ABC filed an emergency petition to the Federal Communications Commission on May 1 to force TWC to restore the affected stations; the FCC ruled in favor of ABC, ordering Time Warner Cable to restore the stations, doing so on the afternoon of May 2. ABC ended the 2000–01 season as the most-watched network, ahead of NBC.", "In 1952, when the release of the FCC's Sixth Report and Order announced the end of its freeze on new station license applications, among the issues the Commission was slated to address was whether to approve the UPT-ABC merger. One FCC Commissioner saw the possibility of ABC, funded by UPT, becoming a viable and competitive third television network. On February 9, 1953, the FCC approved UPT's purchase of ABC in exchange for $25 million in shares. The merged company, renamed American Broadcasting-Paramount Theatres, Inc. and headquartered in the Paramount Building at 1501 Broadway in Manhattan, owned six AM and several FM radio stations, five television stations and 644 cinemas in 300 U.S. cities. To comply with FCC ownership restrictions in effect at the time that barred common ownership of two television stations in the same market, UPT sold its Chicago television station, WBKB-TV, to CBS (which subsequently changed the station's call letters to WBBM-TV) for $6 million, while it kept ABC's existing Chicago station, WENR-TV. The merged company acquired the WBKB call letters for channel 7, which would eventually become WLS-TV. Goldenson began to sell some of the older theaters to help finance the new television network."]</t>
-        </is>
-      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -5176,21 +3646,6 @@
 When finally Edward the Confessor returned from his father's refuge in 1041, at the invitation of his half-brother Harthacnut, he brought with him a Norman-educated mind. He also brought many Norman counsellors and fighters, some of whom established an English cavalry force. This concept never really took root, but it is a typical example of the attitudes of Edward. He appointed Robert of Jumièges archbishop of Canterbury and made Ralph the Timid earl of Hereford. He invited his brother-in-law Eustace II, Count of Boulogne to his court in 1051, an event which resulted in the greatest of early conflicts between Saxon and Norman and ultimately resulted in the exile of Earl Godwin of Wessex.</t>
         </is>
       </c>
-      <c r="F103" t="inlineStr">
-        <is>
-          <t>[101, 63, 842, 123, 573]</t>
-        </is>
-      </c>
-      <c r="G103" t="inlineStr">
-        <is>
-          <t>[0.8186925649642944, 0.7635119557380676, 0.7616726160049438, 0.75580894947052, 0.7516316175460815]</t>
-        </is>
-      </c>
-      <c r="H103" t="inlineStr">
-        <is>
-          <t>["The pattern of warfare, followed by brief periods of peace, continued for nearly another quarter-century. The warfare was definitively quelled in 1598, when Henry of Navarre, having succeeded to the French throne as Henry IV, and having recanted Protestantism in favour of Roman Catholicism, issued the Edict of Nantes. The Edict reaffirmed Catholicism as the state religion of France, but granted the Protestants equality with Catholics under the throne and a degree of religious and political freedom within their domains. The Edict simultaneously protected Catholic interests by discouraging the founding of new Protestant churches in Catholic-controlled regions.[citation needed]", "Despite the disagreements on the Eucharist, the Marburg Colloquy paved the way for the signing in 1530 of the Augsburg Confession, and for the formation of the Schmalkaldic League the following year by leading Protestant nobles such as John of Saxony, Philip of Hesse, and George, Margrave of Brandenburg-Ansbach. The Swiss cities, however, did not sign these agreements.", "Bethencourt took the title of King of the Canary Islands, as vassal to Henry III of Castile. In 1418, Jean's nephew Maciot de Bethencourt sold the rights to the islands to Enrique Pérez de Guzmán, 2nd Count de Niebla.", "Huguenot numbers peaked near an estimated two million by 1562, concentrated mainly in the southern and central parts of France, about one-eighth the number of French Catholics. As Huguenots gained influence and more openly displayed their faith, Catholic hostility grew, in spite of increasingly liberal political concessions and edicts of toleration from the French crown. A series of religious conflicts followed, known as the Wars of Religion, fought intermittently from 1562 to 1598. The wars finally ended with the granting of the Edict of Nantes, which granted the Huguenots substantial religious, political and military autonomy.", "When finally Edward the Confessor returned from his father's refuge in 1041, at the invitation of his half-brother Harthacnut, he brought with him a Norman-educated mind. He also brought many Norman counsellors and fighters, some of whom established an English cavalry force. This concept never really took root, but it is a typical example of the attitudes of Edward. He appointed Robert of Jumièges archbishop of Canterbury and made Ralph the Timid earl of Hereford. He invited his brother-in-law Eustace II, Count of Boulogne to his court in 1051, an event which resulted in the greatest of early conflicts between Saxon and Norman and ultimately resulted in the exile of Earl Godwin of Wessex."]</t>
-        </is>
-      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -5222,21 +3677,6 @@
 University of Chicago scholars have played a major role in the development of various academic disciplines, including: the Chicago school of economics, the Chicago school of sociology, the law and economics movement in legal analysis, the Chicago school of literary criticism, the Chicago school of religion, and the behavioralism school of political science. Chicago's physics department helped develop the world's first man-made, self-sustaining nuclear reaction beneath the university's Stagg Field. Chicago's research pursuits have been aided by unique affiliations with world-renowned institutions like the nearby Fermilab and Argonne National Laboratory, as well as the Marine Biological Laboratory. The university is also home to the University of Chicago Press, the largest university press in the United States. With an estimated completion date of 2020, the Barack Obama Presidential Center will be housed at the university and include both the Obama presidential library and offices of the Obama Foundation.</t>
         </is>
       </c>
-      <c r="F104" t="inlineStr">
-        <is>
-          <t>[290, 102, 437, 3, 442]</t>
-        </is>
-      </c>
-      <c r="G104" t="inlineStr">
-        <is>
-          <t>[0.7631736397743225, 0.7378835082054138, 0.7270313501358032, 0.719382107257843, 0.6829115748405457]</t>
-        </is>
-      </c>
-      <c r="H104" t="inlineStr">
-        <is>
-          <t>["Women remained segregated at Radcliffe, though more and more took Harvard classes. Nonetheless, Harvard's undergraduate population remained predominantly male, with about four men attending Harvard College for every woman studying at Radcliffe. Following the merger of Harvard and Radcliffe admissions in 1977, the proportion of female undergraduates steadily increased, mirroring a trend throughout higher education in the United States. Harvard's graduate schools, which had accepted females and other groups in greater numbers even before the college, also became more diverse in the post-World War II period.", "Harvard's 2,400 professors, lecturers, and instructors instruct 7,200 undergraduates and 14,000 graduate students. The school color is crimson, which is also the name of the Harvard sports teams and the daily newspaper, The Harvard Crimson. The color was unofficially adopted (in preference to magenta) by an 1875 vote of the student body, although the association with some form of red can be traced back to 1858, when Charles William Eliot, a young graduate student who would later become Harvard's 21st and longest-serving president (1869–1909), bought red bandanas for his crew so they could more easily be distinguished by spectators at a regatta.", "In the early 1950s, student applications declined as a result of increasing crime and poverty in the Hyde Park neighborhood. In response, the university became a major sponsor of a controversial urban renewal project for Hyde Park, which profoundly affected both the neighborhood's architecture and street plan. During this period the university, like Shimer College and 10 others, adopted an early entrant program that allowed very young students to attend college; in addition, students enrolled at Shimer were enabled to transfer automatically to the University of Chicago after their second year, having taken comparable or identical examinations and courses.", "The university runs a number of academic institutions and programs apart from its undergraduate and postgraduate schools. It operates the University of Chicago Laboratory Schools (a private day school for K-12 students and day care), the Sonia Shankman Orthogenic School (a residential treatment program for those with behavioral and emotional problems), and four public charter schools on the South Side of Chicago administered by the university's Urban Education Institute. In addition, the Hyde Park Day School, a school for students with learning disabilities, maintains a location on the University of Chicago campus. Since 1983, the University of Chicago has maintained the University of Chicago School Mathematics Project, a mathematics program used in urban primary and secondary schools. The university runs a program called the Council on Advanced Studies in the Social Sciences and Humanities, which administers interdisciplinary workshops to provide a forum for graduate students, faculty, and visiting scholars to present scholarly work in progress. The university also operates the University of Chicago Press, the largest university press in the United States.", "University of Chicago scholars have played a major role in the development of various academic disciplines, including: the Chicago school of economics, the Chicago school of sociology, the law and economics movement in legal analysis, the Chicago school of literary criticism, the Chicago school of religion, and the behavioralism school of political science. Chicago's physics department helped develop the world's first man-made, self-sustaining nuclear reaction beneath the university's Stagg Field. Chicago's research pursuits have been aided by unique affiliations with world-renowned institutions like the nearby Fermilab and Argonne National Laboratory, as well as the Marine Biological Laboratory. The university is also home to the University of Chicago Press, the largest university press in the United States. With an estimated completion date of 2020, the Barack Obama Presidential Center will be housed at the university and include both the Obama presidential library and offices of the Obama Foundation."]</t>
-        </is>
-      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -5268,21 +3708,6 @@
 The American Broadcasting Company (ABC) (stylized in its logo as abc since 1957) is an American commercial broadcast television network that is owned by the Disney–ABC Television Group, a subsidiary of Disney Media Networks division of The Walt Disney Company. The network is part of the Big Three television networks. The network is headquartered on Columbus Avenue and West 66th Street in Manhattan, with additional major offices and production facilities in New York City, Los Angeles and Burbank, California.</t>
         </is>
       </c>
-      <c r="F105" t="inlineStr">
-        <is>
-          <t>[103, 773, 462, 735, 732]</t>
-        </is>
-      </c>
-      <c r="G105" t="inlineStr">
-        <is>
-          <t>[0.8947772979736328, 0.8472180962562561, 0.8346245288848877, 0.8269910216331482, 0.8223757147789001]</t>
-        </is>
-      </c>
-      <c r="H105" t="inlineStr">
-        <is>
-          <t>["On July 31, 1995, The Walt Disney Company announced an agreement to merge with Capital Cities/ABC for $19 billion. Disney shareholders approved the merger at a special conference in New York City on January 4, 1996, with the acquisition of Capital Cities/ABC being completed on February 9; following the sale, Disney renamed its new subsidiary ABC Inc. In addition to the ABC network, the Disney acquisition integrated ABC's ten owned-and-operated television and 21 radio stations; its 80% interest in ESPN, ownership interests in The History Channel, A&amp;E Television Networks, and Lifetime Entertainment; and Capital Cities/ABC's magazine and newspaper properties into the company. As FCC ownership rules forbade the company from keeping both it and KABC-TV, Disney sold Los Angeles independent station KCAL-TV to Young Broadcasting for $387 million. On April 4, Disney sold the four newspapers that ABC had controlled under Capital Cities to Knight Ridder for $1.65 billion. Following the merger, Thomas S. Murphy left ABC with Robert Iger taking his place as president and CEO. Around the time of the merger, Disney's television production units had already produced series for the network such as Home Improvement and Boy Meets World, while the deal also allowed ABC access to", "In 1959, Walt Disney Productions, having improved its financial situation, had purchased ABC's shares in the Disneyland theme park for $7.5 million and initiated discussions to renew ABC's television contract for Walt Disney Presents, which was due to expire in 1961. Walt Disney was approached by NBC to produce color broadcasts of his anthology series (which would be renamed Walt Disney's Wonderful World of Color). Goldenson said ABC could not counter the offer, because the network did not have the technical and financial resources to carry the program in the format. As a result, ABC and Disney's first television collaboration ended in 1961 (the network would resume its relationship with Disney in 1985, when the anthology series returned to the network for a three-season run as the Disney Sunday Movie until it lost the rights to NBC again in 1988; the Disney anthology series would return to ABC in 1996, following the company's purchase of the future Capital Cities/ABC, as The Wonderful World of Disney).", "In 1968, ABC took advantage of new FCC ownership regulations that allowed broadcasting companies to own a maximum of seven radio stations nationwide in order to purchase Houston radio stations KXYZ and KXYZ-FM for $1 million in shares and $1.5 million in bonds. That year, Roone Arledge was named president of ABC Sports; the company also founded ABC Pictures, a film production company which released its first picture that year, the Ralph Nelson-directed Charly. It was renamed ABC Motion Pictures in 1979; the unit was dissolved in 1985. The studio also operated two subsidiaries, Palomar Pictures International and Selmur Pictures. In July 1968, ABC continued its acquisitions in the amusement parks sector with the opening of ABC Marine World in Redwood City, California; that park was sold in 1972 and demolished in 1986, with the land that occupied the park later becoming home to the headquarters of Oracle Corporation.", "Between May and September 2005, rumors circulated that Disney–ABC was considering a sale of ABC Radio, with Clear Channel Communications and Westwood One (which had earlier purchased NBC's radio division, as well as the distribution rights to CBS's, and the Mutual Broadcasting System during the 1990s) as potential buyers. On October 19, 2005, ABC announced the restructuring of the group into six divisions: Entertainment Communications, Communications Resources, Kids Communications, News Communications, Corporate Communications, and International Communications.", "The American Broadcasting Company (ABC) (stylized in its logo as abc since 1957) is an American commercial broadcast television network that is owned by the Disney–ABC Television Group, a subsidiary of Disney Media Networks division of The Walt Disney Company. The network is part of the Big Three television networks. The network is headquartered on Columbus Avenue and West 66th Street in Manhattan, with additional major offices and production facilities in New York City, Los Angeles and Burbank, California."]</t>
-        </is>
-      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -5314,21 +3739,6 @@
 Warsaw was occupied by Germany from 4 August 1915 until November 1918. The Allied Armistice terms required in Article 12 that Germany withdraw from areas controlled by Russia in 1914, which included Warsaw. Germany did so, and underground leader Piłsudski returned to Warsaw on 11 November and set up what became the Second Polish Republic, with Warsaw the capital. In the course of the Polish-Bolshevik War of 1920, the huge Battle of Warsaw was fought on the eastern outskirts of the city in which the capital was successfully defended and the Red Army defeated. Poland stopped by itself the full brunt of the Red Army and defeated an idea of the "export of the revolution".</t>
         </is>
       </c>
-      <c r="F106" t="inlineStr">
-        <is>
-          <t>[105, 26, 337, 35, 396]</t>
-        </is>
-      </c>
-      <c r="G106" t="inlineStr">
-        <is>
-          <t>[0.8556464910507202, 0.7878593802452087, 0.7804685831069946, 0.7740026116371155, 0.7646973133087158]</t>
-        </is>
-      </c>
-      <c r="H106" t="inlineStr">
-        <is>
-          <t>["Warsaw's name in the Polish language is Warszawa, approximately /vɑːrˈʃɑːvə/ (also formerly spelled Warszewa and Warszowa), meaning \"belonging to Warsz\", Warsz being a shortened form of the masculine name of Slavic origin Warcisław; see also etymology of Wrocław. Folk etymology attributes the city name to a fisherman, Wars, and his wife, Sawa. According to legend, Sawa was a mermaid living in the Vistula River with whom Wars fell in love. In actuality, Warsz was a 12th/13th-century nobleman who owned a village located at the modern-day site of Mariensztat neighbourhood. See also the Vršovci family which had escaped to Poland. The official city name in full is miasto stołeczne Warszawa (English: \"The Capital City of Warsaw\"). A native or resident of Warsaw is known as a Varsovian – in Polish warszawiak (male), warszawianka (female), warszawiacy (plural).", "In 1529, Warsaw for the first time became the seat of the General Sejm, permanent from 1569. In 1573 the city gave its name to the Warsaw Confederation, formally establishing religious freedom in the Polish–Lithuanian Commonwealth. Due to its central location between the Commonwealth's capitals of Kraków and Vilnius, Warsaw became the capital of the Commonwealth and the Crown of the Kingdom of Poland when King Sigismund III Vasa moved his court from Kraków to Warsaw in 1596. In the following years the town expanded towards the suburbs. Several private independent districts were established, the property of aristocrats and the gentry, which were ruled by their own laws. Three times between 1655–1658 the city was under siege and three times it was taken and pillaged by the Swedish, Brandenburgian and Transylvanian forces.", "Warsaw remained the capital of the Polish–Lithuanian Commonwealth until 1796, when it was annexed by the Kingdom of Prussia to become the capital of the province of South Prussia. Liberated by Napoleon's army in 1806, Warsaw was made the capital of the newly created Duchy of Warsaw. Following the Congress of Vienna of 1815, Warsaw became the centre of the Congress Poland, a constitutional monarchy under a personal union with Imperial Russia. The Royal University of Warsaw was established in 1816.", "In 2012 the Economist Intelligence Unit ranked Warsaw as the 32nd most liveable city in the world. It was also ranked as one of the most liveable cities in Central Europe. Today Warsaw is considered an \"Alpha–\" global city, a major international tourist destination and a significant cultural, political and economic hub. Warsaw's economy, by a wide variety of industries, is characterised by FMCG manufacturing, metal processing, steel and electronic manufacturing and food processing. The city is a significant centre of research and development, BPO, ITO, as well as of the Polish media industry. The Warsaw Stock Exchange is one of the largest and most important in Central and Eastern Europe. Frontex, the European Union agency for external border security, has its headquarters in Warsaw. It has been said that Warsaw, together with Frankfurt, London, Paris and Barcelona is one of the cities with the highest number of skyscrapers in the European Union. Warsaw has also been called \"Eastern Europe’s chic cultural capital with thriving art and club scenes and serious restaurants\".", "Warsaw was occupied by Germany from 4 August 1915 until November 1918. The Allied Armistice terms required in Article 12 that Germany withdraw from areas controlled by Russia in 1914, which included Warsaw. Germany did so, and underground leader Piłsudski returned to Warsaw on 11 November and set up what became the Second Polish Republic, with Warsaw the capital. In the course of the Polish-Bolshevik War of 1920, the huge Battle of Warsaw was fought on the eastern outskirts of the city in which the capital was successfully defended and the Red Army defeated. Poland stopped by itself the full brunt of the Red Army and defeated an idea of the \"export of the revolution\"."]</t>
-        </is>
-      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -5360,21 +3770,6 @@
 After the revocation of the Edict of Nantes, the Dutch Republic received the largest group of Huguenot refugees, an estimated total of 75,000 to 100,000 people. Amongst them were 200 clergy. Many came from the region of the Cévennes, for instance, the village of Fraissinet-de-Lozère. This was a huge influx as the entire population of the Dutch Republic amounted to ca. 2 million at that time. Around 1700, it is estimated that nearly 25% of the Amsterdam population was Huguenot.[citation needed] In 1705, Amsterdam and the area of West Frisia were the first areas to provide full citizens rights to Huguenot immigrants, followed by the Dutch Republic in 1715. Huguenots intermarried with Dutch from the outset.</t>
         </is>
       </c>
-      <c r="F107" t="inlineStr">
-        <is>
-          <t>[725, 106, 745, 525, 240]</t>
-        </is>
-      </c>
-      <c r="G107" t="inlineStr">
-        <is>
-          <t>[0.848737359046936, 0.8253918886184692, 0.8142426609992981, 0.7977233529090881, 0.797457218170166]</t>
-        </is>
-      </c>
-      <c r="H107" t="inlineStr">
-        <is>
-          <t>["Huguenot immigrants did not disperse or settle in different parts of the country, but rather, formed three societies or congregations; one in the city of New York, another 21 miles north of New York in a town which they named New Rochelle, and a third further upstate in New Paltz. The \"Huguenot Street Historic District\" in New Paltz has been designated a National Historic Landmark site and contains the oldest street in the United States of America. A small group of Huguenots also settled on the south shore of Staten Island along the New York Harbor, for which the current neighborhood of Huguenot was named.", "In the early years, many Huguenots also settled in the area of present-day Charleston, South Carolina. In 1685, Rev. Elie Prioleau from the town of Pons in France, was among the first to settle there. He became pastor of the first Huguenot church in North America in that city. After the Revocation of the Edict of Nantes in 1685, several Huguenot families of Norman and Carolingian nobility and descent, including Edmund Bohun of Suffolk England from the Humphrey de Bohun line of French royalty descended from Charlemagne, Jean Postell of Dieppe France, Alexander Pepin, Antoine Poitevin of Orsement France, and Jacques de Bordeaux of Grenoble, immigrated to the Charleston Orange district. They were very successful at marriage and property speculation. After petitioning the British Crown in 1697 for the right to own land in the Baronies, they prospered as slave owners on the Cooper, Ashepoo, Ashley and Santee River plantations they purchased from the British Landgrave Edmund Bellinger. Some of their descendants moved into the Deep South and Texas, where they developed new plantations.", "Barred by the government from settling in New France, Huguenots led by Jessé de Forest, sailed to North America in 1624 and settled instead in the Dutch colony of New Netherland (later incorporated into New York and New Jersey); as well as Great Britain's colonies, including Nova Scotia. A number of New Amsterdam's families were of Huguenot origin, often having emigrated as refugees to the Netherlands in the previous century. In 1628 the Huguenots established a congregation as L'Église française à la Nouvelle-Amsterdam (the French church in New Amsterdam). This parish continues today as L'Eglise du Saint-Esprit, part of the Episcopal (Anglican) communion, and welcomes Francophone New Yorkers from all over the world. Upon their arrival in New Amsterdam, Huguenots were offered land directly across from Manhattan on Long Island for a permanent settlement and chose the harbor at the end of Newtown Creek, becoming the first Europeans to live in Brooklyn, then known as Boschwick, in the neighborhood now known as Bushwick.", "A number of Huguenots served as mayors in Dublin, Cork, Youghal and Waterford in the 17th and 18th centuries. Numerous signs of Huguenot presence can still be seen with names still in use, and with areas of the main towns and cities named after the people who settled there. Examples include the Huguenot District and French Church Street in Cork City; and D'Olier Street in Dublin, named after a High Sheriff and one of the founders of the Bank of Ireland. A French church in Portarlington dates back to 1696, and was built to serve the significant new Huguenot community in the town. At the time, they constituted the majority of the townspeople.", "After the revocation of the Edict of Nantes, the Dutch Republic received the largest group of Huguenot refugees, an estimated total of 75,000 to 100,000 people. Amongst them were 200 clergy. Many came from the region of the Cévennes, for instance, the village of Fraissinet-de-Lozère. This was a huge influx as the entire population of the Dutch Republic amounted to ca. 2 million at that time. Around 1700, it is estimated that nearly 25% of the Amsterdam population was Huguenot.[citation needed] In 1705, Amsterdam and the area of West Frisia were the first areas to provide full citizens rights to Huguenot immigrants, followed by the Dutch Republic in 1715. Huguenots intermarried with Dutch from the outset."]</t>
-        </is>
-      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -5406,21 +3801,6 @@
 In The Church of Jesus Christ of Latter-day Saints (LDS Church), the teacher is an office in the Aaronic priesthood, generally conferred on young boys or recent converts, and has little in common with the "spiritual teacher" archetype. The role of "spiritual teacher" may be filled by many individuals in the LDS Church, often a trusted friend, who may hold any office, from Elder to Bishop, or no office at all. The emphasis on spiritual mentorship in the LDS Church is similar to that in the more "low-church" traditions of Protestantism, with a stronger emphasis placed on the husband and father of a family to provide spiritual guidance for all of his family, ideally in consultation with his wife, even if the husband is not a member of the LDS Church, based on interpretatios of certain Biblical texts which proclaim the spiritual authority of husbands in marriage. Even Priesthood representatives are expected to defer to the father of the house when in his home. Further, additional spiritual guidance is offered by those holding the office of Patriarch, which is supposed by Latter-day Saints to grant certain gifts of the Spirit, such as the ability to prophesy, to its holders. This</t>
         </is>
       </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>[338, 107, 683, 384, 860]</t>
-        </is>
-      </c>
-      <c r="G108" t="inlineStr">
-        <is>
-          <t>[0.8190984725952148, 0.8150198459625244, 0.7663912773132324, 0.7662370800971985, 0.7394217848777771]</t>
-        </is>
-      </c>
-      <c r="H108" t="inlineStr">
-        <is>
-          <t>["In education, teachers facilitate student learning, often in a school or academy or perhaps in another environment such as outdoors. A teacher who teaches on an individual basis may be described as a tutor.", "In some countries, formal education can take place through home schooling. Informal learning may be assisted by a teacher occupying a transient or ongoing role, such as a family member, or by anyone with knowledge or skills in the wider community setting.", "The objective is typically a course of study, lesson plan, or a practical skill. A teacher may follow standardized curricula as determined by the relevant authority. The teacher may interact with students of different ages, from infants to adults, students with different abilities and students with learning disabilities.", "The objective is typically accomplished through either an informal or formal approach to learning, including a course of study and lesson plan that teaches skills, knowledge and/or thinking skills. Different ways to teach are often referred to as pedagogy. When deciding what teaching method to use teachers consider students' background knowledge, environment, and their learning goals as well as standardized curricula as determined by the relevant authority. Many times, teachers assist in learning outside of the classroom by accompanying students on field trips. The increasing use of technology, specifically the rise of the internet over the past decade, has begun to shape the way teachers approach their roles in the classroom.", "In The Church of Jesus Christ of Latter-day Saints (LDS Church), the teacher is an office in the Aaronic priesthood, generally conferred on young boys or recent converts, and has little in common with the \"spiritual teacher\" archetype. The role of \"spiritual teacher\" may be filled by many individuals in the LDS Church, often a trusted friend, who may hold any office, from Elder to Bishop, or no office at all. The emphasis on spiritual mentorship in the LDS Church is similar to that in the more \"low-church\" traditions of Protestantism, with a stronger emphasis placed on the husband and father of a family to provide spiritual guidance for all of his family, ideally in consultation with his wife, even if the husband is not a member of the LDS Church, based on interpretatios of certain Biblical texts which proclaim the spiritual authority of husbands in marriage. Even Priesthood representatives are expected to defer to the father of the house when in his home. Further, additional spiritual guidance is offered by those holding the office of Patriarch, which is supposed by Latter-day Saints to grant certain gifts of the Spirit, such as the ability to prophesy, to its holders. This"]</t>
-        </is>
-      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -5452,21 +3832,6 @@
 wages due to the nature of the job, since there is a relative shortage of workers for the particular position. Professional and labor organizations may limit the supply of workers which results in higher demand and greater incomes for members. Members may also receive higher wages through collective bargaining, political influence, or corruption.</t>
         </is>
       </c>
-      <c r="F109" t="inlineStr">
-        <is>
-          <t>[93, 243, 743, 482, 407]</t>
-        </is>
-      </c>
-      <c r="G109" t="inlineStr">
-        <is>
-          <t>[0.8985971808433533, 0.8031179904937744, 0.7807430624961853, 0.7797146439552307, 0.7782220840454102]</t>
-        </is>
-      </c>
-      <c r="H109" t="inlineStr">
-        <is>
-          <t>["During the mass high school education movement from 1910–1940, there was an increase in skilled workers, which led to a decrease in the price of skilled labor. High school education during the period was designed to equip students with necessary skill sets to be able to perform at work. In fact, it differs from the present high school education, which is regarded as a stepping-stone to acquire college and advanced degrees. This decrease in wages caused a period of compression and decreased inequality between skilled and unskilled workers. Education is very important for the growth of the economy, however educational inequality in gender also influence towards the economy. Lagerlof and Galor stated that gender inequality in education can result to low economic growth, and continued gender inequality in education, thus creating a poverty trap. It is suggested that a large gap in male and female education may indicate backwardness and so may be associated with lower economic growth, which can explain why there is economic inequality between countries.", "An important factor in the creation of inequality is variation in individuals' access to education. Education, especially in an area where there is a high demand for workers, creates high wages for those with this education, however, increases in education first increase and then decrease growth as well as income inequality. As a result, those who are unable to afford an education, or choose not to pursue optional education, generally receive much lower wages. The justification for this is that a lack of education leads directly to lower incomes, and thus lower aggregate savings and investment. Conversely, education raises incomes and promotes growth because it helps to unleash the productive potential of the poor.", "In 2014, economists with the Standard &amp; Poor's rating agency concluded that the widening disparity between the U.S.'s wealthiest citizens and the rest of the nation had slowed its recovery from the 2008-2009 recession and made it more prone to boom-and-bust cycles. To partially remedy the wealth gap and the resulting slow growth, S&amp;P recommended increasing access to education. It estimated that if the average United States worker had completed just one more year of school, it would add an additional $105 billion in growth to the country's economy over five years.", "Sociologist Jake Rosenfield of the University of Washington asserts that the decline of organized labor in the United States has played a more significant role in expanding the income gap than technological changes and globalization, which were also experienced by other industrialized nations that didn't experience steep surges in inequality. He points out that nations with high rates of unionization, particularly in Scandinavia, have very low levels of inequality, and concludes \"the historical pattern is clear; the cross-national pattern is clear: high inequality goes hand-in-hand with weak labor movements and vice-versa.\"", "wages due to the nature of the job, since there is a relative shortage of workers for the particular position. Professional and labor organizations may limit the supply of workers which results in higher demand and greater incomes for members. Members may also receive higher wages through collective bargaining, political influence, or corruption."]</t>
-        </is>
-      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -5498,21 +3863,6 @@
 During the 1970s and sometimes later, Western and pro-Western governments often supported sometimes fledgling Islamists and Islamist groups that later came to be seen as dangerous enemies. Islamists were considered by Western governments bulwarks against—what were thought to be at the time—more dangerous leftist/communist/nationalist insurgents/opposition, which Islamists were correctly seen as opposing. The US spent billions of dollars to aid the mujahideen Muslim Afghanistan enemies of the Soviet Union, and non-Afghan veterans of the war returned home with their prestige, "experience, ideology, and weapons", and had considerable impact.</t>
         </is>
       </c>
-      <c r="F110" t="inlineStr">
-        <is>
-          <t>[108, 760, 182, 255, 23]</t>
-        </is>
-      </c>
-      <c r="G110" t="inlineStr">
-        <is>
-          <t>[0.781732439994812, 0.7626890540122986, 0.7566120028495789, 0.7501788139343262, 0.7418280839920044]</t>
-        </is>
-      </c>
-      <c r="H110" t="inlineStr">
-        <is>
-          <t>["Some elements of the Brotherhood, though perhaps against orders, did engage in violence against the government, and its founder Al-Banna was assassinated in 1949 in retaliation for the assassination of Egypt's premier Mahmud Fami Naqrashi three months earlier. The Brotherhood has suffered periodic repression in Egypt and has been banned several times, in 1948 and several years later following confrontations with Egyptian president Gamal Abdul Nasser, who jailed thousands of members for several years.", "Some forms of civil disobedience, such as illegal boycotts, refusals to pay taxes, draft dodging, distributed denial-of-service attacks, and sit-ins, make it more difficult for a system to function. In this way, they might be considered coercive. Brownlee notes that \"although civil disobedients are constrained in their use of coercion by their conscientious aim to engage in moral dialogue, nevertheless they may find it necessary to employ limited coercion in order to get their issue onto the table.\" The Plowshares organization temporarily closed GCSB Waihopai by padlocking the gates and using sickles to deflate one of the large domes covering two satellite dishes.", "Civil disobedients have chosen a variety of different illegal acts. Bedau writes, \"There is a whole class of acts, undertaken in the name of civil disobedience, which, even if they were widely practiced, would in themselves constitute hardly more than a nuisance (e.g. trespassing at a nuclear-missile installation)...Such acts are often just a harassment and, at least to the bystander, somewhat inane...The remoteness of the connection between the disobedient act and the objectionable law lays such acts open to the charge of ineffectiveness and absurdity.\" Bedau also notes, though, that the very harmlessness of such entirely symbolic illegal protests toward public policy goals may serve a propaganda purpose. Some civil disobedients, such as the proprietors of illegal medical cannabis dispensaries and Voice in the Wilderness, which brought medicine to Iraq without the permission of the U.S. Government, directly achieve a desired social goal (such as the provision of medication to the sick) while openly breaking the law. Julia Butterfly Hill lived in Luna, a 180-foot (55 m)-tall, 600-year-old California Redwood tree for 738 days, successfully preventing it from being cut down.", "Another of the Egyptian groups which employed violence in their struggle for Islamic order was al-Gama'a al-Islamiyya (Islamic Group). Victims of their campaign against the Egyptian state in the 1990s included the head of the counter-terrorism police (Major General Raouf Khayrat), a parliamentary speaker (Rifaat al-Mahgoub), dozens of European tourists and Egyptian bystanders, and over 100 Egyptian police. Ultimately the campaign to overthrow the government was unsuccessful, and the major jihadi group, Jamaa Islamiya (or al-Gama'a al-Islamiyya), renounced violence in 2003. Other lesser known groups include the Islamic Liberation Party, Salvation from Hell and Takfir wal-Hijra, and these groups have variously been involved in activities such as attempted assassinations of political figures, arson of video shops and attempted takeovers of government buildings.", "During the 1970s and sometimes later, Western and pro-Western governments often supported sometimes fledgling Islamists and Islamist groups that later came to be seen as dangerous enemies. Islamists were considered by Western governments bulwarks against—what were thought to be at the time—more dangerous leftist/communist/nationalist insurgents/opposition, which Islamists were correctly seen as opposing. The US spent billions of dollars to aid the mujahideen Muslim Afghanistan enemies of the Soviet Union, and non-Afghan veterans of the war returned home with their prestige, \"experience, ideology, and weapons\", and had considerable impact."]</t>
-        </is>
-      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -5544,21 +3894,6 @@
 The Upper Rhine region was changed significantly by a Rhine straightening program in the 19th Century. The rate of flow was increased and the ground water level fell significantly. Dead branches dried up and the amount of forests on the flood plains decreased sharply. On the French side, the Grand Canal d'Alsace was dug, which carries a significant part of the river water, and all of the traffic. In some places, there are large compensation pools, for example the huge Bassin de compensation de Plobsheim in Alsace.</t>
         </is>
       </c>
-      <c r="F111" t="inlineStr">
-        <is>
-          <t>[109, 43, 747, 68, 345]</t>
-        </is>
-      </c>
-      <c r="G111" t="inlineStr">
-        <is>
-          <t>[0.8245474696159363, 0.7722309827804565, 0.7718028426170349, 0.7704314589500427, 0.7622818350791931]</t>
-        </is>
-      </c>
-      <c r="H111" t="inlineStr">
-        <is>
-          <t>["A regulation of the Rhine was called for, with an upper canal near Diepoldsau and a lower canal at Fußach, in order to counteract the constant flooding and strong sedimentation in the western Rhine Delta. The Dornbirner Ach had to be diverted, too, and it now flows parallel to the canalized Rhine into the lake. Its water has a darker color than the Rhine; the latter's lighter suspended load comes from higher up the mountains. It is expected that the continuous input of sediment into the lake will silt up the lake. This has already happened to the former Lake Tuggenersee.", "At the begin of the Holocene (~11,700 years ago), the Rhine occupied its Late-Glacial valley. As a meandering river, it reworked its ice-age braidplain. As sea-level continued to rise in the Netherlands, the formation of the Holocene Rhine-Meuse delta began (~8,000 years ago). Coeval absolute sea-level rise and tectonic subsidence have strongly influenced delta evolution. Other factors of importance to the shape of the delta are the local tectonic activities of the Peel Boundary Fault, the substrate and geomorphology, as inherited from the Last Glacial and the coastal-marine dynamics, such as barrier and tidal inlet formations.", "The mouth of the Rhine into Lake Constance forms an inland delta. The delta is delimited in the West by the Alter Rhein (\"Old Rhine\") and in the East by a modern canalized section. Most of the delta is a nature reserve and bird sanctuary. It includes the Austrian towns of Gaißau, Höchst and Fußach. The natural Rhine originally branched into at least two arms and formed small islands by precipitating sediments. In the local Alemannic dialect, the singular is pronounced \"Isel\" and this is also the local pronunciation of Esel (\"Donkey\"). Many local fields have an official name containing this element.", "The hydrography of the current delta is characterized by the delta's main arms, disconnected arms (Hollandse IJssel, Linge, Vecht, etc.) and smaller rivers and streams. Many rivers have been closed (\"dammed\") and now serve as drainage channels for the numerous polders. The construction of Delta Works changed the Delta in the second half of the 20th Century fundamentally. Currently Rhine water runs into the sea, or into former marine bays now separated from the sea, in five places, namely at the mouths of the Nieuwe Merwede, Nieuwe Waterway (Nieuwe Maas), Dordtse Kil, Spui and IJssel.", "The Upper Rhine region was changed significantly by a Rhine straightening program in the 19th Century. The rate of flow was increased and the ground water level fell significantly. Dead branches dried up and the amount of forests on the flood plains decreased sharply. On the French side, the Grand Canal d'Alsace was dug, which carries a significant part of the river water, and all of the traffic. In some places, there are large compensation pools, for example the huge Bassin de compensation de Plobsheim in Alsace."]</t>
-        </is>
-      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -5590,21 +3925,6 @@
 The most frequent musical contributor during the first 15 years was Dudley Simpson, who is also well known for his theme and incidental music for Blake's 7, and for his haunting theme music and score for the original 1970s version of The Tomorrow People. Simpson's first Doctor Who score was Planet of Giants (1964) and he went on to write music for many adventures of the 1960s and 1970s, including most of the stories of the Jon Pertwee/Tom Baker periods, ending with The Horns of Nimon (1979). He also made a cameo appearance in The Talons of Weng-Chiang (as a Music hall conductor).</t>
         </is>
       </c>
-      <c r="F112" t="inlineStr">
-        <is>
-          <t>[110, 36, 776, 37, 665]</t>
-        </is>
-      </c>
-      <c r="G112" t="inlineStr">
-        <is>
-          <t>[0.8280532360076904, 0.8032209873199463, 0.8021425604820251, 0.7926058173179626, 0.7787353992462158]</t>
-        </is>
-      </c>
-      <c r="H112" t="inlineStr">
-        <is>
-          <t>["A new arrangement of the theme, once again by Gold, was introduced in the 2007 Christmas special episode, \"Voyage of the Damned\"; Gold returned as composer for the 2010 series. He was responsible for a new version of the theme which was reported to have had a hostile reception from some viewers. In 2011, the theme tune charted at number 228 of radio station Classic FM's Hall of Fame, a survey of classical music tastes. A revised version of Gold's 2010 arrangement had its debut over the opening titles of the 2012 Christmas special \"The Snowmen\", and a further revision of the arrangement was made for the 50th Anniversary special \"The Day of the Doctor\" in November 2013.[citation needed]", "In 1998, the network began using a minimalist graphical identity, designed by Pittard Sullivan, featuring a small black-and-white \"ABC Circle\" logo on a yellow background (promotions during this time also featured a sequence of still photos of the stars of its programs during the timeslot card as well as the schedule sequence that began each night's prime time lineup). A new four-note theme tune was introduced alongside the package, based around the network's \"We Love TV\" image campaign introduced that year, creating an audio signature on par with the NBC chimes, CBS' various three-note soundmarks (including the current version used since 2000) and the Fox Fanfare. The four-note signature has been updated with every television season thereafter (though variants of it used since the 1998–99 season remain in use during the production company vanity cards shown following the closing credits of most programs). In the fall of 2015, ABC is stopped with its 1998–2002 four-note jingles for promotions and production company vanity cards following the closing credits of most of its programs over seventeen years, now it have a different and adventure-type music (with the drums of the network's four-note signature in the ending). The old four-note theme tune is", "as a selection of classics based on the theme of space and time. The event was presented by Freema Agyeman and guest-presented by various other stars of the show with numerous monsters participating in the proceedings. It also featured the specially filmed mini-episode \"Music of the Spheres\", written by Russell T Davies and starring David Tennant.", "stopped with its 1998–2002 four-note jingles for promotions and production company vanity cards following the closing credits of most of its programs over seventeen years, now it have a different and adventure-type music (with the drums of the network's four-note signature in the ending). The old four-note theme tune is still used by ABC on Demand to the beginning of the ABC show.", "The most frequent musical contributor during the first 15 years was Dudley Simpson, who is also well known for his theme and incidental music for Blake's 7, and for his haunting theme music and score for the original 1970s version of The Tomorrow People. Simpson's first Doctor Who score was Planet of Giants (1964) and he went on to write music for many adventures of the 1960s and 1970s, including most of the stories of the Jon Pertwee/Tom Baker periods, ending with The Horns of Nimon (1979). He also made a cameo appearance in The Talons of Weng-Chiang (as a Music hall conductor)."]</t>
-        </is>
-      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -5636,21 +3956,6 @@
 Michael Oppenheimer, a long-time participant in the IPCC and coordinating lead author of the Fifth Assessment Report conceded in Science Magazine's State of the Planet 2008-2009 some limitations of the IPCC consensus approach and asks for concurring, smaller assessments of special problems instead of the large scale approach as in the previous IPCC assessment reports. It has become more important to provide a broader exploration of uncertainties. Others see as well mixed blessings of the drive for consensus within the IPCC process and ask to include dissenting or minority positions or to improve statements about uncertainties.</t>
         </is>
       </c>
-      <c r="F113" t="inlineStr">
-        <is>
-          <t>[664, 730, 827, 390, 414]</t>
-        </is>
-      </c>
-      <c r="G113" t="inlineStr">
-        <is>
-          <t>[0.7341638207435608, 0.711736261844635, 0.7106855511665344, 0.7053391337394714, 0.7026218771934509]</t>
-        </is>
-      </c>
-      <c r="H113" t="inlineStr">
-        <is>
-          <t>["The 1970s and 1980s saw the emergence of many graphical imaging packages for the network in which based the logo's setting mainly on special lighting effects then under development including white, blue, pink, rainbow neon and glittering dotted lines. Among the \"ABC Circle\" logo's many variants was a 1977 ID sequence that featured a bubble on a black background representing the circle with glossy gold letters, and as such, was the first ABC identification card to have a three-dimensional appearance.", "In general, there are three sectors of construction: buildings, infrastructure and industrial. Building construction is usually further divided into residential and non-residential (commercial/institutional). Infrastructure is often called heavy/highway, heavy civil or heavy engineering. It includes large public works, dams, bridges, highways, water/wastewater and utility distribution. Industrial includes refineries, process chemical, power generation, mills and manufacturing plants. There are other ways to break the industry into sectors or markets.", "United States and Western Europe than in China (due to a greater tendency to take on debts).[unreliable source?][unreliable source?] Anthony Shorrocks, the lead author of the Credit Suisse report which is one of the sources of Oxfam's data, considers the criticism about debt to be a \"silly argument\" and \"a non-issue . . . a diversion.\"", "less than 700 preparations, their properties, modes of action, and their indications. He devoted in fact a whole volume to simple drugs in The Canon of Medicine. Of great impact were also the works by al-Maridini of Baghdad and Cairo, and Ibn al-Wafid (1008–1074), both of which were printed in Latin more than fifty times, appearing as De Medicinis universalibus et particularibus by 'Mesue' the younger, and the Medicamentis simplicibus by 'Abenguefit'. Peter of Abano (1250–1316) translated and added a supplement to the work of al-Maridini under the title De Veneris. Al-Muwaffaq’s contributions in the field are also pioneering. Living in the 10th century, he wrote The foundations of the true properties of Remedies, amongst others describing arsenious oxide, and being acquainted with silicic acid. He made clear distinction between sodium carbonate and potassium carbonate, and drew attention to the poisonous nature of copper compounds, especially copper vitriol, and also lead compounds. He also describes the distillation of sea-water for drinking.[verification needed]", "Michael Oppenheimer, a long-time participant in the IPCC and coordinating lead author of the Fifth Assessment Report conceded in Science Magazine's State of the Planet 2008-2009 some limitations of the IPCC consensus approach and asks for concurring, smaller assessments of special problems instead of the large scale approach as in the previous IPCC assessment reports. It has become more important to provide a broader exploration of uncertainties. Others see as well mixed blessings of the drive for consensus within the IPCC process and ask to include dissenting or minority positions or to improve statements about uncertainties."]</t>
-        </is>
-      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -5682,21 +3987,6 @@
 The Dalek race, which first appeared in the show's second serial in 1963, are Doctor Who's oldest villains. The Daleks are Kaleds from the planet Skaro, mutated by the scientist Davros and housed in mechanical armour shells for mobility. The actual creatures resemble octopi with large, pronounced brains. Their armour shells have a single eye-stalk, a sink-plunger-like device that serves the purpose of a hand, and a directed-energy weapon. Their main weakness is their eyestalk; attacks upon them using various weapons can blind a Dalek, making it go mad. Their chief role in the series plot, as they frequently remark in their instantly recognisable metallic voices, is to "exterminate" all non-Dalek beings. They even attack the Time Lords in the Time War, as shown during the 50th Anniversary of the show. They continue to be a recurring 'monster' within the Doctor Who franchise, their most recent appearances being in the 2015 episodes "The Witch's Familiar" and "Hell Bent". Davros has also been a recurring figure since his debut in Genesis of the Daleks, although played by several different actors.</t>
         </is>
       </c>
-      <c r="F114" t="inlineStr">
-        <is>
-          <t>[112, 20, 184, 185, 748]</t>
-        </is>
-      </c>
-      <c r="G114" t="inlineStr">
-        <is>
-          <t>[0.8268134593963623, 0.817301332950592, 0.7930781245231628, 0.7913696765899658, 0.7839435935020447]</t>
-        </is>
-      </c>
-      <c r="H114" t="inlineStr">
-        <is>
-          <t>["Doctor Who originally ran for 26 seasons on BBC One, from 23 November 1963 until 6 December 1989. During the original run, each weekly episode formed part of a story (or \"serial\") — usually of four to six parts in earlier years and three to four in later years. Notable exceptions were: The Daleks' Master Plan, which aired in 12 episodes (plus an earlier one-episode teaser, \"Mission to the Unknown\", featuring none of the regular cast); almost an entire season of seven-episode serials (season 7); the 10-episode serial The War Games; and The Trial of a Time Lord, which ran for 14 episodes (albeit divided into three production codes and four narrative segments) during season 23. Occasionally serials were loosely connected by a storyline, such as season 8 being devoted to the Doctor battling a rogue Time Lord called The Master, season 16's quest for The Key to Time, season 18's journey through E-Space and the theme of entropy, and season 20's Black Guardian Trilogy.", "With the show's 2005 revival, executive producer Russell T Davies stated his intention to reintroduce classic icons of Doctor Who one step at a time: the Autons with the Nestene Consciousness and Daleks in series 1, Cybermen in series 2, the Macra and the Master in series 3, the Sontarans and Davros in series 4, and the Time Lords (Rassilon) in the 2009–10 Specials. Davies' successor, Steven Moffat, has continued the trend by reviving the Silurians in series 5, Cybermats in series 6, the Great Intelligence and the Ice Warriors in Series 7, and Zygons in the 50th Anniversary Special. Since its 2005 return, the series has also introduced new recurring aliens: Slitheen (Raxacoricofallapatorian), Ood, Judoon, Weeping Angels and the Silence.", "Following the success of the 2005 series produced by Russell T Davies, the BBC commissioned Davies to produce a 13-part spin-off series titled Torchwood (an anagram of \"Doctor Who\"), set in modern-day Cardiff and investigating alien activities and crime. The series debuted on BBC Three on 22 October 2006. John Barrowman reprised his role of Jack Harkness from the 2005 series of Doctor Who. Two other actresses who appeared in Doctor Who also star in the series; Eve Myles as Gwen Cooper, who also played the similarly named servant girl Gwyneth in the 2005 Doctor Who episode \"The Unquiet Dead\", and Naoko Mori who reprised her role as Toshiko Sato first seen in \"Aliens of London\". A second series of Torchwood aired in 2008; for three episodes, the cast was joined by Freema Agyeman reprising her Doctor Who role of Martha Jones. A third series was broadcast from 6 to 10 July 2009, and consisted of a single five-part story called Children of Earth which was set largely in London. A fourth series, Torchwood: Miracle Day jointly produced by BBC Wales, BBC Worldwide and the American entertainment company Starz debuted in 2011. The series was predominantly set in the United", "10 July 2009, and consisted of a single five-part story called Children of Earth which was set largely in London. A fourth series, Torchwood: Miracle Day jointly produced by BBC Wales, BBC Worldwide and the American entertainment company Starz debuted in 2011. The series was predominantly set in the United States, though Wales remained part of the show's setting.", "The Dalek race, which first appeared in the show's second serial in 1963, are Doctor Who's oldest villains. The Daleks are Kaleds from the planet Skaro, mutated by the scientist Davros and housed in mechanical armour shells for mobility. The actual creatures resemble octopi with large, pronounced brains. Their armour shells have a single eye-stalk, a sink-plunger-like device that serves the purpose of a hand, and a directed-energy weapon. Their main weakness is their eyestalk; attacks upon them using various weapons can blind a Dalek, making it go mad. Their chief role in the series plot, as they frequently remark in their instantly recognisable metallic voices, is to \"exterminate\" all non-Dalek beings. They even attack the Time Lords in the Time War, as shown during the 50th Anniversary of the show. They continue to be a recurring 'monster' within the Doctor Who franchise, their most recent appearances being in the 2015 episodes \"The Witch's Familiar\" and \"Hell Bent\". Davros has also been a recurring figure since his debut in Genesis of the Daleks, although played by several different actors."]</t>
-        </is>
-      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -5728,21 +4018,6 @@
 In the late 17th century, Robert Boyle proved that air is necessary for combustion. English chemist John Mayow (1641–1679) refined this work by showing that fire requires only a part of air that he called spiritus nitroaereus or just nitroaereus. In one experiment he found that placing either a mouse or a lit candle in a closed container over water caused the water to rise and replace one-fourteenth of the air's volume before extinguishing the subjects. From this he surmised that nitroaereus is consumed in both respiration and combustion.</t>
         </is>
       </c>
-      <c r="F115" t="inlineStr">
-        <is>
-          <t>[827, 109, 664, 831, 428]</t>
-        </is>
-      </c>
-      <c r="G115" t="inlineStr">
-        <is>
-          <t>[0.7218897342681885, 0.7214215993881226, 0.7175269722938538, 0.7089757919311523, 0.7085909843444824]</t>
-        </is>
-      </c>
-      <c r="H115" t="inlineStr">
-        <is>
-          <t>["United States and Western Europe than in China (due to a greater tendency to take on debts).[unreliable source?][unreliable source?] Anthony Shorrocks, the lead author of the Credit Suisse report which is one of the sources of Oxfam's data, considers the criticism about debt to be a \"silly argument\" and \"a non-issue . . . a diversion.\"", "A regulation of the Rhine was called for, with an upper canal near Diepoldsau and a lower canal at Fußach, in order to counteract the constant flooding and strong sedimentation in the western Rhine Delta. The Dornbirner Ach had to be diverted, too, and it now flows parallel to the canalized Rhine into the lake. Its water has a darker color than the Rhine; the latter's lighter suspended load comes from higher up the mountains. It is expected that the continuous input of sediment into the lake will silt up the lake. This has already happened to the former Lake Tuggenersee.", "The 1970s and 1980s saw the emergence of many graphical imaging packages for the network in which based the logo's setting mainly on special lighting effects then under development including white, blue, pink, rainbow neon and glittering dotted lines. Among the \"ABC Circle\" logo's many variants was a 1977 ID sequence that featured a bubble on a black background representing the circle with glossy gold letters, and as such, was the first ABC identification card to have a three-dimensional appearance.", "Since 7500 yr ago, a situation with tides and currents, very similar to present has existed. Rates of sea-level rise had dropped so far, that natural sedimentation by the Rhine and coastal processes together, could compensate the transgression by the sea; in the last 7000 years, the coast line was roughly at the same location. In the southern North Sea, due to ongoing tectonic subsidence, the sea level is still rising, at the rate of about 1–3 cm (0.39–1.18 in) per century (1 metre or 39 inches in last 3000 years).", "In the late 17th century, Robert Boyle proved that air is necessary for combustion. English chemist John Mayow (1641–1679) refined this work by showing that fire requires only a part of air that he called spiritus nitroaereus or just nitroaereus. In one experiment he found that placing either a mouse or a lit candle in a closed container over water caused the water to rise and replace one-fourteenth of the air's volume before extinguishing the subjects. From this he surmised that nitroaereus is consumed in both respiration and combustion."]</t>
-        </is>
-      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -5774,21 +4049,6 @@
 seen as an affront and insult to Genghis Khan. Outraged, Genghis Khan planned one of his largest invasion campaigns by organizing together around 100,000 soldiers (10 tumens), his most capable generals and some of his sons. He left a commander and number of troops in China, designated his successors to be his family members and likely appointed Ögedei to be his immediate successor and then went out to Khwarezmia.</t>
         </is>
       </c>
-      <c r="F116" t="inlineStr">
-        <is>
-          <t>[114, 80, 494, 803, 45]</t>
-        </is>
-      </c>
-      <c r="G116" t="inlineStr">
-        <is>
-          <t>[0.8950733542442322, 0.828593909740448, 0.8217741250991821, 0.8094630837440491, 0.780948281288147]</t>
-        </is>
-      </c>
-      <c r="H116" t="inlineStr">
-        <is>
-          <t>["The Mongol military was also successful in siege warfare, cutting off resources for cities and towns by diverting certain rivers, taking enemy prisoners and driving them in front of the army, and adopting new ideas, techniques and tools from the people they conquered, particularly in employing Muslim and Chinese siege engines and engineers to aid the Mongol cavalry in capturing cities. Another standard tactic of the Mongol military was the commonly practiced feigned retreat to break enemy formations and to lure small enemy groups away from the larger group and defended position for ambush and counterattack.", "The Shah's army was split by diverse internecine feuds and by the Shah's decision to divide his army into small groups concentrated in various cities. This fragmentation was decisive in Khwarezmia's defeats, as it allowed the Mongols, although exhausted from the long journey, to immediately set about defeating small fractions of the Khwarzemi forces instead of facing a unified defense. The Mongol army quickly seized the town of Otrar, relying on superior strategy and tactics. Genghis Khan ordered the wholesale massacre of many of the civilians, enslaved the rest of the population and executed Inalchuq by pouring molten silver into his ears and eyes, as retribution for his actions. Near the end of the battle the Shah fled rather than surrender. Genghis Khan ordered Subutai and Jebe to hunt him down, giving them 20,000 men and two years to do this. The Shah died under mysterious circumstances on a small island within his empire.", "With such a small force, the invading Mongols were forced to change strategies and resort to inciting internal revolt among Kuchlug's supporters, leaving the Qara Khitai more vulnerable to Mongol conquest. As a result, Kuchlug's army was defeated west of Kashgar. Kuchlug fled again, but was soon hunted down by Jebe's army and executed. By 1218, as a result of defeat of Qara Khitai, the Mongol Empire and its control extended as far west as Lake Balkhash, which bordered the Khwarezmia (Khwarezmid Empire), a Muslim state that reached the Caspian Sea to the west and Persian Gulf and the Arabian Sea to the south.", "After the defeat of the Khwarezmian Empire in 1220, Genghis Khan gathered his forces in Persia and Armenia to return to the Mongolian steppes. Under the suggestion of Subutai, the Mongol army was split into two forces. Genghis Khan led the main army on a raid through Afghanistan and northern India towards Mongolia, while another 20,000 (two tumen) contingent marched through the Caucasus and into Russia under generals Jebe and Subutai. They pushed deep into Armenia and Azerbaijan. The Mongols destroyed the kingdom of Georgia, sacked the Genoese trade-fortress of Caffa in Crimea and overwintered near the Black Sea. Heading home, Subutai's forces attacked the allied forces of the Cuman–Kipchaks and the poorly coordinated 80,000 Kievan Rus' troops led by Mstislav the Bold of Halych and Mstislav III of Kiev who went out to stop the Mongols' actions in the area. Subutai sent emissaries to the Slavic princes calling for a separate peace, but the emissaries were executed. At the Battle of Kalka River in 1223, Subutai's forces defeated the larger Kievan force. They also may have fought against the neighboring Volga Bulgars. There is no historical record except a short account by the Arab historian Ibn al-Athir, writing in", "seen as an affront and insult to Genghis Khan. Outraged, Genghis Khan planned one of his largest invasion campaigns by organizing together around 100,000 soldiers (10 tumens), his most capable generals and some of his sons. He left a commander and number of troops in China, designated his successors to be his family members and likely appointed Ögedei to be his immediate successor and then went out to Khwarezmia."]</t>
-        </is>
-      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -5820,21 +4080,6 @@
 Economist Joseph Stiglitz argues that rather than explaining concentrations of wealth and income, market forces should serve as a brake on such concentration, which may better be explained by the non-market force known as "rent-seeking". While the market will bid up compensation for rare and desired skills to reward wealth creation, greater productivity, etc., it will also prevent successful entrepreneurs from earning excess profits by fostering competition to cut prices, profits and large compensation. A better explainer of growing inequality, according to Stiglitz, is the use of political power generated by wealth by certain groups to shape government policies financially beneficial to them. This process, known to economists as rent-seeking, brings income not from creation of wealth but from "grabbing a larger share of the wealth that would otherwise have been produced without their effort"</t>
         </is>
       </c>
-      <c r="F117" t="inlineStr">
-        <is>
-          <t>[115, 400, 241, 743, 409]</t>
-        </is>
-      </c>
-      <c r="G117" t="inlineStr">
-        <is>
-          <t>[0.7911558747291565, 0.7738929986953735, 0.7628395557403564, 0.759792685508728, 0.7588297724723816]</t>
-        </is>
-      </c>
-      <c r="H117" t="inlineStr">
-        <is>
-          <t>["Economist Joseph Stiglitz presented evidence in 2009 that both global inequality and inequality within countries prevent growth by limiting aggregate demand. Economist Branko Milanovic, wrote in 2001 that, \"The view that income inequality harms growth – or that improved equality can help sustain growth – has become more widely held in recent years. ... The main reason for this shift is the increasing importance of human capital in development. When physical capital mattered most, savings and investments were key. Then it was important to have a large contingent of rich people who could save a greater proportion of their income than the poor and invest it in physical capital. But now that human capital is scarcer than machines, widespread education has become the secret to growth.\"", "Some theories developed in the 1970s established possible avenues through which inequality may have a positive effect on economic development. According to a 1955 review, savings by the wealthy, if these increase with inequality, were thought to offset reduced consumer demand. A 2013 report on Nigeria suggests that growth has risen with increased income inequality. Some theories popular from the 1950s to 2011 incorrectly stated that inequality had a positive effect on economic development. Analyses based on comparing yearly equality figures to yearly growth rates were misleading because it takes several years for effects to manifest as changes to economic growth. IMF economists found a strong association between lower levels of inequality in developing countries and sustained periods of economic growth. Developing countries with high inequality have \"succeeded in initiating growth at high rates for a few years\" but \"longer growth spells are robustly associated with more equality in the income distribution.\"", "While acknowledging the central role economic growth can potentially play in human development, poverty reduction and the achievement of the Millennium Development Goals, it is becoming widely understood amongst the development community that special efforts must be made to ensure poorer sections of society are able to participate in economic growth. The effect of economic growth on poverty reduction – the growth elasticity of poverty – can depend on the existing level of inequality. For instance, with low inequality a country with a growth rate of 2% per head and 40% of its population living in poverty, can halve poverty in ten years, but a country with high inequality would take nearly 60 years to achieve the same reduction. In the words of the Secretary General of the United Nations Ban Ki-Moon: \"While economic growth is necessary, it is not sufficient for progress on reducing poverty.\"", "In 2014, economists with the Standard &amp; Poor's rating agency concluded that the widening disparity between the U.S.'s wealthiest citizens and the rest of the nation had slowed its recovery from the 2008-2009 recession and made it more prone to boom-and-bust cycles. To partially remedy the wealth gap and the resulting slow growth, S&amp;P recommended increasing access to education. It estimated that if the average United States worker had completed just one more year of school, it would add an additional $105 billion in growth to the country's economy over five years.", "Economist Joseph Stiglitz argues that rather than explaining concentrations of wealth and income, market forces should serve as a brake on such concentration, which may better be explained by the non-market force known as \"rent-seeking\". While the market will bid up compensation for rare and desired skills to reward wealth creation, greater productivity, etc., it will also prevent successful entrepreneurs from earning excess profits by fostering competition to cut prices, profits and large compensation. A better explainer of growing inequality, according to Stiglitz, is the use of political power generated by wealth by certain groups to shape government policies financially beneficial to them. This process, known to economists as rent-seeking, brings income not from creation of wealth but from \"grabbing a larger share of the wealth that would otherwise have been produced without their effort\""]</t>
-        </is>
-      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -5866,21 +4111,6 @@
 The network's troubles with sustaining existing series and gaining new hits spilled over into its 2010–11 schedule: ABC's dramas during that season continued to fail, with the midseason forensic investigation drama Body of Proof being the only one that was renewed for a second season. The network also struggled to establish new comedies to support the previous year's debuts, with only late-season premiere Happy Endings earning a second season. Meanwhile, the new lows hit by Brothers &amp; Sisters led to its cancellation, and the previous year's only drama renewal, V, also failed to earn another season after a low-rated midseason run. Despite this and another noticeable ratings decline, ABC would manage to outrate NBC for third place by a larger margin than the previous year.</t>
         </is>
       </c>
-      <c r="F118" t="inlineStr">
-        <is>
-          <t>[356, 779, 401, 810, 259]</t>
-        </is>
-      </c>
-      <c r="G118" t="inlineStr">
-        <is>
-          <t>[0.786691427230835, 0.7635387182235718, 0.7529079914093018, 0.7495690584182739, 0.7369594573974609]</t>
-        </is>
-      </c>
-      <c r="H118" t="inlineStr">
-        <is>
-          <t>["On April 14, 2011, ABC canceled the long-running soap operas All My Children and One Life to Live after 41 and 43 years on the air, respectively (following backlash from fans, ABC sold the rights to both shows to Prospect Park, which eventually revived the soaps on Hulu for one additional season in 2013 and with both companies suing one another for allegations of interference with the process of reviving the shows, failure to pay licensing fees and issues over ABC's use of certain characters from One Live to Live on General Hospital during the transition). The talk/lifestyle show that replaced One Life to Live, The Revolution, failed to generate satisfactory ratings and was in turn canceled after only seven months. The 2011–12 season saw ABC drop to fourth place in the 18–49 demographic despite renewing a handful of new shows (including freshmen dramas Scandal, Revenge and Once Upon a Time) for second seasons.", "In addition to Who Wants to Be a Millionaire, the network entered the 2000s with hits held over from the previous decade such as The Practice, NYPD Blue and The Wonderful World of Disney and new series such as My Wife and Kids and According to Jim, all of which managed to help ABC stay ahead of the competition in the ratings in spite of the later departure of Millionaire. 2000 saw the end of \"TGIF\", which was struggling to find new hits (with Boy Meets World and Sabrina, the Teenage Witch, the latter of which moved to The WB in September 2000, beginning to wane as well by this point) following the loss of Family Matters and Step by Step to CBS as part of its own failed attempt at a family-oriented Friday comedy block in the 1997–98 season. Outside of Friday stalwart 20/20, Friday nights remained a weak spot for ABC for the next 11 years.", "Networks affiliates approved a two-year affiliate agreement in 2002. In September, Disney Chairman/CEO Michael Eisner outlined a proposed realignment of the ABC broadcast network day parts with the similar unit in its cable channels: ABC Saturday mornings with Disney Channels (Toon &amp; Playhouse), ABC daytime with Soapnet and ABC prime time with ABC Family. 2002 saw the debut of the network's first hit reality series, The Bachelor (the elimination-style dating show's success led to a spinoff, The Bachelorette, which premiered the following year, as well as two additional spinoffs that later debuted in the early 2010s).", "ABC dominated the American television landscape during the 1970s and early 1980s (by 1980, the three major networks represented 90% of all prime-time television viewership in the U.S.). Several flagship series debuted on the network during this time including Dynasty, an opulent drama from Aaron Spelling that became a hit when it premiered as a midseason series in 1981, five months before Spelling's other ABC hit Charlie's Angels ended its run. The network was also propelled during the early 1980s by the continued successes of Happy Days, Three's Company, Laverne &amp; Shirley and Fantasy Island, and gained new hits in Too Close for Comfort, Soap spinoff Benson and Happy Days spinoff Mork &amp; Mindy. In 1981, ABC (through its ABC Video Services division) launched the Alpha Repertory Television Service (ARTS), a cable channel operated as a joint venture with the Hearst Corporation offering cultural and arts programming, which aired as a nighttime service over the channel space of Nickelodeon.", "The network's troubles with sustaining existing series and gaining new hits spilled over into its 2010–11 schedule: ABC's dramas during that season continued to fail, with the midseason forensic investigation drama Body of Proof being the only one that was renewed for a second season. The network also struggled to establish new comedies to support the previous year's debuts, with only late-season premiere Happy Endings earning a second season. Meanwhile, the new lows hit by Brothers &amp; Sisters led to its cancellation, and the previous year's only drama renewal, V, also failed to earn another season after a low-rated midseason run. Despite this and another noticeable ratings decline, ABC would manage to outrate NBC for third place by a larger margin than the previous year."]</t>
-        </is>
-      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -5912,21 +4142,6 @@
 One of the more unusual collections is that of Eadweard Muybridge's photographs of Animal Locomotion of 1887, this consists of 781 plates. These sequences of photographs taken a fraction of a second apart capture images of different animals and humans performimg various actions. There are several of John Thomson's 1876-7 images of Street Life in London in the collection. The museum also holds James Lafayette's society portraits, a collection of more than 600 photographs dating from the late 19th to early 20th centuries and portraying a wide range of society figures of the period, including bishops, generals, society ladies, Indian maharajas, Ethiopian rulers and other foreign leaders, actresses, people posing in their motor cars and a sequence of photographs recording the guests at the famous fancy-dress ball held at Devonshire House in 1897 to celebrate Queen Victoria's diamond jubilee.</t>
         </is>
       </c>
-      <c r="F119" t="inlineStr">
-        <is>
-          <t>[340, 787, 117, 519, 285]</t>
-        </is>
-      </c>
-      <c r="G119" t="inlineStr">
-        <is>
-          <t>[0.8367286920547485, 0.8071867823600769, 0.7952327728271484, 0.7858848571777344, 0.7646950483322144]</t>
-        </is>
-      </c>
-      <c r="H119" t="inlineStr">
-        <is>
-          <t>["Not only the work of British artists and craftspeople is on display, but also work produced by European artists that was purchased or commissioned by British patrons, as well as imports from Asia, including porcelain, cloth and wallpaper. Designers and artists whose work is on display in the galleries include Gian Lorenzo Bernini, Grinling Gibbons, Daniel Marot, Louis Laguerre, Antonio Verrio, Sir James Thornhill, William Kent, Robert Adam, Josiah Wedgwood, Matthew Boulton, Canova, Thomas Chippendale, Pugin, William Morris. Patrons who have influenced taste are also represented by works of art from their collections, these include: Horace Walpole (a major influence on the Gothic Revival), William Thomas Beckford and Thomas Hope.", "With the opening of the Dorothy and Michael Hintze sculpture galleries in 2006 it was decided to extend the chronology of the works on display up to 1950; this has involved loans by other museums, including Tate Britain, so works by Henry Moore and Jacob Epstein along with other of their contemporaries are now on view. These galleries concentrate on works dated 1600 to 1950 by British sculptors, works by continental sculptors who worked in Britain, and works bought by British patrons from the continental sculptors, such as Canova's Theseus and the Minotaur. The galleries overlooking the garden are arranged by theme, tomb sculpture, portraiture, garden sculpture and mythology. Then there is a section that covers late 19th-century and early 20th-century sculpture, this includes work by Rodin and other French sculptors such as Dalou who spent several years in Britain where he taught sculpture.", "Sculptors both British and Europeans who were based in Britain and whose work is in the collection include Nicholas Stone, Caius Gabriel Cibber, Grinling Gibbons, John Michael Rysbrack, Louis-François Roubiliac, Peter Scheemakers, Sir Henry Cheere, Agostino Carlini, Thomas Banks, Joseph Nollekens, Joseph Wilton, John Flaxman, Sir Francis Chantrey, John Gibson, Edward Hodges Baily, Lord Leighton, Alfred Stevens, Thomas Brock, Alfred Gilbert, George Frampton, and Eric Gill. A sample of some of these sculptors' work is on display in the British Galleries.", "The sculpture collection at the V&amp;A is the most comprehensive holding of post-classical European sculpture in the world. There are approximately 22,000 objects in the collection that cover the period from about 400 AD to 1914. This covers among other periods Byzantine and Anglo Saxon ivory sculptures, British, French and Spanish medieval statues and carvings, the Renaissance, Baroque, Neo-Classical, Victorian and Art Nouveau periods. All uses of sculpture are represented, from tomb and memorial, to portrait, allegorical, religious, mythical, statues for gardens including fountains, as well as architectural decorations. Materials used include, marble, alabaster, stone, terracotta, wood (history of wood carving), ivory, gesso, plaster, bronze, lead and ceramics.", "One of the more unusual collections is that of Eadweard Muybridge's photographs of Animal Locomotion of 1887, this consists of 781 plates. These sequences of photographs taken a fraction of a second apart capture images of different animals and humans performimg various actions. There are several of John Thomson's 1876-7 images of Street Life in London in the collection. The museum also holds James Lafayette's society portraits, a collection of more than 600 photographs dating from the late 19th to early 20th centuries and portraying a wide range of society figures of the period, including bishops, generals, society ladies, Indian maharajas, Ethiopian rulers and other foreign leaders, actresses, people posing in their motor cars and a sequence of photographs recording the guests at the famous fancy-dress ball held at Devonshire House in 1897 to celebrate Queen Victoria's diamond jubilee."]</t>
-        </is>
-      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -5958,21 +4173,6 @@
 Early in 1537, Johannes Agricola (1494–1566) – serving at the time as pastor in Luther's birthplace, Eisleben – preached a sermon in which he claimed that God's gospel, not God's moral law (the Ten Commandments), revealed God's wrath to Christians. Based on this sermon and others by Agricola, Luther suspected that Agricola was behind certain anonymous antinomian theses circulating in Wittenberg. These theses asserted that the law is no longer to be taught to Christians but belonged only to city hall. Luther responded to these theses with six series of theses against Agricola and the antinomians, four of which became the basis for disputations between 1538 and 1540. He also responded to these assertions in other writings, such as his 1539 open letter to C. Güttel Against the Antinomians, and his book On the Councils and the Church from the same year.</t>
         </is>
       </c>
-      <c r="F120" t="inlineStr">
-        <is>
-          <t>[398, 572, 118, 324, 336]</t>
-        </is>
-      </c>
-      <c r="G120" t="inlineStr">
-        <is>
-          <t>[0.8091687560081482, 0.7948890924453735, 0.7849951386451721, 0.7782987356185913, 0.7764351963996887]</t>
-        </is>
-      </c>
-      <c r="H120" t="inlineStr">
-        <is>
-          <t>["Luther's rediscovery of \"Christ and His salvation\" was the first of two points that became the foundation for the Reformation. His railing against the sale of indulgences was based on it.", "(1528), drafted by Melanchthon with Luther's approval, stressed the role of repentance in the forgiveness of sins, despite Luther's position that faith alone ensures justification. The Eisleben reformer Johannes Agricola challenged this compromise, and Luther condemned him for teaching that faith is separate from works. The Instruction is a problematic document for those seeking a consistent evolution in Luther's thought and practice.", "Sir Charles Lyell first published his famous book, Principles of Geology, in 1830. This book, which influenced the thought of Charles Darwin, successfully promoted the doctrine of uniformitarianism. This theory states that slow geological processes have occurred throughout the Earth's history and are still occurring today. In contrast, catastrophism is the theory that Earth's features formed in single, catastrophic events and remained unchanged thereafter. Though Hutton believed in uniformitarianism, the idea was not widely accepted at the time.", "In October 1529, Philip I, Landgrave of Hesse, convoked an assembly of German and Swiss theologians at the Marburg Colloquy, to establish doctrinal unity in the emerging Protestant states. Agreement was achieved on fourteen points out of fifteen, the exception being the nature of the Eucharist – the sacrament of the Lord's Supper—an issue crucial to Luther.", "Early in 1537, Johannes Agricola (1494–1566) – serving at the time as pastor in Luther's birthplace, Eisleben – preached a sermon in which he claimed that God's gospel, not God's moral law (the Ten Commandments), revealed God's wrath to Christians. Based on this sermon and others by Agricola, Luther suspected that Agricola was behind certain anonymous antinomian theses circulating in Wittenberg. These theses asserted that the law is no longer to be taught to Christians but belonged only to city hall. Luther responded to these theses with six series of theses against Agricola and the antinomians, four of which became the basis for disputations between 1538 and 1540. He also responded to these assertions in other writings, such as his 1539 open letter to C. Güttel Against the Antinomians, and his book On the Councils and the Church from the same year."]</t>
-        </is>
-      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -6004,21 +4204,6 @@
 During the mid-Eocene, it is believed that the drainage basin of the Amazon was split along the middle of the continent by the Purus Arch. Water on the eastern side flowed toward the Atlantic, while to the west water flowed toward the Pacific across the Amazonas Basin. As the Andes Mountains rose, however, a large basin was created that enclosed a lake; now known as the Solimões Basin. Within the last 5–10 million years, this accumulating water broke through the Purus Arch, joining the easterly flow toward the Atlantic.</t>
         </is>
       </c>
-      <c r="F121" t="inlineStr">
-        <is>
-          <t>[5, 555, 200, 594, 565]</t>
-        </is>
-      </c>
-      <c r="G121" t="inlineStr">
-        <is>
-          <t>[0.8723031282424927, 0.8014264106750488, 0.7877436876296997, 0.758863627910614, 0.7543541789054871]</t>
-        </is>
-      </c>
-      <c r="H121" t="inlineStr">
-        <is>
-          <t>["The first European to travel the length of the Amazon River was Francisco de Orellana in 1542. The BBC's Unnatural Histories presents evidence that Orellana, rather than exaggerating his claims as previously thought, was correct in his observations that a complex civilization was flourishing along the Amazon in the 1540s. It is believed that the civilization was later devastated by the spread of diseases from Europe, such as smallpox. Since the 1970s, numerous geoglyphs have been discovered on deforested land dating between AD 0–1250, furthering claims about Pre-Columbian civilizations. Ondemar Dias is accredited with first discovering the geoglyphs in 1977 and Alceu Ranzi with furthering their discovery after flying over Acre. The BBC's Unnatural Histories presented evidence that the Amazon rainforest, rather than being a pristine wilderness, has been shaped by man for at least 11,000 years through practices such as forest gardening and terra preta.", "For a long time, it was thought that the Amazon rainforest was only ever sparsely populated, as it was impossible to sustain a large population through agriculture given the poor soil. Archeologist Betty Meggers was a prominent proponent of this idea, as described in her book Amazonia: Man and Culture in a Counterfeit Paradise. She claimed that a population density of 0.2 inhabitants per square kilometre (0.52/sq mi) is the maximum that can be sustained in the rainforest through hunting, with agriculture needed to host a larger population. However, recent anthropological findings have suggested that the region was actually densely populated. Some 5 million people may have lived in the Amazon region in AD 1500, divided between dense coastal settlements, such as that at Marajó, and inland dwellers. By 1900 the population had fallen to 1 million and by the early 1980s it was less than 200,000.", "The area of the modern city of Jacksonville has been inhabited for thousands of years. On Black Hammock Island in the national Timucuan Ecological and Historic Preserve, a University of North Florida team discovered some of the oldest remnants of pottery in the United States, dating to 2500 BC. In the 16th century, the beginning of the historical era, the region was inhabited by the Mocama, a coastal subgroup of the Timucua people. At the time of contact with Europeans, all Mocama villages in present-day Jacksonville were part of the powerful chiefdom known as the Saturiwa, centered around the mouth of the St. Johns River. One early map shows a village called Ossachite at the site of what is now downtown Jacksonville; this may be the earliest recorded name for that area.", "Following the Cretaceous–Paleogene extinction event, the extinction of the dinosaurs and the wetter climate may have allowed the tropical rainforest to spread out across the continent. From 66–34 Mya, the rainforest extended as far south as 45°. Climate fluctuations during the last 34 million years have allowed savanna regions to expand into the tropics. During the Oligocene, for example, the rainforest spanned a relatively narrow band. It expanded again during the Middle Miocene, then retracted to a mostly inland formation at the last glacial maximum. However, the rainforest still managed to thrive during these glacial periods, allowing for the survival and evolution of a broad diversity of species.", "During the mid-Eocene, it is believed that the drainage basin of the Amazon was split along the middle of the continent by the Purus Arch. Water on the eastern side flowed toward the Atlantic, while to the west water flowed toward the Pacific across the Amazonas Basin. As the Andes Mountains rose, however, a large basin was created that enclosed a lake; now known as the Solimões Basin. Within the last 5–10 million years, this accumulating water broke through the Purus Arch, joining the easterly flow toward the Atlantic."]</t>
-        </is>
-      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -6048,21 +4233,6 @@
 in interceptions. In week 10, Manning suffered a partial tear of the plantar fasciitis in his left foot. He set the NFL's all-time record for career passing yards in this game, but was benched after throwing four interceptions in favor of backup quarterback Brock Osweiler, who took over as the starter for most of the remainder of the regular season. Osweiler was injured, however, leading to Manning's return during the Week 17 regular season finale, where the Broncos were losing 13–7 against the 4–11 San Diego Chargers, resulting in Manning re-claiming the starting quarterback position for the playoffs by leading the team to a key 27–20 win that enabled the team to clinch the number one overall AFC seed. Under defensive coordinator Wade Phillips, the Broncos' defense ranked number one in total yards allowed, passing yards allowed and sacks, and like the previous three seasons, the team has continued to set numerous individual, league and franchise records. With the defense carrying the team despite the issues with the offense, the Broncos finished the regular season with a 12–4 record and earned home-field advantage throughout the AFC playoffs.
 After each team punted, Panthers quarterback Cam Newton appeared to complete a 24-yard pass Jerricho Cotchery, but the call was ruled an incompletion and upheld after a replay challenge. CBS analyst and retired referee Mike Carey stated he disagreed with the call and felt the review clearly showed the pass was complete. A few plays later, on 3rd-and-10 from the 15-yard line, linebacker Von Miller knocked the ball out of Newton's hands while sacking him, and Malik Jackson recovered it in the end zone for a Broncos touchdown, giving the team a 10–0 lead. This was the first fumble return touchdown in a Super Bowl since Super Bowl XXVIII at the end of the 1993 season.
 Manning finished the year with a career-low 67.9 passer rating, throwing for 2,249 yards and nine touchdowns, with 17 interceptions. In contrast, Osweiler threw for 1,967 yards, 10 touchdowns and six interceptions for a rating of 86.4. Veteran receiver Demaryius Thomas led the team with 105 receptions for 1,304 yards and six touchdowns, while Emmanuel Sanders caught 76 passes for 1,135 yards and six scores, while adding another 106 yards returning punts. Tight end Owen Daniels was also a big element of the passing game with 46 receptions for 517 yards. Running back C. J. Anderson was the team's leading rusher 863 yards and seven touchdowns, while also catching 25 passes for 183 yards. Running back Ronnie Hillman also made a big impact with 720 yards, five touchdowns, 24 receptions, and a 4.7 yards per carry average. Overall, the offense ranked 19th in scoring with 355 points and did not have any Pro Bowl selections.</t>
-        </is>
-      </c>
-      <c r="F122" t="inlineStr">
-        <is>
-          <t>[119, 523, 206, 608, 652]</t>
-        </is>
-      </c>
-      <c r="G122" t="inlineStr">
-        <is>
-          <t>[0.8460533022880554, 0.8457133173942566, 0.8147562742233276, 0.8142878413200378, 0.8141229152679443]</t>
-        </is>
-      </c>
-      <c r="H122" t="inlineStr">
-        <is>
-          <t>["Manning finished the game 13 of 23 for 141 yards with one interception and zero touchdowns. Sanders was his top receiver with six receptions for 83 yards. Anderson was the game's leading rusher with 90 yards and a touchdown, along with four receptions for 10 yards. Miller had six total tackles (five solo), 2½ sacks, and two forced fumbles. Ware had five total tackles and two sacks. Ward had seven total tackles, a fumble recovery, and an interception. McManus made all four of his field goals, making him perfect on all 11 attempts during the post-season. Newton completed 18 of 41 passes for 265 yards, with one interception. He was also the team's leading rusher with 45 yards on six carries. Brown caught four passes for 80 yards, while Ginn had four receptions for 74. Ealy was the top defensive performer for Carolina with four total tackles, three sacks, a forced fumble, a fumble recovery, and an interception. Defensive End Charles Johnson had four total tackles, a sack, and a forced fumble. Linebacker Luke Kuechly had 11 total tackles, while Thomas Davis had seven, despite playing just two weeks after breaking his right arm in the NFC title game.", "The Broncos' defense ranked first in the NFL yards allowed (4,530) for the first time in franchise history, and fourth in points allowed (296). Defensive ends Derek Wolfe and Malik Jackson each had 5½ sacks. Pro Bowl linebacker Von Miller led the team with 11 sacks, forced four fumbles, and recovered three. Linebacker DeMarcus Ware was selected to play in the Pro Bowl for the ninth time in his career, ranking second on the team with 7½ sacks. Linebacker Brandon Marshall led the team in total tackles with 109, while Danny Trevathan ranked second with 102. Cornerbacks Aqib Talib (three interceptions) and Chris Harris, Jr. (two interceptions) were the other two Pro Bowl selections from the defense.", "in interceptions. In week 10, Manning suffered a partial tear of the plantar fasciitis in his left foot. He set the NFL's all-time record for career passing yards in this game, but was benched after throwing four interceptions in favor of backup quarterback Brock Osweiler, who took over as the starter for most of the remainder of the regular season. Osweiler was injured, however, leading to Manning's return during the Week 17 regular season finale, where the Broncos were losing 13–7 against the 4–11 San Diego Chargers, resulting in Manning re-claiming the starting quarterback position for the playoffs by leading the team to a key 27–20 win that enabled the team to clinch the number one overall AFC seed. Under defensive coordinator Wade Phillips, the Broncos' defense ranked number one in total yards allowed, passing yards allowed and sacks, and like the previous three seasons, the team has continued to set numerous individual, league and franchise records. With the defense carrying the team despite the issues with the offense, the Broncos finished the regular season with a 12–4 record and earned home-field advantage throughout the AFC playoffs.", "After each team punted, Panthers quarterback Cam Newton appeared to complete a 24-yard pass Jerricho Cotchery, but the call was ruled an incompletion and upheld after a replay challenge. CBS analyst and retired referee Mike Carey stated he disagreed with the call and felt the review clearly showed the pass was complete. A few plays later, on 3rd-and-10 from the 15-yard line, linebacker Von Miller knocked the ball out of Newton's hands while sacking him, and Malik Jackson recovered it in the end zone for a Broncos touchdown, giving the team a 10–0 lead. This was the first fumble return touchdown in a Super Bowl since Super Bowl XXVIII at the end of the 1993 season.", "Manning finished the year with a career-low 67.9 passer rating, throwing for 2,249 yards and nine touchdowns, with 17 interceptions. In contrast, Osweiler threw for 1,967 yards, 10 touchdowns and six interceptions for a rating of 86.4. Veteran receiver Demaryius Thomas led the team with 105 receptions for 1,304 yards and six touchdowns, while Emmanuel Sanders caught 76 passes for 1,135 yards and six scores, while adding another 106 yards returning punts. Tight end Owen Daniels was also a big element of the passing game with 46 receptions for 517 yards. Running back C. J. Anderson was the team's leading rusher 863 yards and seven touchdowns, while also catching 25 passes for 183 yards. Running back Ronnie Hillman also made a big impact with 720 yards, five touchdowns, 24 receptions, and a 4.7 yards per carry average. Overall, the offense ranked 19th in scoring with 355 points and did not have any Pro Bowl selections."]</t>
         </is>
       </c>
     </row>
@@ -6108,21 +4278,6 @@
 3, in hematite and rust), and calcium carbonate (in limestone). The rest of the Earth's crust is also made of oxygen compounds, in particular various complex silicates (in silicate minerals). The Earth's mantle, of much larger mass than the crust, is largely composed of silicates of magnesium and iron.</t>
         </is>
       </c>
-      <c r="F123" t="inlineStr">
-        <is>
-          <t>[419, 120, 441, 326, 315]</t>
-        </is>
-      </c>
-      <c r="G123" t="inlineStr">
-        <is>
-          <t>[0.7500335574150085, 0.7384543418884277, 0.7383394241333008, 0.6763467192649841, 0.6718812584877014]</t>
-        </is>
-      </c>
-      <c r="H123" t="inlineStr">
-        <is>
-          <t>["Due to its electronegativity, oxygen forms chemical bonds with almost all other elements to give corresponding oxides. The surface of most metals, such as aluminium and titanium, are oxidized in the presence of air and become coated with a thin film of oxide that passivates the metal and slows further corrosion. Many oxides of the transition metals are non-stoichiometric compounds, with slightly less metal than the chemical formula would show. For example, the mineral FeO (wüstite) is written as Fe\n1 − xO, where x is usually around 0.05.", "Highly concentrated sources of oxygen promote rapid combustion. Fire and explosion hazards exist when concentrated oxidants and fuels are brought into close proximity; an ignition event, such as heat or a spark, is needed to trigger combustion. Oxygen is the oxidant, not the fuel, but nevertheless the source of most of the chemical energy released in combustion. Combustion hazards also apply to compounds of oxygen with a high oxidative potential, such as peroxides, chlorates, nitrates, perchlorates, and dichromates because they can donate oxygen to a fire.", "Among the most important classes of organic compounds that contain oxygen are (where \"R\" is an organic group): alcohols (R-OH); ethers (R-O-R); ketones (R-CO-R); aldehydes (R-CO-H); carboxylic acids (R-COOH); esters (R-COO-R); acid anhydrides (R-CO-O-CO-R); and amides (R-C(O)-NR\n2). There are many important organic solvents that contain oxygen, including: acetone, methanol, ethanol, isopropanol, furan, THF, diethyl ether, dioxane, ethyl acetate, DMF, DMSO, acetic acid, and formic acid. Acetone ((CH\n3)\n2CO) and phenol (C\n6H\n5OH) are used as feeder materials in the synthesis of many different substances. Other important organic compounds that contain oxygen are: glycerol, formaldehyde, glutaraldehyde, citric acid, acetic anhydride, and acetamide. Epoxides are ethers in which the oxygen atom is part of a ring of three atoms.", "To fix carbon dioxide into sugar molecules in the process of photosynthesis, chloroplasts use an enzyme called rubisco. Rubisco has a problem—it has trouble distinguishing between carbon dioxide and oxygen, so at high oxygen concentrations, rubisco starts accidentally adding oxygen to sugar precursors. This has the end result of ATP energy being wasted and CO2 being released, all with no sugar being produced. This is a big problem, since O2 is produced by the initial light reactions of photosynthesis, causing issues down the line in the Calvin cycle which uses rubisco.", "Oxygen is present in the atmosphere in trace quantities in the form of carbon dioxide (CO\n2). The Earth's crustal rock is composed in large part of oxides of silicon (silica SiO\n2, as found in granite and quartz), aluminium (aluminium oxide Al\n2O\n3, in bauxite and corundum), iron (iron(III) oxide Fe\n2O\n3, in hematite and rust), and calcium carbonate (in limestone). The rest of the Earth's crust is also made of oxygen compounds, in particular various complex silicates (in silicate minerals). The Earth's mantle, of much larger mass than the crust, is largely composed of silicates of magnesium and iron."]</t>
-        </is>
-      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -6154,21 +4309,6 @@
 In 1998, the network began using a minimalist graphical identity, designed by Pittard Sullivan, featuring a small black-and-white "ABC Circle" logo on a yellow background (promotions during this time also featured a sequence of still photos of the stars of its programs during the timeslot card as well as the schedule sequence that began each night's prime time lineup). A new four-note theme tune was introduced alongside the package, based around the network's "We Love TV" image campaign introduced that year, creating an audio signature on par with the NBC chimes, CBS' various three-note soundmarks (including the current version used since 2000) and the Fox Fanfare. The four-note signature has been updated with every television season thereafter (though variants of it used since the 1998–99 season remain in use during the production company vanity cards shown following the closing credits of most programs). In the fall of 2015, ABC is stopped with its 1998–2002 four-note jingles for promotions and production company vanity cards following the closing credits of most of its programs over seventeen years, now it have a different and adventure-type music (with the drums of the network's four-note signature in the ending). The old four-note theme tune is</t>
         </is>
       </c>
-      <c r="F124" t="inlineStr">
-        <is>
-          <t>[121, 824, 37, 541, 36]</t>
-        </is>
-      </c>
-      <c r="G124" t="inlineStr">
-        <is>
-          <t>[0.7830983996391296, 0.7632771730422974, 0.7550470232963562, 0.7455083131790161, 0.7387986183166504]</t>
-        </is>
-      </c>
-      <c r="H124" t="inlineStr">
-        <is>
-          <t>["CBS set the base rate for a 30-second advertisement at $5,000,000, a record high price for a Super Bowl ad. As of January 26, the advertisements had not yet sold out. CBS mandated that all advertisers purchase a package covering time on both the television and digital broadcasts of the game, meaning that for the first time, digital streams of the game would carry all national advertising in pattern with the television broadcast. This would be the final year in a multi-year contract with Anheuser-Busch InBev that allowed the beer manufacturer to air multiple advertisements during the game at a steep discount. It was also the final year that Doritos, a longtime sponsor of the game, held its \"Crash the Super Bowl\" contest that allowed viewers to create their own Doritos ads for a chance to have it aired during the game. Nintendo and The Pokémon Company also made their Super Bowl debut, promoting the 20th anniversary of the Pokémon video game and media franchise.", "On June 16, 2007, ABC began to phase in a new imaging campaign for the upcoming 2007–08 season, \"Start Here\". Also developed by Troika, the on-air design was intended to emphasize the availability of ABC content across multiple platforms (in particular, using a system of icons representing different devices, such as television, computers and mobile devices), and \"simplify and bring a lot more consistency and continuity to the visual representation of ABC\". The ABC logo was also significantly redesigned as part of the transition, with a glossy \"ball\" effect that was specifically designed for HD. On-air, the logo was accompanied by animated water and ribbon effects. Red ribbons were used to represent the entertainment division, while blue ribbons were used for ABC News.", "stopped with its 1998–2002 four-note jingles for promotions and production company vanity cards following the closing credits of most of its programs over seventeen years, now it have a different and adventure-type music (with the drums of the network's four-note signature in the ending). The old four-note theme tune is still used by ABC on Demand to the beginning of the ABC show.", "The service started on 1 September 1993 based on the idea from the then chief executive officer, Sam Chisholm and Rupert Murdoch, of converting the company business strategy to an entirely fee-based concept. The new package included four channels formerly available free-to-air, broadcasting on Astra's satellites, as well as introducing new channels. The service continued until the closure of BSkyB's analogue service on 27 September 2001, due to the launch and expansion of the Sky Digital platform. Some of the channels did broadcast either in the clear or soft encrypted (whereby a Videocrypt decoder was required to decode, without a subscription card) prior to their addition to the Sky Multichannels package. Within two months of the launch, BSkyB gained 400,000 new subscribers, with the majority taking at least one premium channel as well, which helped BSkyB reach 3.5 million households by mid-1994. Michael Grade criticized the operations in front of the Select Committee on National Heritage, mainly for the lack of original programming on many of the new channels.", "In 1998, the network began using a minimalist graphical identity, designed by Pittard Sullivan, featuring a small black-and-white \"ABC Circle\" logo on a yellow background (promotions during this time also featured a sequence of still photos of the stars of its programs during the timeslot card as well as the schedule sequence that began each night's prime time lineup). A new four-note theme tune was introduced alongside the package, based around the network's \"We Love TV\" image campaign introduced that year, creating an audio signature on par with the NBC chimes, CBS' various three-note soundmarks (including the current version used since 2000) and the Fox Fanfare. The four-note signature has been updated with every television season thereafter (though variants of it used since the 1998–99 season remain in use during the production company vanity cards shown following the closing credits of most programs). In the fall of 2015, ABC is stopped with its 1998–2002 four-note jingles for promotions and production company vanity cards following the closing credits of most of its programs over seventeen years, now it have a different and adventure-type music (with the drums of the network's four-note signature in the ending). The old four-note theme tune is"]</t>
-        </is>
-      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -6200,21 +4340,6 @@
 Civil disobedients have chosen a variety of different illegal acts. Bedau writes, "There is a whole class of acts, undertaken in the name of civil disobedience, which, even if they were widely practiced, would in themselves constitute hardly more than a nuisance (e.g. trespassing at a nuclear-missile installation)...Such acts are often just a harassment and, at least to the bystander, somewhat inane...The remoteness of the connection between the disobedient act and the objectionable law lays such acts open to the charge of ineffectiveness and absurdity." Bedau also notes, though, that the very harmlessness of such entirely symbolic illegal protests toward public policy goals may serve a propaganda purpose. Some civil disobedients, such as the proprietors of illegal medical cannabis dispensaries and Voice in the Wilderness, which brought medicine to Iraq without the permission of the U.S. Government, directly achieve a desired social goal (such as the provision of medication to the sick) while openly breaking the law. Julia Butterfly Hill lived in Luna, a 180-foot (55 m)-tall, 600-year-old California Redwood tree for 738 days, successfully preventing it from being cut down.</t>
         </is>
       </c>
-      <c r="F125" t="inlineStr">
-        <is>
-          <t>[122, 416, 514, 362, 182]</t>
-        </is>
-      </c>
-      <c r="G125" t="inlineStr">
-        <is>
-          <t>[0.8086053133010864, 0.7483088374137878, 0.7200848460197449, 0.7163118124008179, 0.7125861644744873]</t>
-        </is>
-      </c>
-      <c r="H125" t="inlineStr">
-        <is>
-          <t>["One of the oldest depictions of civil disobedience is in Sophocles' play Antigone, in which Antigone, one of the daughters of former King of Thebes, Oedipus, defies Creon, the current King of Thebes, who is trying to stop her from giving her brother Polynices a proper burial. She gives a stirring speech in which she tells him that she must obey her conscience rather than human law. She is not at all afraid of the death he threatens her with (and eventually carries out), but she is afraid of how her conscience will smite her if she does not do this.", "Following the Peterloo massacre of 1819, poet Percy Shelley wrote the political poem The Mask of Anarchy later that year, that begins with the images of what he thought to be the unjust forms of authority of his time—and then imagines the stirrings of a new form of social action. It is perhaps the first modern[vague] statement of the principle of nonviolent protest. A version was taken up by the author Henry David Thoreau in his essay Civil Disobedience, and later by Gandhi in his doctrine of Satyagraha. Gandhi's Satyagraha was partially influenced and inspired by Shelley's nonviolence in protest and political action. In particular, it is known that Gandhi would often quote Shelley's Masque of Anarchy to vast audiences during the campaign for a free India.", "In cases where the criminalized behavior is pure speech, civil disobedience can consist simply of engaging in the forbidden speech. An example would be WBAI's broadcasting the track \"Filthy Words\" from a George Carlin comedy album, which eventually led to the 1978 Supreme Court case of FCC v. Pacifica Foundation. Threatening government officials is another classic way of expressing defiance toward the government and unwillingness to stand for its policies. For example, Joseph Haas was arrested for allegedly sending an email to the Lebanon, New Hampshire city councilors stating, \"Wise up or die.\"", "The earliest recorded incidents of collective civil disobedience took place during the Roman Empire[citation needed]. Unarmed Jews gathered in the streets to prevent the installation of pagan images in the Temple in Jerusalem.[citation needed][original research?] In modern times, some activists who commit civil disobedience as a group collectively refuse to sign bail until certain demands are met, such as favorable bail conditions, or the release of all the activists. This is a form of jail solidarity.[page needed] There have also been many instances of solitary civil disobedience, such as that committed by Thoreau, but these sometimes go unnoticed. Thoreau, at the time of his arrest, was not yet a well-known author, and his arrest was not covered in any newspapers in the days, weeks and months after it happened. The tax collector who arrested him rose to higher political office, and Thoreau's essay was not published until after the end of the Mexican War.", "Civil disobedients have chosen a variety of different illegal acts. Bedau writes, \"There is a whole class of acts, undertaken in the name of civil disobedience, which, even if they were widely practiced, would in themselves constitute hardly more than a nuisance (e.g. trespassing at a nuclear-missile installation)...Such acts are often just a harassment and, at least to the bystander, somewhat inane...The remoteness of the connection between the disobedient act and the objectionable law lays such acts open to the charge of ineffectiveness and absurdity.\" Bedau also notes, though, that the very harmlessness of such entirely symbolic illegal protests toward public policy goals may serve a propaganda purpose. Some civil disobedients, such as the proprietors of illegal medical cannabis dispensaries and Voice in the Wilderness, which brought medicine to Iraq without the permission of the U.S. Government, directly achieve a desired social goal (such as the provision of medication to the sick) while openly breaking the law. Julia Butterfly Hill lived in Luna, a 180-foot (55 m)-tall, 600-year-old California Redwood tree for 738 days, successfully preventing it from being cut down."]</t>
-        </is>
-      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -6246,21 +4371,6 @@
 Approximately one million Protestants in modern France represent some 2% of its population. Most are concentrated in Alsace in northeast France and the Cévennes mountain region in the south, who still regard themselves as Huguenots to this day.[citation needed] A diaspora of French Australians still considers itself Huguenot, even after centuries of exile. Long integrated into Australian society, it is encouraged by the Huguenot Society of Australia to embrace and conserve its cultural heritage, aided by the Society's genealogical research services.</t>
         </is>
       </c>
-      <c r="F126" t="inlineStr">
-        <is>
-          <t>[123, 521, 489, 240, 531]</t>
-        </is>
-      </c>
-      <c r="G126" t="inlineStr">
-        <is>
-          <t>[0.8663129210472107, 0.854246973991394, 0.8507106304168701, 0.8398133516311646, 0.8368486762046814]</t>
-        </is>
-      </c>
-      <c r="H126" t="inlineStr">
-        <is>
-          <t>["Huguenot numbers peaked near an estimated two million by 1562, concentrated mainly in the southern and central parts of France, about one-eighth the number of French Catholics. As Huguenots gained influence and more openly displayed their faith, Catholic hostility grew, in spite of increasingly liberal political concessions and edicts of toleration from the French crown. A series of religious conflicts followed, known as the Wars of Religion, fought intermittently from 1562 to 1598. The wars finally ended with the granting of the Edict of Nantes, which granted the Huguenots substantial religious, political and military autonomy.", "The Catholic Church in France and many of its members opposed the Huguenots. Some Huguenot preachers and congregants were attacked as they attempted to meet for worship. The height of this persecution was the St. Bartholomew's Day massacre when 5,000 to 30,000 were killed, although there were also underlying political reasons for this as well, as some of the Huguenots were nobles trying to establish separate centers of power in southern France. Retaliating against the French Catholics, the Huguenots had their own militia.", "Both before and after the 1708 passage of the Foreign Protestants Naturalization Act, an estimated 50,000 Protestant Walloons and Huguenots fled to England, with many moving on to Ireland and elsewhere. In relative terms, this was one of the largest waves of immigration ever of a single ethnic community to Britain. Andrew Lortie (born André Lortie), a leading Huguenot theologian and writer who led the exiled community in London, became known for articulating their criticism of the Pope and the doctrine of transubstantiation during Mass.", "After the revocation of the Edict of Nantes, the Dutch Republic received the largest group of Huguenot refugees, an estimated total of 75,000 to 100,000 people. Amongst them were 200 clergy. Many came from the region of the Cévennes, for instance, the village of Fraissinet-de-Lozère. This was a huge influx as the entire population of the Dutch Republic amounted to ca. 2 million at that time. Around 1700, it is estimated that nearly 25% of the Amsterdam population was Huguenot.[citation needed] In 1705, Amsterdam and the area of West Frisia were the first areas to provide full citizens rights to Huguenot immigrants, followed by the Dutch Republic in 1715. Huguenots intermarried with Dutch from the outset.", "Approximately one million Protestants in modern France represent some 2% of its population. Most are concentrated in Alsace in northeast France and the Cévennes mountain region in the south, who still regard themselves as Huguenots to this day.[citation needed] A diaspora of French Australians still considers itself Huguenot, even after centuries of exile. Long integrated into Australian society, it is encouraged by the Huguenot Society of Australia to embrace and conserve its cultural heritage, aided by the Society's genealogical research services."]</t>
-        </is>
-      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -6292,21 +4402,6 @@
 The most useful instrument for analyzing the performance of steam engines is the steam engine indicator. Early versions were in use by 1851, but the most successful indicator was developed for the high speed engine inventor and manufacturer Charles Porter by Charles Richard and exhibited at London Exhibition in 1862. The steam engine indicator traces on paper the pressure in the cylinder throughout the cycle, which can be used to spot various problems and calculate developed horsepower. It was routinely used by engineers, mechanics and insurance inspectors. The engine indicator can also be used on internal combustion engines. See image of indicator diagram below (in Types of motor units section).</t>
         </is>
       </c>
-      <c r="F127" t="inlineStr">
-        <is>
-          <t>[124, 242, 506, 554, 284]</t>
-        </is>
-      </c>
-      <c r="G127" t="inlineStr">
-        <is>
-          <t>[0.8429484367370605, 0.820589005947113, 0.7933021187782288, 0.7766405344009399, 0.7683526277542114]</t>
-        </is>
-      </c>
-      <c r="H127" t="inlineStr">
-        <is>
-          <t>["In 1781 James Watt patented a steam engine that produced continuous rotary motion. Watt's ten-horsepower engines enabled a wide range of manufacturing machinery to be powered. The engines could be sited anywhere that water and coal or wood fuel could be obtained. By 1883, engines that could provide 10,000 hp had become feasible. The stationary steam engine was a key component of the Industrial Revolution, allowing factories to locate where water power was unavailable. The atmospheric engines of Newcomen and Watt were large compared to the amount of power they produced, but high pressure steam engines were light enough to be applied to vehicles such as traction engines and the railway locomotives.", "The next major step occurred when James Watt developed (1763–1775) an improved version of Newcomen's engine, with a separate condenser. Boulton and Watt's early engines used half as much coal as John Smeaton's improved version of Newcomen's. Newcomen's and Watt's early engines were \"atmospheric\". They were powered by air pressure pushing a piston into the partial vacuum generated by condensing steam, instead of the pressure of expanding steam. The engine cylinders had to be large because the only usable force acting on them was due to atmospheric pressure.", "Around 1800 Richard Trevithick and, separately, Oliver Evans in 1801 introduced engines using high-pressure steam; Trevithick obtained his high-pressure engine patent in 1802. These were much more powerful for a given cylinder size than previous engines and could be made small enough for transport applications. Thereafter, technological developments and improvements in manufacturing techniques (partly brought about by the adoption of the steam engine as a power source) resulted in the design of more efficient engines that could be smaller, faster, or more powerful, depending on the intended application.", "Near the end of the 19th century compound engines came into widespread use. Compound engines exhausted steam in to successively larger cylinders to accommodate the higher volumes at reduced pressures, giving improved efficiency. These stages were called expansions, with double and triple expansion engines being common, especially in shipping where efficiency was important to reduce the weight of coal carried. Steam engines remained the dominant source of power until the early 20th century, when advances in the design of electric motors and internal combustion engines gradually resulted in the replacement of reciprocating (piston) steam engines, with shipping in the 20th-century relying upon the steam turbine.", "The most useful instrument for analyzing the performance of steam engines is the steam engine indicator. Early versions were in use by 1851, but the most successful indicator was developed for the high speed engine inventor and manufacturer Charles Porter by Charles Richard and exhibited at London Exhibition in 1862. The steam engine indicator traces on paper the pressure in the cylinder throughout the cycle, which can be used to spot various problems and calculate developed horsepower. It was routinely used by engineers, mechanics and insurance inspectors. The engine indicator can also be used on internal combustion engines. See image of indicator diagram below (in Types of motor units section)."]</t>
-        </is>
-      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -6338,21 +4433,6 @@
 Although the European Union does not have a codified constitution, like every political body it has laws which "constitute" its basic governance structure. The EU's primary constitutional sources are the Treaty on European Union (TEU) and the Treaty on the Functioning of the European Union (TFEU), which have been agreed or adhered to among the governments of all 28 member states. The Treaties establish the EU's institutions, list their powers and responsibilities, and explain the areas in which the EU can legislate with Directives or Regulations. The European Commission has the initiative to propose legislation. During the ordinary legislative procedure, the Council (which are ministers from member state governments) and the European Parliament (elected by citizens) can make amendments and must give their consent for laws to pass. The Commission oversees departments and various agencies that execute or enforce EU law. The "European Council" (rather than the Council, made up of different government Ministers) is composed of the Prime Ministers or executive Presidents of the member states. It appoints the Commissioners and the board of the European Central Bank. The European Court of Justice is the supreme judicial body which interprets EU law, and develops it through precedent. The Court</t>
         </is>
       </c>
-      <c r="F128" t="inlineStr">
-        <is>
-          <t>[422, 298, 125, 874, 592]</t>
-        </is>
-      </c>
-      <c r="G128" t="inlineStr">
-        <is>
-          <t>[0.812178373336792, 0.8104715943336487, 0.8088741898536682, 0.7819502949714661, 0.7782793641090393]</t>
-        </is>
-      </c>
-      <c r="H128" t="inlineStr">
-        <is>
-          <t>["European Union law is applied by the courts of member states and the Court of Justice of the European Union. Where the laws of member states provide for lesser rights European Union law can be enforced by the courts of member states. In case of European Union law which should have been transposed into the laws of member states, such as Directives, the European Commission can take proceedings against the member state under the Treaty on the Functioning of the European Union. The European Court of Justice is the highest court able to interpret European Union law. Supplementary sources of European Union law include case law by the Court of Justice, international law and general principles of European Union law.", "The primary law of the EU consists mainly of the founding treaties, the \"core\" treaties being the Treaty on European Union (TEU) and the Treaty on the Functioning of the European Union (TFEU). The Treaties contain formal and substantive provisions, which frame policies of the European Union institutions and determine the division of competences between the European Union and its member states. The TEU establishes that European Union law applies to the metropolitan territories of the member states, as well as certain islands and overseas territories, including Madeira, the Canary Islands and the French overseas departments. European Union law also applies in territories where a member state is responsible for external relations, for example Gibraltar and the Åland islands. The TEU allows the European Council to make specific provisions for regions, as for example done for customs matters in Gibraltar and Saint-Pierre-et-Miquelon. The TEU specifically excludes certain regions, for example the Faroe Islands, from the jurisdiction of European Union law. Treaties apply as soon as they enter into force, unless stated otherwise, and are generally concluded for an unlimited period. The TEU provides that commitments entered into by the member states between themselves before the treaty was signed no longer", "European Union law is a body of treaties and legislation, such as Regulations and Directives, which have direct effect or indirect effect on the laws of European Union member states. The three sources of European Union law are primary law, secondary law and supplementary law. The main sources of primary law are the Treaties establishing the European Union. Secondary sources include regulations and directives which are based on the Treaties. The legislature of the European Union is principally composed of the European Parliament and the Council of the European Union, which under the Treaties may establish secondary law to pursue the objective set out in the Treaties.", "Since its founding, the EU has operated among an increasing plurality of national and globalising legal systems. This has meant both the European Court of Justice and the highest national courts have had to develop principles to resolve conflicts of laws between different systems. Within the EU itself, the Court of Justice's view is that if EU law conflicts with a provision of national law, then EU law has primacy. In the first major case in 1964, Costa v ENEL, a Milanese lawyer, and former shareholder of an energy company, named Mr Costa refused to pay his electricity bill to Enel, as a protest against the nationalisation of the Italian energy corporations. He claimed the Italian nationalisation law conflicted with the Treaty of Rome, and requested a reference be made to both the Italian Constitutional Court and the Court of Justice under TFEU article 267. The Italian Constitutional Court gave an opinion that because the nationalisation law was from 1962, and the treaty was in force from 1958, Costa had no claim. By contrast, the Court of Justice held that ultimately the Treaty of Rome in no way prevented energy nationalisation, and in any case under the Treaty provisions only", "Although the European Union does not have a codified constitution, like every political body it has laws which \"constitute\" its basic governance structure. The EU's primary constitutional sources are the Treaty on European Union (TEU) and the Treaty on the Functioning of the European Union (TFEU), which have been agreed or adhered to among the governments of all 28 member states. The Treaties establish the EU's institutions, list their powers and responsibilities, and explain the areas in which the EU can legislate with Directives or Regulations. The European Commission has the initiative to propose legislation. During the ordinary legislative procedure, the Council (which are ministers from member state governments) and the European Parliament (elected by citizens) can make amendments and must give their consent for laws to pass. The Commission oversees departments and various agencies that execute or enforce EU law. The \"European Council\" (rather than the Council, made up of different government Ministers) is composed of the Prime Ministers or executive Presidents of the member states. It appoints the Commissioners and the board of the European Central Bank. The European Court of Justice is the supreme judicial body which interprets EU law, and develops it through precedent. The Court"]</t>
-        </is>
-      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -6384,21 +4464,6 @@
 In 2004, the V&amp;A alongside Royal Institute of British Architects opened the first permanent gallery in the UK covering the history of architecture with displays using models, photographs, elements from buildings and original drawings. With the opening of the new gallery, the RIBA Drawings and Archives Collection has been transferred to the museum, joining the already extensive collection held by the V&amp;A. With over 600,000 drawings, over 750,000 papers and paraphernalia, and over 700,000 photographs from around the world, together they form the world's most comprehensive architectural resource.</t>
         </is>
       </c>
-      <c r="F129" t="inlineStr">
-        <is>
-          <t>[126, 540, 561, 703, 79]</t>
-        </is>
-      </c>
-      <c r="G129" t="inlineStr">
-        <is>
-          <t>[0.8616623878479004, 0.7916635274887085, 0.7642150521278381, 0.755953311920166, 0.7551968097686768]</t>
-        </is>
-      </c>
-      <c r="H129" t="inlineStr">
-        <is>
-          <t>["Harvard operates several arts, cultural, and scientific museums. The Harvard Art Museums comprises three museums. The Arthur M. Sackler Museum includes collections of ancient, Asian, Islamic and later Indian art, the Busch-Reisinger Museum, formerly the Germanic Museum, covers central and northern European art, and the Fogg Museum of Art, covers Western art from the Middle Ages to the present emphasizing Italian early Renaissance, British pre-Raphaelite, and 19th-century French art. The Harvard Museum of Natural History includes the Harvard Mineralogical Museum, Harvard University Herbaria featuring the Blaschka Glass Flowers exhibit, and the Museum of Comparative Zoology. Other museums include the Carpenter Center for the Visual Arts, designed by Le Corbusier, housing the film archive, the Peabody Museum of Archaeology and Ethnology, specializing in the cultural history and civilizations of the Western Hemisphere, and the Semitic Museum featuring artifacts from excavations in the Middle East.", "As interesting examples of expositions the most notable are: the world's first Museum of Posters boasting one of the largest collections of art posters in the world, Museum of Hunting and Riding and the Railway Museum. From among Warsaw's 60 museums, the most prestigious ones are National Museum with a collection of works whose origin ranges in time from antiquity till the present epoch as well as one of the best collections of paintings in the country including some paintings from Adolf Hitler's private collection, and Museum of the Polish Army whose set portrays the history of arms.", "was referred to as the Art School or Art Training School, later to become the Royal College of Art which finally achieved full independence in 1949. From the 1860s to the 1880s the scientific collections had been moved from the main museum site to various improvised galleries to the west of Exhibition Road. In 1893 the \"Science Museum\" had effectively come into existence when a separate director was appointed.", "There are several museums and galleries in Newcastle, including the Centre for Life with its Science Village; the Discovery Museum a museum highlighting life on Tyneside, including Tyneside's shipbuilding heritage, and inventions which changed the world; the Great North Museum; in 2009 the Newcastle on Tyne Museum of Antiquities merged with the Great North Museum (Hancock Museum); Seven Stories a museum dedicated to children's books, the Side Gallery historical and contemporary photography from around the world and Northern England and the Newburn Hall Motor Museum.", "In 2004, the V&amp;A alongside Royal Institute of British Architects opened the first permanent gallery in the UK covering the history of architecture with displays using models, photographs, elements from buildings and original drawings. With the opening of the new gallery, the RIBA Drawings and Archives Collection has been transferred to the museum, joining the already extensive collection held by the V&amp;A. With over 600,000 drawings, over 750,000 papers and paraphernalia, and over 700,000 photographs from around the world, together they form the world's most comprehensive architectural resource."]</t>
-        </is>
-      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -6430,21 +4495,6 @@
 Between 1402 and 1405, the expedition led by the Norman noble Jean de Bethencourt and the Poitevine Gadifer de la Salle conquered the Canarian islands of Lanzarote, Fuerteventura and El Hierro off the Atlantic coast of Africa. Their troops were gathered in Normandy, Gascony and were later reinforced by Castilian colonists.</t>
         </is>
       </c>
-      <c r="F130" t="inlineStr">
-        <is>
-          <t>[487, 502, 127, 28, 55]</t>
-        </is>
-      </c>
-      <c r="G130" t="inlineStr">
-        <is>
-          <t>[0.7750291228294373, 0.7638592720031738, 0.7633119821548462, 0.7539690136909485, 0.7534828782081604]</t>
-        </is>
-      </c>
-      <c r="H130" t="inlineStr">
-        <is>
-          <t>["The War of the Austrian Succession (whose North American theater is known as King George's War) formally ended in 1748 with the signing of the Treaty of Aix-la-Chapelle. The treaty was primarily focused on resolving issues in Europe. The issues of conflicting territorial claims between British and French colonies in North America were turned over to a commission to resolve, but it reached no decision. Frontiers from between Nova Scotia and Acadia in the north, to the Ohio Country in the south, were claimed by both sides. The disputes also extended into the Atlantic Ocean, where both powers wanted access to the rich fisheries of the Grand Banks off Newfoundland.", "members of the Reformed Church) involved in the Amboise plot of 1560: a foiled attempt to wrest power in France from the influential House of Guise. The move would have had the side effect of fostering relations with the Swiss. Thus, Hugues plus Eidgenosse by way of Huisgenoten supposedly became Huguenot, a nickname associating the Protestant cause with politics unpopular in France.[citation needed]", "Colonel Monckton, in the sole British success that year, captured Fort Beauséjour in June 1755, cutting the French fortress at Louisbourg off from land-based reinforcements. To cut vital supplies to Louisbourg, Nova Scotia's Governor Charles Lawrence ordered the deportation of the French-speaking Acadian population from the area. Monckton's forces, including companies of Rogers' Rangers, forcibly removed thousands of Acadians, chasing down many who resisted, and sometimes committing atrocities. More than any other factor, the cutting off of supplies to Louisbourg led to its demise. The Acadian resistance, in concert with native allies, including the Mi'kmaq, was sometimes quite stiff, with ongoing frontier raids (against Dartmouth and Lunenburg among others). Other than the campaigns to expel the Acadians (ranging around the Bay of Fundy, on the Petitcodiac and St. John rivers, and Île Saint-Jean), the only clashes of any size were at Petitcodiac in 1755 and at Bloody Creek near Annapolis Royal in 1757.", "Loudoun, a capable administrator but a cautious field commander, planned one major operation for 1757: an attack on New France's capital, Quebec. Leaving a sizable force at Fort William Henry to distract Montcalm, he began organizing for the expedition to Quebec. He was then ordered by William Pitt, the Secretary of State responsible for the colonies, to attack Louisbourg first. Beset by delays of all kinds, the expedition was finally ready to sail from Halifax, Nova Scotia in early August. In the meantime French ships had escaped the British blockade of the French coast, and a fleet outnumbering the British one awaited Loudoun at Louisbourg. Faced with this strength, Loudoun returned to New York amid news that a massacre had occurred at Fort William Henry.", "Between 1402 and 1405, the expedition led by the Norman noble Jean de Bethencourt and the Poitevine Gadifer de la Salle conquered the Canarian islands of Lanzarote, Fuerteventura and El Hierro off the Atlantic coast of Africa. Their troops were gathered in Normandy, Gascony and were later reinforced by Castilian colonists."]</t>
-        </is>
-      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -6476,21 +4526,6 @@
 Alternatively, glucose monomers in the chloroplast can be linked together to make starch, which accumulates into the starch grains found in the chloroplast. Under conditions such as high atmospheric CO2 concentrations, these starch grains may grow very large, distorting the grana and thylakoids. The starch granules displace the thylakoids, but leave them intact. Waterlogged roots can also cause starch buildup in the chloroplasts, possibly due to less sucrose being exported out of the chloroplast (or more accurately, the plant cell). This depletes a plant's free phosphate supply, which indirectly stimulates chloroplast starch synthesis. While linked to low photosynthesis rates, the starch grains themselves may not necessarily interfere significantly with the efficiency of photosynthesis, and might simply be a side effect of another photosynthesis-depressing factor.</t>
         </is>
       </c>
-      <c r="F131" t="inlineStr">
-        <is>
-          <t>[90, 360, 326, 164, 300]</t>
-        </is>
-      </c>
-      <c r="G131" t="inlineStr">
-        <is>
-          <t>[0.8287343382835388, 0.8079965710639954, 0.7617941498756409, 0.7274967432022095, 0.7135007381439209]</t>
-        </is>
-      </c>
-      <c r="H131" t="inlineStr">
-        <is>
-          <t>["One of the main functions of the chloroplast is its role in photosynthesis, the process by which light is transformed into chemical energy, to subsequently produce food in the form of sugars. Water (H2O) and carbon dioxide (CO2) are used in photosynthesis, and sugar and oxygen (O2) is made, using light energy. Photosynthesis is divided into two stages—the light reactions, where water is split to produce oxygen, and the dark reactions, or Calvin cycle, which builds sugar molecules from carbon dioxide. The two phases are linked by the energy carriers adenosine triphosphate (ATP) and nicotinamide adenine dinucleotide phosphate (NADP+).", "Chloroplasts' main role is to conduct photosynthesis, where the photosynthetic pigment chlorophyll captures the energy from sunlight and converts it and stores it in the energy-storage molecules ATP and NADPH while freeing oxygen from water. They then use the ATP and NADPH to make organic molecules from carbon dioxide in a process known as the Calvin cycle. Chloroplasts carry out a number of other functions, including fatty acid synthesis, much amino acid synthesis, and the immune response in plants. The number of chloroplasts per cell varies from 1 in algae up to 100 in plants like Arabidopsis and wheat.", "To fix carbon dioxide into sugar molecules in the process of photosynthesis, chloroplasts use an enzyme called rubisco. Rubisco has a problem—it has trouble distinguishing between carbon dioxide and oxygen, so at high oxygen concentrations, rubisco starts accidentally adding oxygen to sugar precursors. This has the end result of ATP energy being wasted and CO2 being released, all with no sugar being produced. This is a big problem, since O2 is produced by the initial light reactions of photosynthesis, causing issues down the line in the Calvin cycle which uses rubisco.", "Photorespiration can occur when the oxygen concentration is too high. Rubisco cannot distinguish between oxygen and carbon dioxide very well, so it can accidentally add O2 instead of CO2 to RuBP. This process reduces the efficiency of photosynthesis—it consumes ATP and oxygen, releases CO2, and produces no sugar. It can waste up to half the carbon fixed by the Calvin cycle. Several mechanisms have evolved in different lineages that raise the carbon dioxide concentration relative to oxygen within the chloroplast, increasing the efficiency of photosynthesis. These mechanisms are called carbon dioxide concentrating mechanisms, or CCMs. These include Crassulacean acid metabolism, C4 carbon fixation, and pyrenoids. Chloroplasts in C4 plants are notable as they exhibit a distinct chloroplast dimorphism.", "Alternatively, glucose monomers in the chloroplast can be linked together to make starch, which accumulates into the starch grains found in the chloroplast. Under conditions such as high atmospheric CO2 concentrations, these starch grains may grow very large, distorting the grana and thylakoids. The starch granules displace the thylakoids, but leave them intact. Waterlogged roots can also cause starch buildup in the chloroplasts, possibly due to less sucrose being exported out of the chloroplast (or more accurately, the plant cell). This depletes a plant's free phosphate supply, which indirectly stimulates chloroplast starch synthesis. While linked to low photosynthesis rates, the starch grains themselves may not necessarily interfere significantly with the efficiency of photosynthesis, and might simply be a side effect of another photosynthesis-depressing factor."]</t>
-        </is>
-      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -6522,21 +4557,6 @@
 A regulation of the Rhine was called for, with an upper canal near Diepoldsau and a lower canal at Fußach, in order to counteract the constant flooding and strong sedimentation in the western Rhine Delta. The Dornbirner Ach had to be diverted, too, and it now flows parallel to the canalized Rhine into the lake. Its water has a darker color than the Rhine; the latter's lighter suspended load comes from higher up the mountains. It is expected that the continuous input of sediment into the lake will silt up the lake. This has already happened to the former Lake Tuggenersee.</t>
         </is>
       </c>
-      <c r="F132" t="inlineStr">
-        <is>
-          <t>[128, 661, 68, 612, 109]</t>
-        </is>
-      </c>
-      <c r="G132" t="inlineStr">
-        <is>
-          <t>[0.9081704616546631, 0.8528642654418945, 0.8489307761192322, 0.845065712928772, 0.8258143663406372]</t>
-        </is>
-      </c>
-      <c r="H132" t="inlineStr">
-        <is>
-          <t>["The other third of the water flows through the Pannerdens Kanaal and redistributes in the IJssel and Nederrijn. The IJssel branch carries one ninth of the water flow of the Rhine north into the IJsselmeer (a former bay), while the Nederrijn carries approximately two ninths of the flow west along a route parallel to the Waal. However, at Wijk bij Duurstede, the Nederrijn changes its name and becomes the Lek. It flows farther west, to rejoin the Noord River into the Nieuwe Maas and to the North Sea.", "The shape of the Rhine delta is determined by two bifurcations: first, at Millingen aan de Rijn, the Rhine splits into Waal and Pannerdens Kanaal, which changes its name to Nederrijn at Angeren, and second near Arnhem, the IJssel branches off from the Nederrijn. This creates three main flows, two of which change names rather often. The largest and southern main branch begins as Waal and continues as Boven Merwede (\"Upper Merwede\"), Beneden Merwede (\"Lower Merwede\"), Noord River (\"North River\"), Nieuwe Maas (\"New Meuse\"), Het Scheur (\"the Rip\") and Nieuwe Waterweg (\"New Waterway\"). The middle flow begins as Nederrijn, then changes into Lek, then joins the Noord, thereby forming Nieuwe Maas. The northern flow keeps the name IJssel until it flows into Lake IJsselmeer. Three more flows carry significant amounts of water: the Nieuwe Merwede (\"New Merwede\"), which branches off from the southern branch where it changes from Boven to Beneden Merwede; the Oude Maas (\"Old Meuse\"), which branches off from the southern branch where it changes from Beneden Merwede into Noord, and Dordtse Kil, which branches off from Oude Maas.", "The hydrography of the current delta is characterized by the delta's main arms, disconnected arms (Hollandse IJssel, Linge, Vecht, etc.) and smaller rivers and streams. Many rivers have been closed (\"dammed\") and now serve as drainage channels for the numerous polders. The construction of Delta Works changed the Delta in the second half of the 20th Century fundamentally. Currently Rhine water runs into the sea, or into former marine bays now separated from the sea, in five places, namely at the mouths of the Nieuwe Merwede, Nieuwe Waterway (Nieuwe Maas), Dordtse Kil, Spui and IJssel.", "The name Rijn, from here on, is used only for smaller streams farther to the north, which together formed the main river Rhine in Roman times. Though they retained the name, these streams no longer carry water from the Rhine, but are used for draining the surrounding land and polders. From Wijk bij Duurstede, the old north branch of the Rhine is called Kromme Rijn (\"Bent Rhine\") past Utrecht, first Leidse Rijn (\"Rhine of Leiden\") and then, Oude Rijn (\"Old Rhine\"). The latter flows west into a sluice at Katwijk, where its waters can be discharged into the North Sea. This branch once formed the line along which the Limes Germanicus were built. During periods of lower sea levels within the various ice ages, the Rhine took a left turn, creating the Channel River, the course of which now lies below the English Channel.", "A regulation of the Rhine was called for, with an upper canal near Diepoldsau and a lower canal at Fußach, in order to counteract the constant flooding and strong sedimentation in the western Rhine Delta. The Dornbirner Ach had to be diverted, too, and it now flows parallel to the canalized Rhine into the lake. Its water has a darker color than the Rhine; the latter's lighter suspended load comes from higher up the mountains. It is expected that the continuous input of sediment into the lake will silt up the lake. This has already happened to the former Lake Tuggenersee."]</t>
-        </is>
-      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -6568,21 +4588,6 @@
 On April 12, 1961, Soviet cosmonaut Yuri Gagarin became the first person to fly in space, reinforcing American fears about being left behind in a technological competition with the Soviet Union. At a meeting of the US House Committee on Science and Astronautics one day after Gagarin's flight, many congressmen pledged their support for a crash program aimed at ensuring that America would catch up. Kennedy was circumspect in his response to the news, refusing to make a commitment on America's response to the Soviets.</t>
         </is>
       </c>
-      <c r="F133" t="inlineStr">
-        <is>
-          <t>[129, 827, 749, 245, 244]</t>
-        </is>
-      </c>
-      <c r="G133" t="inlineStr">
-        <is>
-          <t>[0.8143095374107361, 0.7436031103134155, 0.741310715675354, 0.7382842302322388, 0.7328624725341797]</t>
-        </is>
-      </c>
-      <c r="H133" t="inlineStr">
-        <is>
-          <t>["On August 15, 1971, the United States unilaterally pulled out of the Bretton Woods Accord. The US abandoned the Gold Exchange Standard whereby the value of the dollar had been pegged to the price of gold and all other currencies were pegged to the dollar, whose value was left to \"float\" (rise and fall according to market demand). Shortly thereafter, Britain followed, floating the pound sterling. The other industrialized nations followed suit with their respective currencies. Anticipating that currency values would fluctuate unpredictably for a time, the industrialized nations increased their reserves (by expanding their money supplies) in amounts far greater than before. The result was a depreciation of the dollar and other industrialized nations' currencies. Because oil was priced in dollars, oil producers' real income decreased. In September 1971, OPEC issued a joint communiqué stating that, from then on, they would price oil in terms of a fixed amount of gold.", "United States and Western Europe than in China (due to a greater tendency to take on debts).[unreliable source?][unreliable source?] Anthony Shorrocks, the lead author of the Credit Suisse report which is one of the sources of Oxfam's data, considers the criticism about debt to be a \"silly argument\" and \"a non-issue . . . a diversion.\"", "The embargo had a negative influence on the US economy by causing immediate demands to address the threats to U.S. energy security. On an international level, the price increases changed competitive positions in many industries, such as automobiles. Macroeconomic problems consisted of both inflationary and deflationary impacts. The embargo left oil companies searching for new ways to increase oil supplies, even in rugged terrain such as the Arctic. Finding oil and developing new fields usually required five to ten years before significant production.", "The principal Treaties that form the European Union began with common rules for coal and steel, and then atomic energy, but more complete and formal institutions were established through the Treaty of Rome 1957 and the Maastricht Treaty 1992 (now: TFEU). Minor amendments were made during the 1960s and 1970s. Major amending treaties were signed to complete the development of a single, internal market in the Single European Act 1986, to further the development of a more social Europe in the Treaty of Amsterdam 1997, and to make minor amendments to the relative power of member states in the EU institutions in the Treaty of Nice 2001 and the Treaty of Lisbon 2007. Since its establishment, more member states have joined through a series of accession treaties, from the UK, Ireland, Denmark and Norway in 1972 (though Norway did not end up joining), Greece in 1979, Spain and Portugal 1985, Austria, Finland, Norway and Sweden in 1994 (though again Norway failed to join, because of lack of support in the referendum), the Czech Republic, Cyprus, Estonia, Hungary, Latvia, Lithuania, Malta, Poland, Slovakia and Slovenia in 2004, Romania and Bulgaria in 2007 and Croatia in 2013. Greenland signed a Treaty in", "On April 12, 1961, Soviet cosmonaut Yuri Gagarin became the first person to fly in space, reinforcing American fears about being left behind in a technological competition with the Soviet Union. At a meeting of the US House Committee on Science and Astronautics one day after Gagarin's flight, many congressmen pledged their support for a crash program aimed at ensuring that America would catch up. Kennedy was circumspect in his response to the news, refusing to make a commitment on America's response to the Soviets."]</t>
-        </is>
-      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -6614,21 +4619,6 @@
 Dynamic equilibrium was first described by Galileo who noticed that certain assumptions of Aristotelian physics were contradicted by observations and logic. Galileo realized that simple velocity addition demands that the concept of an "absolute rest frame" did not exist. Galileo concluded that motion in a constant velocity was completely equivalent to rest. This was contrary to Aristotle's notion of a "natural state" of rest that objects with mass naturally approached. Simple experiments showed that Galileo's understanding of the equivalence of constant velocity and rest were correct. For example, if a mariner dropped a cannonball from the crow's nest of a ship moving at a constant velocity, Aristotelian physics would have the cannonball fall straight down while the ship moved beneath it. Thus, in an Aristotelian universe, the falling cannonball would land behind the foot of the mast of a moving ship. However, when this experiment is actually conducted, the cannonball always falls at the foot of the mast, as if the cannonball knows to travel with the ship despite being separated from it. Since there is no forward horizontal force being applied on the cannonball as it falls, the only conclusion left is that the cannonball continues to move with</t>
         </is>
       </c>
-      <c r="F134" t="inlineStr">
-        <is>
-          <t>[130, 601, 621, 754, 369]</t>
-        </is>
-      </c>
-      <c r="G134" t="inlineStr">
-        <is>
-          <t>[0.8742043375968933, 0.7804858684539795, 0.7740042805671692, 0.7738820910453796, 0.7677196264266968]</t>
-        </is>
-      </c>
-      <c r="H134" t="inlineStr">
-        <is>
-          <t>["Torque is the rotation equivalent of force in the same way that angle is the rotational equivalent for position, angular velocity for velocity, and angular momentum for momentum. As a consequence of Newton's First Law of Motion, there exists rotational inertia that ensures that all bodies maintain their angular momentum unless acted upon by an unbalanced torque. Likewise, Newton's Second Law of Motion can be used to derive an analogous equation for the instantaneous angular acceleration of the rigid body:", "The shortcomings of Aristotelian physics would not be fully corrected until the 17th century work of Galileo Galilei, who was influenced by the late Medieval idea that objects in forced motion carried an innate force of impetus. Galileo constructed an experiment in which stones and cannonballs were both rolled down an incline to disprove the Aristotelian theory of motion early in the 17th century. He showed that the bodies were accelerated by gravity to an extent that was independent of their mass and argued that objects retain their velocity unless acted on by a force, for example friction.", "Aristotle provided a philosophical discussion of the concept of a force as an integral part of Aristotelian cosmology. In Aristotle's view, the terrestrial sphere contained four elements that come to rest at different \"natural places\" therein. Aristotle believed that motionless objects on Earth, those composed mostly of the elements earth and water, to be in their natural place on the ground and that they will stay that way if left alone. He distinguished between the innate tendency of objects to find their \"natural place\" (e.g., for heavy bodies to fall), which led to \"natural motion\", and unnatural or forced motion, which required continued application of a force. This theory, based on the everyday experience of how objects move, such as the constant application of a force needed to keep a cart moving, had conceptual trouble accounting for the behavior of projectiles, such as the flight of arrows. The place where the archer moves the projectile was at the start of the flight, and while the projectile sailed through the air, no discernible efficient cause acts on it. Aristotle was aware of this problem and proposed that the air displaced through the projectile's path carries the projectile to its target. This", "Newton's laws and Newtonian mechanics in general were first developed to describe how forces affect idealized point particles rather than three-dimensional objects. However, in real life, matter has extended structure and forces that act on one part of an object might affect other parts of an object. For situations where lattice holding together the atoms in an object is able to flow, contract, expand, or otherwise change shape, the theories of continuum mechanics describe the way forces affect the material. For example, in extended fluids, differences in pressure result in forces being directed along the pressure gradients as follows:", "Dynamic equilibrium was first described by Galileo who noticed that certain assumptions of Aristotelian physics were contradicted by observations and logic. Galileo realized that simple velocity addition demands that the concept of an \"absolute rest frame\" did not exist. Galileo concluded that motion in a constant velocity was completely equivalent to rest. This was contrary to Aristotle's notion of a \"natural state\" of rest that objects with mass naturally approached. Simple experiments showed that Galileo's understanding of the equivalence of constant velocity and rest were correct. For example, if a mariner dropped a cannonball from the crow's nest of a ship moving at a constant velocity, Aristotelian physics would have the cannonball fall straight down while the ship moved beneath it. Thus, in an Aristotelian universe, the falling cannonball would land behind the foot of the mast of a moving ship. However, when this experiment is actually conducted, the cannonball always falls at the foot of the mast, as if the cannonball knows to travel with the ship despite being separated from it. Since there is no forward horizontal force being applied on the cannonball as it falls, the only conclusion left is that the cannonball continues to move with"]</t>
-        </is>
-      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -6660,21 +4650,6 @@
 A computational problem can be viewed as an infinite collection of instances together with a solution for every instance. The input string for a computational problem is referred to as a problem instance, and should not be confused with the problem itself. In computational complexity theory, a problem refers to the abstract question to be solved. In contrast, an instance of this problem is a rather concrete utterance, which can serve as the input for a decision problem. For example, consider the problem of primality testing. The instance is a number (e.g. 15) and the solution is "yes" if the number is prime and "no" otherwise (in this case "no"). Stated another way, the instance is a particular input to the problem, and the solution is the output corresponding to the given input.</t>
         </is>
       </c>
-      <c r="F135" t="inlineStr">
-        <is>
-          <t>[131, 475, 533, 814, 71]</t>
-        </is>
-      </c>
-      <c r="G135" t="inlineStr">
-        <is>
-          <t>[0.9054017663002014, 0.8486523628234863, 0.8468760251998901, 0.8459096550941467, 0.8381496667861938]</t>
-        </is>
-      </c>
-      <c r="H135" t="inlineStr">
-        <is>
-          <t>["A problem is regarded as inherently difficult if its solution requires significant resources, whatever the algorithm used. The theory formalizes this intuition, by introducing mathematical models of computation to study these problems and quantifying the amount of resources needed to solve them, such as time and storage. Other complexity measures are also used, such as the amount of communication (used in communication complexity), the number of gates in a circuit (used in circuit complexity) and the number of processors (used in parallel computing). One of the roles of computational complexity theory is to determine the practical limits on what computers can and cannot do.", "Many important complexity classes can be defined by bounding the time or space used by the algorithm. Some important complexity classes of decision problems defined in this manner are the following:", "Analogous definitions can be made for space requirements. Although time and space are the most well-known complexity resources, any complexity measure can be viewed as a computational resource. Complexity measures are very generally defined by the Blum complexity axioms. Other complexity measures used in complexity theory include communication complexity, circuit complexity, and decision tree complexity.", "Closely related fields in theoretical computer science are analysis of algorithms and computability theory. A key distinction between analysis of algorithms and computational complexity theory is that the former is devoted to analyzing the amount of resources needed by a particular algorithm to solve a problem, whereas the latter asks a more general question about all possible algorithms that could be used to solve the same problem. More precisely, it tries to classify problems that can or cannot be solved with appropriately restricted resources. In turn, imposing restrictions on the available resources is what distinguishes computational complexity from computability theory: the latter theory asks what kind of problems can, in principle, be solved algorithmically.", "A computational problem can be viewed as an infinite collection of instances together with a solution for every instance. The input string for a computational problem is referred to as a problem instance, and should not be confused with the problem itself. In computational complexity theory, a problem refers to the abstract question to be solved. In contrast, an instance of this problem is a rather concrete utterance, which can serve as the input for a decision problem. For example, consider the problem of primality testing. The instance is a number (e.g. 15) and the solution is \"yes\" if the number is prime and \"no\" otherwise (in this case \"no\"). Stated another way, the instance is a particular input to the problem, and the solution is the output corresponding to the given input."]</t>
-        </is>
-      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -6706,21 +4681,6 @@
 justified as part of the public policy of promoting the Irish language, but only if the measure was not disproportionate. By contrast in Angonese v Cassa di Risparmio di Bolzano SpA a bank in Bolzano, Italy, was not allowed to require Mr Angonese to have a bilingual certificate that could only be obtained in Bolzano. The Court of Justice, giving "horizontal" direct effect to TFEU article 45, reasoned that people from other countries would have little chance of acquiring the certificate, and because it was "impossible to submit proof of the required linguistic knowledge by any other means", the measure was disproportionate. Second, article 7(2) requires equal treatment in respect of tax. In Finanzamt Köln Altstadt v Schumacker the Court of Justice held that it contravened TFEU art 45 to deny tax benefits (e.g. for married couples, and social insurance expense deductions) to a man who worked in Germany, but was resident in Belgium when other German residents got the benefits. By contrast in Weigel v Finanzlandesdirektion für Vorarlberg the Court of Justice rejected Mr Weigel's claim that a re-registration charge upon bringing his car to Austria violated his right to free movement. Although the tax was "likely to have</t>
         </is>
       </c>
-      <c r="F136" t="inlineStr">
-        <is>
-          <t>[876, 874, 134, 875, 281]</t>
-        </is>
-      </c>
-      <c r="G136" t="inlineStr">
-        <is>
-          <t>[0.8416346907615662, 0.822268545627594, 0.8183003664016724, 0.8167518973350525, 0.8157950639724731]</t>
-        </is>
-      </c>
-      <c r="H136" t="inlineStr">
-        <is>
-          <t>["domestic legal provisions, however framed... without the legal basis of the community itself being called into question.\" This meant any \"subsequent unilateral act\" of the member state inapplicable. Similarly, in Amministrazione delle Finanze v Simmenthal SpA, a company, Simmenthal SpA, claimed that a public health inspection fee under an Italian law of 1970 for importing beef from France to Italy was contrary to two Regulations from 1964 and 1968. In \"accordance with the principle of the precedence of Community law,\" said the Court of Justice, the \"directly applicable measures of the institutions\" (such as the Regulations in the case) \"render automatically inapplicable any conflicting provision of current national law\". This was necessary to prevent a \"corresponding denial\" of Treaty \"obligations undertaken unconditionally and irrevocably by member states\", that could \"imperil the very foundations of the\" EU. But despite the views of the Court of Justice, the national courts of member states have not accepted the same analysis.", "Since its founding, the EU has operated among an increasing plurality of national and globalising legal systems. This has meant both the European Court of Justice and the highest national courts have had to develop principles to resolve conflicts of laws between different systems. Within the EU itself, the Court of Justice's view is that if EU law conflicts with a provision of national law, then EU law has primacy. In the first major case in 1964, Costa v ENEL, a Milanese lawyer, and former shareholder of an energy company, named Mr Costa refused to pay his electricity bill to Enel, as a protest against the nationalisation of the Italian energy corporations. He claimed the Italian nationalisation law conflicted with the Treaty of Rome, and requested a reference be made to both the Italian Constitutional Court and the Court of Justice under TFEU article 267. The Italian Constitutional Court gave an opinion that because the nationalisation law was from 1962, and the treaty was in force from 1958, Costa had no claim. By contrast, the Court of Justice held that ultimately the Treaty of Rome in no way prevented energy nationalisation, and in any case under the Treaty provisions only", "had to be \"chocolate substitute\". All Italian chocolate was made from cocoa butter alone, but British, Danish and Irish manufacturers used other vegetable fats. They claimed the law infringed article 34. The Court of Justice held that a low content of vegetable fat did not justify a \"chocolate substitute\" label. This was derogatory in the consumers' eyes. A ‘neutral and objective statement’ was enough to protect consumers. If member states place considerable obstacles on the use of a product, this can also infringe article 34. So, in a 2009 case, Commission v Italy, the Court of Justice held that an Italian law prohibiting motorcycles or mopeds pulling trailers infringed article 34. Again, the law applied neutrally to everyone, but disproportionately affected importers, because Italian companies did not make trailers. This was not a product requirement, but the Court reasoned that the prohibition would deter people from buying it: it would have \"a considerable influence on the behaviour of consumers\" that \"affects the access of that product to the market\". It would require justification under article 36, or as a mandatory requirement.", "an opinion that because the nationalisation law was from 1962, and the treaty was in force from 1958, Costa had no claim. By contrast, the Court of Justice held that ultimately the Treaty of Rome in no way prevented energy nationalisation, and in any case under the Treaty provisions only the Commission could have brought a claim, not Mr Costa. However, in principle, Mr Costa was entitled to plead that the Treaty conflicted with national law, and the court would have a duty to consider his claim to make a reference if there would be no appeal against its decision. The Court of Justice, repeating its view in Van Gend en Loos, said member states \"albeit within limited spheres, have restricted their sovereign rights and created a body of law applicable both to their nationals and to themselves\" on the \"basis of reciprocity\". EU law would not \"be overridden by domestic legal provisions, however framed... without the legal basis of the community itself being called into question.\" This meant any \"subsequent unilateral act\" of the member state inapplicable. Similarly, in Amministrazione delle Finanze v Simmenthal SpA, a company, Simmenthal SpA, claimed that a public health inspection fee under an Italian", "justified as part of the public policy of promoting the Irish language, but only if the measure was not disproportionate. By contrast in Angonese v Cassa di Risparmio di Bolzano SpA a bank in Bolzano, Italy, was not allowed to require Mr Angonese to have a bilingual certificate that could only be obtained in Bolzano. The Court of Justice, giving \"horizontal\" direct effect to TFEU article 45, reasoned that people from other countries would have little chance of acquiring the certificate, and because it was \"impossible to submit proof of the required linguistic knowledge by any other means\", the measure was disproportionate. Second, article 7(2) requires equal treatment in respect of tax. In Finanzamt Köln Altstadt v Schumacker the Court of Justice held that it contravened TFEU art 45 to deny tax benefits (e.g. for married couples, and social insurance expense deductions) to a man who worked in Germany, but was resident in Belgium when other German residents got the benefits. By contrast in Weigel v Finanzlandesdirektion für Vorarlberg the Court of Justice rejected Mr Weigel's claim that a re-registration charge upon bringing his car to Austria violated his right to free movement. Although the tax was \"likely to have"]</t>
-        </is>
-      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -6752,21 +4712,6 @@
 There are over 10,000 objects made from silver or gold in the collection, the display (about 15% of the collection) is divided into secular and sacred covering both Christian (Roman Catholic, Anglican and Greek Orthodox) and Jewish liturgical vessels and items. The main silver gallery is divided into these areas: British silver pre-1800; British silver 1800 to 1900; modernist to contemporary silver; European silver. The collection includes the earliest known piece of English silver with a dated hallmark, a silver gilt beaker dated 1496–97. Silversmiths' whose work is represented in the collection include Paul de Lamerie and Paul Storr whose Castlereagh Inkstand dated 1817–19 is one of his finest works. The main iron work gallery covers European wrought and cast iron from the mediaeval period to the early 20th century. The master of wrought ironwork Jean Tijou is represented by both examples of his work and designs on paper. One of the largest items is the Hereford Screen, weighing nearly 8 tonnes, 10.5 metres high and 11 metres wide, designed by Sir George Gilbert Scott in 1862 for the chancel in Hereford Cathedral, from which it was removed in 1967. It was made by Skidmore &amp; Company. Its structure of</t>
         </is>
       </c>
-      <c r="F137" t="inlineStr">
-        <is>
-          <t>[135, 158, 688, 820, 695]</t>
-        </is>
-      </c>
-      <c r="G137" t="inlineStr">
-        <is>
-          <t>[0.8189235925674438, 0.7811620235443115, 0.763403594493866, 0.751703143119812, 0.7427474856376648]</t>
-        </is>
-      </c>
-      <c r="H137" t="inlineStr">
-        <is>
-          <t>["The glass collection covers 4000 years of glass making, and has over 6000 items from Africa, Britain, Europe, America and Asia. The earliest glassware on display comes from Ancient Egypt and continues through the Ancient Roman, Medieval, Renaissance covering areas such as Venetian glass and Bohemian glass and more recent periods, including Art Nouveau glass by Louis Comfort Tiffany and Émile Gallé, the Art Deco style is represented by several examples by René Lalique. There are many examples of crystal chandeliers both English, displayed in the British galleries and foreign for example Venetian (attributed to Giuseppe Briati) dated c1750 are in the collection. The stained glass collection is possibly the finest in the world, covering the medieval to modern periods, and covering Europe as well as Britain. Several examples of English 16th-century heraldic glass is displayed in the British Galleries. Many well-known designers of stained glass are represented in the collection including, from the 19th century: Dante Gabriel Rossetti, Edward Burne-Jones and William Morris. There is also an example of Frank Lloyd Wright's work in the collection. 20th-century designers include Harry Clarke, John Piper, Patrick Reyntiens, Veronica Whall and Brian Clarke.", "There are a set of beautiful inlaid doors, dated 1580 from Antwerp City Hall, attributed to Hans Vredeman de Vries. One of the finest pieces of continental furniture in the collection is the Rococo Augustus Rex Bureau Cabinet dated c1750 from Germany, with especially fine marquetry and ormolu mounts. One of the grandest pieces of 19th-century furniture is the highly elaborate French Cabinet dated 1861–1867 made by M. Fourdinois, made from ebony inlaid with box, lime, holly, pear, walnut and mahogany woods as well as marble with gilded carvings. Furniture designed by Ernest Gimson, Edward William Godwin, Charles Voysey, Adolf Loos and Otto Wagner are among the late 19th-century and early 20th-century examples in the collection. The work of modernists in the collection include Le Corbusier, Marcel Breuer, Charles and Ray Eames, and Giò Ponti.", "The main gallery was redesigned in 1994, the glass balustrade on the staircase and mezzanine are the work of Danny Lane, the gallery covering contemporary glass opened in 2004 and the sacred silver and stained-glass gallery in 2005. In this latter gallery stained glass is displayed alongside silverware starting in the 12th century and continuing to the present. Some of the most outstanding stained glass, dated 1243–48 comes from the Sainte-Chapelle, is displayed along with other examples in the new Medieval &amp; Renaissance galleries. The important 13th-century glass beaker known as the Luck of Edenhall is also displayed in these galleries. Examples of British stained glass are displayed in the British Galleries. One of the most spectacular items in the collection is the chandelier by Dale Chihuly in the rotunda at the Museum's main entrance.", "Well represented in the collection is Meissen porcelain, from the first factory in Europe to discover the Chinese method of making porcelain. Among the finest examples are the Meissen Vulture from 1731 and the Möllendorff Dinner Service, designed in 1762 by Frederick II the Great. Ceramics from the Manufacture nationale de Sèvres are extensive, especially from the 18th and 19th centuries. The collection of 18th-century British porcelain is the largest and finest in the world. Examples from every factory are represented, the collections of Chelsea porcelain and Worcester Porcelain being especially fine. All the major 19th-century British factories are also represented. A major boost to the collections was the Salting Bequest made in 1909, which enriched the museum's stock of Chinese and Japanese ceramics. This bequest forms part of the finest collection of East Asian pottery and porcelain in the world, including Kakiemon ware.", "There are over 10,000 objects made from silver or gold in the collection, the display (about 15% of the collection) is divided into secular and sacred covering both Christian (Roman Catholic, Anglican and Greek Orthodox) and Jewish liturgical vessels and items. The main silver gallery is divided into these areas: British silver pre-1800; British silver 1800 to 1900; modernist to contemporary silver; European silver. The collection includes the earliest known piece of English silver with a dated hallmark, a silver gilt beaker dated 1496–97. Silversmiths' whose work is represented in the collection include Paul de Lamerie and Paul Storr whose Castlereagh Inkstand dated 1817–19 is one of his finest works. The main iron work gallery covers European wrought and cast iron from the mediaeval period to the early 20th century. The master of wrought ironwork Jean Tijou is represented by both examples of his work and designs on paper. One of the largest items is the Hereford Screen, weighing nearly 8 tonnes, 10.5 metres high and 11 metres wide, designed by Sir George Gilbert Scott in 1862 for the chancel in Hereford Cathedral, from which it was removed in 1967. It was made by Skidmore &amp; Company. Its structure of"]</t>
-        </is>
-      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -6798,21 +4743,6 @@
 Chloroplasts' main role is to conduct photosynthesis, where the photosynthetic pigment chlorophyll captures the energy from sunlight and converts it and stores it in the energy-storage molecules ATP and NADPH while freeing oxygen from water. They then use the ATP and NADPH to make organic molecules from carbon dioxide in a process known as the Calvin cycle. Chloroplasts carry out a number of other functions, including fatty acid synthesis, much amino acid synthesis, and the immune response in plants. The number of chloroplasts per cell varies from 1 in algae up to 100 in plants like Arabidopsis and wheat.</t>
         </is>
       </c>
-      <c r="F138" t="inlineStr">
-        <is>
-          <t>[136, 513, 367, 90, 360]</t>
-        </is>
-      </c>
-      <c r="G138" t="inlineStr">
-        <is>
-          <t>[0.8271632194519043, 0.7493924498558044, 0.7312986850738525, 0.7051749229431152, 0.6963510513305664]</t>
-        </is>
-      </c>
-      <c r="H138" t="inlineStr">
-        <is>
-          <t>["In cpDNA, there are several A → G deamination gradients. DNA becomes susceptible to deamination events when it is single stranded. When replication forks form, the strand not being copied is single stranded, and thus at risk for A → G deamination. Therefore, gradients in deamination indicate that replication forks were most likely present and the direction that they initially opened (the highest gradient is most likely nearest the start site because it was single stranded for the longest amount of time). This mechanism is still the leading theory today; however, a second theory suggests that most cpDNA is actually linear and replicates through homologous recombination. It further contends that only a minority of the genetic material is kept in circular chromosomes while the rest is in branched, linear, or other complex structures.", "The inverted repeat regions are highly conserved among land plants, and accumulate few mutations. Similar inverted repeats exist in the genomes of cyanobacteria and the other two chloroplast lineages (glaucophyta and rhodophyceæ), suggesting that they predate the chloroplast, though some chloroplast DNAs have since lost or flipped the inverted repeats (making them direct repeats). It is possible that the inverted repeats help stabilize the rest of the chloroplast genome, as chloroplast DNAs which have lost some of the inverted repeat segments tend to get rearranged more.", "It is likely that a multicomponent, adaptive immune system arose with the first vertebrates, as invertebrates do not generate lymphocytes or an antibody-based humoral response. Many species, however, utilize mechanisms that appear to be precursors of these aspects of vertebrate immunity. Immune systems appear even in the structurally most simple forms of life, with bacteria using a unique defense mechanism, called the restriction modification system to protect themselves from viral pathogens, called bacteriophages. Prokaryotes also possess acquired immunity, through a system that uses CRISPR sequences to retain fragments of the genomes of phage that they have come into contact with in the past, which allows them to block virus replication through a form of RNA interference. Offensive elements of the immune systems are also present in unicellular eukaryotes, but studies of their roles in defense are few.", "One of the main functions of the chloroplast is its role in photosynthesis, the process by which light is transformed into chemical energy, to subsequently produce food in the form of sugars. Water (H2O) and carbon dioxide (CO2) are used in photosynthesis, and sugar and oxygen (O2) is made, using light energy. Photosynthesis is divided into two stages—the light reactions, where water is split to produce oxygen, and the dark reactions, or Calvin cycle, which builds sugar molecules from carbon dioxide. The two phases are linked by the energy carriers adenosine triphosphate (ATP) and nicotinamide adenine dinucleotide phosphate (NADP+).", "Chloroplasts' main role is to conduct photosynthesis, where the photosynthetic pigment chlorophyll captures the energy from sunlight and converts it and stores it in the energy-storage molecules ATP and NADPH while freeing oxygen from water. They then use the ATP and NADPH to make organic molecules from carbon dioxide in a process known as the Calvin cycle. Chloroplasts carry out a number of other functions, including fatty acid synthesis, much amino acid synthesis, and the immune response in plants. The number of chloroplasts per cell varies from 1 in algae up to 100 in plants like Arabidopsis and wheat."]</t>
-        </is>
-      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -6844,21 +4774,6 @@
 Parliament typically sits Tuesdays, Wednesdays and Thursdays from early January to late June and from early September to mid December, with two-week recesses in April and October. Plenary meetings in the debating chamber usually take place on Wednesday afternoons from 2 pm to 6 pm and on Thursdays from 9:15 am to 6 pm. Chamber debates and committee meetings are open to the public. Entry is free, but booking in advance is recommended due to limited space. Meetings are broadcast on the Parliament's own channel Holyrood.tv and on the BBC's parliamentary channel BBC Parliament. Proceedings are also recorded in text form, in print and online, in the Official Report, which is the substantially verbatim transcript of parliamentary debates.</t>
         </is>
       </c>
-      <c r="F139" t="inlineStr">
-        <is>
-          <t>[137, 635, 714, 653, 208]</t>
-        </is>
-      </c>
-      <c r="G139" t="inlineStr">
-        <is>
-          <t>[0.7924456596374512, 0.7858152389526367, 0.7742476463317871, 0.7622222900390625, 0.7582756280899048]</t>
-        </is>
-      </c>
-      <c r="H139" t="inlineStr">
-        <is>
-          <t>["Following a referendum in 1997, in which the Scottish electorate voted for devolution, the current Parliament was convened by the Scotland Act 1998, which sets out its powers as a devolved legislature. The Act delineates the legislative competence of the Parliament – the areas in which it can make laws – by explicitly specifying powers that are \"reserved\" to the Parliament of the United Kingdom. The Scottish Parliament has the power to legislate in all areas that are not explicitly reserved to Westminster. The British Parliament retains the ability to amend the terms of reference of the Scottish Parliament, and can extend or reduce the areas in which it can make laws. The first meeting of the new Parliament took place on 12 May 1999.", "Under the Scotland Act 1998, ordinary general elections for the Scottish Parliament are held on the first Thursday in May every four years (1999, 2003, 2007 and so on). The date of the poll may be varied by up to one month either way by the Monarch on the proposal of the Presiding Officer. If the Parliament itself resolves that it should be dissolved (with at least two-thirds of the Members voting in favour), or if the Parliament fails to nominate one of its members to be First Minister within 28 days of a General Election or of the position becoming vacant, the Presiding Officer proposes a date for an extraordinary general election and the Parliament is dissolved by the Queen by royal proclamation. Extraordinary general elections are in addition to ordinary general elections, unless held less than six months before the due date of an ordinary general election, in which case they supplant it. The following ordinary election reverts to the first Thursday in May, a multiple of four years after 1999 (i.e., 5 May 2011, 7 May 2015, etc.).", "A procedural consequence of the establishment of the Scottish Parliament is that Scottish MPs sitting in the UK House of Commons are able to vote on domestic legislation that applies only to England, Wales and Northern Ireland – whilst English, Scottish, Welsh and Northern Irish Westminster MPs are unable to vote on the domestic legislation of the Scottish Parliament. This phenomenon is known as the West Lothian question and has led to criticism. Following the Conservative victory in the 2015 UK election, standing orders of the House of Commons were changed to give MPs representing English constituencies a new \"veto\" over laws only affecting England.", "Royal assent: After the bill has been passed, the Presiding Officer submits it to the Monarch for royal assent and it becomes an Act of the Scottish Parliament. However he cannot do so until a 4-week period has elapsed, during which the Law Officers of the Scottish Government or UK Government can refer the bill to the Supreme Court of the United Kingdom for a ruling on whether it is within the powers of the Parliament. Acts of the Scottish Parliament do not begin with a conventional enacting formula. Instead they begin with a phrase that reads: \"The Bill for this Act of the Scottish Parliament was passed by the Parliament on [Date] and received royal assent on [Date]\".", "Parliament typically sits Tuesdays, Wednesdays and Thursdays from early January to late June and from early September to mid December, with two-week recesses in April and October. Plenary meetings in the debating chamber usually take place on Wednesday afternoons from 2 pm to 6 pm and on Thursdays from 9:15 am to 6 pm. Chamber debates and committee meetings are open to the public. Entry is free, but booking in advance is recommended due to limited space. Meetings are broadcast on the Parliament's own channel Holyrood.tv and on the BBC's parliamentary channel BBC Parliament. Proceedings are also recorded in text form, in print and online, in the Official Report, which is the substantially verbatim transcript of parliamentary debates."]</t>
-        </is>
-      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -6890,21 +4805,6 @@
 In the early 1950s, student applications declined as a result of increasing crime and poverty in the Hyde Park neighborhood. In response, the university became a major sponsor of a controversial urban renewal project for Hyde Park, which profoundly affected both the neighborhood's architecture and street plan. During this period the university, like Shimer College and 10 others, adopted an early entrant program that allowed very young students to attend college; in addition, students enrolled at Shimer were enabled to transfer automatically to the University of Chicago after their second year, having taken comparable or identical examinations and courses.</t>
         </is>
       </c>
-      <c r="F140" t="inlineStr">
-        <is>
-          <t>[138, 174, 442, 3, 437]</t>
-        </is>
-      </c>
-      <c r="G140" t="inlineStr">
-        <is>
-          <t>[0.852772057056427, 0.803546667098999, 0.7973294258117676, 0.7633465528488159, 0.7603757977485657]</t>
-        </is>
-      </c>
-      <c r="H140" t="inlineStr">
-        <is>
-          <t>["After the 1940s, the Gothic style on campus began to give way to modern styles. In 1955, Eero Saarinen was contracted to develop a second master plan, which led to the construction of buildings both north and south of the Midway, including the Laird Bell Law Quadrangle (a complex designed by Saarinen); a series of arts buildings; a building designed by Ludwig Mies van der Rohe for the university's School of Social Service Administration;, a building which is to become the home of the Harris School of Public Policy Studies by Edward Durrell Stone, and the Regenstein Library, the largest building on campus, a brutalist structure designed by Walter Netsch of the Chicago firm Skidmore, Owings &amp; Merrill. Another master plan, designed in 1999 and updated in 2004, produced the Gerald Ratner Athletics Center (2003), the Max Palevsky Residential Commons (2001), South Campus Residence Hall and dining commons (2009), a new children's hospital, and other construction, expansions, and restorations. In 2011, the university completed the glass dome-shaped Joe and Rika Mansueto Library, which provides a grand reading room for the university library and prevents the need for an off-campus book depository.", "The first buildings of the University of Chicago campus, which make up what is now known as the Main Quadrangles, were part of a \"master plan\" conceived by two University of Chicago trustees and plotted by Chicago architect Henry Ives Cobb. The Main Quadrangles consist of six quadrangles, each surrounded by buildings, bordering one larger quadrangle. The buildings of the Main Quadrangles were designed by Cobb, Shepley, Rutan and Coolidge, Holabird &amp; Roche, and other architectural firms in a mixture of the Victorian Gothic and Collegiate Gothic styles, patterned on the colleges of the University of Oxford. (Mitchell Tower, for example, is modeled after Oxford's Magdalen Tower, and the university Commons, Hutchinson Hall, replicates Christ Church Hall.)", "University of Chicago scholars have played a major role in the development of various academic disciplines, including: the Chicago school of economics, the Chicago school of sociology, the law and economics movement in legal analysis, the Chicago school of literary criticism, the Chicago school of religion, and the behavioralism school of political science. Chicago's physics department helped develop the world's first man-made, self-sustaining nuclear reaction beneath the university's Stagg Field. Chicago's research pursuits have been aided by unique affiliations with world-renowned institutions like the nearby Fermilab and Argonne National Laboratory, as well as the Marine Biological Laboratory. The university is also home to the University of Chicago Press, the largest university press in the United States. With an estimated completion date of 2020, the Barack Obama Presidential Center will be housed at the university and include both the Obama presidential library and offices of the Obama Foundation.", "The university runs a number of academic institutions and programs apart from its undergraduate and postgraduate schools. It operates the University of Chicago Laboratory Schools (a private day school for K-12 students and day care), the Sonia Shankman Orthogenic School (a residential treatment program for those with behavioral and emotional problems), and four public charter schools on the South Side of Chicago administered by the university's Urban Education Institute. In addition, the Hyde Park Day School, a school for students with learning disabilities, maintains a location on the University of Chicago campus. Since 1983, the University of Chicago has maintained the University of Chicago School Mathematics Project, a mathematics program used in urban primary and secondary schools. The university runs a program called the Council on Advanced Studies in the Social Sciences and Humanities, which administers interdisciplinary workshops to provide a forum for graduate students, faculty, and visiting scholars to present scholarly work in progress. The university also operates the University of Chicago Press, the largest university press in the United States.", "In the early 1950s, student applications declined as a result of increasing crime and poverty in the Hyde Park neighborhood. In response, the university became a major sponsor of a controversial urban renewal project for Hyde Park, which profoundly affected both the neighborhood's architecture and street plan. During this period the university, like Shimer College and 10 others, adopted an early entrant program that allowed very young students to attend college; in addition, students enrolled at Shimer were enabled to transfer automatically to the University of Chicago after their second year, having taken comparable or identical examinations and courses."]</t>
-        </is>
-      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -6936,21 +4836,6 @@
 creating "synforms". If the tops of the rock units within the folds remain pointing upwards, they are called anticlines and synclines, respectively. If some of the units in the fold are facing downward, the structure is called an overturned anticline or syncline, and if all of the rock units are overturned or the correct up-direction is unknown, they are simply called by the most general terms, antiforms and synforms.</t>
         </is>
       </c>
-      <c r="F141" t="inlineStr">
-        <is>
-          <t>[139, 15, 590, 254, 218]</t>
-        </is>
-      </c>
-      <c r="G141" t="inlineStr">
-        <is>
-          <t>[0.8771372437477112, 0.8268440365791321, 0.7657442688941956, 0.7654327154159546, 0.7450404763221741]</t>
-        </is>
-      </c>
-      <c r="H141" t="inlineStr">
-        <is>
-          <t>["In the laboratory, biostratigraphers analyze rock samples from outcrop and drill cores for the fossils found in them. These fossils help scientists to date the core and to understand the depositional environment in which the rock units formed. Geochronologists precisely date rocks within the stratigraphic section in order to provide better absolute bounds on the timing and rates of deposition. Magnetic stratigraphers look for signs of magnetic reversals in igneous rock units within the drill cores. Other scientists perform stable isotope studies on the rocks to gain information about past climate.", "For many geologic applications, isotope ratios of radioactive elements are measured in minerals that give the amount of time that has passed since a rock passed through its particular closure temperature, the point at which different radiometric isotopes stop diffusing into and out of the crystal lattice. These are used in geochronologic and thermochronologic studies. Common methods include uranium-lead dating, potassium-argon dating, argon-argon dating and uranium-thorium dating. These methods are used for a variety of applications. Dating of lava and volcanic ash layers found within a stratigraphic sequence can provide absolute age data for sedimentary rock units which do not contain radioactive isotopes and calibrate relative dating techniques. These methods can also be used to determine ages of pluton emplacement. Thermochemical techniques can be used to determine temperature profiles within the crust, the uplift of mountain ranges, and paleotopography.", "Among the most well-known experiments in structural geology are those involving orogenic wedges, which are zones in which mountains are built along convergent tectonic plate boundaries. In the analog versions of these experiments, horizontal layers of sand are pulled along a lower surface into a back stop, which results in realistic-looking patterns of faulting and the growth of a critically tapered (all angles remain the same) orogenic wedge. Numerical models work in the same way as these analog models, though they are often more sophisticated and can include patterns of erosion and uplift in the mountain belt. This helps to show the relationship between erosion and the shape of the mountain range. These studies can also give useful information about pathways for metamorphism through pressure, temperature, space, and time.", "The principle of inclusions and components states that, with sedimentary rocks, if inclusions (or clasts) are found in a formation, then the inclusions must be older than the formation that contains them. For example, in sedimentary rocks, it is common for gravel from an older formation to be ripped up and included in a newer layer. A similar situation with igneous rocks occurs when xenoliths are found. These foreign bodies are picked up as magma or lava flows, and are incorporated, later to cool in the matrix. As a result, xenoliths are older than the rock which contains them.", "creating \"synforms\". If the tops of the rock units within the folds remain pointing upwards, they are called anticlines and synclines, respectively. If some of the units in the fold are facing downward, the structure is called an overturned anticline or syncline, and if all of the rock units are overturned or the correct up-direction is unknown, they are simply called by the most general terms, antiforms and synforms."]</t>
-        </is>
-      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -6982,21 +4867,6 @@
 were designed by Reuben Townroe who also designed the plaster work in the library, Sir John Taylor designed the book shelves and cases, also this was the first part of the museum to have electric lighting. This completed the northern half of the site, creating a quadrangle with the garden at its centre, but left the museum without a proper façade. In 1890 the government launched a competition to design new buildings for the museum, with architect Alfred Waterhouse as one of the judges; this would give the museum a new imposing front entrance.</t>
         </is>
       </c>
-      <c r="F142" t="inlineStr">
-        <is>
-          <t>[560, 561, 582, 738, 588]</t>
-        </is>
-      </c>
-      <c r="G142" t="inlineStr">
-        <is>
-          <t>[0.7206369638442993, 0.7194111943244934, 0.7177601456642151, 0.7171826958656311, 0.7160288095474243]</t>
-        </is>
-      </c>
-      <c r="H142" t="inlineStr">
-        <is>
-          <t>["The official opening by Queen Victoria was on 22 June 1857. In the following year, late night openings were introduced, made possible by the use of gas lighting. This was to enable in the words of Cole \"to ascertain practically what hours are most convenient to the working classes\"—this was linked to the use of the collections of both applied art and science as educational resources to help boost productive industry. In these early years the practical use of the collection was very much emphasised as opposed to that of \"High Art\" at the National Gallery and scholarship at the British Museum. George Wallis (1811–1891), the first Keeper of Fine Art Collection, passionately promoted the idea of wide art education through the museum collections. This led to the transfer to the museum of the School of Design that had been founded in 1837 at Somerset House; after the transfer it was referred to as the Art School or Art Training School, later to become the Royal College of Art which finally achieved full independence in 1949. From the 1860s to the 1880s the scientific collections had been moved from the main museum site to various improvised galleries to the west", "was referred to as the Art School or Art Training School, later to become the Royal College of Art which finally achieved full independence in 1949. From the 1860s to the 1880s the scientific collections had been moved from the main museum site to various improvised galleries to the west of Exhibition Road. In 1893 the \"Science Museum\" had effectively come into existence when a separate director was appointed.", "The fourth Yuan emperor, Buyantu Khan (Ayurbarwada), was a competent emperor. He was the first Yuan emperor to actively support and adopt mainstream Chinese culture after the reign of Kublai, to the discontent of some Mongol elite. He had been mentored by Li Meng, a Confucian academic. He made many reforms, including the liquidation of the Department of State Affairs (Chinese: 尚書省), which resulted in the execution of five of the highest-ranking officials. Starting in 1313 the traditional imperial examinations were reintroduced for prospective officials, testing their knowledge on significant historical works. Also, he codified much of the law, as well as publishing or translating a number of Chinese books and works.", "The Literary and Philosophical Society of Newcastle upon Tyne (popularly known as the 'Lit &amp; Phil') is the largest independent library outside London, housing more than 150,000 books. Its music library contains 8000 CDs and 10,000 LPs. The current Lit and Phil premises were built in 1825 and the building was designed by John and Benjamin Green. Operating since 1793 and founded as a ‘conversation club,’ its lecture theatre was the first public building to be lit by electric light, during a lecture by Joseph Swan on 20 October 1880.", "were designed by Reuben Townroe who also designed the plaster work in the library, Sir John Taylor designed the book shelves and cases, also this was the first part of the museum to have electric lighting. This completed the northern half of the site, creating a quadrangle with the garden at its centre, but left the museum without a proper façade. In 1890 the government launched a competition to design new buildings for the museum, with architect Alfred Waterhouse as one of the judges; this would give the museum a new imposing front entrance."]</t>
-        </is>
-      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -7028,21 +4898,6 @@
 Between 1402 and 1405, the expedition led by the Norman noble Jean de Bethencourt and the Poitevine Gadifer de la Salle conquered the Canarian islands of Lanzarote, Fuerteventura and El Hierro off the Atlantic coast of Africa. Their troops were gathered in Normandy, Gascony and were later reinforced by Castilian colonists.</t>
         </is>
       </c>
-      <c r="F143" t="inlineStr">
-        <is>
-          <t>[141, 594, 32, 5, 55]</t>
-        </is>
-      </c>
-      <c r="G143" t="inlineStr">
-        <is>
-          <t>[0.8538378477096558, 0.7453623414039612, 0.7393973469734192, 0.7287804484367371, 0.7280310988426208]</t>
-        </is>
-      </c>
-      <c r="H143" t="inlineStr">
-        <is>
-          <t>["The African Great Lakes region, which Kenya is a part of, has been inhabited by humans since the Lower Paleolithic period. By the first millennium AD, the Bantu expansion had reached the area from West-Central Africa. The borders of the modern state consequently comprise the crossroads of the Niger-Congo, Nilo-Saharan and Afroasiatic areas of the continent, representing most major ethnolinguistic groups found in Africa. Bantu and Nilotic populations together constitute around 97% of the nation's residents. European and Arab presence in coastal Mombasa dates to the Early Modern period; European exploration of the interior began in the 19th century. The British Empire established the East Africa Protectorate in 1895, which starting in 1920 gave way to the Kenya Colony. Kenya obtained independence in December 1963. Following a referendum in August 2010 and adoption of a new constitution, Kenya is now divided into 47 semi-autonomous counties, governed by elected governors.", "Following the Cretaceous–Paleogene extinction event, the extinction of the dinosaurs and the wetter climate may have allowed the tropical rainforest to spread out across the continent. From 66–34 Mya, the rainforest extended as far south as 45°. Climate fluctuations during the last 34 million years have allowed savanna regions to expand into the tropics. During the Oligocene, for example, the rainforest spanned a relatively narrow band. It expanded again during the Middle Miocene, then retracted to a mostly inland formation at the last glacial maximum. However, the rainforest still managed to thrive during these glacial periods, allowing for the survival and evolution of a broad diversity of species.", "The Swahili built Mombasa into a major port city and established trade links with other nearby city-states, as well as commercial centres in Persia, Arabia, and even India. By the 15th-century, Portuguese voyager Duarte Barbosa claimed that \"Mombasa is a place of great traffic and has a good harbour in which there are always moored small craft of many kinds and also great ships, both of which are bound from Sofala and others which come from Cambay and Melinde and others which sail to the island of Zanzibar.\"", "The first European to travel the length of the Amazon River was Francisco de Orellana in 1542. The BBC's Unnatural Histories presents evidence that Orellana, rather than exaggerating his claims as previously thought, was correct in his observations that a complex civilization was flourishing along the Amazon in the 1540s. It is believed that the civilization was later devastated by the spread of diseases from Europe, such as smallpox. Since the 1970s, numerous geoglyphs have been discovered on deforested land dating between AD 0–1250, furthering claims about Pre-Columbian civilizations. Ondemar Dias is accredited with first discovering the geoglyphs in 1977 and Alceu Ranzi with furthering their discovery after flying over Acre. The BBC's Unnatural Histories presented evidence that the Amazon rainforest, rather than being a pristine wilderness, has been shaped by man for at least 11,000 years through practices such as forest gardening and terra preta.", "Between 1402 and 1405, the expedition led by the Norman noble Jean de Bethencourt and the Poitevine Gadifer de la Salle conquered the Canarian islands of Lanzarote, Fuerteventura and El Hierro off the Atlantic coast of Africa. Their troops were gathered in Normandy, Gascony and were later reinforced by Castilian colonists."]</t>
-        </is>
-      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -7074,21 +4929,6 @@
 in January 2015, Oxfam reported that the wealthiest 1 percent will own more than half of the global wealth by 2016. An October 2014 study by Credit Suisse also claims that the top 1% now own nearly half of the world's wealth and that the accelerating disparity could trigger a recession. In October 2015, Credit Suisse published a study which shows global inequality continues to increase, and that half of the world's wealth is now in the hands of those in the top percentile, whose assets each exceed $759,900. A 2016 report by Oxfam claims that the 62 wealthiest individuals own as much wealth as the poorer half of the global population combined. Oxfam's claims have however been questioned on the basis of the methodology used: by using net wealth (adding up assets and subtracting debts), the Oxfam report, for instance, finds that there are more poor people in the United States and Western Europe than in China (due to a greater tendency to take on debts).[unreliable source?][unreliable source?] Anthony Shorrocks, the lead author of the Credit Suisse report which is one of the sources of Oxfam's data, considers the criticism about debt to be a "silly argument" and "a</t>
         </is>
       </c>
-      <c r="F144" t="inlineStr">
-        <is>
-          <t>[142, 691, 102, 819, 826]</t>
-        </is>
-      </c>
-      <c r="G144" t="inlineStr">
-        <is>
-          <t>[0.883831262588501, 0.787255048751831, 0.7612414956092834, 0.7429308891296387, 0.7117429971694946]</t>
-        </is>
-      </c>
-      <c r="H144" t="inlineStr">
-        <is>
-          <t>["Harvard has the largest university endowment in the world. As of September 2011[update], it had nearly regained the loss suffered during the 2008 recession. It was worth $32 billion in 2011, up from $28 billion in September 2010 and $26 billion in 2009. It suffered about 30% loss in 2008-09. In December 2008, Harvard announced that its endowment had lost 22% (approximately $8 billion) from July to October 2008, necessitating budget cuts. Later reports suggest the loss was actually more than double that figure, a reduction of nearly 50% of its endowment in the first four months alone. Forbes in March 2009 estimated the loss to be in the range of $12 billion. One of the most visible results of Harvard's attempt to re-balance its budget was their halting of construction of the $1.2 billion Allston Science Complex that had been scheduled to be completed by 2011, resulting in protests from local residents. As of 2012[update], Harvard University had a total financial aid reserve of $159 million for students, and a Pell Grant reserve of $4.093 million available for disbursement.", "From the mid-2000s, the university began a number of multimillion-dollar expansion projects. In 2008, the University of Chicago announced plans to establish the Milton Friedman Institute which attracted both support and controversy from faculty members and students. The institute will cost around $200 million and occupy the buildings of the Chicago Theological Seminary. During the same year, investor David G. Booth donated $300 million to the university's Booth School of Business, which is the largest gift in the university's history and the largest gift ever to any business school. In 2009, planning or construction on several new buildings, half of which cost $100 million or more, was underway. Since 2011, major construction projects have included the Jules and Gwen Knapp Center for Biomedical Discovery, a ten-story medical research center, and further additions to the medical campus of the University of Chicago Medical Center. In 2014 the University launched the public phase of a $4.5 billion fundraising campaign. In September 2015, the University received $100 million from The Pearson Family Foundation to establish The Pearson Institute for the Study and Resolution of Global Conflicts and The Pearson Global Forum at the Harris School of Public Policy Studies.", "Harvard's 2,400 professors, lecturers, and instructors instruct 7,200 undergraduates and 14,000 graduate students. The school color is crimson, which is also the name of the Harvard sports teams and the daily newspaper, The Harvard Crimson. The color was unofficially adopted (in preference to magenta) by an 1875 vote of the student body, although the association with some form of red can be traced back to 1858, when Charles William Eliot, a young graduate student who would later become Harvard's 21st and longest-serving president (1869–1909), bought red bandanas for his crew so they could more easily be distinguished by spectators at a regatta.", "For the 2012–13 school year annual tuition was $38,000, with a total cost of attendance of $57,000. Beginning 2007, families with incomes below $60,000 pay nothing for their children to attend, including room and board. Families with incomes between $60,000 to $80,000 pay only a few thousand dollars per year, and families earning between $120,000 and $180,000 pay no more than 10% of their annual incomes. In 2009, Harvard offered grants totaling $414 million across all eleven divisions;[further explanation needed] $340 million came from institutional funds, $35 million from federal support, and $39 million from other outside support. Grants total 88% of Harvard's aid for undergraduate students, with aid also provided by loans (8%) and work-study (4%).", "in January 2015, Oxfam reported that the wealthiest 1 percent will own more than half of the global wealth by 2016. An October 2014 study by Credit Suisse also claims that the top 1% now own nearly half of the world's wealth and that the accelerating disparity could trigger a recession. In October 2015, Credit Suisse published a study which shows global inequality continues to increase, and that half of the world's wealth is now in the hands of those in the top percentile, whose assets each exceed $759,900. A 2016 report by Oxfam claims that the 62 wealthiest individuals own as much wealth as the poorer half of the global population combined. Oxfam's claims have however been questioned on the basis of the methodology used: by using net wealth (adding up assets and subtracting debts), the Oxfam report, for instance, finds that there are more poor people in the United States and Western Europe than in China (due to a greater tendency to take on debts).[unreliable source?][unreliable source?] Anthony Shorrocks, the lead author of the Credit Suisse report which is one of the sources of Oxfam's data, considers the criticism about debt to be a \"silly argument\" and \"a"]</t>
-        </is>
-      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -7120,21 +4960,6 @@
 "wide test", to determine what could potentially be an unlawful restriction on trade, applies equally to actions by quasi-government bodies, such as the former "Buy Irish" company that had government appointees. It also means states can be responsible for private actors. For instance, in Commission v France French farmer vigilantes were continually sabotaging shipments of Spanish strawberries, and even Belgian tomato imports. France was liable for these hindrances to trade because the authorities ‘manifestly and persistently abstained' from preventing the sabotage. Generally speaking, if a member state has laws or practices that directly discriminate against imports (or exports under TFEU article 35) then it must be justified under article 36. The justifications include public morality, policy or security, "protection of health and life of humans, animals or plants", "national treasures" of "artistic, historic or archaeological value" and "industrial and commercial property." In addition, although not clearly listed, environmental protection can justify restrictions on trade as an overriding requirement derived from TFEU article 11. More generally, it has been increasingly acknowledged that fundamental human rights should take priority over all trade rules. So, in Schmidberger v Austria the Court of Justice held that Austria did not infringe article 34 by failing</t>
         </is>
       </c>
-      <c r="F145" t="inlineStr">
-        <is>
-          <t>[143, 287, 876, 281, 837]</t>
-        </is>
-      </c>
-      <c r="G145" t="inlineStr">
-        <is>
-          <t>[0.8336015939712524, 0.7998631596565247, 0.7975821495056152, 0.7825984358787537, 0.7792646884918213]</t>
-        </is>
-      </c>
-      <c r="H145" t="inlineStr">
-        <is>
-          <t>["Citizenship of the EU has increasingly been seen as a \"fundamental\" status of member state nationals by the Court of Justice, and has accordingly increased the number of social services that people can access wherever they move. The Court has required that higher education, along with other forms of vocational training, should be more access, albeit with qualifying periods. In Commission v Austria the Court held that Austria was not entitled to restrict places in Austrian universities to Austrian students to avoid \"structural, staffing and financial problems\" if (mainly German) foreign students applied for places because there was little evidence of an actual problem.", "While the Treaties and Regulations will have direct effect (if clear, unconditional and immediate), Directives do not generally give citizens (as opposed to the member state) standing to sue other citizens. In theory, this is because TFEU article 288 says Directives are addressed to the member states and usually \"leave to the national authorities the choice of form and methods\" to implement. In part this reflects that directives often create minimum standards, leaving member states to apply higher standards. For example, the Working Time Directive requires that every worker has at least 4 weeks paid holidays each year, but most member states require more than 28 days in national law. However, on the current position adopted by the Court of Justice, citizens have standing to make claims based on national laws that implement Directives, but not from Directives themselves. Directives do not have so called \"horizontal\" direct effect (i.e. between non-state parties). This view was instantly controversial, and in the early 1990s three Advocate Generals persuasively argued that Directives should create rights and duties for all citizens. The Court of Justice refused, but there are five large exceptions.", "domestic legal provisions, however framed... without the legal basis of the community itself being called into question.\" This meant any \"subsequent unilateral act\" of the member state inapplicable. Similarly, in Amministrazione delle Finanze v Simmenthal SpA, a company, Simmenthal SpA, claimed that a public health inspection fee under an Italian law of 1970 for importing beef from France to Italy was contrary to two Regulations from 1964 and 1968. In \"accordance with the principle of the precedence of Community law,\" said the Court of Justice, the \"directly applicable measures of the institutions\" (such as the Regulations in the case) \"render automatically inapplicable any conflicting provision of current national law\". This was necessary to prevent a \"corresponding denial\" of Treaty \"obligations undertaken unconditionally and irrevocably by member states\", that could \"imperil the very foundations of the\" EU. But despite the views of the Court of Justice, the national courts of member states have not accepted the same analysis.", "justified as part of the public policy of promoting the Irish language, but only if the measure was not disproportionate. By contrast in Angonese v Cassa di Risparmio di Bolzano SpA a bank in Bolzano, Italy, was not allowed to require Mr Angonese to have a bilingual certificate that could only be obtained in Bolzano. The Court of Justice, giving \"horizontal\" direct effect to TFEU article 45, reasoned that people from other countries would have little chance of acquiring the certificate, and because it was \"impossible to submit proof of the required linguistic knowledge by any other means\", the measure was disproportionate. Second, article 7(2) requires equal treatment in respect of tax. In Finanzamt Köln Altstadt v Schumacker the Court of Justice held that it contravened TFEU art 45 to deny tax benefits (e.g. for married couples, and social insurance expense deductions) to a man who worked in Germany, but was resident in Belgium when other German residents got the benefits. By contrast in Weigel v Finanzlandesdirektion für Vorarlberg the Court of Justice rejected Mr Weigel's claim that a re-registration charge upon bringing his car to Austria violated his right to free movement. Although the tax was \"likely to have", "\"wide test\", to determine what could potentially be an unlawful restriction on trade, applies equally to actions by quasi-government bodies, such as the former \"Buy Irish\" company that had government appointees. It also means states can be responsible for private actors. For instance, in Commission v France French farmer vigilantes were continually sabotaging shipments of Spanish strawberries, and even Belgian tomato imports. France was liable for these hindrances to trade because the authorities ‘manifestly and persistently abstained' from preventing the sabotage. Generally speaking, if a member state has laws or practices that directly discriminate against imports (or exports under TFEU article 35) then it must be justified under article 36. The justifications include public morality, policy or security, \"protection of health and life of humans, animals or plants\", \"national treasures\" of \"artistic, historic or archaeological value\" and \"industrial and commercial property.\" In addition, although not clearly listed, environmental protection can justify restrictions on trade as an overriding requirement derived from TFEU article 11. More generally, it has been increasingly acknowledged that fundamental human rights should take priority over all trade rules. So, in Schmidberger v Austria the Court of Justice held that Austria did not infringe article 34 by failing"]</t>
-        </is>
-      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -7166,21 +4991,6 @@
 members of the Reformed Church) involved in the Amboise plot of 1560: a foiled attempt to wrest power in France from the influential House of Guise. The move would have had the side effect of fostering relations with the Swiss. Thus, Hugues plus Eidgenosse by way of Huisgenoten supposedly became Huguenot, a nickname associating the Protestant cause with politics unpopular in France.[citation needed]</t>
         </is>
       </c>
-      <c r="F146" t="inlineStr">
-        <is>
-          <t>[144, 267, 145, 212, 502]</t>
-        </is>
-      </c>
-      <c r="G146" t="inlineStr">
-        <is>
-          <t>[0.8115085363388062, 0.7892394065856934, 0.7887643575668335, 0.7864276766777039, 0.7811938524246216]</t>
-        </is>
-      </c>
-      <c r="H146" t="inlineStr">
-        <is>
-          <t>["The war in North America officially ended with the signing of the Treaty of Paris on 10 February 1763, and war in the European theatre of the Seven Years' War was settled by the Treaty of Hubertusburg on 15 February 1763. The British offered France the choice of surrendering either its continental North American possessions east of the Mississippi or the Caribbean islands of Guadeloupe and Martinique, which had been occupied by the British. France chose to cede the former, but was able to negotiate the retention of Saint Pierre and Miquelon, two small islands in the Gulf of St. Lawrence, along with fishing rights in the area. They viewed the economic value of the Caribbean islands' sugar cane to be greater and easier to defend than the furs from the continent. The contemporaneous French philosopher Voltaire referred to Canada disparagingly as nothing more than a few acres of snow. The British, for their part, were happy to take New France, as defence of their North American colonies would no longer be an issue and also because they already had ample places from which to obtain sugar. Spain, which traded Florida to Britain to regain Cuba, also gained Louisiana, including", "It became a moral justification to lift the world up to French standards by bringing Christianity and French culture. In 1884 the leading exponent of colonialism, Jules Ferry declared France had a civilising mission: \"The higher races have a right over the lower races, they have a duty to civilize the inferior\". Full citizenship rights – ‘’assimilation’’ – were offered, although in reality assimilation was always on the distant horizon. Contrasting from Britain, France sent small numbers of settlers to its colonies, with the only notable exception of Algeria, where French settlers nevertheless always remained a small minority.", "The British, for their part, were happy to take New France, as defence of their North American colonies would no longer be an issue and also because they already had ample places from which to obtain sugar. Spain, which traded Florida to Britain to regain Cuba, also gained Louisiana, including New Orleans, from France in compensation for its losses. Great Britain and Spain also agreed that navigation on the Mississippi River was to be open to vessels of all nations.", "Since the Peace of Westphalia, the Upper Rhine formed a contentious border between France and Germany. Establishing \"natural borders\" on the Rhine was a long-term goal of French foreign policy, since the Middle Ages, though the language border was – and is – far more to the west. French leaders, such as Louis XIV and Napoleon Bonaparte, tried with varying degrees of success to annex lands west of the Rhine. The Confederation of the Rhine was established by Napoleon, as a French client state, in 1806 and lasted until 1814, during which time it served as a significant source of resources and military manpower for the First French Empire. In 1840, the Rhine crisis, prompted by French prime minister Adolphe Thiers's desire to reinstate the Rhine as a natural border, led to a diplomatic crisis and a wave of nationalism in Germany.", "members of the Reformed Church) involved in the Amboise plot of 1560: a foiled attempt to wrest power in France from the influential House of Guise. The move would have had the side effect of fostering relations with the Swiss. Thus, Hugues plus Eidgenosse by way of Huisgenoten supposedly became Huguenot, a nickname associating the Protestant cause with politics unpopular in France.[citation needed]"]</t>
-        </is>
-      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -7212,21 +5022,6 @@
 A new arrangement of the theme, once again by Gold, was introduced in the 2007 Christmas special episode, "Voyage of the Damned"; Gold returned as composer for the 2010 series. He was responsible for a new version of the theme which was reported to have had a hostile reception from some viewers. In 2011, the theme tune charted at number 228 of radio station Classic FM's Hall of Fame, a survey of classical music tastes. A revised version of Gold's 2010 arrangement had its debut over the opening titles of the 2012 Christmas special "The Snowmen", and a further revision of the arrangement was made for the 50th Anniversary special "The Day of the Doctor" in November 2013.[citation needed]</t>
         </is>
       </c>
-      <c r="F147" t="inlineStr">
-        <is>
-          <t>[185, 776, 665, 868, 110]</t>
-        </is>
-      </c>
-      <c r="G147" t="inlineStr">
-        <is>
-          <t>[0.7909352779388428, 0.7883536219596863, 0.7875199317932129, 0.7869905233383179, 0.7815312147140503]</t>
-        </is>
-      </c>
-      <c r="H147" t="inlineStr">
-        <is>
-          <t>["10 July 2009, and consisted of a single five-part story called Children of Earth which was set largely in London. A fourth series, Torchwood: Miracle Day jointly produced by BBC Wales, BBC Worldwide and the American entertainment company Starz debuted in 2011. The series was predominantly set in the United States, though Wales remained part of the show's setting.", "as a selection of classics based on the theme of space and time. The event was presented by Freema Agyeman and guest-presented by various other stars of the show with numerous monsters participating in the proceedings. It also featured the specially filmed mini-episode \"Music of the Spheres\", written by Russell T Davies and starring David Tennant.", "The most frequent musical contributor during the first 15 years was Dudley Simpson, who is also well known for his theme and incidental music for Blake's 7, and for his haunting theme music and score for the original 1970s version of The Tomorrow People. Simpson's first Doctor Who score was Planet of Giants (1964) and he went on to write music for many adventures of the 1960s and 1970s, including most of the stories of the Jon Pertwee/Tom Baker periods, ending with The Horns of Nimon (1979). He also made a cameo appearance in The Talons of Weng-Chiang (as a Music hall conductor).", "Six soundtrack releases have been released since 2005. The first featured tracks from the first two series, the second and third featured music from the third and fourth series respectively. The fourth was released on 4 October 2010 as a two disc special edition and contained music from the 2008–2010 specials (The Next Doctor to End of Time Part 2). The soundtrack for Series 5 was released on 8 November 2010. In February 2011, a soundtrack was released for the 2010 Christmas special: \"A Christmas Carol\", and in December 2011 the soundtrack for Series 6 was released, both by Silva Screen Records.", "A new arrangement of the theme, once again by Gold, was introduced in the 2007 Christmas special episode, \"Voyage of the Damned\"; Gold returned as composer for the 2010 series. He was responsible for a new version of the theme which was reported to have had a hostile reception from some viewers. In 2011, the theme tune charted at number 228 of radio station Classic FM's Hall of Fame, a survey of classical music tastes. A revised version of Gold's 2010 arrangement had its debut over the opening titles of the 2012 Christmas special \"The Snowmen\", and a further revision of the arrangement was made for the 50th Anniversary special \"The Day of the Doctor\" in November 2013.[citation needed]"]</t>
-        </is>
-      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -7258,21 +5053,6 @@
 run for about 4 × 1010 years, which is the same order of magnitude as the age of the universe. Even with a much faster computer, the program would only be useful for very small instances and in that sense the intractability of a problem is somewhat independent of technological progress. Nevertheless, a polynomial time algorithm is not always practical. If its running time is, say, n15, it is unreasonable to consider it efficient and it is still useless except on small instances.</t>
         </is>
       </c>
-      <c r="F148" t="inlineStr">
-        <is>
-          <t>[147, 475, 278, 234, 605]</t>
-        </is>
-      </c>
-      <c r="G148" t="inlineStr">
-        <is>
-          <t>[0.853864312171936, 0.7969574928283691, 0.7945928573608398, 0.7939085960388184, 0.7922728061676025]</t>
-        </is>
-      </c>
-      <c r="H148" t="inlineStr">
-        <is>
-          <t>["But bounding the computation time above by some concrete function f(n) often yields complexity classes that depend on the chosen machine model. For instance, the language {xx | x is any binary string} can be solved in linear time on a multi-tape Turing machine, but necessarily requires quadratic time in the model of single-tape Turing machines. If we allow polynomial variations in running time, Cobham-Edmonds thesis states that \"the time complexities in any two reasonable and general models of computation are polynomially related\" (Goldreich 2008, Chapter 1.2). This forms the basis for the complexity class P, which is the set of decision problems solvable by a deterministic Turing machine within polynomial time. The corresponding set of function problems is FP.", "Many important complexity classes can be defined by bounding the time or space used by the algorithm. Some important complexity classes of decision problems defined in this manner are the following:", "However, some computational problems are easier to analyze in terms of more unusual resources. For example, a non-deterministic Turing machine is a computational model that is allowed to branch out to check many different possibilities at once. The non-deterministic Turing machine has very little to do with how we physically want to compute algorithms, but its branching exactly captures many of the mathematical models we want to analyze, so that non-deterministic time is a very important resource in analyzing computational problems.", "The most commonly used reduction is a polynomial-time reduction. This means that the reduction process takes polynomial time. For example, the problem of squaring an integer can be reduced to the problem of multiplying two integers. This means an algorithm for multiplying two integers can be used to square an integer. Indeed, this can be done by giving the same input to both inputs of the multiplication algorithm. Thus we see that squaring is not more difficult than multiplication, since squaring can be reduced to multiplication.", "run for about 4 × 1010 years, which is the same order of magnitude as the age of the universe. Even with a much faster computer, the program would only be useful for very small instances and in that sense the intractability of a problem is somewhat independent of technological progress. Nevertheless, a polynomial time algorithm is not always practical. If its running time is, say, n15, it is unreasonable to consider it efficient and it is still useless except on small instances."]</t>
-        </is>
-      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -7304,21 +5084,6 @@
 New techniques of building construction are being researched, made possible by advances in 3D printing technology. In a form of additive building construction, similar to the additive manufacturing techniques for manufactured parts, building printing is making it possible to flexibly construct small commercial buildings and private habitations in around 20 hours, with built-in plumbing and electrical facilities, in one continuous build, using large 3D printers. Working versions of 3D-printing building technology are already printing 2 metres (6 ft 7 in) of building material per hour as of January 2013[update], with the next-generation printers capable of 3.5 metres (11 ft) per hour, sufficient to complete a building in a week. Dutch architect Janjaap Ruijssenaars's performative architecture 3D-printed building is scheduled to be built in 2014.</t>
         </is>
       </c>
-      <c r="F149" t="inlineStr">
-        <is>
-          <t>[148, 788, 618, 433, 849]</t>
-        </is>
-      </c>
-      <c r="G149" t="inlineStr">
-        <is>
-          <t>[0.8248428106307983, 0.7767413258552551, 0.7594218254089355, 0.7554294466972351, 0.7536492943763733]</t>
-        </is>
-      </c>
-      <c r="H149" t="inlineStr">
-        <is>
-          <t>["Construction is the process of constructing a building or infrastructure. Construction differs from manufacturing in that manufacturing typically involves mass production of similar items without a designated purchaser, while construction typically takes place on location for a known client. Construction as an industry comprises six to nine percent of the gross domestic product of developed countries. Construction starts with planning,[citation needed] design, and financing and continues until the project is built and ready for use.", "Large-scale construction requires collaboration across multiple disciplines. An architect normally manages the job, and a construction manager, design engineer, construction engineer or project manager supervises it. For the successful execution of a project, effective planning is essential. Those involved with the design and execution of the infrastructure in question must consider zoning requirements, the environmental impact of the job, the successful scheduling, budgeting, construction-site safety, availability and transportation of building materials, logistics, inconvenience to the public caused by construction delays and bidding, etc. The largest construction projects are referred to as megaprojects.", "The owner produces a list of requirements for a project, giving an overall view of the project's goals. Several D&amp;B contractors present different ideas about how to accomplish these goals. The owner selects the ideas he or she likes best and hires the appropriate contractor. Often, it is not just one contractor, but a consortium of several contractors working together. Once these have been hired, they begin building the first phase of the project. As they build phase 1, they design phase 2. This is in contrast to a design-bid-build contract, where the project is completely designed by the owner, then bid on, then completed.", "The Standard Industrial Classification and the newer North American Industry Classification System have a classification system for companies that perform or otherwise engage in construction. To recognize the differences of companies in this sector, it is divided into three subsectors: building construction, heavy and civil engineering construction, and specialty trade contractors. There are also categories for construction service firms (e.g., engineering, architecture) and construction managers (firms engaged in managing construction projects without assuming direct financial responsibility for completion of the construction project).", "New techniques of building construction are being researched, made possible by advances in 3D printing technology. In a form of additive building construction, similar to the additive manufacturing techniques for manufactured parts, building printing is making it possible to flexibly construct small commercial buildings and private habitations in around 20 hours, with built-in plumbing and electrical facilities, in one continuous build, using large 3D printers. Working versions of 3D-printing building technology are already printing 2 metres (6 ft 7 in) of building material per hour as of January 2013[update], with the next-generation printers capable of 3.5 metres (11 ft) per hour, sufficient to complete a building in a week. Dutch architect Janjaap Ruijssenaars's performative architecture 3D-printed building is scheduled to be built in 2014."]</t>
-        </is>
-      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -7350,21 +5115,6 @@
 (1528), drafted by Melanchthon with Luther's approval, stressed the role of repentance in the forgiveness of sins, despite Luther's position that faith alone ensures justification. The Eisleben reformer Johannes Agricola challenged this compromise, and Luther condemned him for teaching that faith is separate from works. The Instruction is a problematic document for those seeking a consistent evolution in Luther's thought and practice.</t>
         </is>
       </c>
-      <c r="F150" t="inlineStr">
-        <is>
-          <t>[398, 412, 149, 627, 572]</t>
-        </is>
-      </c>
-      <c r="G150" t="inlineStr">
-        <is>
-          <t>[0.8185694813728333, 0.7945829033851624, 0.7945744395256042, 0.7945278286933899, 0.7913405299186707]</t>
-        </is>
-      </c>
-      <c r="H150" t="inlineStr">
-        <is>
-          <t>["Luther's rediscovery of \"Christ and His salvation\" was the first of two points that became the foundation for the Reformation. His railing against the sale of indulgences was based on it.", "The Lutheran theologian Franz Pieper observed that Luther's teaching about the state of the Christian's soul after death differed from the later Lutheran theologians such as Johann Gerhard. Lessing (1755) had earlier reached the same conclusion in his analysis of Lutheran orthodoxy on this issue.", "Luther came to understand justification as entirely the work of God. This teaching by Luther was clearly expressed in his 1525 publication On the Bondage of the Will, which was written in response to On Free Will by Desiderius Erasmus (1524). Luther based his position on predestination on St. Paul's epistle to the Ephesians 2:8–10. Against the teaching of his day that the righteous acts of believers are performed in cooperation with God, Luther wrote that Christians receive such righteousness entirely from outside themselves; that righteousness not only comes from Christ but actually is the righteousness of Christ, imputed to Christians (rather than infused into them) through faith. \"That is why faith alone makes someone just and fulfills the law,\" he wrote. \"Faith is that which brings the Holy Spirit through the merits of Christ.\" Faith, for Luther, was a gift from God; the experience of being justified by faith was \"as though I had been born again.\" His entry into Paradise, no less, was a discovery about \"the righteousness of God\" – a discovery that \"the just person\" of whom the Bible speaks (as in Romans 1:17) lives by faith. He explained his concept of \"justification\" in the Smalcald", "Martin Luther (/ˈluːθər/ or /ˈluːðər/; German: [ˈmaɐ̯tiːn ˈlʊtɐ] ( listen); 10 November 1483 – 18 February 1546) was a German professor of theology, composer, priest, former monk and a seminal figure in the Protestant Reformation. Luther came to reject several teachings and practices of the Late Medieval Catholic Church. He strongly disputed the claim that freedom from God's punishment for sin could be purchased with money. He proposed an academic discussion of the power and usefulness of indulgences in his Ninety-Five Theses of 1517. His refusal to retract all of his writings at the demand of Pope Leo X in 1520 and the Holy Roman Emperor Charles V at the Diet of Worms in 1521 resulted in his excommunication by the Pope and condemnation as an outlaw by the Emperor.", "(1528), drafted by Melanchthon with Luther's approval, stressed the role of repentance in the forgiveness of sins, despite Luther's position that faith alone ensures justification. The Eisleben reformer Johannes Agricola challenged this compromise, and Luther condemned him for teaching that faith is separate from works. The Instruction is a problematic document for those seeking a consistent evolution in Luther's thought and practice."]</t>
-        </is>
-      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -7396,21 +5146,6 @@
 Tesla theorized that the application of electricity to the brain enhanced intelligence. In 1912, he crafted "a plan to make dull students bright by saturating them unconsciously with electricity," wiring the walls of a schoolroom and, "saturating [the schoolroom] with infinitesimal electric waves vibrating at high frequency. The whole room will thus, Mr. Tesla claims, be converted into a health-giving and stimulating electromagnetic field or 'bath.'" The plan was, at least provisionally approved by then superintendent of New York City schools, William H. Maxwell.</t>
         </is>
       </c>
-      <c r="F151" t="inlineStr">
-        <is>
-          <t>[249, 667, 785, 685, 465]</t>
-        </is>
-      </c>
-      <c r="G151" t="inlineStr">
-        <is>
-          <t>[0.8116275668144226, 0.7915297746658325, 0.7729974985122681, 0.7597134113311768, 0.7563560605049133]</t>
-        </is>
-      </c>
-      <c r="H151" t="inlineStr">
-        <is>
-          <t>["Tesla invented a steam-powered mechanical oscillator—Tesla's oscillator. While experimenting with mechanical oscillators at his Houston Street lab, Tesla allegedly generated a resonance of several buildings. As the speed grew, it is said that the machine oscillated at the resonance frequency of his own building and, belatedly realizing the danger, he was forced to use a sledge hammer to terminate the experiment, just as the police arrived.:162–164 In February 1912, an article—\"Nikola Tesla, Dreamer\" by Allan L. Benson—was published in World Today, in which an artist's illustration appears showing the entire earth cracking in half with the caption, \"Tesla claims that in a few weeks he could set the earth's crust into such a state of vibration that it would rise and fall hundreds of feet and practically destroy civilization. A continuation of this process would, he says, eventually split the earth in two.\"", "Tesla investigated atmospheric electricity, observing lightning signals via his receivers. He stated that he observed stationary waves during this time. The great distances and the nature of what Tesla was detecting from lightning storms confirmed his belief that the earth had a resonant frequency.", "While experimenting, Tesla inadvertently faulted a power station generator, causing a power outage. In August 1917, Tesla explained what had happened in The Electrical Experimenter: \"As an example of what has been done with several hundred kilowatts of high frequency energy liberated, it was found that the dynamos in a power house six miles away were repeatedly burned out, due to the powerful high frequency currents set up in them, and which caused heavy sparks to jump through the windings and destroy the insulation!\"", "During the same year, Tesla wrote a treatise, The Art of Projecting Concentrated Non-dispersive Energy through the Natural Media, concerning charged particle beam weapons. Tesla published the document in an attempt to expound on the technical description of a \"superweapon that would put an end to all war.\" This treatise is currently in the Nikola Tesla Museum archive in Belgrade. It describes an open-ended vacuum tube with a gas jet seal that allows particles to exit, a method of charging particles to millions of volts, and a method of creating and directing non-dispersive particle streams (through electrostatic repulsion). Tesla tried to interest the US War Department, the United Kingdom, the Soviet Union, and Yugoslavia in the device.", "Tesla theorized that the application of electricity to the brain enhanced intelligence. In 1912, he crafted \"a plan to make dull students bright by saturating them unconsciously with electricity,\" wiring the walls of a schoolroom and, \"saturating [the schoolroom] with infinitesimal electric waves vibrating at high frequency. The whole room will thus, Mr. Tesla claims, be converted into a health-giving and stimulating electromagnetic field or 'bath.'\" The plan was, at least provisionally approved by then superintendent of New York City schools, William H. Maxwell."]</t>
-        </is>
-      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -7442,21 +5177,6 @@
 run for about 4 × 1010 years, which is the same order of magnitude as the age of the universe. Even with a much faster computer, the program would only be useful for very small instances and in that sense the intractability of a problem is somewhat independent of technological progress. Nevertheless, a polynomial time algorithm is not always practical. If its running time is, say, n15, it is unreasonable to consider it efficient and it is still useless except on small instances.</t>
         </is>
       </c>
-      <c r="F152" t="inlineStr">
-        <is>
-          <t>[152, 234, 71, 131, 605]</t>
-        </is>
-      </c>
-      <c r="G152" t="inlineStr">
-        <is>
-          <t>[0.8445632457733154, 0.7212565541267395, 0.7163801193237305, 0.7084491848945618, 0.6947909593582153]</t>
-        </is>
-      </c>
-      <c r="H152" t="inlineStr">
-        <is>
-          <t>["A function problem is a computational problem where a single output (of a total function) is expected for every input, but the output is more complex than that of a decision problem, that is, it isn't just yes or no. Notable examples include the traveling salesman problem and the integer factorization problem.", "The most commonly used reduction is a polynomial-time reduction. This means that the reduction process takes polynomial time. For example, the problem of squaring an integer can be reduced to the problem of multiplying two integers. This means an algorithm for multiplying two integers can be used to square an integer. Indeed, this can be done by giving the same input to both inputs of the multiplication algorithm. Thus we see that squaring is not more difficult than multiplication, since squaring can be reduced to multiplication.", "A computational problem can be viewed as an infinite collection of instances together with a solution for every instance. The input string for a computational problem is referred to as a problem instance, and should not be confused with the problem itself. In computational complexity theory, a problem refers to the abstract question to be solved. In contrast, an instance of this problem is a rather concrete utterance, which can serve as the input for a decision problem. For example, consider the problem of primality testing. The instance is a number (e.g. 15) and the solution is \"yes\" if the number is prime and \"no\" otherwise (in this case \"no\"). Stated another way, the instance is a particular input to the problem, and the solution is the output corresponding to the given input.", "A problem is regarded as inherently difficult if its solution requires significant resources, whatever the algorithm used. The theory formalizes this intuition, by introducing mathematical models of computation to study these problems and quantifying the amount of resources needed to solve them, such as time and storage. Other complexity measures are also used, such as the amount of communication (used in communication complexity), the number of gates in a circuit (used in circuit complexity) and the number of processors (used in parallel computing). One of the roles of computational complexity theory is to determine the practical limits on what computers can and cannot do.", "run for about 4 × 1010 years, which is the same order of magnitude as the age of the universe. Even with a much faster computer, the program would only be useful for very small instances and in that sense the intractability of a problem is somewhat independent of technological progress. Nevertheless, a polynomial time algorithm is not always practical. If its running time is, say, n15, it is unreasonable to consider it efficient and it is still useless except on small instances."]</t>
-        </is>
-      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -7488,21 +5208,6 @@
 The Taliban were spawned by the thousands of madrasahs the Deobandi movement established for impoverished Afghan refugees and supported by governmental and religious groups in neighboring Pakistan. The Taliban differed from other Islamist movements to the point where they might be more properly described as Islamic fundamentalist or neofundamentalist, interested in spreading "an idealized and systematized version of conservative tribal village customs" under the label of Sharia to an entire country. Their ideology was also described as being influenced by Wahhabism, and the extremist jihadism of their guest Osama bin Laden.</t>
         </is>
       </c>
-      <c r="F153" t="inlineStr">
-        <is>
-          <t>[153, 625, 386, 23, 258]</t>
-        </is>
-      </c>
-      <c r="G153" t="inlineStr">
-        <is>
-          <t>[0.8842718601226807, 0.8155586123466492, 0.8076122999191284, 0.8059468269348145, 0.78138667345047]</t>
-        </is>
-      </c>
-      <c r="H153" t="inlineStr">
-        <is>
-          <t>["Islamism is a controversial concept not just because it posits a political role for Islam but also because its supporters believe their views merely reflect Islam, while the contrary idea that Islam is, or can be, apolitical is an error. Scholars and observers who do not believe that Islam is merely a political ideology include Fred Halliday, John Esposito and Muslim intellectuals like Javed Ahmad Ghamidi. Hayri Abaza argues the failure to distinguish between Islam and Islamism leads many in the West to support illiberal Islamic regimes, to the detriment of progressive moderates who seek to separate religion from politics.", "Moderate and reformist Islamists who accept and work within the democratic process include parties like the Tunisian Ennahda Movement. Jamaat-e-Islami of Pakistan is basically a socio-political and democratic Vanguard party but has also gained political influence through military coup d'état in past. The Islamist groups like Hezbollah in Lebanon and Hamas in Palestine participate in democratic and political process as well as armed attacks, seeking to abolish the state of Israel. Radical Islamist organizations like al-Qaeda and the Egyptian Islamic Jihad, and groups such as the Taliban, entirely reject democracy, often declaring as kuffar those Muslims who support it (see takfirism), as well as calling for violent/offensive jihad or urging and conducting attacks on a religious basis.", "The views of Ali Shariati, ideologue of the Iranian Revolution, had resemblance with Mohammad Iqbal, ideological father of the State of Pakistan, but Khomeini's beliefs is perceived to be placed somewhere between beliefs of Sunni Islamic thinkers like Mawdudi and Qutb. He believed that complete imitation of the Prophet Mohammad and his successors such as Ali for restoration of Sharia law was essential to Islam, that many secular, Westernizing Muslims were actually agents of the West serving Western interests, and that the acts such as \"plundering\" of Muslim lands was part of a long-term conspiracy against Islam by the Western governments.", "During the 1970s and sometimes later, Western and pro-Western governments often supported sometimes fledgling Islamists and Islamist groups that later came to be seen as dangerous enemies. Islamists were considered by Western governments bulwarks against—what were thought to be at the time—more dangerous leftist/communist/nationalist insurgents/opposition, which Islamists were correctly seen as opposing. The US spent billions of dollars to aid the mujahideen Muslim Afghanistan enemies of the Soviet Union, and non-Afghan veterans of the war returned home with their prestige, \"experience, ideology, and weapons\", and had considerable impact.", "The Taliban were spawned by the thousands of madrasahs the Deobandi movement established for impoverished Afghan refugees and supported by governmental and religious groups in neighboring Pakistan. The Taliban differed from other Islamist movements to the point where they might be more properly described as Islamic fundamentalist or neofundamentalist, interested in spreading \"an idealized and systematized version of conservative tribal village customs\" under the label of Sharia to an entire country. Their ideology was also described as being influenced by Wahhabism, and the extremist jihadism of their guest Osama bin Laden."]</t>
-        </is>
-      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -7534,21 +5239,6 @@
 As interesting examples of expositions the most notable are: the world's first Museum of Posters boasting one of the largest collections of art posters in the world, Museum of Hunting and Riding and the Railway Museum. From among Warsaw's 60 museums, the most prestigious ones are National Museum with a collection of works whose origin ranges in time from antiquity till the present epoch as well as one of the best collections of paintings in the country including some paintings from Adolf Hitler's private collection, and Museum of the Polish Army whose set portrays the history of arms.</t>
         </is>
       </c>
-      <c r="F154" t="inlineStr">
-        <is>
-          <t>[154, 787, 519, 767, 540]</t>
-        </is>
-      </c>
-      <c r="G154" t="inlineStr">
-        <is>
-          <t>[0.7746720314025879, 0.7522373199462891, 0.7331631779670715, 0.7268854975700378, 0.7255305647850037]</t>
-        </is>
-      </c>
-      <c r="H154" t="inlineStr">
-        <is>
-          <t>["By far the most famous work of Norman art is the Bayeux Tapestry, which is not a tapestry but a work of embroidery. It was commissioned by Odo, the Bishop of Bayeux and first Earl of Kent, employing natives from Kent who were learned in the Nordic traditions imported in the previous half century by the Danish Vikings.", "With the opening of the Dorothy and Michael Hintze sculpture galleries in 2006 it was decided to extend the chronology of the works on display up to 1950; this has involved loans by other museums, including Tate Britain, so works by Henry Moore and Jacob Epstein along with other of their contemporaries are now on view. These galleries concentrate on works dated 1600 to 1950 by British sculptors, works by continental sculptors who worked in Britain, and works bought by British patrons from the continental sculptors, such as Canova's Theseus and the Minotaur. The galleries overlooking the garden are arranged by theme, tomb sculpture, portraiture, garden sculpture and mythology. Then there is a section that covers late 19th-century and early 20th-century sculpture, this includes work by Rodin and other French sculptors such as Dalou who spent several years in Britain where he taught sculpture.", "The sculpture collection at the V&amp;A is the most comprehensive holding of post-classical European sculpture in the world. There are approximately 22,000 objects in the collection that cover the period from about 400 AD to 1914. This covers among other periods Byzantine and Anglo Saxon ivory sculptures, British, French and Spanish medieval statues and carvings, the Renaissance, Baroque, Neo-Classical, Victorian and Art Nouveau periods. All uses of sculpture are represented, from tomb and memorial, to portrait, allegorical, religious, mythical, statues for gardens including fountains, as well as architectural decorations. Materials used include, marble, alabaster, stone, terracotta, wood (history of wood carving), ivory, gesso, plaster, bronze, lead and ceramics.", "One of the most dramatic parts of the museum is the Cast Courts in the sculpture wing, comprising two large, skylighted rooms two storeys high housing hundreds of plaster casts of sculptures, friezes and tombs. One of these is dominated by a full-scale replica of Trajan's Column, cut in half in order to fit under the ceiling. The other includes reproductions of various works of Italian Renaissance sculpture and architecture, including a full-size replica of Michelangelo's David. Replicas of two earlier Davids by Donatello's David and Verrocchio's David, are also included, although for conservation reasons the Verrocchio replica is displayed in a glass case.", "As interesting examples of expositions the most notable are: the world's first Museum of Posters boasting one of the largest collections of art posters in the world, Museum of Hunting and Riding and the Railway Museum. From among Warsaw's 60 museums, the most prestigious ones are National Museum with a collection of works whose origin ranges in time from antiquity till the present epoch as well as one of the best collections of paintings in the country including some paintings from Adolf Hitler's private collection, and Museum of the Polish Army whose set portrays the history of arms."]</t>
-        </is>
-      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -7578,21 +5268,6 @@
 the merger, Thomas S. Murphy left ABC with Robert Iger taking his place as president and CEO. Around the time of the merger, Disney's television production units had already produced series for the network such as Home Improvement and Boy Meets World, while the deal also allowed ABC access to Disney's children's programming library for its Saturday morning block. In 1998, ABC premiered the Aaron Sorkin-created sitcom Sports Night, centering on the travails of the staff of a SportsCenter-style sports news program; despite earning critical praise and multiple Emmy Awards, the series was cancelled in 2000 after two seasons.
 Between May and September 2005, rumors circulated that Disney–ABC was considering a sale of ABC Radio, with Clear Channel Communications and Westwood One (which had earlier purchased NBC's radio division, as well as the distribution rights to CBS's, and the Mutual Broadcasting System during the 1990s) as potential buyers. On October 19, 2005, ABC announced the restructuring of the group into six divisions: Entertainment Communications, Communications Resources, Kids Communications, News Communications, Corporate Communications, and International Communications.
 The service started on 1 September 1993 based on the idea from the then chief executive officer, Sam Chisholm and Rupert Murdoch, of converting the company business strategy to an entirely fee-based concept. The new package included four channels formerly available free-to-air, broadcasting on Astra's satellites, as well as introducing new channels. The service continued until the closure of BSkyB's analogue service on 27 September 2001, due to the launch and expansion of the Sky Digital platform. Some of the channels did broadcast either in the clear or soft encrypted (whereby a Videocrypt decoder was required to decode, without a subscription card) prior to their addition to the Sky Multichannels package. Within two months of the launch, BSkyB gained 400,000 new subscribers, with the majority taking at least one premium channel as well, which helped BSkyB reach 3.5 million households by mid-1994. Michael Grade criticized the operations in front of the Select Committee on National Heritage, mainly for the lack of original programming on many of the new channels.</t>
-        </is>
-      </c>
-      <c r="F155" t="inlineStr">
-        <is>
-          <t>[415, 103, 104, 735, 541]</t>
-        </is>
-      </c>
-      <c r="G155" t="inlineStr">
-        <is>
-          <t>[0.8074596524238586, 0.7927190661430359, 0.7911202907562256, 0.7902077436447144, 0.7878879308700562]</t>
-        </is>
-      </c>
-      <c r="H155" t="inlineStr">
-        <is>
-          <t>["ABC maintains several video on demand services for delayed viewing of the network's programming, including a traditional VOD service called ABC on Demand, which is carried on most traditional cable and IPTV providers. The Walt Disney Company is also a part-owner of Hulu (as part of a consortium that includes, among other parties, the respective parent companies of NBC and Fox, NBCUniversal and 21st Century Fox), and has offered full-length episodes of most of ABC's programming through the streaming service since July 6, 2009 (which are available for viewing on Hulu's website and mobile app), as part of an agreement reached in April that year that also allowed Disney to acquire a 27% ownership stake in Hulu.", "On July 31, 1995, The Walt Disney Company announced an agreement to merge with Capital Cities/ABC for $19 billion. Disney shareholders approved the merger at a special conference in New York City on January 4, 1996, with the acquisition of Capital Cities/ABC being completed on February 9; following the sale, Disney renamed its new subsidiary ABC Inc. In addition to the ABC network, the Disney acquisition integrated ABC's ten owned-and-operated television and 21 radio stations; its 80% interest in ESPN, ownership interests in The History Channel, A&amp;E Television Networks, and Lifetime Entertainment; and Capital Cities/ABC's magazine and newspaper properties into the company. As FCC ownership rules forbade the company from keeping both it and KABC-TV, Disney sold Los Angeles independent station KCAL-TV to Young Broadcasting for $387 million. On April 4, Disney sold the four newspapers that ABC had controlled under Capital Cities to Knight Ridder for $1.65 billion. Following the merger, Thomas S. Murphy left ABC with Robert Iger taking his place as president and CEO. Around the time of the merger, Disney's television production units had already produced series for the network such as Home Improvement and Boy Meets World, while the deal also allowed ABC access to", "the merger, Thomas S. Murphy left ABC with Robert Iger taking his place as president and CEO. Around the time of the merger, Disney's television production units had already produced series for the network such as Home Improvement and Boy Meets World, while the deal also allowed ABC access to Disney's children's programming library for its Saturday morning block. In 1998, ABC premiered the Aaron Sorkin-created sitcom Sports Night, centering on the travails of the staff of a SportsCenter-style sports news program; despite earning critical praise and multiple Emmy Awards, the series was cancelled in 2000 after two seasons.", "Between May and September 2005, rumors circulated that Disney–ABC was considering a sale of ABC Radio, with Clear Channel Communications and Westwood One (which had earlier purchased NBC's radio division, as well as the distribution rights to CBS's, and the Mutual Broadcasting System during the 1990s) as potential buyers. On October 19, 2005, ABC announced the restructuring of the group into six divisions: Entertainment Communications, Communications Resources, Kids Communications, News Communications, Corporate Communications, and International Communications.", "The service started on 1 September 1993 based on the idea from the then chief executive officer, Sam Chisholm and Rupert Murdoch, of converting the company business strategy to an entirely fee-based concept. The new package included four channels formerly available free-to-air, broadcasting on Astra's satellites, as well as introducing new channels. The service continued until the closure of BSkyB's analogue service on 27 September 2001, due to the launch and expansion of the Sky Digital platform. Some of the channels did broadcast either in the clear or soft encrypted (whereby a Videocrypt decoder was required to decode, without a subscription card) prior to their addition to the Sky Multichannels package. Within two months of the launch, BSkyB gained 400,000 new subscribers, with the majority taking at least one premium channel as well, which helped BSkyB reach 3.5 million households by mid-1994. Michael Grade criticized the operations in front of the Select Committee on National Heritage, mainly for the lack of original programming on many of the new channels."]</t>
         </is>
       </c>
     </row>
@@ -7635,21 +5310,6 @@
 In the late 17th century, Robert Boyle proved that air is necessary for combustion. English chemist John Mayow (1641–1679) refined this work by showing that fire requires only a part of air that he called spiritus nitroaereus or just nitroaereus. In one experiment he found that placing either a mouse or a lit candle in a closed container over water caused the water to rise and replace one-fourteenth of the air's volume before extinguishing the subjects. From this he surmised that nitroaereus is consumed in both respiration and combustion.</t>
         </is>
       </c>
-      <c r="F156" t="inlineStr">
-        <is>
-          <t>[156, 617, 315, 419, 428]</t>
-        </is>
-      </c>
-      <c r="G156" t="inlineStr">
-        <is>
-          <t>[0.815736711025238, 0.7484197616577148, 0.7433025240898132, 0.7405879497528076, 0.7248865962028503]</t>
-        </is>
-      </c>
-      <c r="H156" t="inlineStr">
-        <is>
-          <t>["Oxygen is the most abundant chemical element by mass in the Earth's biosphere, air, sea and land. Oxygen is the third most abundant chemical element in the universe, after hydrogen and helium. About 0.9% of the Sun's mass is oxygen. Oxygen constitutes 49.2% of the Earth's crust by mass and is the major component of the world's oceans (88.8% by mass). Oxygen gas is the second most common component of the Earth's atmosphere, taking up 20.8% of its volume and 23.1% of its mass (some 1015 tonnes).[d] Earth is unusual among the planets of the Solar System in having such a high concentration of oxygen gas in its atmosphere: Mars (with 0.1% O\n2 by volume) and Venus have far lower concentrations. The O\n2 surrounding these other planets is produced solely by ultraviolet radiation impacting oxygen-containing molecules such as carbon dioxide.", "The unusually high concentration of oxygen gas on Earth is the result of the oxygen cycle. This biogeochemical cycle describes the movement of oxygen within and between its three main reservoirs on Earth: the atmosphere, the biosphere, and the lithosphere. The main driving factor of the oxygen cycle is photosynthesis, which is responsible for modern Earth's atmosphere. Photosynthesis releases oxygen into the atmosphere, while respiration and decay remove it from the atmosphere. In the present equilibrium, production and consumption occur at the same rate of roughly 1/2000th of the entire atmospheric oxygen per year.", "Oxygen is present in the atmosphere in trace quantities in the form of carbon dioxide (CO\n2). The Earth's crustal rock is composed in large part of oxides of silicon (silica SiO\n2, as found in granite and quartz), aluminium (aluminium oxide Al\n2O\n3, in bauxite and corundum), iron (iron(III) oxide Fe\n2O\n3, in hematite and rust), and calcium carbonate (in limestone). The rest of the Earth's crust is also made of oxygen compounds, in particular various complex silicates (in silicate minerals). The Earth's mantle, of much larger mass than the crust, is largely composed of silicates of magnesium and iron.", "Due to its electronegativity, oxygen forms chemical bonds with almost all other elements to give corresponding oxides. The surface of most metals, such as aluminium and titanium, are oxidized in the presence of air and become coated with a thin film of oxide that passivates the metal and slows further corrosion. Many oxides of the transition metals are non-stoichiometric compounds, with slightly less metal than the chemical formula would show. For example, the mineral FeO (wüstite) is written as Fe\n1 − xO, where x is usually around 0.05.", "In the late 17th century, Robert Boyle proved that air is necessary for combustion. English chemist John Mayow (1641–1679) refined this work by showing that fire requires only a part of air that he called spiritus nitroaereus or just nitroaereus. In one experiment he found that placing either a mouse or a lit candle in a closed container over water caused the water to rise and replace one-fourteenth of the air's volume before extinguishing the subjects. From this he surmised that nitroaereus is consumed in both respiration and combustion."]</t>
-        </is>
-      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -7681,21 +5341,6 @@
 Despite their soft, gelatinous bodies, fossils thought to represent ctenophores, apparently with no tentacles but many more comb-rows than modern forms, have been found in lagerstätten as far back as the early Cambrian, about 515 million years ago. The position of the ctenophores in the evolutionary family tree of animals has long been debated, and the majority view at present, based on molecular phylogenetics, is that cnidarians and bilaterians are more closely related to each other than either is to ctenophores. A recent molecular phylogenetics analysis concluded that the common ancestor of all modern ctenophores was cydippid-like, and that all the modern groups appeared relatively recently, probably after the Cretaceous–Paleogene extinction event 66 million years ago. Evidence accumulating since the 1980s indicates that the "cydippids" are not monophyletic, in other words do not include all and only the descendants of a single common ancestor, because all the other traditional ctenophore groups are descendants of various cydippids.</t>
         </is>
       </c>
-      <c r="F157" t="inlineStr">
-        <is>
-          <t>[157, 513, 786, 778, 349]</t>
-        </is>
-      </c>
-      <c r="G157" t="inlineStr">
-        <is>
-          <t>[0.749467670917511, 0.7105928659439087, 0.6945489048957825, 0.6925673484802246, 0.6872993111610413]</t>
-        </is>
-      </c>
-      <c r="H157" t="inlineStr">
-        <is>
-          <t>["These chloroplasts, which can be traced back directly to a cyanobacterial ancestor, are known as primary plastids (\"plastid\" in this context means almost the same thing as chloroplast). All primary chloroplasts belong to one of three chloroplast lineages—the glaucophyte chloroplast lineage, the rhodophyte, or red algal chloroplast lineage, or the chloroplastidan, or green chloroplast lineage. The second two are the largest, and the green chloroplast lineage is the one that contains the land plants.", "The inverted repeat regions are highly conserved among land plants, and accumulate few mutations. Similar inverted repeats exist in the genomes of cyanobacteria and the other two chloroplast lineages (glaucophyta and rhodophyceæ), suggesting that they predate the chloroplast, though some chloroplast DNAs have since lost or flipped the inverted repeats (making them direct repeats). It is possible that the inverted repeats help stabilize the rest of the chloroplast genome, as chloroplast DNAs which have lost some of the inverted repeat segments tend to get rearranged more.", "The chloroplastidan chloroplasts, or green chloroplasts, are another large, highly diverse primary chloroplast lineage. Their host organisms are commonly known as the green algae and land plants. They differ from glaucophyte and red algal chloroplasts in that they have lost their phycobilisomes, and contain chlorophyll b instead. Most green chloroplasts are (obviously) green, though some aren't, like some forms of Hæmatococcus pluvialis, due to accessory pigments that override the chlorophylls' green colors. Chloroplastidan chloroplasts have lost the peptidoglycan wall between their double membrane, and have replaced it with an intermembrane space. Some plants seem to have kept the genes for the synthesis of the peptidoglycan layer, though they've been repurposed for use in chloroplast division instead.", "The alga Cyanophora, a glaucophyte, is thought to be one of the first organisms to contain a chloroplast. The glaucophyte chloroplast group is the smallest of the three primary chloroplast lineages, being found in only 13 species, and is thought to be the one that branched off the earliest. Glaucophytes have chloroplasts that retain a peptidoglycan wall between their double membranes, like their cyanobacterial parent. For this reason, glaucophyte chloroplasts are also known as muroplasts. Glaucophyte chloroplasts also contain concentric unstacked thylakoids, which surround a carboxysome - an icosahedral structure that glaucophyte chloroplasts and cyanobacteria keep their carbon fixation enzyme rubisco in. The starch that they synthesize collects outside the chloroplast. Like cyanobacteria, glaucophyte chloroplast thylakoids are studded with light collecting structures called phycobilisomes. For these reasons, glaucophyte chloroplasts are considered a primitive intermediate between cyanobacteria and the more evolved chloroplasts in red algae and plants.", "Despite their soft, gelatinous bodies, fossils thought to represent ctenophores, apparently with no tentacles but many more comb-rows than modern forms, have been found in lagerstätten as far back as the early Cambrian, about 515 million years ago. The position of the ctenophores in the evolutionary family tree of animals has long been debated, and the majority view at present, based on molecular phylogenetics, is that cnidarians and bilaterians are more closely related to each other than either is to ctenophores. A recent molecular phylogenetics analysis concluded that the common ancestor of all modern ctenophores was cydippid-like, and that all the modern groups appeared relatively recently, probably after the Cretaceous–Paleogene extinction event 66 million years ago. Evidence accumulating since the 1980s indicates that the \"cydippids\" are not monophyletic, in other words do not include all and only the descendants of a single common ancestor, because all the other traditional ctenophore groups are descendants of various cydippids."]</t>
-        </is>
-      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -7727,21 +5372,6 @@
 Continuing the style of the earlier buildings, various designers were responsible for the decoration, the terracotta embellishments were again the work of Godfrey Sykes, although sgraffito was used to decorate the east side of the building designed by F. W. Moody, a final embellishment were the wrought iron gates made as late as 1885 designed by Starkie Gardner, these lead to a passage through the building. Scott also designed the two Cast Courts 1870–73 to the southeast of the garden (the site of the "Brompton Boilers"), these vast spaces have ceilings 70 feet (21 m) in height to accommodate the plaster casts of parts of famous buildings, including Trajan's Column (in two separate pieces). The final part of the museum designed by Scott was the Art Library and what is now the sculpture gallery on the south side of the garden, built 1877–83, the exterior mosaic panels in the parapet were designed by Reuben Townroe who also designed the plaster work in the library, Sir John Taylor designed the book shelves and cases, also this was the first part of the museum to have electric lighting. This completed the northern half of the site, creating a quadrangle with the garden</t>
         </is>
       </c>
-      <c r="F158" t="inlineStr">
-        <is>
-          <t>[717, 158, 599, 688, 587]</t>
-        </is>
-      </c>
-      <c r="G158" t="inlineStr">
-        <is>
-          <t>[0.7912874221801758, 0.7904323935508728, 0.7771570086479187, 0.7771496772766113, 0.7732900381088257]</t>
-        </is>
-      </c>
-      <c r="H158" t="inlineStr">
-        <is>
-          <t>["(later transferred to the Tate Gallery) and now used as the picture galleries and tapestry gallery respectively. The North and South Courts, were then built, both of which opened by June 1862. They now form the galleries for temporary exhibitions and are directly behind the Sheepshanks Gallery. On the very northern edge of the site is situated the Secretariat Wing, also built in 1862 this houses the offices and board room etc. and is not open to the public.", "There are a set of beautiful inlaid doors, dated 1580 from Antwerp City Hall, attributed to Hans Vredeman de Vries. One of the finest pieces of continental furniture in the collection is the Rococo Augustus Rex Bureau Cabinet dated c1750 from Germany, with especially fine marquetry and ormolu mounts. One of the grandest pieces of 19th-century furniture is the highly elaborate French Cabinet dated 1861–1867 made by M. Fourdinois, made from ebony inlaid with box, lime, holly, pear, walnut and mahogany woods as well as marble with gilded carvings. Furniture designed by Ernest Gimson, Edward William Godwin, Charles Voysey, Adolf Loos and Otto Wagner are among the late 19th-century and early 20th-century examples in the collection. The work of modernists in the collection include Le Corbusier, Marcel Breuer, Charles and Ray Eames, and Giò Ponti.", "Prince Albert appears within the main arch above the twin entrances, Queen Victoria above the frame around the arches and entrance, sculpted by Alfred Drury. These façades surround four levels of galleries. Other areas designed by Webb include the Entrance Hall and Rotunda, the East and West Halls, the areas occupied by the shop and Asian Galleries as well as the Costume Gallery. The interior makes much use of marble in the entrance hall and flanking staircases, although the galleries as originally designed were white with restrained classical detail and mouldings, very much in contrast to the elaborate decoration of the Victorian galleries, although much of this decoration was removed in the early 20th century.", "The main gallery was redesigned in 1994, the glass balustrade on the staircase and mezzanine are the work of Danny Lane, the gallery covering contemporary glass opened in 2004 and the sacred silver and stained-glass gallery in 2005. In this latter gallery stained glass is displayed alongside silverware starting in the 12th century and continuing to the present. Some of the most outstanding stained glass, dated 1243–48 comes from the Sainte-Chapelle, is displayed along with other examples in the new Medieval &amp; Renaissance galleries. The important 13th-century glass beaker known as the Luck of Edenhall is also displayed in these galleries. Examples of British stained glass are displayed in the British Galleries. One of the most spectacular items in the collection is the chandelier by Dale Chihuly in the rotunda at the Museum's main entrance.", "Continuing the style of the earlier buildings, various designers were responsible for the decoration, the terracotta embellishments were again the work of Godfrey Sykes, although sgraffito was used to decorate the east side of the building designed by F. W. Moody, a final embellishment were the wrought iron gates made as late as 1885 designed by Starkie Gardner, these lead to a passage through the building. Scott also designed the two Cast Courts 1870–73 to the southeast of the garden (the site of the \"Brompton Boilers\"), these vast spaces have ceilings 70 feet (21 m) in height to accommodate the plaster casts of parts of famous buildings, including Trajan's Column (in two separate pieces). The final part of the museum designed by Scott was the Art Library and what is now the sculpture gallery on the south side of the garden, built 1877–83, the exterior mosaic panels in the parapet were designed by Reuben Townroe who also designed the plaster work in the library, Sir John Taylor designed the book shelves and cases, also this was the first part of the museum to have electric lighting. This completed the northern half of the site, creating a quadrangle with the garden"]</t>
-        </is>
-      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -7773,21 +5403,6 @@
 The main gallery was redesigned in 1994, the glass balustrade on the staircase and mezzanine are the work of Danny Lane, the gallery covering contemporary glass opened in 2004 and the sacred silver and stained-glass gallery in 2005. In this latter gallery stained glass is displayed alongside silverware starting in the 12th century and continuing to the present. Some of the most outstanding stained glass, dated 1243–48 comes from the Sainte-Chapelle, is displayed along with other examples in the new Medieval &amp; Renaissance galleries. The important 13th-century glass beaker known as the Luck of Edenhall is also displayed in these galleries. Examples of British stained glass are displayed in the British Galleries. One of the most spectacular items in the collection is the chandelier by Dale Chihuly in the rotunda at the Museum's main entrance.</t>
         </is>
       </c>
-      <c r="F159" t="inlineStr">
-        <is>
-          <t>[159, 519, 787, 767, 688]</t>
-        </is>
-      </c>
-      <c r="G159" t="inlineStr">
-        <is>
-          <t>[0.8393174409866333, 0.818558394908905, 0.8063251972198486, 0.798420786857605, 0.7587502598762512]</t>
-        </is>
-      </c>
-      <c r="H159" t="inlineStr">
-        <is>
-          <t>["The Toshiba gallery of Japanese art opened in December 1986. The majority of exhibits date from 1550 to 1900, but one of the oldest pieces displayed is the 13th-century sculpture of Amida Nyorai. Examples of classic Japanese armour from the mid-19th century, steel sword blades (Katana), Inrō, lacquerware including the Mazarin Chest dated c1640 is one of the finest surviving pieces from Kyoto, porcelain including Imari, Netsuke, woodblock prints including the work of Ando Hiroshige, graphic works include printed books, as well as a few paintings, scrolls and screens, textiles and dress including kimonos are some of the objects on display. One of the finest objects displayed is Suzuki Chokichi's bronze incense burner (koro) dated 1875, standing at over 2.25 metres high and 1.25 metres in diameter it is also one of the largest examples made. The museum also holds some cloisonné pieces from the Japanese art production company, Ando Cloisonné.", "The sculpture collection at the V&amp;A is the most comprehensive holding of post-classical European sculpture in the world. There are approximately 22,000 objects in the collection that cover the period from about 400 AD to 1914. This covers among other periods Byzantine and Anglo Saxon ivory sculptures, British, French and Spanish medieval statues and carvings, the Renaissance, Baroque, Neo-Classical, Victorian and Art Nouveau periods. All uses of sculpture are represented, from tomb and memorial, to portrait, allegorical, religious, mythical, statues for gardens including fountains, as well as architectural decorations. Materials used include, marble, alabaster, stone, terracotta, wood (history of wood carving), ivory, gesso, plaster, bronze, lead and ceramics.", "With the opening of the Dorothy and Michael Hintze sculpture galleries in 2006 it was decided to extend the chronology of the works on display up to 1950; this has involved loans by other museums, including Tate Britain, so works by Henry Moore and Jacob Epstein along with other of their contemporaries are now on view. These galleries concentrate on works dated 1600 to 1950 by British sculptors, works by continental sculptors who worked in Britain, and works bought by British patrons from the continental sculptors, such as Canova's Theseus and the Minotaur. The galleries overlooking the garden are arranged by theme, tomb sculpture, portraiture, garden sculpture and mythology. Then there is a section that covers late 19th-century and early 20th-century sculpture, this includes work by Rodin and other French sculptors such as Dalou who spent several years in Britain where he taught sculpture.", "One of the most dramatic parts of the museum is the Cast Courts in the sculpture wing, comprising two large, skylighted rooms two storeys high housing hundreds of plaster casts of sculptures, friezes and tombs. One of these is dominated by a full-scale replica of Trajan's Column, cut in half in order to fit under the ceiling. The other includes reproductions of various works of Italian Renaissance sculpture and architecture, including a full-size replica of Michelangelo's David. Replicas of two earlier Davids by Donatello's David and Verrocchio's David, are also included, although for conservation reasons the Verrocchio replica is displayed in a glass case.", "The main gallery was redesigned in 1994, the glass balustrade on the staircase and mezzanine are the work of Danny Lane, the gallery covering contemporary glass opened in 2004 and the sacred silver and stained-glass gallery in 2005. In this latter gallery stained glass is displayed alongside silverware starting in the 12th century and continuing to the present. Some of the most outstanding stained glass, dated 1243–48 comes from the Sainte-Chapelle, is displayed along with other examples in the new Medieval &amp; Renaissance galleries. The important 13th-century glass beaker known as the Luck of Edenhall is also displayed in these galleries. Examples of British stained glass are displayed in the British Galleries. One of the most spectacular items in the collection is the chandelier by Dale Chihuly in the rotunda at the Museum's main entrance."]</t>
-        </is>
-      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -7819,21 +5434,6 @@
 In the United States, the game was televised by CBS, as part of a cycle between the three main broadcast television partners of the NFL. The network's lead broadcast team of Jim Nantz and Phil Simms called the contest, with Tracy Wolfson and Evan Washburn on the sidelines. CBS introduced new features during the telecast, including pylon cameras and microphones along with EyeVision 360—an array of 36 cameras along the upper deck that can be used to provide a 360-degree view of plays and "bullet time" effects. (An earlier version of EyeVision was last used in Super Bowl XXXV; for Super Bowl 50, the cameras were upgraded to 5K resolution.)</t>
         </is>
       </c>
-      <c r="F160" t="inlineStr">
-        <is>
-          <t>[160, 39, 418, 263, 353]</t>
-        </is>
-      </c>
-      <c r="G160" t="inlineStr">
-        <is>
-          <t>[0.8297154903411865, 0.8081313967704773, 0.8069614171981812, 0.798603892326355, 0.7932020425796509]</t>
-        </is>
-      </c>
-      <c r="H160" t="inlineStr">
-        <is>
-          <t>["As opposed to broadcasts of primetime series, CBS broadcast special episodes of its late night talk shows as its lead-out programs for Super Bowl 50, beginning with a special episode of The Late Show with Stephen Colbert following the game. Following a break for late local programming, CBS also aired a special episode of The Late Late Show with James Corden.", "CBS broadcast Super Bowl 50 in the U.S., and charged an average of $5 million for a 30-second commercial during the game. The Super Bowl 50 halftime show was headlined by the British rock group Coldplay with special guest performers Beyoncé and Bruno Mars, who headlined the Super Bowl XLVII and Super Bowl XLVIII halftime shows, respectively. It was the third-most watched U.S. broadcast ever.", "In early 2012, NFL Commissioner Roger Goodell stated that the league planned to make the 50th Super Bowl \"spectacular\" and that it would be \"an important game for us as a league\".", "Super Bowl 50 was an American football game to determine the champion of the National Football League (NFL) for the 2015 season. The American Football Conference (AFC) champion Denver Broncos defeated the National Football Conference (NFC) champion Carolina Panthers 24–10 to earn their third Super Bowl title. The game was played on February 7, 2016, at Levi's Stadium in the San Francisco Bay Area at Santa Clara, California. As this was the 50th Super Bowl, the league emphasized the \"golden anniversary\" with various gold-themed initiatives, as well as temporarily suspending the tradition of naming each Super Bowl game with Roman numerals (under which the game would have been known as \"Super Bowl L\"), so that the logo could prominently feature the Arabic numerals 50.", "In the United States, the game was televised by CBS, as part of a cycle between the three main broadcast television partners of the NFL. The network's lead broadcast team of Jim Nantz and Phil Simms called the contest, with Tracy Wolfson and Evan Washburn on the sidelines. CBS introduced new features during the telecast, including pylon cameras and microphones along with EyeVision 360—an array of 36 cameras along the upper deck that can be used to provide a 360-degree view of plays and \"bullet time\" effects. (An earlier version of EyeVision was last used in Super Bowl XXXV; for Super Bowl 50, the cameras were upgraded to 5K resolution.)"]</t>
-        </is>
-      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -7865,21 +5465,6 @@
 While experimenting, Tesla inadvertently faulted a power station generator, causing a power outage. In August 1917, Tesla explained what had happened in The Electrical Experimenter: "As an example of what has been done with several hundred kilowatts of high frequency energy liberated, it was found that the dynamos in a power house six miles away were repeatedly burned out, due to the powerful high frequency currents set up in them, and which caused heavy sparks to jump through the windings and destroy the insulation!"</t>
         </is>
       </c>
-      <c r="F161" t="inlineStr">
-        <is>
-          <t>[161, 831, 24, 77, 785]</t>
-        </is>
-      </c>
-      <c r="G161" t="inlineStr">
-        <is>
-          <t>[0.8453885912895203, 0.6686620712280273, 0.6608587503433228, 0.6558754444122314, 0.6529285907745361]</t>
-        </is>
-      </c>
-      <c r="H161" t="inlineStr">
-        <is>
-          <t>["NASA's CALIPSO satellite has measured the amount of dust transported by wind from the Sahara to the Amazon: an average 182 million tons of dust are windblown out of the Sahara each year, at 15 degrees west longitude, across 1,600 miles (2,600 km) over the Atlantic Ocean (some dust falls into the Atlantic), then at 35 degrees West longitude at the eastern coast of South America, 27.7 million tons (15%) of dust fall over the Amazon basin, 132 million tons of dust remain in the air, 43 million tons of dust are windblown and falls on the Caribbean Sea, past 75 degrees west longitude.", "Since 7500 yr ago, a situation with tides and currents, very similar to present has existed. Rates of sea-level rise had dropped so far, that natural sedimentation by the Rhine and coastal processes together, could compensate the transgression by the sea; in the last 7000 years, the coast line was roughly at the same location. In the southern North Sea, due to ongoing tectonic subsidence, the sea level is still rising, at the rate of about 1–3 cm (0.39–1.18 in) per century (1 metre or 39 inches in last 3000 years).", "In 2010 the Amazon rainforest experienced another severe drought, in some ways more extreme than the 2005 drought. The affected region was approximate 1,160,000 square miles (3,000,000 km2) of rainforest, compared to 734,000 square miles (1,900,000 km2) in 2005. The 2010 drought had three epicenters where vegetation died off, whereas in 2005 the drought was focused on the southwestern part. The findings were published in the journal Science. In a typical year the Amazon absorbs 1.5 gigatons of carbon dioxide; during 2005 instead 5 gigatons were released and in 2010 8 gigatons were released.", "Most of the Rhine's current course was not under the ice during the last Ice Age; although, its source must still have been a glacier. A tundra, with Ice Age flora and fauna, stretched across middle Europe, from Asia to the Atlantic Ocean. Such was the case during the Last Glacial Maximum, ca. 22,000–14,000 yr BP, when ice-sheets covered Scandinavia, the Baltics, Scotland and the Alps, but left the space between as open tundra. The loess or wind-blown dust over that tundra, settled in and around the Rhine Valley, contributing to its current agricultural usefulness.", "While experimenting, Tesla inadvertently faulted a power station generator, causing a power outage. In August 1917, Tesla explained what had happened in The Electrical Experimenter: \"As an example of what has been done with several hundred kilowatts of high frequency energy liberated, it was found that the dynamos in a power house six miles away were repeatedly burned out, due to the powerful high frequency currents set up in them, and which caused heavy sparks to jump through the windings and destroy the insulation!\""]</t>
-        </is>
-      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -7911,21 +5496,6 @@
 are expected to defer to the father of the house when in his home. Further, additional spiritual guidance is offered by those holding the office of Patriarch, which is supposed by Latter-day Saints to grant certain gifts of the Spirit, such as the ability to prophesy, to its holders. This guidance is generally offered during a ceremony called the patriarchal blessing.</t>
         </is>
       </c>
-      <c r="F162" t="inlineStr">
-        <is>
-          <t>[162, 163, 860, 633, 861]</t>
-        </is>
-      </c>
-      <c r="G162" t="inlineStr">
-        <is>
-          <t>[0.8200721144676208, 0.8072803616523743, 0.7485798001289368, 0.7445328831672668, 0.7401888966560364]</t>
-        </is>
-      </c>
-      <c r="H162" t="inlineStr">
-        <is>
-          <t>["There are many forms of spiritual or religious teachers in Christianity, across all three major traditions - (Roman) Catholic, (Eastern) Orthodox Catholic, and Protestant/Non-Denominational, with a stronger tradition of spiritual formation in the more historic and authoritarian/hierarchical Christian traditions with a long tradition of \"discernment of spirits\", of vocations, and other aspects of spiritual life, especially the Roman and Orthodox Catholic Churches. These positions include: the honoured but informal position of starets or elder - a man (or, less often, woman), often a monastic, considered to be graced by God with certain gifts for the guidance of souls and the detection and correction of prelest (spiritual pride or deception) - who acts as a spiritual guide or father in the Orthodox Catholic tradition, especially Russian Orthodoxy (see Optina Monastery, which had a long line of said starets); the Priest or Confessor in Roman Catholicism, who is often a man in Holy Orders but may be a monastic or other person respected for his spiritual accomplishments or acumen (even the Pope of Rome has a Confessor, who is not always a bishop, and, due to the hierarchical structure of the Roman Church, can not be his equal in authority), which is", "Holy Orders but may be a monastic or other person respected for his spiritual accomplishments or acumen (even the Pope of Rome has a Confessor, who is not always a bishop, and, due to the hierarchical structure of the Roman Church, can not be his equal in authority), which is often a semi-official to official position, as opposed to the unofficial positions of spiritual guides in the Orthodox Catholic and Protestant traditions; and the almost-exclusively informal arrangements (generally formal only in members who are under some form of church discipline) of mentorship (both of adults and children, in the latter case often a youth pastor) in the Protestant and Non-Denominational traditions, which boundaries can be blurred with the more typically Roman \"confessor\" position in some of the more historic and conservative Reformation Churches, such as some of the Lutheran and Anglican. In keeping with the individualistic nature of most Protestant denominations, the emphasis on being guided in spiritual development is small, with a heavy emphasis placed on heavy reading and personal, Spirit-enlightened interpretation of the Holy Bible.", "In The Church of Jesus Christ of Latter-day Saints (LDS Church), the teacher is an office in the Aaronic priesthood, generally conferred on young boys or recent converts, and has little in common with the \"spiritual teacher\" archetype. The role of \"spiritual teacher\" may be filled by many individuals in the LDS Church, often a trusted friend, who may hold any office, from Elder to Bishop, or no office at all. The emphasis on spiritual mentorship in the LDS Church is similar to that in the more \"low-church\" traditions of Protestantism, with a stronger emphasis placed on the husband and father of a family to provide spiritual guidance for all of his family, ideally in consultation with his wife, even if the husband is not a member of the LDS Church, based on interpretatios of certain Biblical texts which proclaim the spiritual authority of husbands in marriage. Even Priesthood representatives are expected to defer to the father of the house when in his home. Further, additional spiritual guidance is offered by those holding the office of Patriarch, which is supposed by Latter-day Saints to grant certain gifts of the Spirit, such as the ability to prophesy, to its holders. This", "Deacons are called by God, affirmed by the church, and ordained by a bishop to servant leadership within the church.They are ordained to ministries of word, service, compassion, and justice. They may be appointed to ministry within the local church or to an extension ministry that supports the mission of the church. Deacons give leadership, preach the Word, contribute in worship, conduct marriages, bury the dead, and aid the church in embodying its mission within the world. Deacons assist elders in the sacraments of Holy Communion and Baptism, and may be granted sacramental authority if they are appointed as the pastor in a local church. Deacons serve a term of 2–3 years as provisional deacons prior to their ordination.", "are expected to defer to the father of the house when in his home. Further, additional spiritual guidance is offered by those holding the office of Patriarch, which is supposed by Latter-day Saints to grant certain gifts of the Spirit, such as the ability to prophesy, to its holders. This guidance is generally offered during a ceremony called the patriarchal blessing."]</t>
-        </is>
-      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -7957,21 +5527,6 @@
 In addition to chlorophylls, another group of yellow–orange pigments called carotenoids are also found in the photosystems. There are about thirty photosynthetic carotenoids. They help transfer and dissipate excess energy, and their bright colors sometimes override the chlorophyll green, like during the fall, when the leaves of some land plants change color. β-carotene is a bright red-orange carotenoid found in nearly all chloroplasts, like chlorophyll a. Xanthophylls, especially the orange-red zeaxanthin, are also common. Many other forms of carotenoids exist that are only found in certain groups of chloroplasts.</t>
         </is>
       </c>
-      <c r="F163" t="inlineStr">
-        <is>
-          <t>[326, 164, 90, 360, 223]</t>
-        </is>
-      </c>
-      <c r="G163" t="inlineStr">
-        <is>
-          <t>[0.8437896966934204, 0.804824709892273, 0.7483727335929871, 0.7393100261688232, 0.7113282084465027]</t>
-        </is>
-      </c>
-      <c r="H163" t="inlineStr">
-        <is>
-          <t>["To fix carbon dioxide into sugar molecules in the process of photosynthesis, chloroplasts use an enzyme called rubisco. Rubisco has a problem—it has trouble distinguishing between carbon dioxide and oxygen, so at high oxygen concentrations, rubisco starts accidentally adding oxygen to sugar precursors. This has the end result of ATP energy being wasted and CO2 being released, all with no sugar being produced. This is a big problem, since O2 is produced by the initial light reactions of photosynthesis, causing issues down the line in the Calvin cycle which uses rubisco.", "Photorespiration can occur when the oxygen concentration is too high. Rubisco cannot distinguish between oxygen and carbon dioxide very well, so it can accidentally add O2 instead of CO2 to RuBP. This process reduces the efficiency of photosynthesis—it consumes ATP and oxygen, releases CO2, and produces no sugar. It can waste up to half the carbon fixed by the Calvin cycle. Several mechanisms have evolved in different lineages that raise the carbon dioxide concentration relative to oxygen within the chloroplast, increasing the efficiency of photosynthesis. These mechanisms are called carbon dioxide concentrating mechanisms, or CCMs. These include Crassulacean acid metabolism, C4 carbon fixation, and pyrenoids. Chloroplasts in C4 plants are notable as they exhibit a distinct chloroplast dimorphism.", "One of the main functions of the chloroplast is its role in photosynthesis, the process by which light is transformed into chemical energy, to subsequently produce food in the form of sugars. Water (H2O) and carbon dioxide (CO2) are used in photosynthesis, and sugar and oxygen (O2) is made, using light energy. Photosynthesis is divided into two stages—the light reactions, where water is split to produce oxygen, and the dark reactions, or Calvin cycle, which builds sugar molecules from carbon dioxide. The two phases are linked by the energy carriers adenosine triphosphate (ATP) and nicotinamide adenine dinucleotide phosphate (NADP+).", "Chloroplasts' main role is to conduct photosynthesis, where the photosynthetic pigment chlorophyll captures the energy from sunlight and converts it and stores it in the energy-storage molecules ATP and NADPH while freeing oxygen from water. They then use the ATP and NADPH to make organic molecules from carbon dioxide in a process known as the Calvin cycle. Chloroplasts carry out a number of other functions, including fatty acid synthesis, much amino acid synthesis, and the immune response in plants. The number of chloroplasts per cell varies from 1 in algae up to 100 in plants like Arabidopsis and wheat.", "In addition to chlorophylls, another group of yellow–orange pigments called carotenoids are also found in the photosystems. There are about thirty photosynthetic carotenoids. They help transfer and dissipate excess energy, and their bright colors sometimes override the chlorophyll green, like during the fall, when the leaves of some land plants change color. β-carotene is a bright red-orange carotenoid found in nearly all chloroplasts, like chlorophyll a. Xanthophylls, especially the orange-red zeaxanthin, are also common. Many other forms of carotenoids exist that are only found in certain groups of chloroplasts."]</t>
-        </is>
-      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -8003,21 +5558,6 @@
 The reason for the majority rule is the high risk of a conflict of interest and/or the avoidance of absolute powers. Otherwise, the physician has a financial self-interest in "diagnosing" as many conditions as possible, and in exaggerating their seriousness, because he or she can then sell more medications to the patient. Such self-interest directly conflicts with the patient's interest in obtaining cost-effective medication and avoiding the unnecessary use of medication that may have side-effects. This system reflects much similarity to the checks and balances system of the U.S. and many other governments.[citation needed]</t>
         </is>
       </c>
-      <c r="F164" t="inlineStr">
-        <is>
-          <t>[827, 686, 491, 414, 607]</t>
-        </is>
-      </c>
-      <c r="G164" t="inlineStr">
-        <is>
-          <t>[0.7221654653549194, 0.7143991589546204, 0.6981547474861145, 0.6936350464820862, 0.6929702162742615]</t>
-        </is>
-      </c>
-      <c r="H164" t="inlineStr">
-        <is>
-          <t>["United States and Western Europe than in China (due to a greater tendency to take on debts).[unreliable source?][unreliable source?] Anthony Shorrocks, the lead author of the Credit Suisse report which is one of the sources of Oxfam's data, considers the criticism about debt to be a \"silly argument\" and \"a non-issue . . . a diversion.\"", "LeGrande writes that \"the formulation of a single all-encompassing definition of the term is extremely difficult, if not impossible. In reviewing the voluminous literature on the subject, the student of civil disobedience rapidly finds himself surrounded by a maze of semantical problems and grammatical niceties. Like Alice in Wonderland, he often finds that specific terminology has no more (or no less) meaning than the individual orator intends it to have.\" He encourages a distinction between lawful protest demonstration, nonviolent civil disobedience, and violent civil disobedience.", "According to Sheldon Ungar's comparison with global warming, the actors in the ozone depletion case had a better understanding of scientific ignorance and uncertainties. The ozone case communicated to lay persons \"with easy-to-understand bridging metaphors derived from the popular culture\" and related to \"immediate risks with everyday relevance\", while the public opinion on climate change sees no imminent danger. The stepwise mitigation of the ozone layer challenge was based as well on successfully reducing regional burden sharing conflicts. In case of the IPCC conclusions and the failure of the Kyoto Protocol, varying regional cost-benefit analysis and burden-sharing conflicts with regard to the distribution of emission reductions remain an unsolved problem. In the UK, a report for a House of Lords committee asked to urge the IPCC to involve better assessments of costs and benefits of climate change but the Stern Review ordered by the UK government made a stronger argument in favor to combat human-made climate change.", "Michael Oppenheimer, a long-time participant in the IPCC and coordinating lead author of the Fifth Assessment Report conceded in Science Magazine's State of the Planet 2008-2009 some limitations of the IPCC consensus approach and asks for concurring, smaller assessments of special problems instead of the large scale approach as in the previous IPCC assessment reports. It has become more important to provide a broader exploration of uncertainties. Others see as well mixed blessings of the drive for consensus within the IPCC process and ask to include dissenting or minority positions or to improve statements about uncertainties.", "The reason for the majority rule is the high risk of a conflict of interest and/or the avoidance of absolute powers. Otherwise, the physician has a financial self-interest in \"diagnosing\" as many conditions as possible, and in exaggerating their seriousness, because he or she can then sell more medications to the patient. Such self-interest directly conflicts with the patient's interest in obtaining cost-effective medication and avoiding the unnecessary use of medication that may have side-effects. This system reflects much similarity to the checks and balances system of the U.S. and many other governments.[citation needed]"]</t>
-        </is>
-      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -8049,21 +5589,6 @@
 Some of the oldest schools in South Africa are private church schools that were established by missionaries in the early nineteenth century. The private sector has grown ever since. After the abolition of apartheid, the laws governing private education in South Africa changed significantly. The South African Schools Act of 1996 recognises two categories of schools: "public" (state-controlled) and "independent" (which includes traditional private schools and schools which are privately governed[clarification needed].)</t>
         </is>
       </c>
-      <c r="F165" t="inlineStr">
-        <is>
-          <t>[166, 524, 660, 207, 772]</t>
-        </is>
-      </c>
-      <c r="G165" t="inlineStr">
-        <is>
-          <t>[0.8814725279808044, 0.8184941411018372, 0.7946382164955139, 0.7648248672485352, 0.7566242814064026]</t>
-        </is>
-      </c>
-      <c r="H165" t="inlineStr">
-        <is>
-          <t>["There are eleven LEA-funded 11 to 18 schools and seven independent schools with sixth forms in Newcastle. There are a number of successful state schools, including Walker Technology College, Gosforth High School, Heaton Manor School, St Cuthbert's High School, St. Mary's Catholic Comprehensive School, Kenton School, George Stephenson High School, Sacred Heart and Benfield School. The largest co-ed independent school is the Royal Grammar School. The largest girls' independent school is Newcastle High School for Girls. Both schools are located on the same street in Jesmond. Newcastle School for Boys is the only independent boys' only school in the city and is situated in Gosforth. Newcastle College is the largest general further education college in the North East and is a beacon status college; there are two smaller colleges in the Newcastle area. St Cuthbert's High School and Sacred Heart are the two primary state-Catholic run high schools, and are both achieving results on par with the independent schools in Newcastle.", "Private schools generally prefer to be called independent schools, because of their freedom to operate outside of government and local government control. Some of these are also known as public schools. Preparatory schools in the UK prepare pupils aged up to 13 years old to enter public schools. The name \"public school\" is based on the fact that the schools were open to pupils from anywhere, and not merely to those from a certain locality, and of any religion or occupation. According to The Good Schools Guide approximately 9 per cent of children being educated in the UK are doing so at fee-paying schools at GSCE level and 13 per cent at A-level.[citation needed] Many independent schools are single-sex (though this is becoming less common). Fees range from under £3,000 to £21,000 and above per year for day pupils, rising to £27,000+ per year for boarders. For details in Scotland, see \"Meeting the Cost\".", "Private schools are often Anglican, such as King's College and Diocesan School for Girls in Auckland, St Paul's Collegiate School in Hamilton, St Peter's School in Cambridge, Samuel Marsden Collegiate School in Wellington, and Christ's College and St Margaret's College in Christchurch; or Presbyterian, such as Saint Kentigern College and St Cuthbert's College in Auckland, Scots College and Queen Margaret College in Wellington, and St Andrew's College and Rangi Ruru Girls' School in Christchurch. Academic Colleges Group is a recent group of private schools run as a business, with schools throughout Auckland, including ACG Senior College in Auckland’s CBD, ACG Parnell College in Parnell, and international school ACG New Zealand International College. There are three private schools (including the secondary school, St Dominic's College) operated by the Catholic schismatic group, the Society of St Pius X in Wanganui.", "In the final years of the apartheid era, parents at white government schools were given the option to convert to a \"semi-private\" form called Model C, and many of these schools changed their admissions policies to accept children of other races. Following the transition to democracy, the legal form of \"Model C\" was abolished, however, the term continues to be used to describe government schools formerly reserved for white children.. These schools tend to produce better academic results than government schools formerly reserved for other race groups . Former \"Model C\" schools are not private schools, as they are state-controlled. All schools in South Africa (including both independent schools and public schools) have the right to set compulsory school fees, and formerly model C schools tend to set much higher school fees than other public schools.", "Some of the oldest schools in South Africa are private church schools that were established by missionaries in the early nineteenth century. The private sector has grown ever since. After the abolition of apartheid, the laws governing private education in South Africa changed significantly. The South African Schools Act of 1996 recognises two categories of schools: \"public\" (state-controlled) and \"independent\" (which includes traditional private schools and schools which are privately governed[clarification needed].)"]</t>
-        </is>
-      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -8095,21 +5620,6 @@
 were very few North Chinese or Southerners reaching the highest-post in the government compared with the possibility that Persians did so in the Ilkhanate. Later the Yongle Emperor of the Ming dynasty also mentioned the discrimination that existed during the Yuan dynasty. In response to an objection against the use of "barbarians" in his government, the Yongle Emperor answered: "... Discrimination was used by the Mongols during the Yuan dynasty, who employed only "Mongols and Tartars" and discarded northern and southern Chinese and this was precisely the cause that brought disaster upon them".</t>
         </is>
       </c>
-      <c r="F166" t="inlineStr">
-        <is>
-          <t>[167, 140, 499, 582, 364]</t>
-        </is>
-      </c>
-      <c r="G166" t="inlineStr">
-        <is>
-          <t>[0.9014887809753418, 0.8094683885574341, 0.7704184055328369, 0.765084445476532, 0.762753427028656]</t>
-        </is>
-      </c>
-      <c r="H166" t="inlineStr">
-        <is>
-          <t>["One of the more notable applications of printing technology was the chao, the paper money of the Yuan. Chao were made from the bark of mulberry trees. The Yuan government used woodblocks to print paper money, but switched to bronze plates in 1275. The Mongols experimented with establishing the Chinese-style paper monetary system in Mongol-controlled territories outside of China. The Yuan minister Bolad was sent to Iran, where he explained Yuan paper money to the Il-khanate court of Gaykhatu. The Il-khanate government issued paper money in 1294, but public distrust of the exotic new currency doomed the experiment.", "The Mongol rulers patronized the Yuan printing industry. Chinese printing technology was transferred to the Mongols through Kingdom of Qocho and Tibetan intermediaries. Some Yuan documents such as Wang Zhen's Nong Shu were printed with earthenware movable type, a technology invented in the 12th century. However, most published works were still produced through traditional block printing techniques. The publication of a Taoist text inscribed with the name of Töregene Khatun, Ögedei's wife, is one of the first printed works sponsored by the Mongols. In 1273, the Mongols created the Imperial Library Directorate, a government-sponsored printing office. The Yuan government established centers for printing throughout China. Local schools and government agencies were funded to support the publishing of books.", "The Yuan undertook extensive public works. Among Kublai Khan's top engineers and scientists was the astronomer Guo Shoujing, who was tasked with many public works projects and helped the Yuan reform the lunisolar calendar to provide an accuracy of 365.2425 days of the year, which was only 26 seconds off the modern Gregorian calendar's measurement. Road and water communications were reorganized and improved. To provide against possible famines, granaries were ordered built throughout the empire. The city of Beijing was rebuilt with new palace grounds that included artificial lakes, hills and mountains, and parks. During the Yuan period, Beijing became the terminus of the Grand Canal of China, which was completely renovated. These commercially oriented improvements encouraged overland and maritime commerce throughout Asia and facilitated direct Chinese contacts with Europe. Chinese travelers to the West were able to provide assistance in such areas as hydraulic engineering. Contacts with the West also brought the introduction to China of a major food crop, sorghum, along with other foreign food products and methods of preparation.", "The fourth Yuan emperor, Buyantu Khan (Ayurbarwada), was a competent emperor. He was the first Yuan emperor to actively support and adopt mainstream Chinese culture after the reign of Kublai, to the discontent of some Mongol elite. He had been mentored by Li Meng, a Confucian academic. He made many reforms, including the liquidation of the Department of State Affairs (Chinese: 尚書省), which resulted in the execution of five of the highest-ranking officials. Starting in 1313 the traditional imperial examinations were reintroduced for prospective officials, testing their knowledge on significant historical works. Also, he codified much of the law, as well as publishing or translating a number of Chinese books and works.", "were very few North Chinese or Southerners reaching the highest-post in the government compared with the possibility that Persians did so in the Ilkhanate. Later the Yongle Emperor of the Ming dynasty also mentioned the discrimination that existed during the Yuan dynasty. In response to an objection against the use of \"barbarians\" in his government, the Yongle Emperor answered: \"... Discrimination was used by the Mongols during the Yuan dynasty, who employed only \"Mongols and Tartars\" and discarded northern and southern Chinese and this was precisely the cause that brought disaster upon them\"."]</t>
-        </is>
-      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -8141,21 +5651,6 @@
 Justifying Grace or Accepting Grace is that grace, offered by God to all people, that we receive by faith and trust in Christ, through which God pardons the believer of sin. It is in justifying grace we are received by God, in spite of our sin. In this reception, we are forgiven through the atoning work of Jesus Christ on the cross. The justifying grace cancels our guilt and empowers us to resist the power of sin and to fully love God and neighbor. Today, justifying grace is also known as conversion, "accepting Jesus as your personal Lord and Savior," or being "born again". John Wesley originally called this experience the New Birth. This experience can occur in different ways; it can be one transforming moment, such as an altar call experience, or it may involve a series of decisions across a period of time.</t>
         </is>
       </c>
-      <c r="F167" t="inlineStr">
-        <is>
-          <t>[168, 610, 495, 398, 65]</t>
-        </is>
-      </c>
-      <c r="G167" t="inlineStr">
-        <is>
-          <t>[0.8448802828788757, 0.807860255241394, 0.8057610988616943, 0.7967115640640259, 0.7620871663093567]</t>
-        </is>
-      </c>
-      <c r="H167" t="inlineStr">
-        <is>
-          <t>["He insisted that, since forgiveness was God's alone to grant, those who claimed that indulgences absolved buyers from all punishments and granted them salvation were in error. Christians, he said, must not slacken in following Christ on account of such false assurances.", "However, this oft-quoted saying of Tetzel was by no means representative of contemporary Catholic teaching on indulgences, but rather a reflection of his capacity to exaggerate. Yet if Tetzel overstated the matter in regard to indulgences for the dead, his teaching on indulgences for the living was in line with Catholic dogma of the time.", "In the summer of 1521, Luther widened his target from individual pieties like indulgences and pilgrimages to doctrines at the heart of Church practices. In On the Abrogation of the Private Mass, he condemned as idolatry the idea that the mass is a sacrifice, asserting instead that it is a gift, to be received with thanksgiving by the whole congregation. His essay On Confession, Whether the Pope has the Power to Require It rejected compulsory confession and encouraged private confession and absolution, since \"every Christian is a confessor.\" In November, Luther wrote The Judgement of Martin Luther on Monastic Vows. He assured monks and nuns that they could break their vows without sin, because vows were an illegitimate and vain attempt to win salvation.", "Luther's rediscovery of \"Christ and His salvation\" was the first of two points that became the foundation for the Reformation. His railing against the sale of indulgences was based on it.", "Justifying Grace or Accepting Grace is that grace, offered by God to all people, that we receive by faith and trust in Christ, through which God pardons the believer of sin. It is in justifying grace we are received by God, in spite of our sin. In this reception, we are forgiven through the atoning work of Jesus Christ on the cross. The justifying grace cancels our guilt and empowers us to resist the power of sin and to fully love God and neighbor. Today, justifying grace is also known as conversion, \"accepting Jesus as your personal Lord and Savior,\" or being \"born again\". John Wesley originally called this experience the New Birth. This experience can occur in different ways; it can be one transforming moment, such as an altar call experience, or it may involve a series of decisions across a period of time."]</t>
-        </is>
-      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -8187,21 +5682,6 @@
 By the opening of the 2008 General Conference, total UMC membership was estimated at 11.4 million, with about 7.9 million in the U.S. and 3.5 million overseas. Significantly, about 20% of the conference delegates were from Africa, with Filipinos and Europeans making up another 10%. During the conference, the delegates voted to finalize the induction of the Methodist Church of the Ivory Coast and its 700,000 members into the denomination. Given current trends in the UMC—with overseas churches growing, especially in Africa, and U.S. churches collectively losing about 1,000 members a week—it has been estimated that Africans will make up at least 30% of the delegates at the 2012 General Conference, and it is also possible that 40% of the delegates will be from outside the U.S. One Congolese bishop has estimated that typical Sunday attendance of the UMC is higher in his country than in the entire United States.</t>
         </is>
       </c>
-      <c r="F168" t="inlineStr">
-        <is>
-          <t>[169, 219, 796, 354, 674]</t>
-        </is>
-      </c>
-      <c r="G168" t="inlineStr">
-        <is>
-          <t>[0.7732163667678833, 0.7577083706855774, 0.7357963919639587, 0.7118159532546997, 0.7018125057220459]</t>
-        </is>
-      </c>
-      <c r="H168" t="inlineStr">
-        <is>
-          <t>["The Book of Discipline is the guidebook for local churches and pastors and describes in considerable detail the organizational structure of local United Methodist churches. All UM churches must have a board of trustees with at least three members and no more than nine members and it is recommended that no gender should hold more than a 2/3 majority. All churches must also have a nominations committee, a finance committee and a church council or administrative council. Other committees are suggested but not required such as a missions committee, or evangelism or worship committee. Term limits are set for some committees but not for all. The church conference is an annual meeting of all the officers of the church and any interested members. This committee has the exclusive power to set pastors' salaries (compensation packages for tax purposes) and to elect officers to the committees.", "Decisions in-between the four-year meetings are made by the Mission Council (usually consisting of church bishops). One of the most high profile decisions in recent years by one of the councils was a decision by the Mission Council of the South Central Jurisdiction which in March 2007 approved a 99-year lease of 36 acres (150,000 m2) at Southern Methodist University for the George W. Bush Presidential Library. The decision generated controversy in light of Bush's support of the Iraq War which the church bishops have criticized. A debate over whether the decision should or could be submitted for approval by the Southern Jurisdictional Conference at its July 2008 meeting in Dallas, Texas, remains unresolved.", "in the legislative process still remains limited because no member can actually or pass legislation without the Commission and Council, meaning power (\"kratia\") is not in the hands of directly elected representatives of the people (\"demos\"): in the EU it is not yet true that \"the administration is in the hands of the many and not of the few.\"", "Immediately after Decision Time a \"Members Debate\" is held, which lasts for 45 minutes. Members Business is a debate on a motion proposed by an MSP who is not a Scottish minister. Such motions are on issues which may be of interest to a particular area such as a member's own constituency, an upcoming or past event or any other item which would otherwise not be accorded official parliamentary time. As well as the proposer, other members normally contribute to the debate. The relevant minister, whose department the debate and motion relate to \"winds up\" the debate by speaking after all other participants.", "By the opening of the 2008 General Conference, total UMC membership was estimated at 11.4 million, with about 7.9 million in the U.S. and 3.5 million overseas. Significantly, about 20% of the conference delegates were from Africa, with Filipinos and Europeans making up another 10%. During the conference, the delegates voted to finalize the induction of the Methodist Church of the Ivory Coast and its 700,000 members into the denomination. Given current trends in the UMC—with overseas churches growing, especially in Africa, and U.S. churches collectively losing about 1,000 members a week—it has been estimated that Africans will make up at least 30% of the delegates at the 2012 General Conference, and it is also possible that 40% of the delegates will be from outside the U.S. One Congolese bishop has estimated that typical Sunday attendance of the UMC is higher in his country than in the entire United States."]</t>
-        </is>
-      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -8233,21 +5713,6 @@
 Luther had published his German translation of the New Testament in 1522, and he and his collaborators completed the translation of the Old Testament in 1534, when the whole Bible was published. He continued to work on refining the translation until the end of his life. Others had translated the Bible into German, but Luther tailored his translation to his own doctrine. When he was criticised for inserting the word "alone" after "faith" in Romans 3:28, he replied in part: "[T]he text itself and the meaning of St. Paul urgently require and demand it. For in that very passage he is dealing with the main point of Christian doctrine, namely, that we are justified by faith in Christ without any works of the Law. ... But when works are so completely cut away – and that must mean that faith alone justifies – whoever would speak plainly and clearly about this cutting away of works will have to say, 'Faith alone justifies us, and not works'."</t>
         </is>
       </c>
-      <c r="F169" t="inlineStr">
-        <is>
-          <t>[648, 398, 572, 305, 214]</t>
-        </is>
-      </c>
-      <c r="G169" t="inlineStr">
-        <is>
-          <t>[0.8836939334869385, 0.8733492493629456, 0.869311511516571, 0.8673022389411926, 0.8639667630195618]</t>
-        </is>
-      </c>
-      <c r="H169" t="inlineStr">
-        <is>
-          <t>["Luther taught that salvation and subsequently eternal life is not earned by good deeds but is received only as a free gift of God's grace through faith in Jesus Christ as redeemer from sin. His theology challenged the authority and office of the Pope by teaching that the Bible is the only source of divinely revealed knowledge from God and opposed sacerdotalism by considering all baptized Christians to be a holy priesthood. Those who identify with these, and all of Luther's wider teachings, are called Lutherans even though Luther insisted on Christian or Evangelical as the only acceptable names for individuals who professed Christ.", "Luther's rediscovery of \"Christ and His salvation\" was the first of two points that became the foundation for the Reformation. His railing against the sale of indulgences was based on it.", "(1528), drafted by Melanchthon with Luther's approval, stressed the role of repentance in the forgiveness of sins, despite Luther's position that faith alone ensures justification. The Eisleben reformer Johannes Agricola challenged this compromise, and Luther condemned him for teaching that faith is separate from works. The Instruction is a problematic document for those seeking a consistent evolution in Luther's thought and practice.", "In his theses and disputations against the antinomians, Luther reviews and reaffirms, on the one hand, what has been called the \"second use of the law,\" that is, the law as the Holy Spirit's tool to work sorrow over sin in man's heart, thus preparing him for Christ's fulfillment of the law offered in the gospel. Luther states that everything that is used to work sorrow over sin is called the law, even if it is Christ's life, Christ's death for sin, or God's goodness experienced in creation. Simply refusing to preach the Ten Commandments among Christians – thereby, as it were, removing the three letters l-a-w from the church – does not eliminate the accusing law. Claiming that the law – in any form – should not be preached to Christians anymore would be tantamount to asserting that Christians are no longer sinners in themselves and that the church consists only of essentially holy people.", "Luther had published his German translation of the New Testament in 1522, and he and his collaborators completed the translation of the Old Testament in 1534, when the whole Bible was published. He continued to work on refining the translation until the end of his life. Others had translated the Bible into German, but Luther tailored his translation to his own doctrine. When he was criticised for inserting the word \"alone\" after \"faith\" in Romans 3:28, he replied in part: \"[T]he text itself and the meaning of St. Paul urgently require and demand it. For in that very passage he is dealing with the main point of Christian doctrine, namely, that we are justified by faith in Christ without any works of the Law. ... But when works are so completely cut away – and that must mean that faith alone justifies – whoever would speak plainly and clearly about this cutting away of works will have to say, 'Faith alone justifies us, and not works'.\""]</t>
-        </is>
-      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -8279,21 +5744,6 @@
 In early 2012, NFL Commissioner Roger Goodell stated that the league planned to make the 50th Super Bowl "spectacular" and that it would be "an important game for us as a league".</t>
         </is>
       </c>
-      <c r="F170" t="inlineStr">
-        <is>
-          <t>[171, 39, 37, 121, 418]</t>
-        </is>
-      </c>
-      <c r="G170" t="inlineStr">
-        <is>
-          <t>[0.7979496121406555, 0.7390866279602051, 0.7380450367927551, 0.7276219725608826, 0.7187849283218384]</t>
-        </is>
-      </c>
-      <c r="H170" t="inlineStr">
-        <is>
-          <t>["20th Century Fox, Lionsgate, Paramount Pictures, Universal Studios and Walt Disney Studios paid for movie trailers to be aired during the Super Bowl. Fox paid for Deadpool, X-Men: Apocalypse, Independence Day: Resurgence and Eddie the Eagle, Lionsgate paid for Gods of Egypt, Paramount paid for Teenage Mutant Ninja Turtles: Out of the Shadows and 10 Cloverfield Lane, Universal paid for The Secret Life of Pets and the debut trailer for Jason Bourne and Disney paid for Captain America: Civil War, The Jungle Book and Alice Through the Looking Glass.[citation needed]", "CBS broadcast Super Bowl 50 in the U.S., and charged an average of $5 million for a 30-second commercial during the game. The Super Bowl 50 halftime show was headlined by the British rock group Coldplay with special guest performers Beyoncé and Bruno Mars, who headlined the Super Bowl XLVII and Super Bowl XLVIII halftime shows, respectively. It was the third-most watched U.S. broadcast ever.", "stopped with its 1998–2002 four-note jingles for promotions and production company vanity cards following the closing credits of most of its programs over seventeen years, now it have a different and adventure-type music (with the drums of the network's four-note signature in the ending). The old four-note theme tune is still used by ABC on Demand to the beginning of the ABC show.", "CBS set the base rate for a 30-second advertisement at $5,000,000, a record high price for a Super Bowl ad. As of January 26, the advertisements had not yet sold out. CBS mandated that all advertisers purchase a package covering time on both the television and digital broadcasts of the game, meaning that for the first time, digital streams of the game would carry all national advertising in pattern with the television broadcast. This would be the final year in a multi-year contract with Anheuser-Busch InBev that allowed the beer manufacturer to air multiple advertisements during the game at a steep discount. It was also the final year that Doritos, a longtime sponsor of the game, held its \"Crash the Super Bowl\" contest that allowed viewers to create their own Doritos ads for a chance to have it aired during the game. Nintendo and The Pokémon Company also made their Super Bowl debut, promoting the 20th anniversary of the Pokémon video game and media franchise.", "In early 2012, NFL Commissioner Roger Goodell stated that the league planned to make the 50th Super Bowl \"spectacular\" and that it would be \"an important game for us as a league\"."]</t>
-        </is>
-      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -8325,21 +5775,6 @@
 For the next several years, Hoelun and her children lived in poverty, surviving primarily on wild fruits and ox carcasses, marmots, and other small game killed by Temüjin and his brothers. Begter, Temujin's older half-brother, began to exercise the power of the eldest male in the family and eventually Temujin's mother Hoelun (not Begter's mother) would have to accept him as her husband if and when he became an adult. Temujin's resentment erupted during one hunting excursion that Temüjin and his brother Khasar killed their half-brother Begter.</t>
         </is>
       </c>
-      <c r="F171" t="inlineStr">
-        <is>
-          <t>[172, 493, 791, 558, 190]</t>
-        </is>
-      </c>
-      <c r="G171" t="inlineStr">
-        <is>
-          <t>[0.8594177961349487, 0.7228624224662781, 0.7151615023612976, 0.7128396034240723, 0.7061353325843811]</t>
-        </is>
-      </c>
-      <c r="H171" t="inlineStr">
-        <is>
-          <t>["Near the end of his life, Tesla walked to the park every day to feed the pigeons and even brought injured ones into his hotel room to nurse back to health. He said that he had been visited by a specific injured white pigeon daily. Tesla spent over $2,000, including building a device that comfortably supported her so her bones could heal, to fix her broken wing and leg. Tesla stated,", "In 1874, Tesla evaded being drafted into the Austro-Hungarian Army in Smiljan by running away to Tomingaj, near Gračac. There, he explored the mountains in hunter's garb. Tesla said that this contact with nature made him stronger, both physically and mentally. He read many books while in Tomingaj, and later said that Mark Twain's works had helped him to miraculously recover from his earlier illness.", "In the Sandgate area, to the east of the city and beside the river, resided the close-knit community of keelmen and their families. They were so called because they worked on the keels, boats that were used to transfer coal from the river banks to the waiting colliers, for export to London and elsewhere. In the 1630s about 7,000 out of 20,000 inhabitants of Newcastle died of plague, more than one-third of the population. Specifically within the year 1636, it is roughly estimated with evidence held by the Society of Antiquaries that 47% of the then population of Newcastle died from the epidemic; this may also have been the most devastating loss in any British City in this period.", "to further the story by requesting exposition from the Doctor and manufacturing peril for the Doctor to resolve. The Doctor regularly gains new companions and loses old ones; sometimes they return home or find new causes — or loves — on worlds they have visited. Some have died during the course of the series. Companions are usually human, or humanoid aliens.", "For the next several years, Hoelun and her children lived in poverty, surviving primarily on wild fruits and ox carcasses, marmots, and other small game killed by Temüjin and his brothers. Begter, Temujin's older half-brother, began to exercise the power of the eldest male in the family and eventually Temujin's mother Hoelun (not Begter's mother) would have to accept him as her husband if and when he became an adult. Temujin's resentment erupted during one hunting excursion that Temüjin and his brother Khasar killed their half-brother Begter."]</t>
-        </is>
-      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -8371,21 +5806,6 @@
 The 1970s and 1980s saw the emergence of many graphical imaging packages for the network in which based the logo's setting mainly on special lighting effects then under development including white, blue, pink, rainbow neon and glittering dotted lines. Among the "ABC Circle" logo's many variants was a 1977 ID sequence that featured a bubble on a black background representing the circle with glossy gold letters, and as such, was the first ABC identification card to have a three-dimensional appearance.</t>
         </is>
       </c>
-      <c r="F172" t="inlineStr">
-        <is>
-          <t>[173, 379, 7, 770, 664]</t>
-        </is>
-      </c>
-      <c r="G172" t="inlineStr">
-        <is>
-          <t>[0.7694688439369202, 0.7651798129081726, 0.7633441090583801, 0.763314962387085, 0.7528460621833801]</t>
-        </is>
-      </c>
-      <c r="H172" t="inlineStr">
-        <is>
-          <t>["The Saturn IB was an upgraded version of the Saturn I. The S-IB first stage increased the thrust to 1,600,000 pounds-force (7,120 kN), and the second stage replaced the S-IV with the S-IVB-200, powered by a single J-2 engine burning liquid hydrogen fuel with LOX, to produce 200,000 lbf (890 kN) of thrust. A restartable version of the S-IVB was used as the third stage of the Saturn V. The Saturn IB could send over 40,000 pounds (18,100 kg) into low Earth orbit, sufficient for a partially fueled CSM or the LM. Saturn IB launch vehicles and flights were designated with an AS-200 series number, \"AS\" indicating \"Apollo Saturn\" and the \"2\" indicating the second member of the Saturn rocket family.", "In December 1966, the AS-205 mission was canceled, since the validation of the CSM would be accomplished on the 14-day first flight, and AS-205 would have been devoted to space experiments and contribute no new engineering knowledge about the spacecraft. Its Saturn IB was allocated to the dual mission, now redesignated AS-205/208 or AS-258, planned for August 1967. McDivitt, Scott and Schweickart were promoted to the prime AS-258 crew, and Schirra, Eisele and Cunningham were reassigned as the Apollo 1 backup crew.", "Seamans' establishment of an ad-hoc committee headed by his special technical assistant Nicholas E. Golovin in July 1961, to recommend a launch vehicle to be used in the Apollo program, represented a turning point in NASA's mission mode decision. This committee recognized that the chosen mode was an important part of the launch vehicle choice, and recommended in favor of a hybrid EOR-LOR mode. Its consideration of LOR —as well as Houbolt's ceaseless work— played an important role in publicizing the workability of the approach. In late 1961 and early 1962, members of the Manned Spacecraft Center began to come around to support LOR, including the newly hired deputy director of the Office of Manned Space Flight, Joseph Shea, who became a champion of LOR. The engineers at Marshall Space Flight Center (MSFC) took longer to become convinced of its merits, but their conversion was announced by Wernher von Braun at a briefing in June 1962.", "About the time of the first landing in 1969, it was decided to use an existing Saturn V to launch the Skylab orbital laboratory pre-built on the ground, replacing the original plan to construct it in orbit from several Saturn IB launches; this eliminated Apollo 20. NASA's yearly budget also began to shrink in light of the successful landing, and NASA also had to make funds available for the development of the upcoming Space Shuttle. By 1971, the decision was made to also cancel missions 18 and 19. The two unused Saturn Vs became museum exhibits at the John F. Kennedy Space Center on Merritt Island, Florida, George C. Marshall Space Center in Huntsville, Alabama, Michoud Assembly Facility in New Orleans, Louisiana, and Lyndon B. Johnson Space Center in Houston, Texas.", "The 1970s and 1980s saw the emergence of many graphical imaging packages for the network in which based the logo's setting mainly on special lighting effects then under development including white, blue, pink, rainbow neon and glittering dotted lines. Among the \"ABC Circle\" logo's many variants was a 1977 ID sequence that featured a bubble on a black background representing the circle with glossy gold letters, and as such, was the first ABC identification card to have a three-dimensional appearance."]</t>
-        </is>
-      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -8417,21 +5837,6 @@
 were designed by Reuben Townroe who also designed the plaster work in the library, Sir John Taylor designed the book shelves and cases, also this was the first part of the museum to have electric lighting. This completed the northern half of the site, creating a quadrangle with the garden at its centre, but left the museum without a proper façade. In 1890 the government launched a competition to design new buildings for the museum, with architect Alfred Waterhouse as one of the judges; this would give the museum a new imposing front entrance.</t>
         </is>
       </c>
-      <c r="F173" t="inlineStr">
-        <is>
-          <t>[174, 680, 138, 316, 588]</t>
-        </is>
-      </c>
-      <c r="G173" t="inlineStr">
-        <is>
-          <t>[0.7718218564987183, 0.7653807401657104, 0.7502463459968567, 0.7400222420692444, 0.7395358681678772]</t>
-        </is>
-      </c>
-      <c r="H173" t="inlineStr">
-        <is>
-          <t>["The first buildings of the University of Chicago campus, which make up what is now known as the Main Quadrangles, were part of a \"master plan\" conceived by two University of Chicago trustees and plotted by Chicago architect Henry Ives Cobb. The Main Quadrangles consist of six quadrangles, each surrounded by buildings, bordering one larger quadrangle. The buildings of the Main Quadrangles were designed by Cobb, Shepley, Rutan and Coolidge, Holabird &amp; Roche, and other architectural firms in a mixture of the Victorian Gothic and Collegiate Gothic styles, patterned on the colleges of the University of Oxford. (Mitchell Tower, for example, is modeled after Oxford's Magdalen Tower, and the university Commons, Hutchinson Hall, replicates Christ Church Hall.)", "The main façade, built from red brick and Portland stone, stretches 720 feet (220 m) along Cromwell Gardens and was designed by Aston Webb after winning a competition in 1891 to extend the museum. Construction took place between 1899 and 1909. Stylistically it is a strange hybrid, although much of the detail belongs to the Renaissance there are medieval influences at work. The main entrance consisting of a series of shallow arches supported by slender columns and niches with twin doors separated by pier is Romanesque in form but Classical in detail. Likewise the tower above the main entrance has an open work crown surmounted by a statue of fame, a feature of late Gothic architecture and a feature common in Scotland, but the detail is Classical. The main windows to the galleries are also mullioned and transomed, again a Gothic feature, the top row of windows are interspersed with statues of many of the British artists whose work is displayed in the museum.", "After the 1940s, the Gothic style on campus began to give way to modern styles. In 1955, Eero Saarinen was contracted to develop a second master plan, which led to the construction of buildings both north and south of the Midway, including the Laird Bell Law Quadrangle (a complex designed by Saarinen); a series of arts buildings; a building designed by Ludwig Mies van der Rohe for the university's School of Social Service Administration;, a building which is to become the home of the Harris School of Public Policy Studies by Edward Durrell Stone, and the Regenstein Library, the largest building on campus, a brutalist structure designed by Walter Netsch of the Chicago firm Skidmore, Owings &amp; Merrill. Another master plan, designed in 1999 and updated in 2004, produced the Gerald Ratner Athletics Center (2003), the Max Palevsky Residential Commons (2001), South Campus Residence Hall and dining commons (2009), a new children's hospital, and other construction, expansions, and restorations. In 2011, the university completed the glass dome-shaped Joe and Rika Mansueto Library, which provides a grand reading room for the university library and prevents the need for an off-campus book depository.", "The Tyneside flat was the dominant housing form constructed at the time when the industrial centres on Tyneside were growing most rapidly. They can still be found in areas such as South Heaton in Newcastle but once dominated the streetscape on both sides of the Tyne. Tyneside flats were built as terraces, one of each pair of doors led to an upstairs flat while the other led into the ground-floor flat, each of two or three rooms. A new development in the Ouseburn valley has recreated them; Architects Cany Ash and Robert Sakula were attracted by the possibilities of high density without building high and getting rid of common areas.", "were designed by Reuben Townroe who also designed the plaster work in the library, Sir John Taylor designed the book shelves and cases, also this was the first part of the museum to have electric lighting. This completed the northern half of the site, creating a quadrangle with the garden at its centre, but left the museum without a proper façade. In 1890 the government launched a competition to design new buildings for the museum, with architect Alfred Waterhouse as one of the judges; this would give the museum a new imposing front entrance."]</t>
-        </is>
-      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -8463,21 +5868,6 @@
 The Colorado experiments had prepared Tesla for the establishment of the trans-Atlantic wireless telecommunications facility known as Wardenclyffe near Shoreham, Long Island.</t>
         </is>
       </c>
-      <c r="F174" t="inlineStr">
-        <is>
-          <t>[175, 318, 339, 606, 444]</t>
-        </is>
-      </c>
-      <c r="G174" t="inlineStr">
-        <is>
-          <t>[0.8285174369812012, 0.72670978307724, 0.7178396582603455, 0.7098785042762756, 0.7077628374099731]</t>
-        </is>
-      </c>
-      <c r="H174" t="inlineStr">
-        <is>
-          <t>["For exercise, Tesla walked between 8 to 10 miles per day. He squished his toes one hundred times for each foot every night, saying that it stimulated his brain cells.", "Tesla was renowned for his achievements and showmanship, eventually earning him a reputation in popular culture as an archetypal \"mad scientist\". His patents earned him a considerable amount of money, much of which was used to finance his own projects with varying degrees of success.:121,154 He lived most of his life in a series of New York hotels, through his retirement. Tesla died on 7 January 1943. His work fell into relative obscurity after his death, but in 1960 the General Conference on Weights and Measures named the SI unit of magnetic flux density the tesla in his honor. There has been a resurgence in popular interest in Tesla since the 1990s.", "During that year, Tesla worked in Pittsburgh, helping to create an alternating current system to power the city's streetcars. He found the time there frustrating because of conflicts between him and the other Westinghouse engineers over how best to implement AC power. Between them, they settled on a 60-cycle AC current system Tesla proposed (to match the working frequency of Tesla's motor), although they soon found that, since Tesla's induction motor could only run at a constant speed, it would not work for street cars. They ended up using a DC traction motor instead.", "Many of Tesla's writings are freely available on the web, including the article \"The Problem of Increasing Human Energy,\" published in The Century Magazine in 1900, and the article \"Experiments With Alternate Currents Of High Potential And High Frequency,\" published in his book Inventions, Researches and Writings of Nikola Tesla.", "The Colorado experiments had prepared Tesla for the establishment of the trans-Atlantic wireless telecommunications facility known as Wardenclyffe near Shoreham, Long Island."]</t>
-        </is>
-      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -8509,21 +5899,6 @@
 A new arrangement of the theme, once again by Gold, was introduced in the 2007 Christmas special episode, "Voyage of the Damned"; Gold returned as composer for the 2010 series. He was responsible for a new version of the theme which was reported to have had a hostile reception from some viewers. In 2011, the theme tune charted at number 228 of radio station Classic FM's Hall of Fame, a survey of classical music tastes. A revised version of Gold's 2010 arrangement had its debut over the opening titles of the 2012 Christmas special "The Snowmen", and a further revision of the arrangement was made for the 50th Anniversary special "The Day of the Doctor" in November 2013.[citation needed]</t>
         </is>
       </c>
-      <c r="F175" t="inlineStr">
-        <is>
-          <t>[176, 37, 776, 563, 110]</t>
-        </is>
-      </c>
-      <c r="G175" t="inlineStr">
-        <is>
-          <t>[0.7531571388244629, 0.7055341601371765, 0.7044075727462769, 0.6979140043258667, 0.6954566836357117]</t>
-        </is>
-      </c>
-      <c r="H175" t="inlineStr">
-        <is>
-          <t>["Six-time Grammy winner and Academy Award nominee Lady Gaga performed the national anthem, while Academy Award winner Marlee Matlin provided American Sign Language (ASL) translation.", "stopped with its 1998–2002 four-note jingles for promotions and production company vanity cards following the closing credits of most of its programs over seventeen years, now it have a different and adventure-type music (with the drums of the network's four-note signature in the ending). The old four-note theme tune is still used by ABC on Demand to the beginning of the ABC show.", "as a selection of classics based on the theme of space and time. The event was presented by Freema Agyeman and guest-presented by various other stars of the show with numerous monsters participating in the proceedings. It also featured the specially filmed mini-episode \"Music of the Spheres\", written by Russell T Davies and starring David Tennant.", "Pink Floyd, the Australian string ensemble Fourplay, New Zealand punk band Blam Blam Blam, The Pogues, Thin Lizzy, Dub Syndicate, and the comedians Bill Bailey and Mitch Benn. Both the theme and obsessive fans were satirised on The Chaser's War on Everything. The theme tune has also appeared on many compilation CDs, and has made its way into mobile-phone ringtones. Fans have also produced and distributed their own remixes of the theme. In January 2011 the Mankind version was released as a digital download on the album Gallifrey And Beyond.", "A new arrangement of the theme, once again by Gold, was introduced in the 2007 Christmas special episode, \"Voyage of the Damned\"; Gold returned as composer for the 2010 series. He was responsible for a new version of the theme which was reported to have had a hostile reception from some viewers. In 2011, the theme tune charted at number 228 of radio station Classic FM's Hall of Fame, a survey of classical music tastes. A revised version of Gold's 2010 arrangement had its debut over the opening titles of the 2012 Christmas special \"The Snowmen\", and a further revision of the arrangement was made for the 50th Anniversary special \"The Day of the Doctor\" in November 2013.[citation needed]"]</t>
-        </is>
-      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -8555,21 +5930,6 @@
 the vast majority of large electric generating stations, turbines are directly connected to generators with no reduction gearing. Typical speeds are 3600 revolutions per minute (RPM) in the USA with 60 Hertz power, 3000 RPM in Europe and other countries with 50 Hertz electric power systems. In nuclear power applications the turbines typically run at half these speeds, 1800 RPM and 1500 RPM. A turbine rotor is also only capable of providing power when rotating in one direction. Therefore, a reversing stage or gearbox is usually required where power is required in the opposite direction.[citation needed]</t>
         </is>
       </c>
-      <c r="F176" t="inlineStr">
-        <is>
-          <t>[262, 177, 686, 847, 178]</t>
-        </is>
-      </c>
-      <c r="G176" t="inlineStr">
-        <is>
-          <t>[0.738521158695221, 0.7253786325454712, 0.7165806889533997, 0.7067357301712036, 0.7047494053840637]</t>
-        </is>
-      </c>
-      <c r="H176" t="inlineStr">
-        <is>
-          <t>["It is possible to use a mechanism based on a pistonless rotary engine such as the Wankel engine in place of the cylinders and valve gear of a conventional reciprocating steam engine. Many such engines have been designed, from the time of James Watt to the present day, but relatively few were actually built and even fewer went into quantity production; see link at bottom of article for more details. The major problem is the difficulty of sealing the rotors to make them steam-tight in the face of wear and thermal expansion; the resulting leakage made them very inefficient. Lack of expansive working, or any means of control of the cutoff is also a serious problem with many such designs.[citation needed]", "A steam turbine consists of one or more rotors (rotating discs) mounted on a drive shaft, alternating with a series of stators (static discs) fixed to the turbine casing. The rotors have a propeller-like arrangement of blades at the outer edge. Steam acts upon these blades, producing rotary motion. The stator consists of a similar, but fixed, series of blades that serve to redirect the steam flow onto the next rotor stage. A steam turbine often exhausts into a surface condenser that provides a vacuum. The stages of a steam turbine are typically arranged to extract the maximum potential work from a specific velocity and pressure of steam, giving rise to a series of variably sized high- and low-pressure stages. Turbines are only efficient if they rotate at relatively high speed, therefore they are usually connected to reduction gearing to drive lower speed applications, such as a ship's propeller. In the vast majority of large electric generating stations, turbines are directly connected to generators with no reduction gearing. Typical speeds are 3600 revolutions per minute (RPM) in the USA with 60 Hertz power, 3000 RPM in Europe and other countries with 50 Hertz electric power systems. In nuclear power applications", "LeGrande writes that \"the formulation of a single all-encompassing definition of the term is extremely difficult, if not impossible. In reviewing the voluminous literature on the subject, the student of civil disobedience rapidly finds himself surrounded by a maze of semantical problems and grammatical niceties. Like Alice in Wonderland, he often finds that specific terminology has no more (or no less) meaning than the individual orator intends it to have.\" He encourages a distinction between lawful protest demonstration, nonviolent civil disobedience, and violent civil disobedience.", "Ranging from about 1 millimeter (0.039 in) to 1.5 meters (4.9 ft) in size, ctenophores are the largest non-colonial animals that use cilia (\"hairs\") as their main method of locomotion. Most species have eight strips, called comb rows, that run the length of their bodies and bear comb-like bands of cilia, called \"ctenes,\" stacked along the comb rows so that when the cilia beat, those of each comb touch the comb below. The name \"ctenophora\" means \"comb-bearing\", from the Greek κτείς (stem-form κτεν-) meaning \"comb\" and the Greek suffix -φορος meaning \"carrying\".", "the vast majority of large electric generating stations, turbines are directly connected to generators with no reduction gearing. Typical speeds are 3600 revolutions per minute (RPM) in the USA with 60 Hertz power, 3000 RPM in Europe and other countries with 50 Hertz electric power systems. In nuclear power applications the turbines typically run at half these speeds, 1800 RPM and 1500 RPM. A turbine rotor is also only capable of providing power when rotating in one direction. Therefore, a reversing stage or gearbox is usually required where power is required in the opposite direction.[citation needed]"]</t>
-        </is>
-      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -8601,21 +5961,6 @@
 (1528), drafted by Melanchthon with Luther's approval, stressed the role of repentance in the forgiveness of sins, despite Luther's position that faith alone ensures justification. The Eisleben reformer Johannes Agricola challenged this compromise, and Luther condemned him for teaching that faith is separate from works. The Instruction is a problematic document for those seeking a consistent evolution in Luther's thought and practice.</t>
         </is>
       </c>
-      <c r="F177" t="inlineStr">
-        <is>
-          <t>[179, 398, 480, 468, 572]</t>
-        </is>
-      </c>
-      <c r="G177" t="inlineStr">
-        <is>
-          <t>[0.8222711682319641, 0.8042536377906799, 0.7747495174407959, 0.7691924571990967, 0.7661213278770447]</t>
-        </is>
-      </c>
-      <c r="H177" t="inlineStr">
-        <is>
-          <t>["The effect of Luther's intervention was immediate. After the sixth sermon, the Wittenberg jurist Jerome Schurf wrote to the elector: \"Oh, what joy has Dr. Martin's return spread among us! His words, through divine mercy, are bringing back every day misguided people into the way of the truth.\"", "Luther's rediscovery of \"Christ and His salvation\" was the first of two points that became the foundation for the Reformation. His railing against the sale of indulgences was based on it.", "was one of the worst mistakes Luther made, and, next to the landgrave himself, who was directly responsible for it, history chiefly holds Luther accountable\". Brecht argues that Luther's mistake was not that he gave private pastoral advice, but that he miscalculated the political implications. The affair caused lasting damage to Luther's reputation.", "It was not until January 1518 that friends of Luther translated the 95 Theses from Latin into German and printed and widely copied them, making the controversy one of the first in history to be aided by the printing press. Within two weeks, copies of the theses had spread throughout Germany; within two months, they had spread throughout Europe.", "(1528), drafted by Melanchthon with Luther's approval, stressed the role of repentance in the forgiveness of sins, despite Luther's position that faith alone ensures justification. The Eisleben reformer Johannes Agricola challenged this compromise, and Luther condemned him for teaching that faith is separate from works. The Instruction is a problematic document for those seeking a consistent evolution in Luther's thought and practice."]</t>
-        </is>
-      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -8647,21 +5992,6 @@
 spend $2.5 million to convert 20 acres (80,937 m2) of land in Hollywood into what would become The Prospect Studios, and construct a transmitter on Mount Wilson, in anticipation of the launch of KECA-TV, which was scheduled to begin operations on August 1 (but would not actually sign on until September 16).</t>
         </is>
       </c>
-      <c r="F178" t="inlineStr">
-        <is>
-          <t>[180, 496, 66, 462, 707]</t>
-        </is>
-      </c>
-      <c r="G178" t="inlineStr">
-        <is>
-          <t>[0.8375118374824524, 0.7958711385726929, 0.7552851438522339, 0.7367407083511353, 0.7303292751312256]</t>
-        </is>
-      </c>
-      <c r="H178" t="inlineStr">
-        <is>
-          <t>["In the 1910s, New York–based filmmakers were attracted to Jacksonville's warm climate, exotic locations, excellent rail access, and cheap labor. Over the course of the decade, more than 30 silent film studios were established, earning Jacksonville the title of \"Winter Film Capital of the World\". However, the emergence of Hollywood as a major film production center ended the city's film industry. One converted movie studio site, Norman Studios, remains in Arlington; It has been converted to the Jacksonville Silent Film Museum at Norman Studios.", "The earliest known movie featuring some exterior scenes filmed in the city is On the Night of the Fire (1939), though by and large the action is studio-bound. Later came The Clouded Yellow (1951) and Payroll (1961), both of which feature more extensive scenes filmed in the city. The 1971 film Get Carter was shot on location in and around Newcastle and offers an opportunity to see what Newcastle looked like in the 1960s and early 1970s. The city was also backdrop to another gangster film, the 1988 film noir thriller Stormy Monday, directed by Mike Figgis and starring Tommy Lee Jones, Melanie Griffith, Sting and Sean Bean.", "On the television side, in September 1969, ABC launched the Movie of the Week, a weekly showcase aimed at capitalizing on the growing success of made-for-TV movies since the early 1960s. The Movie of the Week broadcast feature-length dramatic films directed by such talented filmmakers as Aaron Spelling, David Wolper and Steven Spielberg (the latter of whom gained early success through the showcase for his 1971 film Duel) that were produced on an average budget of $400,000–$450,000. Hits for the television network during the late 1960s and early 1970s included The Courtship of Eddie's Father, The Brady Bunch and The Partridge Family.", "In 1968, ABC took advantage of new FCC ownership regulations that allowed broadcasting companies to own a maximum of seven radio stations nationwide in order to purchase Houston radio stations KXYZ and KXYZ-FM for $1 million in shares and $1.5 million in bonds. That year, Roone Arledge was named president of ABC Sports; the company also founded ABC Pictures, a film production company which released its first picture that year, the Ralph Nelson-directed Charly. It was renamed ABC Motion Pictures in 1979; the unit was dissolved in 1985. The studio also operated two subsidiaries, Palomar Pictures International and Selmur Pictures. In July 1968, ABC continued its acquisitions in the amusement parks sector with the opening of ABC Marine World in Redwood City, California; that park was sold in 1972 and demolished in 1986, with the land that occupied the park later becoming home to the headquarters of Oracle Corporation.", "spend $2.5 million to convert 20 acres (80,937 m2) of land in Hollywood into what would become The Prospect Studios, and construct a transmitter on Mount Wilson, in anticipation of the launch of KECA-TV, which was scheduled to begin operations on August 1 (but would not actually sign on until September 16)."]</t>
-        </is>
-      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -8693,21 +6023,6 @@
 Decisions in-between the four-year meetings are made by the Mission Council (usually consisting of church bishops). One of the most high profile decisions in recent years by one of the councils was a decision by the Mission Council of the South Central Jurisdiction which in March 2007 approved a 99-year lease of 36 acres (150,000 m2) at Southern Methodist University for the George W. Bush Presidential Library. The decision generated controversy in light of Bush's support of the Iraq War which the church bishops have criticized. A debate over whether the decision should or could be submitted for approval by the Southern Jurisdictional Conference at its July 2008 meeting in Dallas, Texas, remains unresolved.</t>
         </is>
       </c>
-      <c r="F179" t="inlineStr">
-        <is>
-          <t>[141, 246, 24, 62, 219]</t>
-        </is>
-      </c>
-      <c r="G179" t="inlineStr">
-        <is>
-          <t>[0.7367825508117676, 0.7317453026771545, 0.7296972274780273, 0.7259955406188965, 0.7249631285667419]</t>
-        </is>
-      </c>
-      <c r="H179" t="inlineStr">
-        <is>
-          <t>["The African Great Lakes region, which Kenya is a part of, has been inhabited by humans since the Lower Paleolithic period. By the first millennium AD, the Bantu expansion had reached the area from West-Central Africa. The borders of the modern state consequently comprise the crossroads of the Niger-Congo, Nilo-Saharan and Afroasiatic areas of the continent, representing most major ethnolinguistic groups found in Africa. Bantu and Nilotic populations together constitute around 97% of the nation's residents. European and Arab presence in coastal Mombasa dates to the Early Modern period; European exploration of the interior began in the 19th century. The British Empire established the East Africa Protectorate in 1895, which starting in 1920 gave way to the Kenya Colony. Kenya obtained independence in December 1963. Following a referendum in August 2010 and adoption of a new constitution, Kenya is now divided into 47 semi-autonomous counties, governed by elected governors.", "Austria, Finland, Norway and Sweden in 1994 (though again Norway failed to join, because of lack of support in the referendum), the Czech Republic, Cyprus, Estonia, Hungary, Latvia, Lithuania, Malta, Poland, Slovakia and Slovenia in 2004, Romania and Bulgaria in 2007 and Croatia in 2013. Greenland signed a Treaty in 1985 giving it a special status.", "In 2010 the Amazon rainforest experienced another severe drought, in some ways more extreme than the 2005 drought. The affected region was approximate 1,160,000 square miles (3,000,000 km2) of rainforest, compared to 734,000 square miles (1,900,000 km2) in 2005. The 2010 drought had three epicenters where vegetation died off, whereas in 2005 the drought was focused on the southwestern part. The findings were published in the journal Science. In a typical year the Amazon absorbs 1.5 gigatons of carbon dioxide; during 2005 instead 5 gigatons were released and in 2010 8 gigatons were released.", "The Ottoman Empire was an imperial state that lasted from 1299 to 1923. During the 16th and 17th centuries, in particular at the height of its power under the reign of Suleiman the Magnificent, the Ottoman Empire was a powerful multinational, multilingual empire controlling much of Southeast Europe, Western Asia, the Caucasus, North Africa, and the Horn of Africa. At the beginning of the 17th century the empire contained 32 provinces and numerous vassal states. Some of these were later absorbed into the empire, while others were granted various types of autonomy during the course of centuries.", "Decisions in-between the four-year meetings are made by the Mission Council (usually consisting of church bishops). One of the most high profile decisions in recent years by one of the councils was a decision by the Mission Council of the South Central Jurisdiction which in March 2007 approved a 99-year lease of 36 acres (150,000 m2) at Southern Methodist University for the George W. Bush Presidential Library. The decision generated controversy in light of Bush's support of the Iraq War which the church bishops have criticized. A debate over whether the decision should or could be submitted for approval by the Southern Jurisdictional Conference at its July 2008 meeting in Dallas, Texas, remains unresolved."]</t>
-        </is>
-      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -8739,21 +6054,6 @@
 One theory is that, while disobedience may be helpful, any great amount of it would undermine the law by encouraging general disobedience which is neither conscientious nor of social benefit. Therefore, conscientious lawbreakers must be punished. Michael Bayles argues that if a person violates a law in order to create a test case as to the constitutionality of a law, and then wins his case, then that act did not constitute civil disobedience. It has also been argued that breaking the law for self-gratification, as in the case of a homosexual or cannabis user who does not direct his act at securing the repeal of amendment of the law, is not civil disobedience. Likewise, a protestor who attempts to escape punishment by committing the crime covertly and avoiding attribution, or by denying having committed the crime, or by fleeing the jurisdiction, is generally viewed as not being a civil disobedient.</t>
         </is>
       </c>
-      <c r="F180" t="inlineStr">
-        <is>
-          <t>[182, 760, 686, 683, 536]</t>
-        </is>
-      </c>
-      <c r="G180" t="inlineStr">
-        <is>
-          <t>[0.7480448484420776, 0.7386195659637451, 0.7338002324104309, 0.7328673601150513, 0.719681441783905]</t>
-        </is>
-      </c>
-      <c r="H180" t="inlineStr">
-        <is>
-          <t>["Civil disobedients have chosen a variety of different illegal acts. Bedau writes, \"There is a whole class of acts, undertaken in the name of civil disobedience, which, even if they were widely practiced, would in themselves constitute hardly more than a nuisance (e.g. trespassing at a nuclear-missile installation)...Such acts are often just a harassment and, at least to the bystander, somewhat inane...The remoteness of the connection between the disobedient act and the objectionable law lays such acts open to the charge of ineffectiveness and absurdity.\" Bedau also notes, though, that the very harmlessness of such entirely symbolic illegal protests toward public policy goals may serve a propaganda purpose. Some civil disobedients, such as the proprietors of illegal medical cannabis dispensaries and Voice in the Wilderness, which brought medicine to Iraq without the permission of the U.S. Government, directly achieve a desired social goal (such as the provision of medication to the sick) while openly breaking the law. Julia Butterfly Hill lived in Luna, a 180-foot (55 m)-tall, 600-year-old California Redwood tree for 738 days, successfully preventing it from being cut down.", "Some forms of civil disobedience, such as illegal boycotts, refusals to pay taxes, draft dodging, distributed denial-of-service attacks, and sit-ins, make it more difficult for a system to function. In this way, they might be considered coercive. Brownlee notes that \"although civil disobedients are constrained in their use of coercion by their conscientious aim to engage in moral dialogue, nevertheless they may find it necessary to employ limited coercion in order to get their issue onto the table.\" The Plowshares organization temporarily closed GCSB Waihopai by padlocking the gates and using sickles to deflate one of the large domes covering two satellite dishes.", "LeGrande writes that \"the formulation of a single all-encompassing definition of the term is extremely difficult, if not impossible. In reviewing the voluminous literature on the subject, the student of civil disobedience rapidly finds himself surrounded by a maze of semantical problems and grammatical niceties. Like Alice in Wonderland, he often finds that specific terminology has no more (or no less) meaning than the individual orator intends it to have.\" He encourages a distinction between lawful protest demonstration, nonviolent civil disobedience, and violent civil disobedience.", "The objective is typically a course of study, lesson plan, or a practical skill. A teacher may follow standardized curricula as determined by the relevant authority. The teacher may interact with students of different ages, from infants to adults, students with different abilities and students with learning disabilities.", "One theory is that, while disobedience may be helpful, any great amount of it would undermine the law by encouraging general disobedience which is neither conscientious nor of social benefit. Therefore, conscientious lawbreakers must be punished. Michael Bayles argues that if a person violates a law in order to create a test case as to the constitutionality of a law, and then wins his case, then that act did not constitute civil disobedience. It has also been argued that breaking the law for self-gratification, as in the case of a homosexual or cannabis user who does not direct his act at securing the repeal of amendment of the law, is not civil disobedience. Likewise, a protestor who attempts to escape punishment by committing the crime covertly and avoiding attribution, or by denying having committed the crime, or by fleeing the jurisdiction, is generally viewed as not being a civil disobedient."]</t>
-        </is>
-      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -8785,21 +6085,6 @@
 For the next several years, Hoelun and her children lived in poverty, surviving primarily on wild fruits and ox carcasses, marmots, and other small game killed by Temüjin and his brothers. Begter, Temujin's older half-brother, began to exercise the power of the eldest male in the family and eventually Temujin's mother Hoelun (not Begter's mother) would have to accept him as her husband if and when he became an adult. Temujin's resentment erupted during one hunting excursion that Temüjin and his brother Khasar killed their half-brother Begter.</t>
         </is>
       </c>
-      <c r="F181" t="inlineStr">
-        <is>
-          <t>[183, 311, 668, 366, 190]</t>
-        </is>
-      </c>
-      <c r="G181" t="inlineStr">
-        <is>
-          <t>[0.8368444442749023, 0.8193843960762024, 0.8044835925102234, 0.7864817380905151, 0.7783772945404053]</t>
-        </is>
-      </c>
-      <c r="H181" t="inlineStr">
-        <is>
-          <t>["As Jamukha and Temüjin drifted apart in their friendship, each began consolidating power, and soon became rivals. Jamukha supported the traditional Mongolian aristocracy, while Temüjin followed a meritocratic method, and attracted a broader, though lower class, range of followers. Due to his earlier defeat of the Merkits, and a proclamation by the shaman Kokochu that the Eternal Blue Sky had set aside the world for Temüjin, Temüjin began rising to power. In 1186, Temüjin was elected khan of the Mongols. However, Jamukha, threatened by Temüjin's rapid ascent, quickly moved to stop Temüjin's ambitions. In 1187, he launched an attack against his former friend with an army of thirty thousand troops. Temüjin hastily gathered together his followers to defend against the attack, but he was decisively beaten in the Battle of Dalan Balzhut. Jamukha horrified people greatly and harmed his image by boiling seventy young male captives alive in cauldrons, alienating many of his potential followers and eliciting sympathy for Temüjin. Toghrul, as Temüjin's patron, was exiled to the Qara Khitai. The life of Temüjin for the next ten years is very unclear, as historical records are mostly silent on that period.", "The next direct threat to Temüjin was the Naimans (Naiman Mongols), with whom Jamukha and his followers took refuge. The Naimans did not surrender, although enough sectors again voluntarily sided with Temüjin. In 1201, a khuruldai elected Jamukha as Gür Khan, \"universal ruler\", a title used by the rulers of the Qara Khitai. Jamukha's assumption of this title was the final breach with Temüjin, and Jamukha formed a coalition of tribes to oppose him. Before the conflict, however, several generals abandoned Jamukha, including Subutai, Jelme's well-known younger brother. After several battles, Jamukha was finally turned over to Temüjin by his own men in 1206.", "As a result, by 1206 Temüjin had managed to unite or subdue the Merkits, Naimans, Mongols, Keraites, Tatars, Uyghurs, and other disparate smaller tribes under his rule. It was a monumental feat for the \"Mongols\" (as they became known collectively). At a Khuruldai, a council of Mongol chiefs, Temüjin was acknowledged as \"Khan\" of the consolidated tribes and took the new title \"Genghis Khan\". The title Khagan was not conferred on Genghis until after his death, when his son and successor, Ögedei, took the title for himself and extended it posthumously to his father (as he was also to be posthumously declared the founder of the Yuan dynasty). This unification of all confederations by Genghis Khan established peace between previously warring tribes and a single political and military force under Genghis Khan.", "As previously arranged by his father, Temüjin married Börte of the Onggirat tribe when he was around 16 in order to cement alliances between their respective tribes. Soon after Börte's marriage to Temüjin, she was kidnapped by the Merkits and reportedly given away as a wife. Temüjin rescued her with the help of his friend and future rival, Jamukha, and his protector, Toghrul Khan of the Keraite tribe. She gave birth to a son, Jochi (1185–1226), nine months later, clouding the issue of his parentage. Despite speculation over Jochi, Börte would be Temüjin's only empress, though he did follow tradition by taking several morganatic wives.", "For the next several years, Hoelun and her children lived in poverty, surviving primarily on wild fruits and ox carcasses, marmots, and other small game killed by Temüjin and his brothers. Begter, Temujin's older half-brother, began to exercise the power of the eldest male in the family and eventually Temujin's mother Hoelun (not Begter's mother) would have to accept him as her husband if and when he became an adult. Temujin's resentment erupted during one hunting excursion that Temüjin and his brother Khasar killed their half-brother Begter."]</t>
-        </is>
-      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -8831,21 +6116,6 @@
 Following the series revival in 2005, Derek Jacobi provided the character's re-introduction in the 2007 episode "Utopia". During that story the role was then assumed by John Simm who returned to the role multiple times through the Tenth Doctor's tenure. As of the 2014 episode "Dark Water," it was revealed that the Master had become a female incarnation or "Time Lady," going by the name of "Missy" (short for Mistress, the feminine equivalent of "Master"). This incarnation is played by Michelle Gomez.</t>
         </is>
       </c>
-      <c r="F182" t="inlineStr">
-        <is>
-          <t>[185, 184, 20, 408, 456]</t>
-        </is>
-      </c>
-      <c r="G182" t="inlineStr">
-        <is>
-          <t>[0.8196713924407959, 0.8128653764724731, 0.7105885148048401, 0.7101525664329529, 0.7100846171379089]</t>
-        </is>
-      </c>
-      <c r="H182" t="inlineStr">
-        <is>
-          <t>["10 July 2009, and consisted of a single five-part story called Children of Earth which was set largely in London. A fourth series, Torchwood: Miracle Day jointly produced by BBC Wales, BBC Worldwide and the American entertainment company Starz debuted in 2011. The series was predominantly set in the United States, though Wales remained part of the show's setting.", "Following the success of the 2005 series produced by Russell T Davies, the BBC commissioned Davies to produce a 13-part spin-off series titled Torchwood (an anagram of \"Doctor Who\"), set in modern-day Cardiff and investigating alien activities and crime. The series debuted on BBC Three on 22 October 2006. John Barrowman reprised his role of Jack Harkness from the 2005 series of Doctor Who. Two other actresses who appeared in Doctor Who also star in the series; Eve Myles as Gwen Cooper, who also played the similarly named servant girl Gwyneth in the 2005 Doctor Who episode \"The Unquiet Dead\", and Naoko Mori who reprised her role as Toshiko Sato first seen in \"Aliens of London\". A second series of Torchwood aired in 2008; for three episodes, the cast was joined by Freema Agyeman reprising her Doctor Who role of Martha Jones. A third series was broadcast from 6 to 10 July 2009, and consisted of a single five-part story called Children of Earth which was set largely in London. A fourth series, Torchwood: Miracle Day jointly produced by BBC Wales, BBC Worldwide and the American entertainment company Starz debuted in 2011. The series was predominantly set in the United", "With the show's 2005 revival, executive producer Russell T Davies stated his intention to reintroduce classic icons of Doctor Who one step at a time: the Autons with the Nestene Consciousness and Daleks in series 1, Cybermen in series 2, the Macra and the Master in series 3, the Sontarans and Davros in series 4, and the Time Lords (Rassilon) in the 2009–10 Specials. Davies' successor, Steven Moffat, has continued the trend by reviving the Silurians in series 5, Cybermats in series 6, the Great Intelligence and the Ice Warriors in Series 7, and Zygons in the 50th Anniversary Special. Since its 2005 return, the series has also introduced new recurring aliens: Slitheen (Raxacoricofallapatorian), Ood, Judoon, Weeping Angels and the Silence.", "In addition to those actors who have headlined the series, others have portrayed versions of the Doctor in guest roles. Notably, in 2013, John Hurt guest-starred as a hitherto unknown incarnation of the Doctor known as the War Doctor in the run-up to the show's 50th anniversary special \"The Day of the Doctor\". He is shown in mini-episode \"The Night of the Doctor\" to have been retroactively inserted into the show's fictional chronology between McGann and Eccleston's Doctors, although his introduction was written so as not to disturb the established numerical naming of the Doctors. Another example is from the 1986 serial The Trial of a Time Lord, where Michael Jayston portrayed the Valeyard, who is described as an amalgamation of the darker sides of the Doctor's nature, somewhere between his twelfth and final incarnation.", "Following the series revival in 2005, Derek Jacobi provided the character's re-introduction in the 2007 episode \"Utopia\". During that story the role was then assumed by John Simm who returned to the role multiple times through the Tenth Doctor's tenure. As of the 2014 episode \"Dark Water,\" it was revealed that the Master had become a female incarnation or \"Time Lady,\" going by the name of \"Missy\" (short for Mistress, the feminine equivalent of \"Master\"). This incarnation is played by Michelle Gomez."]</t>
-        </is>
-      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -8877,21 +6147,6 @@
 The 1970s and 1980s saw the emergence of many graphical imaging packages for the network in which based the logo's setting mainly on special lighting effects then under development including white, blue, pink, rainbow neon and glittering dotted lines. Among the "ABC Circle" logo's many variants was a 1977 ID sequence that featured a bubble on a black background representing the circle with glossy gold letters, and as such, was the first ABC identification card to have a three-dimensional appearance.</t>
         </is>
       </c>
-      <c r="F183" t="inlineStr">
-        <is>
-          <t>[186, 187, 285, 225, 664]</t>
-        </is>
-      </c>
-      <c r="G183" t="inlineStr">
-        <is>
-          <t>[0.8609952330589294, 0.7727917432785034, 0.7303101420402527, 0.7070428133010864, 0.7056609988212585]</t>
-        </is>
-      </c>
-      <c r="H183" t="inlineStr">
-        <is>
-          <t>["The Victoria and Albert Museum’s Word and Image Department was under the same pressure being felt in archives around the world, to digitize their collection. A large scale digitization project began in 2007 in that department. That project was entitled the Factory Project to reference Andy Warhol and to create a factory to completely digitize the collection. The first step of the Factory Project was to take photographs utilizing digital cameras. The Word and Image Department had a collection of old photos but they were in black and white and in variant conditions, so new photos were shot. Those new photographs will be accessible to researchers to the Victoria and Albert Museum web-site. 15,000 images were taken during the first year of the Factory Project, including drawings, watercolors, computer-generated art, photographs, posters, and woodcuts. The second step of the Factory Project is to catalog everything. The third step of the Factory Project is to audit the collection. All of those items which were photographed and cataloged, must be audited to make sure everything listed as being in the collection was physically found during the creation of the Factory Project. The fourth goal of the Factory Project is conservation, which means", "Factory Project is to audit the collection. All of those items which were photographed and cataloged, must be audited to make sure everything listed as being in the collection was physically found during the creation of the Factory Project. The fourth goal of the Factory Project is conservation, which means performing some basic preventable procedures to those items in the department. There is a \"Search the Collections\" feature on the Victoria and Albert web-site. The main impetus behind the large-scale digitization project called the Factory Project was to list more items in the collections in those computer databases.", "One of the more unusual collections is that of Eadweard Muybridge's photographs of Animal Locomotion of 1887, this consists of 781 plates. These sequences of photographs taken a fraction of a second apart capture images of different animals and humans performimg various actions. There are several of John Thomson's 1876-7 images of Street Life in London in the collection. The museum also holds James Lafayette's society portraits, a collection of more than 600 photographs dating from the late 19th to early 20th centuries and portraying a wide range of society figures of the period, including bishops, generals, society ladies, Indian maharajas, Ethiopian rulers and other foreign leaders, actresses, people posing in their motor cars and a sequence of photographs recording the guests at the famous fancy-dress ball held at Devonshire House in 1897 to celebrate Queen Victoria's diamond jubilee.", "The Moon landing data was recorded by a special Apollo TV camera which recorded in a format incompatible with broadcast TV. This resulted in lunar footage that had to be converted for the live television broadcast and stored on magnetic telemetry tapes. During the following years, a magnetic tape shortage prompted NASA to remove massive numbers of magnetic tapes from the National Archives and Records Administration to be recorded over with newer satellite data. Stan Lebar, who led the team that designed and built the lunar television camera at Westinghouse Electric Corporation, also worked with Nafzger to try to locate the missing tapes.", "The 1970s and 1980s saw the emergence of many graphical imaging packages for the network in which based the logo's setting mainly on special lighting effects then under development including white, blue, pink, rainbow neon and glittering dotted lines. Among the \"ABC Circle\" logo's many variants was a 1977 ID sequence that featured a bubble on a black background representing the circle with glossy gold letters, and as such, was the first ABC identification card to have a three-dimensional appearance."]</t>
-        </is>
-      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -8923,21 +6178,6 @@
 The game's media day, which was typically held on the Tuesday afternoon prior to the game, was moved to the Monday evening and re-branded as Super Bowl Opening Night. The event was held on February 1, 2016 at SAP Center in San Jose. Alongside the traditional media availabilities, the event featured an opening ceremony with player introductions on a replica of the Golden Gate Bridge.</t>
         </is>
       </c>
-      <c r="F184" t="inlineStr">
-        <is>
-          <t>[550, 194, 263, 39, 188]</t>
-        </is>
-      </c>
-      <c r="G184" t="inlineStr">
-        <is>
-          <t>[0.8334280848503113, 0.8243498206138611, 0.8123905062675476, 0.8106452822685242, 0.8065751194953918]</t>
-        </is>
-      </c>
-      <c r="H184" t="inlineStr">
-        <is>
-          <t>["On May 21, 2013, NFL owners at their spring meetings in Boston voted and awarded the game to Levi's Stadium. The $1.2 billion stadium opened in 2014. It is the first Super Bowl held in the San Francisco Bay Area since Super Bowl XIX in 1985, and the first in California since Super Bowl XXXVII took place in San Diego in 2003.", "The league announced on October 16, 2012, that the two finalists were Sun Life Stadium and Levi's Stadium. The South Florida/Miami area has previously hosted the event 10 times (tied for most with New Orleans), with the most recent one being Super Bowl XLIV in 2010. The San Francisco Bay Area last hosted in 1985 (Super Bowl XIX), held at Stanford Stadium in Stanford, California, won by the home team 49ers. The Miami bid depended on whether the stadium underwent renovations. However, on May 3, 2013, the Florida legislature refused to approve the funding plan to pay for the renovations, dealing a significant blow to Miami's chances.", "Super Bowl 50 was an American football game to determine the champion of the National Football League (NFL) for the 2015 season. The American Football Conference (AFC) champion Denver Broncos defeated the National Football Conference (NFC) champion Carolina Panthers 24–10 to earn their third Super Bowl title. The game was played on February 7, 2016, at Levi's Stadium in the San Francisco Bay Area at Santa Clara, California. As this was the 50th Super Bowl, the league emphasized the \"golden anniversary\" with various gold-themed initiatives, as well as temporarily suspending the tradition of naming each Super Bowl game with Roman numerals (under which the game would have been known as \"Super Bowl L\"), so that the logo could prominently feature the Arabic numerals 50.", "CBS broadcast Super Bowl 50 in the U.S., and charged an average of $5 million for a 30-second commercial during the game. The Super Bowl 50 halftime show was headlined by the British rock group Coldplay with special guest performers Beyoncé and Bruno Mars, who headlined the Super Bowl XLVII and Super Bowl XLVIII halftime shows, respectively. It was the third-most watched U.S. broadcast ever.", "The game's media day, which was typically held on the Tuesday afternoon prior to the game, was moved to the Monday evening and re-branded as Super Bowl Opening Night. The event was held on February 1, 2016 at SAP Center in San Jose. Alongside the traditional media availabilities, the event featured an opening ceremony with player introductions on a replica of the Golden Gate Bridge."]</t>
-        </is>
-      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -8969,21 +6209,6 @@
 Luther came to understand justification as entirely the work of God. This teaching by Luther was clearly expressed in his 1525 publication On the Bondage of the Will, which was written in response to On Free Will by Desiderius Erasmus (1524). Luther based his position on predestination on St. Paul's epistle to the Ephesians 2:8–10. Against the teaching of his day that the righteous acts of believers are performed in cooperation with God, Luther wrote that Christians receive such righteousness entirely from outside themselves; that righteousness not only comes from Christ but actually is the righteousness of Christ, imputed to Christians (rather than infused into them) through faith. "That is why faith alone makes someone just and fulfills the law," he wrote. "Faith is that which brings the Holy Spirit through the merits of Christ." Faith, for Luther, was a gift from God; the experience of being justified by faith was "as though I had been born again." His entry into Paradise, no less, was a discovery about "the righteousness of God" – a discovery that "the just person" of whom the Bible speaks (as in Romans 1:17) lives by faith. He explained his concept of "justification" in the Smalcald</t>
         </is>
       </c>
-      <c r="F185" t="inlineStr">
-        <is>
-          <t>[53, 65, 150, 648, 149]</t>
-        </is>
-      </c>
-      <c r="G185" t="inlineStr">
-        <is>
-          <t>[0.8881345987319946, 0.8398337960243225, 0.8258534669876099, 0.7843132615089417, 0.7842045426368713]</t>
-        </is>
-      </c>
-      <c r="H185" t="inlineStr">
-        <is>
-          <t>["Sanctifying Grace is that grace of God which sustains the believers in the journey toward Christian Perfection: a genuine love of God with heart, soul, mind, and strength, and a genuine love of our neighbors as ourselves. Sanctifying grace enables us to respond to God by leading a Spirit-filled and Christ-like life aimed toward love. Wesley never claimed this state of perfection for himself but instead insisted the attainment of perfection was possible for all Christians. Here the English Reformer parted company with both Luther and Calvin, who denied that a man would ever reach a state in this life in which he could not fall into sin. Such a man can lose all inclination to evil and can gain perfection in this life.", "Justifying Grace or Accepting Grace is that grace, offered by God to all people, that we receive by faith and trust in Christ, through which God pardons the believer of sin. It is in justifying grace we are received by God, in spite of our sin. In this reception, we are forgiven through the atoning work of Jesus Christ on the cross. The justifying grace cancels our guilt and empowers us to resist the power of sin and to fully love God and neighbor. Today, justifying grace is also known as conversion, \"accepting Jesus as your personal Lord and Savior,\" or being \"born again\". John Wesley originally called this experience the New Birth. This experience can occur in different ways; it can be one transforming moment, such as an altar call experience, or it may involve a series of decisions across a period of time.", "was \"as though I had been born again.\" His entry into Paradise, no less, was a discovery about \"the righteousness of God\" – a discovery that \"the just person\" of whom the Bible speaks (as in Romans 1:17) lives by faith. He explained his concept of \"justification\" in the Smalcald Articles:", "Luther taught that salvation and subsequently eternal life is not earned by good deeds but is received only as a free gift of God's grace through faith in Jesus Christ as redeemer from sin. His theology challenged the authority and office of the Pope by teaching that the Bible is the only source of divinely revealed knowledge from God and opposed sacerdotalism by considering all baptized Christians to be a holy priesthood. Those who identify with these, and all of Luther's wider teachings, are called Lutherans even though Luther insisted on Christian or Evangelical as the only acceptable names for individuals who professed Christ.", "Luther came to understand justification as entirely the work of God. This teaching by Luther was clearly expressed in his 1525 publication On the Bondage of the Will, which was written in response to On Free Will by Desiderius Erasmus (1524). Luther based his position on predestination on St. Paul's epistle to the Ephesians 2:8–10. Against the teaching of his day that the righteous acts of believers are performed in cooperation with God, Luther wrote that Christians receive such righteousness entirely from outside themselves; that righteousness not only comes from Christ but actually is the righteousness of Christ, imputed to Christians (rather than infused into them) through faith. \"That is why faith alone makes someone just and fulfills the law,\" he wrote. \"Faith is that which brings the Holy Spirit through the merits of Christ.\" Faith, for Luther, was a gift from God; the experience of being justified by faith was \"as though I had been born again.\" His entry into Paradise, no less, was a discovery about \"the righteousness of God\" – a discovery that \"the just person\" of whom the Bible speaks (as in Romans 1:17) lives by faith. He explained his concept of \"justification\" in the Smalcald"]</t>
-        </is>
-      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -9015,21 +6240,6 @@
 was one of the worst mistakes Luther made, and, next to the landgrave himself, who was directly responsible for it, history chiefly holds Luther accountable". Brecht argues that Luther's mistake was not that he gave private pastoral advice, but that he miscalculated the political implications. The affair caused lasting damage to Luther's reputation.</t>
         </is>
       </c>
-      <c r="F186" t="inlineStr">
-        <is>
-          <t>[348, 877, 189, 398, 480]</t>
-        </is>
-      </c>
-      <c r="G186" t="inlineStr">
-        <is>
-          <t>[0.8027759790420532, 0.7605732679367065, 0.7603802680969238, 0.756118655204773, 0.7558813691139221]</t>
-        </is>
-      </c>
-      <c r="H186" t="inlineStr">
-        <is>
-          <t>["Luther's 1541 hymn \"Christ unser Herr zum Jordan kam\" (\"To Jordan came the Christ our Lord\") reflects the structure and substance of his questions and answers concerning baptism in the Small Catechism. Luther adopted a preexisting Johann Walter tune associated with a hymnic setting of Psalm 67's prayer for grace; Wolf Heintz's four-part setting of the hymn was used to introduce the Lutheran Reformation in Halle in 1541. Preachers and composers of the 18th century, including J. S. Bach, used this rich hymn as a subject for their own work, although its objective baptismal theology was displaced by more subjective hymns under the influence of late-19th-century Lutheran pietism.", "Luther's hymns were included in early Lutheran hymnals and spread the ideas of the Reformation. He supplied four of eight songs of the First Lutheran hymnal Achtliederbuch, 18 of 26 songs of the Erfurt Enchiridion, and 24 of the 32 songs in the first choral hymnal with settings by Johann Walter, Eyn geystlich Gesangk Buchleyn, all published in 1524.", "Luther's hymns inspired composers to write music. Johann Sebastian Bach included several verses as chorales in his cantatas and based chorale cantatas entirely on them, namely Christ lag in Todes Banden, BWV 4, as early as possibly 1707, in his second annual cycle (1724 to 1725) Ach Gott, vom Himmel sieh darein, BWV 2, Christ unser Herr zum Jordan kam, BWV 7, Nun komm, der Heiden Heiland, BWV 62, Gelobet seist du, Jesu Christ, BWV 91, and Aus tiefer Not schrei ich zu dir, BWV 38, later Ein feste Burg ist unser Gott, BWV 80, and in 1735 Wär Gott nicht mit uns diese Zeit, BWV 14.", "Luther's rediscovery of \"Christ and His salvation\" was the first of two points that became the foundation for the Reformation. His railing against the sale of indulgences was based on it.", "was one of the worst mistakes Luther made, and, next to the landgrave himself, who was directly responsible for it, history chiefly holds Luther accountable\". Brecht argues that Luther's mistake was not that he gave private pastoral advice, but that he miscalculated the political implications. The affair caused lasting damage to Luther's reputation."]</t>
-        </is>
-      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -9061,21 +6271,6 @@
 The next direct threat to Temüjin was the Naimans (Naiman Mongols), with whom Jamukha and his followers took refuge. The Naimans did not surrender, although enough sectors again voluntarily sided with Temüjin. In 1201, a khuruldai elected Jamukha as Gür Khan, "universal ruler", a title used by the rulers of the Qara Khitai. Jamukha's assumption of this title was the final breach with Temüjin, and Jamukha formed a coalition of tribes to oppose him. Before the conflict, however, several generals abandoned Jamukha, including Subutai, Jelme's well-known younger brother. After several battles, Jamukha was finally turned over to Temüjin by his own men in 1206.</t>
         </is>
       </c>
-      <c r="F187" t="inlineStr">
-        <is>
-          <t>[719, 190, 366, 183, 311]</t>
-        </is>
-      </c>
-      <c r="G187" t="inlineStr">
-        <is>
-          <t>[0.8572685718536377, 0.8481644988059998, 0.8477796316146851, 0.817672610282898, 0.8090612888336182]</t>
-        </is>
-      </c>
-      <c r="H187" t="inlineStr">
-        <is>
-          <t>["Temüjin had three brothers named Hasar, Hachiun, and Temüge, and one sister named Temülen, as well as two half-brothers named Begter and Belgutei. Like many of the nomads of Mongolia, Temüjin's early life was difficult. His father arranged a marriage for him, and at nine years of age he was delivered by his father to the family of his future wife Börte, who was a member of the tribe Khongirad. Temüjin was to live there in service to Dai Setsen, the head of the new household, until he reached the marriageable age of 12.", "For the next several years, Hoelun and her children lived in poverty, surviving primarily on wild fruits and ox carcasses, marmots, and other small game killed by Temüjin and his brothers. Begter, Temujin's older half-brother, began to exercise the power of the eldest male in the family and eventually Temujin's mother Hoelun (not Begter's mother) would have to accept him as her husband if and when he became an adult. Temujin's resentment erupted during one hunting excursion that Temüjin and his brother Khasar killed their half-brother Begter.", "As previously arranged by his father, Temüjin married Börte of the Onggirat tribe when he was around 16 in order to cement alliances between their respective tribes. Soon after Börte's marriage to Temüjin, she was kidnapped by the Merkits and reportedly given away as a wife. Temüjin rescued her with the help of his friend and future rival, Jamukha, and his protector, Toghrul Khan of the Keraite tribe. She gave birth to a son, Jochi (1185–1226), nine months later, clouding the issue of his parentage. Despite speculation over Jochi, Börte would be Temüjin's only empress, though he did follow tradition by taking several morganatic wives.", "As Jamukha and Temüjin drifted apart in their friendship, each began consolidating power, and soon became rivals. Jamukha supported the traditional Mongolian aristocracy, while Temüjin followed a meritocratic method, and attracted a broader, though lower class, range of followers. Due to his earlier defeat of the Merkits, and a proclamation by the shaman Kokochu that the Eternal Blue Sky had set aside the world for Temüjin, Temüjin began rising to power. In 1186, Temüjin was elected khan of the Mongols. However, Jamukha, threatened by Temüjin's rapid ascent, quickly moved to stop Temüjin's ambitions. In 1187, he launched an attack against his former friend with an army of thirty thousand troops. Temüjin hastily gathered together his followers to defend against the attack, but he was decisively beaten in the Battle of Dalan Balzhut. Jamukha horrified people greatly and harmed his image by boiling seventy young male captives alive in cauldrons, alienating many of his potential followers and eliciting sympathy for Temüjin. Toghrul, as Temüjin's patron, was exiled to the Qara Khitai. The life of Temüjin for the next ten years is very unclear, as historical records are mostly silent on that period.", "The next direct threat to Temüjin was the Naimans (Naiman Mongols), with whom Jamukha and his followers took refuge. The Naimans did not surrender, although enough sectors again voluntarily sided with Temüjin. In 1201, a khuruldai elected Jamukha as Gür Khan, \"universal ruler\", a title used by the rulers of the Qara Khitai. Jamukha's assumption of this title was the final breach with Temüjin, and Jamukha formed a coalition of tribes to oppose him. Before the conflict, however, several generals abandoned Jamukha, including Subutai, Jelme's well-known younger brother. After several battles, Jamukha was finally turned over to Temüjin by his own men in 1206."]</t>
-        </is>
-      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -9107,21 +6302,6 @@
 United States and Western Europe than in China (due to a greater tendency to take on debts).[unreliable source?][unreliable source?] Anthony Shorrocks, the lead author of the Credit Suisse report which is one of the sources of Oxfam's data, considers the criticism about debt to be a "silly argument" and "a non-issue . . . a diversion."</t>
         </is>
       </c>
-      <c r="F188" t="inlineStr">
-        <is>
-          <t>[191, 317, 413, 691, 827]</t>
-        </is>
-      </c>
-      <c r="G188" t="inlineStr">
-        <is>
-          <t>[0.7519713044166565, 0.7366199493408203, 0.7313504815101624, 0.7274993658065796, 0.7226195335388184]</t>
-        </is>
-      </c>
-      <c r="H188" t="inlineStr">
-        <is>
-          <t>["The Super Bowl 50 Host Committee has vowed to be \"the most giving Super Bowl ever\", and will dedicate 25 percent of all money it raises for philanthropic causes in the Bay Area. The committee created the 50 fund as its philanthropic initiative and focuses on providing grants to aid with youth development, community investment and sustainable environments.", "In addition, there are $2 million worth of other ancillary events, including a week-long event at the Santa Clara Convention Center, a beer, wine and food festival at Bellomy Field at Santa Clara University, and a pep rally. A professional fundraiser will aid in finding business sponsors and individual donors, but still may need the city council to help fund the event. Additional funding will be provided by the city council, which has announced plans to set aside seed funding for the event.", "Some of the income was dispensed in the form of aid to other underdeveloped nations whose economies had been caught between higher oil prices and lower prices for their own export commodities, amid shrinking Western demand. Much went for arms purchases that exacerbated political tensions, particularly in the Middle East. Saudi Arabia spent over 100 billion dollars in the ensuing decades for helping spread its fundamentalist interpretation of Islam, known as Wahhabism, throughout the world, via religious charities such al-Haramain Foundation, which often also distributed funds to violent Sunni extremist groups such as Al-Qaeda and the Taliban.", "From the mid-2000s, the university began a number of multimillion-dollar expansion projects. In 2008, the University of Chicago announced plans to establish the Milton Friedman Institute which attracted both support and controversy from faculty members and students. The institute will cost around $200 million and occupy the buildings of the Chicago Theological Seminary. During the same year, investor David G. Booth donated $300 million to the university's Booth School of Business, which is the largest gift in the university's history and the largest gift ever to any business school. In 2009, planning or construction on several new buildings, half of which cost $100 million or more, was underway. Since 2011, major construction projects have included the Jules and Gwen Knapp Center for Biomedical Discovery, a ten-story medical research center, and further additions to the medical campus of the University of Chicago Medical Center. In 2014 the University launched the public phase of a $4.5 billion fundraising campaign. In September 2015, the University received $100 million from The Pearson Family Foundation to establish The Pearson Institute for the Study and Resolution of Global Conflicts and The Pearson Global Forum at the Harris School of Public Policy Studies.", "United States and Western Europe than in China (due to a greater tendency to take on debts).[unreliable source?][unreliable source?] Anthony Shorrocks, the lead author of the Credit Suisse report which is one of the sources of Oxfam's data, considers the criticism about debt to be a \"silly argument\" and \"a non-issue . . . a diversion.\""]</t>
-        </is>
-      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -9153,21 +6333,6 @@
 Tesla was renowned for his achievements and showmanship, eventually earning him a reputation in popular culture as an archetypal "mad scientist". His patents earned him a considerable amount of money, much of which was used to finance his own projects with varying degrees of success.:121,154 He lived most of his life in a series of New York hotels, through his retirement. Tesla died on 7 January 1943. His work fell into relative obscurity after his death, but in 1960 the General Conference on Weights and Measures named the SI unit of magnetic flux density the tesla in his honor. There has been a resurgence in popular interest in Tesla since the 1990s.</t>
         </is>
       </c>
-      <c r="F189" t="inlineStr">
-        <is>
-          <t>[192, 249, 339, 465, 318]</t>
-        </is>
-      </c>
-      <c r="G189" t="inlineStr">
-        <is>
-          <t>[0.7852181196212769, 0.7630321383476257, 0.7585009336471558, 0.7576712369918823, 0.7564729452133179]</t>
-        </is>
-      </c>
-      <c r="H189" t="inlineStr">
-        <is>
-          <t>["Tesla read many works, memorizing complete books, and supposedly possessed a photographic memory.:33 He was a polyglot, speaking eight languages: Serbo-Croatian, Czech, English, French, German, Hungarian, Italian, and Latin.:282 Tesla related in his autobiography that he experienced detailed moments of inspiration. During his early life, Tesla was repeatedly stricken with illness. He suffered a peculiar affliction in which blinding flashes of light would appear before his eyes, often accompanied by visions.:33 Often, the visions were linked to a word or idea he might have come across; at other times they would provide the solution to a particular problem he had encountered. Just by hearing the name of an item, he would be able to envision it in realistic detail.:33 Tesla would visualize an invention in his mind with extreme precision, including all dimensions, before moving to the construction stage, a technique sometimes known as picture thinking. He typically did not make drawings by hand but worked from memory. Beginning in his childhood, Tesla had frequent flashbacks to events that had happened previously in his life.:33", "Tesla invented a steam-powered mechanical oscillator—Tesla's oscillator. While experimenting with mechanical oscillators at his Houston Street lab, Tesla allegedly generated a resonance of several buildings. As the speed grew, it is said that the machine oscillated at the resonance frequency of his own building and, belatedly realizing the danger, he was forced to use a sledge hammer to terminate the experiment, just as the police arrived.:162–164 In February 1912, an article—\"Nikola Tesla, Dreamer\" by Allan L. Benson—was published in World Today, in which an artist's illustration appears showing the entire earth cracking in half with the caption, \"Tesla claims that in a few weeks he could set the earth's crust into such a state of vibration that it would rise and fall hundreds of feet and practically destroy civilization. A continuation of this process would, he says, eventually split the earth in two.\"", "During that year, Tesla worked in Pittsburgh, helping to create an alternating current system to power the city's streetcars. He found the time there frustrating because of conflicts between him and the other Westinghouse engineers over how best to implement AC power. Between them, they settled on a 60-cycle AC current system Tesla proposed (to match the working frequency of Tesla's motor), although they soon found that, since Tesla's induction motor could only run at a constant speed, it would not work for street cars. They ended up using a DC traction motor instead.", "Tesla theorized that the application of electricity to the brain enhanced intelligence. In 1912, he crafted \"a plan to make dull students bright by saturating them unconsciously with electricity,\" wiring the walls of a schoolroom and, \"saturating [the schoolroom] with infinitesimal electric waves vibrating at high frequency. The whole room will thus, Mr. Tesla claims, be converted into a health-giving and stimulating electromagnetic field or 'bath.'\" The plan was, at least provisionally approved by then superintendent of New York City schools, William H. Maxwell.", "Tesla was renowned for his achievements and showmanship, eventually earning him a reputation in popular culture as an archetypal \"mad scientist\". His patents earned him a considerable amount of money, much of which was used to finance his own projects with varying degrees of success.:121,154 He lived most of his life in a series of New York hotels, through his retirement. Tesla died on 7 January 1943. His work fell into relative obscurity after his death, but in 1960 the General Conference on Weights and Measures named the SI unit of magnetic flux density the tesla in his honor. There has been a resurgence in popular interest in Tesla since the 1990s."]</t>
-        </is>
-      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -9199,21 +6364,6 @@
 During 2003–04, the gross value of Victorian agricultural production increased by 17% to $8.7 billion. This represented 24% of national agricultural production total gross value. As of 2004, an estimated 32,463 farms occupied around 136,000 square kilometres (52,500 sq mi) of Victorian land. This comprises more than 60% of the state's total land surface. Victorian farms range from small horticultural outfits to large-scale livestock and grain productions. A quarter of farmland is used to grow consumable crops.</t>
         </is>
       </c>
-      <c r="F190" t="inlineStr">
-        <is>
-          <t>[193, 553, 832, 609, 196]</t>
-        </is>
-      </c>
-      <c r="G190" t="inlineStr">
-        <is>
-          <t>[0.7447278499603271, 0.7160917520523071, 0.6988369822502136, 0.697105884552002, 0.6967316269874573]</t>
-        </is>
-      </c>
-      <c r="H190" t="inlineStr">
-        <is>
-          <t>["The economy of Victoria is highly diversified: service sectors including financial and property services, health, education, wholesale, retail, hospitality and manufacturing constitute the majority of employment. Victoria's total gross state product (GSP) is ranked second in Australia, although Victoria is ranked fourth in terms of GSP per capita because of its limited mining activity. Culturally, Melbourne is home to a number of museums, art galleries and theatres and is also described as the \"sporting capital of Australia\". The Melbourne Cricket Ground is the largest stadium in Australia, and the host of the 1956 Summer Olympics and the 2006 Commonwealth Games. The ground is also considered the \"spiritual home\" of Australian cricket and Australian rules football, and hosts the grand final of the Australian Football League (AFL) each year, usually drawing crowds of over 95,000 people. Victoria includes eight public universities, with the oldest, the University of Melbourne, having been founded in 1853.", "On 1 July 1851, writs were issued for the election of the first Victorian Legislative Council, and the absolute independence of Victoria from New South Wales was established proclaiming a new Colony of Victoria. Days later, still in 1851 gold was discovered near Ballarat, and subsequently at Bendigo. Later discoveries occurred at many sites across Victoria. This triggered one of the largest gold rushes the world has ever seen. The colony grew rapidly in both population and economic power. In ten years the population of Victoria increased sevenfold from 76,000 to 540,000. All sorts of gold records were produced including the \"richest shallow alluvial goldfield in the world\" and the largest gold nugget. Victoria produced in the decade 1851–1860 20 million ounces of gold, one third of the world's output[citation needed].", "British researchers Richard G. Wilkinson and Kate Pickett have found higher rates of health and social problems (obesity, mental illness, homicides, teenage births, incarceration, child conflict, drug use), and lower rates of social goods (life expectancy by country, educational performance, trust among strangers, women's status, social mobility, even numbers of patents issued) in countries and states with higher inequality. Using statistics from 23 developed countries and the 50 states of the US, they found social/health problems lower in countries like Japan and Finland and states like Utah and New Hampshire with high levels of equality, than in countries (US and UK) and states (Mississippi and New York) with large differences in household income.", "Victoria is the centre of dairy farming in Australia. It is home to 60% of Australia's 3 million dairy cattle and produces nearly two-thirds of the nation's milk, almost 6.4 billion litres. The state also has 2.4 million beef cattle, with more than 2.2 million cattle and calves slaughtered each year. In 2003–04, Victorian commercial fishing crews and aquaculture industry produced 11,634 tonnes of seafood valued at nearly A$109 million. Blacklipped abalone is the mainstay of the catch, bringing in A$46 million, followed by southern rock lobster worth A$13.7 million. Most abalone and rock lobster is exported to Asia.", "During 2003–04, the gross value of Victorian agricultural production increased by 17% to $8.7 billion. This represented 24% of national agricultural production total gross value. As of 2004, an estimated 32,463 farms occupied around 136,000 square kilometres (52,500 sq mi) of Victorian land. This comprises more than 60% of the state's total land surface. Victorian farms range from small horticultural outfits to large-scale livestock and grain productions. A quarter of farmland is used to grow consumable crops."]</t>
-        </is>
-      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -9245,21 +6395,6 @@
 Super Bowl 50 was an American football game to determine the champion of the National Football League (NFL) for the 2015 season. The American Football Conference (AFC) champion Denver Broncos defeated the National Football Conference (NFC) champion Carolina Panthers 24–10 to earn their third Super Bowl title. The game was played on February 7, 2016, at Levi's Stadium in the San Francisco Bay Area at Santa Clara, California. As this was the 50th Super Bowl, the league emphasized the "golden anniversary" with various gold-themed initiatives, as well as temporarily suspending the tradition of naming each Super Bowl game with Roman numerals (under which the game would have been known as "Super Bowl L"), so that the logo could prominently feature the Arabic numerals 50.</t>
         </is>
       </c>
-      <c r="F191" t="inlineStr">
-        <is>
-          <t>[194, 325, 550, 289, 263]</t>
-        </is>
-      </c>
-      <c r="G191" t="inlineStr">
-        <is>
-          <t>[0.8150380849838257, 0.7773632407188416, 0.7673671245574951, 0.7580682635307312, 0.7571581602096558]</t>
-        </is>
-      </c>
-      <c r="H191" t="inlineStr">
-        <is>
-          <t>["The league announced on October 16, 2012, that the two finalists were Sun Life Stadium and Levi's Stadium. The South Florida/Miami area has previously hosted the event 10 times (tied for most with New Orleans), with the most recent one being Super Bowl XLIV in 2010. The San Francisco Bay Area last hosted in 1985 (Super Bowl XIX), held at Stanford Stadium in Stanford, California, won by the home team 49ers. The Miami bid depended on whether the stadium underwent renovations. However, on May 3, 2013, the Florida legislature refused to approve the funding plan to pay for the renovations, dealing a significant blow to Miami's chances.", "The league eventually narrowed the bids to three sites: New Orleans' Mercedes-Benz Superdome, Miami's Sun Life Stadium, and the San Francisco Bay Area's Levi's Stadium.", "On May 21, 2013, NFL owners at their spring meetings in Boston voted and awarded the game to Levi's Stadium. The $1.2 billion stadium opened in 2014. It is the first Super Bowl held in the San Francisco Bay Area since Super Bowl XIX in 1985, and the first in California since Super Bowl XXXVII took place in San Diego in 2003.", "The annual NFL Experience was held at the Moscone Center in San Francisco. In addition, \"Super Bowl City\" opened on January 30 at Justin Herman Plaza on The Embarcadero, featuring games and activities that will highlight the Bay Area's technology, culinary creations, and cultural diversity. More than 1 million people are expected to attend the festivities in San Francisco during Super Bowl Week. San Francisco mayor Ed Lee said of the highly visible homeless presence in this area \"they are going to have to leave\". San Francisco city supervisor Jane Kim unsuccessfully lobbied for the NFL to reimburse San Francisco for city services in the amount of $5 million.", "Super Bowl 50 was an American football game to determine the champion of the National Football League (NFL) for the 2015 season. The American Football Conference (AFC) champion Denver Broncos defeated the National Football Conference (NFC) champion Carolina Panthers 24–10 to earn their third Super Bowl title. The game was played on February 7, 2016, at Levi's Stadium in the San Francisco Bay Area at Santa Clara, California. As this was the 50th Super Bowl, the league emphasized the \"golden anniversary\" with various gold-themed initiatives, as well as temporarily suspending the tradition of naming each Super Bowl game with Roman numerals (under which the game would have been known as \"Super Bowl L\"), so that the logo could prominently feature the Arabic numerals 50."]</t>
-        </is>
-      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -9291,21 +6426,6 @@
 less than 700 preparations, their properties, modes of action, and their indications. He devoted in fact a whole volume to simple drugs in The Canon of Medicine. Of great impact were also the works by al-Maridini of Baghdad and Cairo, and Ibn al-Wafid (1008–1074), both of which were printed in Latin more than fifty times, appearing as De Medicinis universalibus et particularibus by 'Mesue' the younger, and the Medicamentis simplicibus by 'Abenguefit'. Peter of Abano (1250–1316) translated and added a supplement to the work of al-Maridini under the title De Veneris. Al-Muwaffaq’s contributions in the field are also pioneering. Living in the 10th century, he wrote The foundations of the true properties of Remedies, amongst others describing arsenious oxide, and being acquainted with silicic acid. He made clear distinction between sodium carbonate and potassium carbonate, and drew attention to the poisonous nature of copper compounds, especially copper vitriol, and also lead compounds. He also describes the distillation of sea-water for drinking.[verification needed]</t>
         </is>
       </c>
-      <c r="F192" t="inlineStr">
-        <is>
-          <t>[195, 579, 271, 607, 390]</t>
-        </is>
-      </c>
-      <c r="G192" t="inlineStr">
-        <is>
-          <t>[0.8706228137016296, 0.7496528029441833, 0.7024112939834595, 0.678053081035614, 0.6744171977043152]</t>
-        </is>
-      </c>
-      <c r="H192" t="inlineStr">
-        <is>
-          <t>["Specialty pharmacies supply high cost injectable, oral, infused, or inhaled medications that are used for chronic and complex disease states such as cancer, hepatitis, and rheumatoid arthritis. Unlike a traditional community pharmacy where prescriptions for any common medication can be brought in and filled, specialty pharmacies carry novel medications that need to be properly stored, administered, carefully monitored, and clinically managed. In addition to supplying these drugs, specialty pharmacies also provide lab monitoring, adherence counseling, and assist patients with cost-containment strategies needed to obtain their expensive specialty drugs. It is currently the fastest growing sector of the pharmaceutical industry with 19 of 28 newly FDA approved medications in 2013 being specialty drugs.", "The word pharmacy is derived from its root word pharma which was a term used since the 15th–17th centuries. However, the original Greek roots from pharmakos imply sorcery or even poison. In addition to pharma responsibilities, the pharma offered general medical advice and a range of services that are now performed solely by other specialist practitioners, such as surgery and midwifery. The pharma (as it was referred to) often operated through a retail shop which, in addition to ingredients for medicines, sold tobacco and patent medicines. Often the place that did this was called an apothecary and several languages have this as the dominant term, though their practices are more akin to a modern pharmacy, in English the term apothecary would today be seen as outdated or only approproriate if herbal remedies were on offer to a large extent. The pharmas also used many other herbs not listed. The Greek word Pharmakeia (Greek: φαρμακεία) derives from pharmakon (φάρμακον), meaning \"drug\", \"medicine\" (or \"poison\").[n 1]", "Anti-inflammatory drugs are often used to control the effects of inflammation. Glucocorticoids are the most powerful of these drugs; however, these drugs can have many undesirable side effects, such as central obesity, hyperglycemia, osteoporosis, and their use must be tightly controlled. Lower doses of anti-inflammatory drugs are often used in conjunction with cytotoxic or immunosuppressive drugs such as methotrexate or azathioprine. Cytotoxic drugs inhibit the immune response by killing dividing cells such as activated T cells. However, the killing is indiscriminate and other constantly dividing cells and their organs are affected, which causes toxic side effects. Immunosuppressive drugs such as cyclosporin prevent T cells from responding to signals correctly by inhibiting signal transduction pathways.", "The reason for the majority rule is the high risk of a conflict of interest and/or the avoidance of absolute powers. Otherwise, the physician has a financial self-interest in \"diagnosing\" as many conditions as possible, and in exaggerating their seriousness, because he or she can then sell more medications to the patient. Such self-interest directly conflicts with the patient's interest in obtaining cost-effective medication and avoiding the unnecessary use of medication that may have side-effects. This system reflects much similarity to the checks and balances system of the U.S. and many other governments.[citation needed]", "less than 700 preparations, their properties, modes of action, and their indications. He devoted in fact a whole volume to simple drugs in The Canon of Medicine. Of great impact were also the works by al-Maridini of Baghdad and Cairo, and Ibn al-Wafid (1008–1074), both of which were printed in Latin more than fifty times, appearing as De Medicinis universalibus et particularibus by 'Mesue' the younger, and the Medicamentis simplicibus by 'Abenguefit'. Peter of Abano (1250–1316) translated and added a supplement to the work of al-Maridini under the title De Veneris. Al-Muwaffaq’s contributions in the field are also pioneering. Living in the 10th century, he wrote The foundations of the true properties of Remedies, amongst others describing arsenious oxide, and being acquainted with silicic acid. He made clear distinction between sodium carbonate and potassium carbonate, and drew attention to the poisonous nature of copper compounds, especially copper vitriol, and also lead compounds. He also describes the distillation of sea-water for drinking.[verification needed]"]</t>
-        </is>
-      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -9337,21 +6457,6 @@
 In 2014, economists with the Standard &amp; Poor's rating agency concluded that the widening disparity between the U.S.'s wealthiest citizens and the rest of the nation had slowed its recovery from the 2008-2009 recession and made it more prone to boom-and-bust cycles. To partially remedy the wealth gap and the resulting slow growth, S&amp;P recommended increasing access to education. It estimated that if the average United States worker had completed just one more year of school, it would add an additional $105 billion in growth to the country's economy over five years.</t>
         </is>
       </c>
-      <c r="F193" t="inlineStr">
-        <is>
-          <t>[196, 425, 866, 736, 743]</t>
-        </is>
-      </c>
-      <c r="G193" t="inlineStr">
-        <is>
-          <t>[0.8208427429199219, 0.7703226804733276, 0.7400650978088379, 0.738728940486908, 0.7219619154930115]</t>
-        </is>
-      </c>
-      <c r="H193" t="inlineStr">
-        <is>
-          <t>["During 2003–04, the gross value of Victorian agricultural production increased by 17% to $8.7 billion. This represented 24% of national agricultural production total gross value. As of 2004, an estimated 32,463 farms occupied around 136,000 square kilometres (52,500 sq mi) of Victorian land. This comprises more than 60% of the state's total land surface. Victorian farms range from small horticultural outfits to large-scale livestock and grain productions. A quarter of farmland is used to grow consumable crops.", "Agriculture is the second largest contributor to Kenya's gross domestic product (GDP), after the service sector. In 2005 agriculture, including forestry and fishing, accounted for 24% of GDP, as well as for 18% of wage employment and 50% of revenue from exports. The principal cash crops are tea, horticultural produce, and coffee. Horticultural produce and tea are the main growth sectors and the two most valuable of all of Kenya's exports. The production of major food staples such as corn is subject to sharp weather-related fluctuations. Production downturns periodically necessitate food aid—for example, in 2004 aid for 1.8 million people because of one of Kenya's intermittent droughts.[citation needed]", "More than 26,000 square kilometres (10,000 sq mi) of Victorian farmland are sown for grain, mostly in the state's west. More than 50% of this area is sown for wheat, 33% for barley and 7% for oats. A further 6,000 square kilometres (2,300 sq mi) is sown for hay. In 2003–04, Victorian farmers produced more than 3 million tonnes of wheat and 2 million tonnes of barley. Victorian farms produce nearly 90% of Australian pears and third of apples. It is also a leader in stone fruit production. The main vegetable crops include asparagus, broccoli, carrots, potatoes and tomatoes. Last year, 121,200 tonnes of pears and 270,000 tonnes of tomatoes were produced.", "Since the 1920s, motion pictures, petroleum and aircraft manufacturing have been major industries. In one of the richest agricultural regions in the U.S., cattle and citrus were major industries until farmlands were turned into suburbs. Although military spending cutbacks have had an impact, aerospace continues to be a major factor.", "In 2014, economists with the Standard &amp; Poor's rating agency concluded that the widening disparity between the U.S.'s wealthiest citizens and the rest of the nation had slowed its recovery from the 2008-2009 recession and made it more prone to boom-and-bust cycles. To partially remedy the wealth gap and the resulting slow growth, S&amp;P recommended increasing access to education. It estimated that if the average United States worker had completed just one more year of school, it would add an additional $105 billion in growth to the country's economy over five years."]</t>
-        </is>
-      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -9383,21 +6488,6 @@
 Courts have distinguished between two types of civil disobedience: "Indirect civil disobedience involves violating a law which is not, itself, the object of protest, whereas direct civil disobedience involves protesting the existence of a particular law by breaking that law." During the Vietnam War, courts typically refused to excuse the perpetrators of illegal protests from punishment on the basis of their challenging the legality of the Vietnam War; the courts ruled it was a political question. The necessity defense has sometimes been used as a shadow defense by civil disobedients to deny guilt without denouncing their politically motivated acts, and to present their political beliefs in the courtroom. However, court cases such as U.S. v. Schoon have greatly curtailed the availability of the political necessity defense. Likewise, when Carter Wentworth was charged for his role in the Clamshell Alliance's 1977 illegal occupation of the Seabrook Station Nuclear Power Plant, the judge instructed the jury to disregard his competing harms defense, and he was found guilty. Fully Informed Jury Association activists have sometimes handed out educational leaflets inside courthouses despite admonitions not to; according to FIJA, many of them have escaped prosecution because "prosecutors have reasoned (correctly) that if they arrest</t>
         </is>
       </c>
-      <c r="F194" t="inlineStr">
-        <is>
-          <t>[760, 602, 182, 19, 33]</t>
-        </is>
-      </c>
-      <c r="G194" t="inlineStr">
-        <is>
-          <t>[0.8508525490760803, 0.845244288444519, 0.8389436602592468, 0.8183149099349976, 0.8131487965583801]</t>
-        </is>
-      </c>
-      <c r="H194" t="inlineStr">
-        <is>
-          <t>["Some forms of civil disobedience, such as illegal boycotts, refusals to pay taxes, draft dodging, distributed denial-of-service attacks, and sit-ins, make it more difficult for a system to function. In this way, they might be considered coercive. Brownlee notes that \"although civil disobedients are constrained in their use of coercion by their conscientious aim to engage in moral dialogue, nevertheless they may find it necessary to employ limited coercion in order to get their issue onto the table.\" The Plowshares organization temporarily closed GCSB Waihopai by padlocking the gates and using sickles to deflate one of the large domes covering two satellite dishes.", "Some theories of civil disobedience hold that civil disobedience is only justified against governmental entities. Brownlee argues that disobedience in opposition to the decisions of non-governmental agencies such as trade unions, banks, and private universities can be justified if it reflects \"a larger challenge to the legal system that permits those decisions to be taken\". The same principle, she argues, applies to breaches of law in protest against international organizations and foreign governments.", "Civil disobedients have chosen a variety of different illegal acts. Bedau writes, \"There is a whole class of acts, undertaken in the name of civil disobedience, which, even if they were widely practiced, would in themselves constitute hardly more than a nuisance (e.g. trespassing at a nuclear-missile installation)...Such acts are often just a harassment and, at least to the bystander, somewhat inane...The remoteness of the connection between the disobedient act and the objectionable law lays such acts open to the charge of ineffectiveness and absurdity.\" Bedau also notes, though, that the very harmlessness of such entirely symbolic illegal protests toward public policy goals may serve a propaganda purpose. Some civil disobedients, such as the proprietors of illegal medical cannabis dispensaries and Voice in the Wilderness, which brought medicine to Iraq without the permission of the U.S. Government, directly achieve a desired social goal (such as the provision of medication to the sick) while openly breaking the law. Julia Butterfly Hill lived in Luna, a 180-foot (55 m)-tall, 600-year-old California Redwood tree for 738 days, successfully preventing it from being cut down.", "Civil disobedience is usually defined as pertaining to a citizen's relation to the state and its laws, as distinguished from a constitutional impasse in which two public agencies, especially two equally sovereign branches of government, conflict. For instance, if the head of government of a country were to refuse to enforce a decision of that country's highest court, it would not be civil disobedience, since the head of government would be acting in her or his capacity as public official rather than private citizen.", "Courts have distinguished between two types of civil disobedience: \"Indirect civil disobedience involves violating a law which is not, itself, the object of protest, whereas direct civil disobedience involves protesting the existence of a particular law by breaking that law.\" During the Vietnam War, courts typically refused to excuse the perpetrators of illegal protests from punishment on the basis of their challenging the legality of the Vietnam War; the courts ruled it was a political question. The necessity defense has sometimes been used as a shadow defense by civil disobedients to deny guilt without denouncing their politically motivated acts, and to present their political beliefs in the courtroom. However, court cases such as U.S. v. Schoon have greatly curtailed the availability of the political necessity defense. Likewise, when Carter Wentworth was charged for his role in the Clamshell Alliance's 1977 illegal occupation of the Seabrook Station Nuclear Power Plant, the judge instructed the jury to disregard his competing harms defense, and he was found guilty. Fully Informed Jury Association activists have sometimes handed out educational leaflets inside courthouses despite admonitions not to; according to FIJA, many of them have escaped prosecution because \"prosecutors have reasoned (correctly) that if they arrest"]</t>
-        </is>
-      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -9429,21 +6519,6 @@
 On June 16, 2007, ABC began to phase in a new imaging campaign for the upcoming 2007–08 season, "Start Here". Also developed by Troika, the on-air design was intended to emphasize the availability of ABC content across multiple platforms (in particular, using a system of icons representing different devices, such as television, computers and mobile devices), and "simplify and bring a lot more consistency and continuity to the visual representation of ABC". The ABC logo was also significantly redesigned as part of the transition, with a glossy "ball" effect that was specifically designed for HD. On-air, the logo was accompanied by animated water and ribbon effects. Red ribbons were used to represent the entertainment division, while blue ribbons were used for ABC News.</t>
         </is>
       </c>
-      <c r="F195" t="inlineStr">
-        <is>
-          <t>[74, 353, 857, 155, 824]</t>
-        </is>
-      </c>
-      <c r="G195" t="inlineStr">
-        <is>
-          <t>[0.8325005769729614, 0.7139379978179932, 0.7024332880973816, 0.7015049457550049, 0.7010223865509033]</t>
-        </is>
-      </c>
-      <c r="H195" t="inlineStr">
-        <is>
-          <t>["CBS provided digital streams of the game via CBSSports.com, and the CBS Sports apps on tablets, Windows 10, Xbox One and other digital media players (such as Chromecast and Roku). Due to Verizon Communications exclusivity, streaming on smartphones was only provided to Verizon Wireless customers via the NFL Mobile service. The ESPN Deportes Spanish broadcast was made available through WatchESPN.", "In the United States, the game was televised by CBS, as part of a cycle between the three main broadcast television partners of the NFL. The network's lead broadcast team of Jim Nantz and Phil Simms called the contest, with Tracy Wolfson and Evan Washburn on the sidelines. CBS introduced new features during the telecast, including pylon cameras and microphones along with EyeVision 360—an array of 36 cameras along the upper deck that can be used to provide a 360-degree view of plays and \"bullet time\" effects. (An earlier version of EyeVision was last used in Super Bowl XXXV; for Super Bowl 50, the cameras were upgraded to 5K resolution.)", "Always in search of new programs that would help it compete with NBC and CBS, ABC's management believed that sports could be a major catalyst in improving the network's market share. On April 29, 1961, ABC debuted Wide World of Sports, an anthology series created by Edgar Scherick through his company Sports Programs, Inc. and produced by a young Roone Arledge which featured a different sporting event each broadcast. ABC purchased Sports Programs, Inc. in exchange for shares in the company, leading it to become the future core of ABC Sports, with Arledge as the executive producer of that division's shows. Wide World of Sports, in particular, was not merely devoted to a single sport, but rather to generally all sporting events.", "In May 2013, ABC launched \"WATCH ABC\", a revamp of its traditional multi-platform streaming services encompassing the network's existing streaming portal at ABC.com and a mobile app for smartphones and tablet computers; in addition to providing full-length episodes of ABC programs, the service allows live programming streams of local ABC affiliates in select markets (the first such offering by a U.S. broadcast network). Similar to sister network ESPN's WatchESPN service (which originated the \"WATCH\" brand used by the streaming services of Disney's television networks), live streams of ABC stations are only available to authenticated subscribers of participating pay television providers in certain markets. New York City O&amp;O WABC-TV and Philadelphia O&amp;O WPVI-TV were the first stations to offer streams of their programming on the service (with a free preview for non-subscribers through June 2013), with the six remaining ABC O&amp;Os offering streams by the start of the 2013–14 season. Hearst Television also reached a deal to offer streams of its ABC affiliates (including stations in Boston, Kansas City, Milwaukee and West Palm Beach) on the service.", "On June 16, 2007, ABC began to phase in a new imaging campaign for the upcoming 2007–08 season, \"Start Here\". Also developed by Troika, the on-air design was intended to emphasize the availability of ABC content across multiple platforms (in particular, using a system of icons representing different devices, such as television, computers and mobile devices), and \"simplify and bring a lot more consistency and continuity to the visual representation of ABC\". The ABC logo was also significantly redesigned as part of the transition, with a glossy \"ball\" effect that was specifically designed for HD. On-air, the logo was accompanied by animated water and ribbon effects. Red ribbons were used to represent the entertainment division, while blue ribbons were used for ABC News."]</t>
-        </is>
-      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -9475,21 +6550,6 @@
 run for about 4 × 1010 years, which is the same order of magnitude as the age of the universe. Even with a much faster computer, the program would only be useful for very small instances and in that sense the intractability of a problem is somewhat independent of technological progress. Nevertheless, a polynomial time algorithm is not always practical. If its running time is, say, n15, it is unreasonable to consider it efficient and it is still useless except on small instances.</t>
         </is>
       </c>
-      <c r="F196" t="inlineStr">
-        <is>
-          <t>[131, 199, 278, 533, 605]</t>
-        </is>
-      </c>
-      <c r="G196" t="inlineStr">
-        <is>
-          <t>[0.7973067760467529, 0.793759286403656, 0.79118812084198, 0.7823069095611572, 0.7796810269355774]</t>
-        </is>
-      </c>
-      <c r="H196" t="inlineStr">
-        <is>
-          <t>["A problem is regarded as inherently difficult if its solution requires significant resources, whatever the algorithm used. The theory formalizes this intuition, by introducing mathematical models of computation to study these problems and quantifying the amount of resources needed to solve them, such as time and storage. Other complexity measures are also used, such as the amount of communication (used in communication complexity), the number of gates in a circuit (used in circuit complexity) and the number of processors (used in parallel computing). One of the roles of computational complexity theory is to determine the practical limits on what computers can and cannot do.", "A Turing machine is a mathematical model of a general computing machine. It is a theoretical device that manipulates symbols contained on a strip of tape. Turing machines are not intended as a practical computing technology, but rather as a thought experiment representing a computing machine—anything from an advanced supercomputer to a mathematician with a pencil and paper. It is believed that if a problem can be solved by an algorithm, there exists a Turing machine that solves the problem. Indeed, this is the statement of the Church–Turing thesis. Furthermore, it is known that everything that can be computed on other models of computation known to us today, such as a RAM machine, Conway's Game of Life, cellular automata or any programming language can be computed on a Turing machine. Since Turing machines are easy to analyze mathematically, and are believed to be as powerful as any other model of computation, the Turing machine is the most commonly used model in complexity theory.", "However, some computational problems are easier to analyze in terms of more unusual resources. For example, a non-deterministic Turing machine is a computational model that is allowed to branch out to check many different possibilities at once. The non-deterministic Turing machine has very little to do with how we physically want to compute algorithms, but its branching exactly captures many of the mathematical models we want to analyze, so that non-deterministic time is a very important resource in analyzing computational problems.", "Analogous definitions can be made for space requirements. Although time and space are the most well-known complexity resources, any complexity measure can be viewed as a computational resource. Complexity measures are very generally defined by the Blum complexity axioms. Other complexity measures used in complexity theory include communication complexity, circuit complexity, and decision tree complexity.", "run for about 4 × 1010 years, which is the same order of magnitude as the age of the universe. Even with a much faster computer, the program would only be useful for very small instances and in that sense the intractability of a problem is somewhat independent of technological progress. Nevertheless, a polynomial time algorithm is not always practical. If its running time is, say, n15, it is unreasonable to consider it efficient and it is still useless except on small instances."]</t>
-        </is>
-      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -9521,21 +6581,6 @@
 Well represented in the collection is Meissen porcelain, from the first factory in Europe to discover the Chinese method of making porcelain. Among the finest examples are the Meissen Vulture from 1731 and the Möllendorff Dinner Service, designed in 1762 by Frederick II the Great. Ceramics from the Manufacture nationale de Sèvres are extensive, especially from the 18th and 19th centuries. The collection of 18th-century British porcelain is the largest and finest in the world. Examples from every factory are represented, the collections of Chelsea porcelain and Worcester Porcelain being especially fine. All the major 19th-century British factories are also represented. A major boost to the collections was the Salting Bequest made in 1909, which enriched the museum's stock of Chinese and Japanese ceramics. This bequest forms part of the finest collection of East Asian pottery and porcelain in the world, including Kakiemon ware.</t>
         </is>
       </c>
-      <c r="F197" t="inlineStr">
-        <is>
-          <t>[200, 632, 381, 5, 820]</t>
-        </is>
-      </c>
-      <c r="G197" t="inlineStr">
-        <is>
-          <t>[0.7578611969947815, 0.7386864423751831, 0.6895065903663635, 0.6887369751930237, 0.6849604249000549]</t>
-        </is>
-      </c>
-      <c r="H197" t="inlineStr">
-        <is>
-          <t>["The area of the modern city of Jacksonville has been inhabited for thousands of years. On Black Hammock Island in the national Timucuan Ecological and Historic Preserve, a University of North Florida team discovered some of the oldest remnants of pottery in the United States, dating to 2500 BC. In the 16th century, the beginning of the historical era, the region was inhabited by the Mocama, a coastal subgroup of the Timucua people. At the time of contact with Europeans, all Mocama villages in present-day Jacksonville were part of the powerful chiefdom known as the Saturiwa, centered around the mouth of the St. Johns River. One early map shows a village called Ossachite at the site of what is now downtown Jacksonville; this may be the earliest recorded name for that area.", "The smaller galleries cover Korea, the Himalayan kingdoms and South East Asia. Korean displays include green-glazed ceramics, silk embroideries from officials' robes and gleaming boxes inlaid with mother-of-pearl made between 500 AD and 2000. Himalayan items include important early Nepalese bronze sculptures, repoussé work and embroidery. Tibetan art from the 14th to the 19th century is represented by notable 14th- and 15th-century religious images in wood and bronze, scroll paintings and ritual objects. Art from Thailand, Burma, Cambodia, Indonesia and Sri Lanka in gold, silver, bronze, stone, terracotta and ivory represents these rich and complex cultures, the displays span the 6th to 19th centuries. Refined Hindu and Buddhist sculptures reflect the influence of India; items on show include betel-nut cutters, ivory combs and bronze palanquin hooks.", "Some modern scholars, such as Fielding H. Garrison, are of the opinion that the origin of the science of geology can be traced to Persia after the Muslim conquests had come to an end. Abu al-Rayhan al-Biruni (973–1048 CE) was one of the earliest Persian geologists, whose works included the earliest writings on the geology of India, hypothesizing that the Indian subcontinent was once a sea. Drawing from Greek and Indian scientific literature that were not destroyed by the Muslim conquests, the Persian scholar Ibn Sina (Avicenna, 981–1037) proposed detailed explanations for the formation of mountains, the origin of earthquakes, and other topics central to modern geology, which provided an essential foundation for the later development of the science. In China, the polymath Shen Kuo (1031–1095) formulated a hypothesis for the process of land formation: based on his observation of fossil animal shells in a geological stratum in a mountain hundreds of miles from the ocean, he inferred that the land was formed by erosion of the mountains and by deposition of silt.", "The first European to travel the length of the Amazon River was Francisco de Orellana in 1542. The BBC's Unnatural Histories presents evidence that Orellana, rather than exaggerating his claims as previously thought, was correct in his observations that a complex civilization was flourishing along the Amazon in the 1540s. It is believed that the civilization was later devastated by the spread of diseases from Europe, such as smallpox. Since the 1970s, numerous geoglyphs have been discovered on deforested land dating between AD 0–1250, furthering claims about Pre-Columbian civilizations. Ondemar Dias is accredited with first discovering the geoglyphs in 1977 and Alceu Ranzi with furthering their discovery after flying over Acre. The BBC's Unnatural Histories presented evidence that the Amazon rainforest, rather than being a pristine wilderness, has been shaped by man for at least 11,000 years through practices such as forest gardening and terra preta.", "Well represented in the collection is Meissen porcelain, from the first factory in Europe to discover the Chinese method of making porcelain. Among the finest examples are the Meissen Vulture from 1731 and the Möllendorff Dinner Service, designed in 1762 by Frederick II the Great. Ceramics from the Manufacture nationale de Sèvres are extensive, especially from the 18th and 19th centuries. The collection of 18th-century British porcelain is the largest and finest in the world. Examples from every factory are represented, the collections of Chelsea porcelain and Worcester Porcelain being especially fine. All the major 19th-century British factories are also represented. A major boost to the collections was the Salting Bequest made in 1909, which enriched the museum's stock of Chinese and Japanese ceramics. This bequest forms part of the finest collection of East Asian pottery and porcelain in the world, including Kakiemon ware."]</t>
-        </is>
-      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -9567,21 +6612,6 @@
 Following the Nice Treaty, there was an attempt to reform the constitutional law of the European Union and make it more transparent; this would have also produced a single constitutional document. However, as a result of the referendum in France and the referendum in the Netherlands, the 2004 Treaty establishing a Constitution for Europe never came into force. Instead, the Lisbon Treaty was enacted. Its substance was very similar to the proposed constitutional treaty, but it was formally an amending treaty, and – though it significantly altered the existing treaties – it did not completely replace them.</t>
         </is>
       </c>
-      <c r="F198" t="inlineStr">
-        <is>
-          <t>[201, 497, 227, 653, 641]</t>
-        </is>
-      </c>
-      <c r="G198" t="inlineStr">
-        <is>
-          <t>[0.8535206913948059, 0.7973272800445557, 0.7175992727279663, 0.7130218744277954, 0.6867468953132629]</t>
-        </is>
-      </c>
-      <c r="H198" t="inlineStr">
-        <is>
-          <t>["In December 2014, President Uhuru Kenyatta signed a Security Laws Amendment Bill, which supporters of the law suggested was necessary to guard against armed groups. Opposition politicians, human rights groups, and nine Western countries criticised the security bill, arguing that it infringed on democratic freedoms. The governments of the United States, Britain, Germany and France also collectively issued a press statement cautioning about the law's potential impact. Through the Jubillee Coalition, the Bill was later passed on 19 December in the National Assembly under acrimonious circumstances.", "A constitutional change was considered that would eliminate the position of Prime Minister and simultaneously reduce the powers of the President. A referendum to vote on the proposed constitution was held on 4 August 2010, and the new constitution passed by a wide margin. Among other things, the new constitution delegates more power to local governments and gives Kenyans a bill of rights. It was promulgated on 27 August 2010 at a euphoric ceremony in Nairobi's Uhuru Park, accompanied by a 21-gun salute. The event was attended by various African leaders and praised by the international community. As of that day, the new constitution heralding the Second Republic came into force.", "The first direct elections for native Kenyans to the Legislative Council took place in 1957. Despite British hopes of handing power to \"moderate\" local rivals, it was the Kenya African National Union (KANU) of Jomo Kenyatta that formed a government. The Colony of Kenya and the Protectorate of Kenya each came to an end on 12 December 1963 with independence being conferred on all of Kenya. The United Kingdom ceded sovereignty over the Colony of Kenya and, under an agreement dated 8 October 1963, the Sultan of Zanzibar agreed that simultaneous with independence for the Colony of Kenya, the Sultan would cease to have sovereignty over the Protectorate of Kenya so that all of Kenya would be one sovereign, independent state. In this way, Kenya became an independent country under the Kenya Independence Act 1963 of the United Kingdom. Exactly 12 months later on 12 December 1964, Kenya became a republic under the name \"Republic of Kenya\".", "Royal assent: After the bill has been passed, the Presiding Officer submits it to the Monarch for royal assent and it becomes an Act of the Scottish Parliament. However he cannot do so until a 4-week period has elapsed, during which the Law Officers of the Scottish Government or UK Government can refer the bill to the Supreme Court of the United Kingdom for a ruling on whether it is within the powers of the Parliament. Acts of the Scottish Parliament do not begin with a conventional enacting formula. Instead they begin with a phrase that reads: \"The Bill for this Act of the Scottish Parliament was passed by the Parliament on [Date] and received royal assent on [Date]\".", "Following the Nice Treaty, there was an attempt to reform the constitutional law of the European Union and make it more transparent; this would have also produced a single constitutional document. However, as a result of the referendum in France and the referendum in the Netherlands, the 2004 Treaty establishing a Constitution for Europe never came into force. Instead, the Lisbon Treaty was enacted. Its substance was very similar to the proposed constitutional treaty, but it was formally an amending treaty, and – though it significantly altered the existing treaties – it did not completely replace them."]</t>
-        </is>
-      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -9611,21 +6641,6 @@
 The hydrography of the current delta is characterized by the delta's main arms, disconnected arms (Hollandse IJssel, Linge, Vecht, etc.) and smaller rivers and streams. Many rivers have been closed ("dammed") and now serve as drainage channels for the numerous polders. The construction of Delta Works changed the Delta in the second half of the 20th Century fundamentally. Currently Rhine water runs into the sea, or into former marine bays now separated from the sea, in five places, namely at the mouths of the Nieuwe Merwede, Nieuwe Waterway (Nieuwe Maas), Dordtse Kil, Spui and IJssel.
 When Céloron's expedition arrived at Logstown, the Native Americans in the area informed Céloron that they owned the Ohio Country and that they would trade with the British regardless of the French. Céloron continued south until his expedition reached the confluence of the Ohio and the Miami rivers, which lay just south of the village of Pickawillany, the home of the Miami chief known as "Old Briton". Céloron threatened "Old Briton" with severe consequences if he continued to trade with the British. "Old Briton" ignored the warning. Disappointed, Céloron returned to Montreal in November 1749.
 The shape of the Rhine delta is determined by two bifurcations: first, at Millingen aan de Rijn, the Rhine splits into Waal and Pannerdens Kanaal, which changes its name to Nederrijn at Angeren, and second near Arnhem, the IJssel branches off from the Nederrijn. This creates three main flows, two of which change names rather often. The largest and southern main branch begins as Waal and continues as Boven Merwede ("Upper Merwede"), Beneden Merwede ("Lower Merwede"), Noord River ("North River"), Nieuwe Maas ("New Meuse"), Het Scheur ("the Rip") and Nieuwe Waterweg ("New Waterway"). The middle flow begins as Nederrijn, then changes into Lek, then joins the Noord, thereby forming Nieuwe Maas. The northern flow keeps the name IJssel until it flows into Lake IJsselmeer. Three more flows carry significant amounts of water: the Nieuwe Merwede ("New Merwede"), which branches off from the southern branch where it changes from Boven to Beneden Merwede; the Oude Maas ("Old Meuse"), which branches off from the southern branch where it changes from Beneden Merwede into Noord, and Dordtse Kil, which branches off from Oude Maas.</t>
-        </is>
-      </c>
-      <c r="F199" t="inlineStr">
-        <is>
-          <t>[612, 747, 68, 709, 661]</t>
-        </is>
-      </c>
-      <c r="G199" t="inlineStr">
-        <is>
-          <t>[0.7576587200164795, 0.7548879384994507, 0.7431272864341736, 0.7398473024368286, 0.7355209589004517]</t>
-        </is>
-      </c>
-      <c r="H199" t="inlineStr">
-        <is>
-          <t>["The name Rijn, from here on, is used only for smaller streams farther to the north, which together formed the main river Rhine in Roman times. Though they retained the name, these streams no longer carry water from the Rhine, but are used for draining the surrounding land and polders. From Wijk bij Duurstede, the old north branch of the Rhine is called Kromme Rijn (\"Bent Rhine\") past Utrecht, first Leidse Rijn (\"Rhine of Leiden\") and then, Oude Rijn (\"Old Rhine\"). The latter flows west into a sluice at Katwijk, where its waters can be discharged into the North Sea. This branch once formed the line along which the Limes Germanicus were built. During periods of lower sea levels within the various ice ages, the Rhine took a left turn, creating the Channel River, the course of which now lies below the English Channel.", "The mouth of the Rhine into Lake Constance forms an inland delta. The delta is delimited in the West by the Alter Rhein (\"Old Rhine\") and in the East by a modern canalized section. Most of the delta is a nature reserve and bird sanctuary. It includes the Austrian towns of Gaißau, Höchst and Fußach. The natural Rhine originally branched into at least two arms and formed small islands by precipitating sediments. In the local Alemannic dialect, the singular is pronounced \"Isel\" and this is also the local pronunciation of Esel (\"Donkey\"). Many local fields have an official name containing this element.", "The hydrography of the current delta is characterized by the delta's main arms, disconnected arms (Hollandse IJssel, Linge, Vecht, etc.) and smaller rivers and streams. Many rivers have been closed (\"dammed\") and now serve as drainage channels for the numerous polders. The construction of Delta Works changed the Delta in the second half of the 20th Century fundamentally. Currently Rhine water runs into the sea, or into former marine bays now separated from the sea, in five places, namely at the mouths of the Nieuwe Merwede, Nieuwe Waterway (Nieuwe Maas), Dordtse Kil, Spui and IJssel.", "When Céloron's expedition arrived at Logstown, the Native Americans in the area informed Céloron that they owned the Ohio Country and that they would trade with the British regardless of the French. Céloron continued south until his expedition reached the confluence of the Ohio and the Miami rivers, which lay just south of the village of Pickawillany, the home of the Miami chief known as \"Old Briton\". Céloron threatened \"Old Briton\" with severe consequences if he continued to trade with the British. \"Old Briton\" ignored the warning. Disappointed, Céloron returned to Montreal in November 1749.", "The shape of the Rhine delta is determined by two bifurcations: first, at Millingen aan de Rijn, the Rhine splits into Waal and Pannerdens Kanaal, which changes its name to Nederrijn at Angeren, and second near Arnhem, the IJssel branches off from the Nederrijn. This creates three main flows, two of which change names rather often. The largest and southern main branch begins as Waal and continues as Boven Merwede (\"Upper Merwede\"), Beneden Merwede (\"Lower Merwede\"), Noord River (\"North River\"), Nieuwe Maas (\"New Meuse\"), Het Scheur (\"the Rip\") and Nieuwe Waterweg (\"New Waterway\"). The middle flow begins as Nederrijn, then changes into Lek, then joins the Noord, thereby forming Nieuwe Maas. The northern flow keeps the name IJssel until it flows into Lake IJsselmeer. Three more flows carry significant amounts of water: the Nieuwe Merwede (\"New Merwede\"), which branches off from the southern branch where it changes from Boven to Beneden Merwede; the Oude Maas (\"Old Meuse\"), which branches off from the southern branch where it changes from Beneden Merwede into Noord, and Dordtse Kil, which branches off from Oude Maas."]</t>
         </is>
       </c>
     </row>
@@ -9674,21 +6689,6 @@
 2 from the air is the essential purpose of respiration, so oxygen supplementation is used in medicine. Treatment not only increases oxygen levels in the patient's blood, but has the secondary effect of decreasing resistance to blood flow in many types of diseased lungs, easing work load on the heart. Oxygen therapy is used to treat emphysema, pneumonia, some heart disorders (congestive heart failure), some disorders that cause increased pulmonary artery pressure, and any disease that impairs the body's ability to take up and use gaseous oxygen.</t>
         </is>
       </c>
-      <c r="F200" t="inlineStr">
-        <is>
-          <t>[203, 0, 86, 710, 10]</t>
-        </is>
-      </c>
-      <c r="G200" t="inlineStr">
-        <is>
-          <t>[0.8409153819084167, 0.8173686861991882, 0.8017300963401794, 0.7868973016738892, 0.7856730222702026]</t>
-        </is>
-      </c>
-      <c r="H200" t="inlineStr">
-        <is>
-          <t>["Breathing pure O\n2 in space applications, such as in some modern space suits, or in early spacecraft such as Apollo, causes no damage due to the low total pressures used. In the case of spacesuits, the O\n2 partial pressure in the breathing gas is, in general, about 30 kPa (1.4 times normal), and the resulting O\n2 partial pressure in the astronaut's arterial blood is only marginally more than normal sea-level O\n2 partial pressure (for more information on this, see space suit and arterial blood gas).", "Hyperbaric (high-pressure) medicine uses special oxygen chambers to increase the partial pressure of O\n2 around the patient and, when needed, the medical staff. Carbon monoxide poisoning, gas gangrene, and decompression sickness (the 'bends') are sometimes treated using these devices. Increased O\n2 concentration in the lungs helps to displace carbon monoxide from the heme group of hemoglobin. Oxygen gas is poisonous to the anaerobic bacteria that cause gas gangrene, so increasing its partial pressure helps kill them. Decompression sickness occurs in divers who decompress too quickly after a dive, resulting in bubbles of inert gas, mostly nitrogen and helium, forming in their blood. Increasing the pressure of O\n2 as soon as possible is part of the treatment.", "Oxygen toxicity to the lungs and central nervous system can also occur in deep scuba diving and surface supplied diving. Prolonged breathing of an air mixture with an O\n2 partial pressure more than 60 kPa can eventually lead to permanent pulmonary fibrosis. Exposure to a O\n2 partial pressures greater than 160 kPa (about 1.6 atm) may lead to convulsions (normally fatal for divers). Acute oxygen toxicity (causing seizures, its most feared effect for divers) can occur by breathing an air mixture with 21% O\n2 at 66 m or more of depth; the same thing can occur by breathing 100% O\n2 at only 6 m.", "Oxygen gas (O\n2) can be toxic at elevated partial pressures, leading to convulsions and other health problems.[j] Oxygen toxicity usually begins to occur at partial pressures more than 50 kilopascals (kPa), equal to about 50% oxygen composition at standard pressure or 2.5 times the normal sea-level O\n2 partial pressure of about 21 kPa. This is not a problem except for patients on mechanical ventilators, since gas supplied through oxygen masks in medical applications is typically composed of only 30%–50% O\n2 by volume (about 30 kPa at standard pressure). (although this figure also is subject to wide variation, depending on type of mask).", "Uptake of O\n2 from the air is the essential purpose of respiration, so oxygen supplementation is used in medicine. Treatment not only increases oxygen levels in the patient's blood, but has the secondary effect of decreasing resistance to blood flow in many types of diseased lungs, easing work load on the heart. Oxygen therapy is used to treat emphysema, pneumonia, some heart disorders (congestive heart failure), some disorders that cause increased pulmonary artery pressure, and any disease that impairs the body's ability to take up and use gaseous oxygen."]</t>
-        </is>
-      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -9720,21 +6720,6 @@
 In the Philippines, the private sector has been a major provider of educational services, accounting for about 7.5% of primary enrollment, 32% of secondary enrollment and about 80% of tertiary enrollment. Private schools have proven to be efficient in resource utilization. Per unit costs in private schools are generally lower when compared to public schools. This situation is more evident at the tertiary level. Government regulations have given private education more flexibility and autonomy in recent years, notably by lifting the moratorium on applications for new courses, new schools and conversions, by liberalizing tuition fee policy for private schools, by replacing values education for third and fourth years with English, mathematics and natural science at the option of the school, and by issuing the revised Manual of Regulations for Private Schools in August 1992.</t>
         </is>
       </c>
-      <c r="F201" t="inlineStr">
-        <is>
-          <t>[219, 390, 207, 589, 204]</t>
-        </is>
-      </c>
-      <c r="G201" t="inlineStr">
-        <is>
-          <t>[0.7287606000900269, 0.7183837890625, 0.7175068855285645, 0.7121680378913879, 0.7092983722686768]</t>
-        </is>
-      </c>
-      <c r="H201" t="inlineStr">
-        <is>
-          <t>["Decisions in-between the four-year meetings are made by the Mission Council (usually consisting of church bishops). One of the most high profile decisions in recent years by one of the councils was a decision by the Mission Council of the South Central Jurisdiction which in March 2007 approved a 99-year lease of 36 acres (150,000 m2) at Southern Methodist University for the George W. Bush Presidential Library. The decision generated controversy in light of Bush's support of the Iraq War which the church bishops have criticized. A debate over whether the decision should or could be submitted for approval by the Southern Jurisdictional Conference at its July 2008 meeting in Dallas, Texas, remains unresolved.", "less than 700 preparations, their properties, modes of action, and their indications. He devoted in fact a whole volume to simple drugs in The Canon of Medicine. Of great impact were also the works by al-Maridini of Baghdad and Cairo, and Ibn al-Wafid (1008–1074), both of which were printed in Latin more than fifty times, appearing as De Medicinis universalibus et particularibus by 'Mesue' the younger, and the Medicamentis simplicibus by 'Abenguefit'. Peter of Abano (1250–1316) translated and added a supplement to the work of al-Maridini under the title De Veneris. Al-Muwaffaq’s contributions in the field are also pioneering. Living in the 10th century, he wrote The foundations of the true properties of Remedies, amongst others describing arsenious oxide, and being acquainted with silicic acid. He made clear distinction between sodium carbonate and potassium carbonate, and drew attention to the poisonous nature of copper compounds, especially copper vitriol, and also lead compounds. He also describes the distillation of sea-water for drinking.[verification needed]", "In the final years of the apartheid era, parents at white government schools were given the option to convert to a \"semi-private\" form called Model C, and many of these schools changed their admissions policies to accept children of other races. Following the transition to democracy, the legal form of \"Model C\" was abolished, however, the term continues to be used to describe government schools formerly reserved for white children.. These schools tend to produce better academic results than government schools formerly reserved for other race groups . Former \"Model C\" schools are not private schools, as they are state-controlled. All schools in South Africa (including both independent schools and public schools) have the right to set compulsory school fees, and formerly model C schools tend to set much higher school fees than other public schools.", "In the United States especially, several high-profile cases such as Debra LaFave, Pamela Rogers, and Mary Kay Letourneau have caused increased scrutiny on teacher misconduct.", "In the Philippines, the private sector has been a major provider of educational services, accounting for about 7.5% of primary enrollment, 32% of secondary enrollment and about 80% of tertiary enrollment. Private schools have proven to be efficient in resource utilization. Per unit costs in private schools are generally lower when compared to public schools. This situation is more evident at the tertiary level. Government regulations have given private education more flexibility and autonomy in recent years, notably by lifting the moratorium on applications for new courses, new schools and conversions, by liberalizing tuition fee policy for private schools, by replacing values education for third and fourth years with English, mathematics and natural science at the option of the school, and by issuing the revised Manual of Regulations for Private Schools in August 1992."]</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>